<commit_message>
smib_build: REEC_D option, hybrid plant controller, 100 MW PV + 100 MW BESS template
- Generators, Electrical control: REEC_A (REECA1), REEC_C (REECCU1), REEC_D
  (REECDU1, USRMDL 102 0 6 77 7 20) per inverter generator.
- Plant, Plant controller: REPC_A (REPCA1 per generator) or REPC_B (one
  PLNTBU1 USRBUS record at the POI, a REAX4BU1 on each generator taking its
  share of the plant's Q and P), laid out as in a hybrid PV + BESS .dyr.
- Plant, REGC_A / REPC_A records: standard REGCA1 / REPCA1 (default) or
  USRMDL REGCAU1 / REPCAU1.
- Dyr_Params: PLANT for the plant controller; ICONn / CONn by position.
- The template is a hybrid plant: 100 MW PV and 100 MW BESS on one
  230/34.5 kV MPT, five feeders each, REPC_B.
- JSON input skips # rows like the workbook; a second run in the same
  second gets a folder of its own; --template never overwrites.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BGsNUhFmVX23f8qnP53zUv
</commit_message>
<xml_diff>
--- a/smib/SMIB_INPUT_TEMPLATE.xlsx
+++ b/smib/SMIB_INPUT_TEMPLATE.xlsx
@@ -157,7 +157,7 @@
       </c>
       <c r="B6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bases, the POI, the grid (SCR and X/R, or short-circuit MVA, or R/X), the gen-tie, the operating point and the PSCAD run settings.</t>
+          <t xml:space="preserve">Bases, the POI, the grid (SCR and X/R, or short-circuit MVA, or R/X), the gen-tie, the operating point, the plant controller and the PSCAD run settings.</t>
         </is>
       </c>
     </row>
@@ -170,120 +170,128 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MPT</t>
-        </is>
-      </c>
+      <c r="A8" s="4"/>
       <c r="B8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">One row per main power transformer; HV winding first. Three windings: TV kV, the three impedances and their bases. Parallel units: identical units in parallel. Tie: a line of its own from HV to it.</t>
+          <t xml:space="preserve">Plant controller (PSS/E .dyr): REPC_A = a REPCA1 on each generator, each holding the POI; REPC_B = one controller for the whole plant (hybrid PV + BESS): PLNTBU1 at the POI, and on each generator a REAX4BU1 that takes its share of the plant's Q (Qmax / sum of Qmax) and P (Pmax / sum of Pmax). REGC_A / REPC_A records: standard = REGCA1 / REPCA1 from the PSS/E library; USRMDL = REGCAU1 / REPCAU1.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Generators</t>
+          <t xml:space="preserve">MPT</t>
         </is>
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">One row per generator (PV, BESS, wind, synchronous ...): the units (count and one unit's data; the model is their aggregate), its GSU (one GSU's data and the count), its collector (FEEDERS: the WECC equivalent of its rows in Feeders; EQUIVALENT: R X B given; NONE), how it shares the POI's Q, and its PSCAD model (vendor library and definition, or blank for a voltage source at the solved terminal voltage: a network check against PSS/E).</t>
+          <t xml:space="preserve">One row per main power transformer; HV winding first. Three windings: TV kV, the three impedances and their bases. Parallel units: identical units in parallel. Tie: a line of its own from HV to it.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Feeders</t>
+          <t xml:space="preserve">Generators</t>
         </is>
       </c>
       <c r="B10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">The collector feeders section by section from the collector bus out: cable, length and the units tapped at the section's far end. A daisy chain needs no From section; a lateral names the section it leaves from (its far end); 0 = straight from the collector bus. Copies: identical feeders. WECC equivalent: Zeq = sum(Zi Wi^2) / W^2, Beq = sum(Bi), Wi = MW of the units downstream of section i.</t>
+          <t xml:space="preserve">One row per generator (PV, BESS, wind, synchronous ...): the units (count and one unit's data; the model is their aggregate), its GSU (one GSU's data and the count), its collector (FEEDERS: the WECC equivalent of its rows in Feeders; EQUIVALENT: R X B given; NONE), how it shares the POI's Q, its electrical control model in the .dyr (REEC_A: REECA1, PV and wind; REEC_C: REECCU1, BESS; REEC_D: REECDU1, PV, BESS and WT4) and its PSCAD model (vendor library and definition, or blank for a voltage source at the solved terminal voltage: a network check against PSS/E).</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cables</t>
+          <t xml:space="preserve">Feeders</t>
         </is>
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cable data per length (R, X in ohm; C in uF or B in uS) and the length unit they are per.</t>
+          <t xml:space="preserve">The collector feeders section by section from the collector bus out: cable, length and the units tapped at the section's far end. A daisy chain needs no From section; a lateral names the section it leaves from (its far end); 0 = straight from the collector bus. Copies: identical feeders. WECC equivalent: Zeq = sum(Zi Wi^2) / W^2, Beq = sum(Bi), Wi = MW of the units downstream of section i.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Collectors</t>
+          <t xml:space="preserve">Cables</t>
         </is>
       </c>
       <c r="B12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Collector systems shared by more than one generator: name and the bus it starts from. Their Feeders rows say whose units each section carries (Units of); the generators on it Connect to its name.</t>
+          <t xml:space="preserve">Cable data per length (R, X in ohm; C in uF or B in uS) and the length unit they are per.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Loads_Shunts</t>
+          <t xml:space="preserve">Collectors</t>
         </is>
       </c>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Auxiliary loads (constant impedance, MW and MVAr at 1 pu) and shunts (MVAr at 1 pu: + capacitor, - reactor) on any bus.</t>
+          <t xml:space="preserve">Collector systems shared by more than one generator: name and the bus it starts from. Their Feeders rows say whose units each section carries (Units of); the generators on it Connect to its name.</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bus_Numbers</t>
+          <t xml:space="preserve">Loads_Shunts</t>
         </is>
       </c>
       <c r="B14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bus numbers or names of your own, by role (the report lists every role and its number).</t>
+          <t xml:space="preserve">Auxiliary loads (constant impedance, MW and MVAr at 1 pu) and shunts (MVAr at 1 pu: + capacitor, - reactor) on any bus.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dyr_Params</t>
+          <t xml:space="preserve">Bus_Numbers</t>
         </is>
       </c>
       <c r="B15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Any parameter of the WECC-approved generic models, by generator, model and PSS/E name (IB for the infinite bus). PV and WT4: REGCA1 + REECA1 + REPCA1 (REGC_A, REEC_A, REPC_A); BESS: REGCAU1 + REECCU1 + REPCAU1 (REGC_A, REEC_C, REPC_A -- USRMDL records: the WECC user-model DLL must be loaded, ADDLIB_IDV / DLLS in the script); WT3: + WTDTA1 WTARA1 WTPTA1 WTTQA1; SYNC: GENROU SEXS TGOV1. The report lists every model's parameters with the values used.</t>
+          <t xml:space="preserve">Bus numbers or names of your own, by role (the report lists every role and its number).</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dyr_Records</t>
+          <t xml:space="preserve">Dyr_Params</t>
         </is>
       </c>
       <c r="B16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Records of your own (vendor or user models), one per row, ending in /. {BUS} {ID} {MBASE} {POI} {IB} {HV} {MV} and {&lt;bus role&gt;} are filled in. Type USER generators have only these. Models in user DLLs: list the DLLs in DLLS in the script for the PSS/E check.</t>
+          <t xml:space="preserve">Any parameter of the WECC-approved generic models, by generator, model and PSS/E name or position (ICON2, CON14) -- IB for the infinite bus, PLANT for the plant controller. Inverters: REGCA1 (REGC_A) + REECA1 / REECCU1 / REECDU1 (REEC_A / C / D) + REPCA1 (REPC_A) or REAX4BU1 (with PLNTBU1, REPC_B); WT3: + WTDTA1 WTARA1 WTPTA1 WTTQA1; SYNC: GENROU SEXS TGOV1. REECCU1, REECDU1, PLNTBU1, REAX4BU1 (and REGCAU1, REPCAU1) are user models: the WECC user-model DLL must be loaded for the PSS/E check (ADDLIB_IDV / DLLS in the script). The report lists every model's parameters with the values used.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
+          <t xml:space="preserve">Dyr_Records</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Records of your own (vendor or user models), one per row, ending in /. {BUS} {ID} {MBASE} {POI} {IB} {HV} {MV} and {&lt;bus role&gt;} are filled in. Type USER generators have only these. Models in user DLLs: list the DLLs in DLLS in the script for the PSS/E check.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">PSCAD_Params</t>
         </is>
       </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="B18" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Parameters of each generator's vendor PSCAD model, as PSCAD takes them.</t>
         </is>
@@ -327,17 +335,17 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"># IB for the infinite bus</t>
+          <t xml:space="preserve"># IB: the infinite bus | PLANT: the plant controller (REPC_B)</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PV/WT4: REGCA1 REECA1 REPCA1 | BESS: REGCAU1 REECCU1 REPCAU1 | WT3: + WTDTA1 WTARA1 WTPTA1 WTTQA1 | SYNC: GENROU SEXS TGOV1 | IB: GENCLS</t>
+          <t xml:space="preserve">REGCA1 (REGCAU1) | REECA1 REECCU1 REECDU1 | REPCA1 (REPCAU1) or REAX4BU1 | PLANT: PLNTBU1 | WT3: + WTDTA1 WTARA1 WTPTA1 WTTQA1 | SYNC: GENROU SEXS TGOV1 | IB: GENCLS</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E name (the report lists them all)</t>
+          <t xml:space="preserve">PSS/E name (the report lists them all) or position: ICON2, CON14</t>
         </is>
       </c>
       <c r="D2" s="2"/>
@@ -345,12 +353,12 @@
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">PV</t>
+          <t xml:space="preserve">PLANT</t>
         </is>
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">REPCA1</t>
+          <t xml:space="preserve">PLNTBU1</t>
         </is>
       </c>
       <c r="C3" s="3" t="inlineStr">
@@ -360,6 +368,26 @@
       </c>
       <c r="D3" s="3">
         <v>1.0</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BESS</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REECCU1</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">SOCini</t>
+        </is>
+      </c>
+      <c r="D4" s="3">
+        <v>0.5</v>
       </c>
     </row>
   </sheetData>
@@ -468,7 +496,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">40</t>
+          <t xml:space="preserve">25</t>
         </is>
       </c>
     </row>
@@ -515,7 +543,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Example_PV_BESS</t>
+          <t xml:space="preserve">Hybrid_PV100_BESS100</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -586,7 +614,7 @@
         </is>
       </c>
       <c r="B6" s="3">
-        <v>345.0</v>
+        <v>230.0</v>
       </c>
       <c r="C6" s="0" t="inlineStr">
         <is>
@@ -717,7 +745,7 @@
         </is>
       </c>
       <c r="B14" s="3">
-        <v>8.0</v>
+        <v>5.0</v>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
@@ -749,7 +777,7 @@
         </is>
       </c>
       <c r="B16" s="3">
-        <v>0.0287</v>
+        <v>0.072</v>
       </c>
       <c r="C16" s="0" t="inlineStr">
         <is>
@@ -769,7 +797,7 @@
         </is>
       </c>
       <c r="B17" s="3">
-        <v>0.37</v>
+        <v>0.495</v>
       </c>
       <c r="C17" s="0" t="inlineStr">
         <is>
@@ -789,7 +817,7 @@
         </is>
       </c>
       <c r="B18" s="3">
-        <v>4.4</v>
+        <v>3.35</v>
       </c>
       <c r="C18" s="0" t="inlineStr">
         <is>
@@ -888,7 +916,7 @@
         </is>
       </c>
       <c r="B24" s="3">
-        <v>600.0</v>
+        <v>400.0</v>
       </c>
       <c r="C24" s="0" t="inlineStr">
         <is>
@@ -1014,51 +1042,45 @@
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSCAD time step</t>
-        </is>
-      </c>
-      <c r="B31" s="3">
-        <v>10.0</v>
-      </c>
-      <c r="C31" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">us</t>
+          <t xml:space="preserve">Plant controller</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REPC_B</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">blank = 10 (the vendor model's own requirement wins)</t>
+          <t xml:space="preserve">PSS/E .dyr -- REPC_A: a REPCA1 on each generator | REPC_B: one for the plant, PLNTBU1 at the POI and a REAX4BU1 on each generator (hybrid plants) (blank = REPC_A)</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSCAD duration</t>
-        </is>
-      </c>
-      <c r="B32" s="3">
-        <v>5.0</v>
-      </c>
-      <c r="C32" s="0" t="inlineStr">
-        <is>
-          <t xml:space="preserve">s</t>
+          <t xml:space="preserve">REGC_A / REPC_A records</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">standard</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">blank = 5</t>
+          <t xml:space="preserve">standard: REGCA1 / REPCA1 (PSS/E library) | USRMDL: REGCAU1 / REPCAU1 (the WECC user-model DLL) (blank = standard)</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSCAD plot step</t>
+          <t xml:space="preserve">PSCAD time step</t>
         </is>
       </c>
       <c r="B33" s="3">
-        <v>100.0</v>
+        <v>10.0</v>
       </c>
       <c r="C33" s="0" t="inlineStr">
         <is>
@@ -1067,49 +1089,95 @@
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">blank = 100</t>
+          <t xml:space="preserve">blank = 10 (the vendor model's own requirement wins)</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSCAD meter at POI</t>
-        </is>
-      </c>
-      <c r="B34" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">YES</t>
+          <t xml:space="preserve">PSCAD duration</t>
+        </is>
+      </c>
+      <c r="B34" s="3">
+        <v>5.0</v>
+      </c>
+      <c r="C34" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">s</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">YES = a multimeter between the grid and the POI</t>
+          <t xml:space="preserve">blank = 5</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
+          <t xml:space="preserve">PSCAD plot step</t>
+        </is>
+      </c>
+      <c r="B35" s="3">
+        <v>100.0</v>
+      </c>
+      <c r="C35" s="0" t="inlineStr">
+        <is>
+          <t xml:space="preserve">us</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">blank = 100</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD meter at POI</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES</t>
+        </is>
+      </c>
+      <c r="D36" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">YES = a multimeter between the grid and the POI</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="4" t="inlineStr">
+        <is>
           <t xml:space="preserve">PSCAD libraries</t>
         </is>
       </c>
-      <c r="B35" s="3"/>
-      <c r="D35" s="2" t="inlineStr">
+      <c r="B37" s="3"/>
+      <c r="D37" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">user-model libraries (.pslx) to load, separated by ;</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="3">
+  <dataValidations count="5">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B15">
       <formula1>"km,mi,kft,m,ft"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B25">
       <formula1>"Q,PF,V"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B34">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B31">
+      <formula1>"REPC_A,REPC_B"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B32">
+      <formula1>"standard,USRMDL"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B36">
       <formula1>"YES,NO"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1413,19 +1481,19 @@
         </is>
       </c>
       <c r="B3" s="3">
-        <v>345.0</v>
+        <v>230.0</v>
       </c>
       <c r="C3" s="3">
         <v>34.5</v>
       </c>
       <c r="D3" s="3"/>
       <c r="E3" s="3">
-        <v>280.0</v>
+        <v>225.0</v>
       </c>
       <c r="F3" s="3"/>
       <c r="G3" s="3"/>
       <c r="H3" s="3">
-        <v>12.0</v>
+        <v>10.0</v>
       </c>
       <c r="I3" s="3"/>
       <c r="J3" s="3"/>
@@ -1433,7 +1501,7 @@
       <c r="L3" s="3"/>
       <c r="M3" s="3"/>
       <c r="N3" s="3">
-        <v>50.0</v>
+        <v>45.0</v>
       </c>
       <c r="O3" s="3"/>
       <c r="P3" s="3" t="inlineStr">
@@ -1450,7 +1518,7 @@
       <c r="S3" s="3"/>
       <c r="T3" s="3"/>
       <c r="U3" s="3">
-        <v>280.0</v>
+        <v>225.0</v>
       </c>
       <c r="V3" s="3"/>
       <c r="W3" s="3"/>
@@ -1502,9 +1570,10 @@
     <col min="29" max="29" width="8" customWidth="1"/>
     <col min="30" max="30" width="8" customWidth="1"/>
     <col min="31" max="31" width="6" customWidth="1"/>
-    <col min="32" max="32" width="18" customWidth="1"/>
-    <col min="33" max="33" width="16" customWidth="1"/>
-    <col min="34" max="34" width="9" customWidth="1"/>
+    <col min="32" max="32" width="9" customWidth="1"/>
+    <col min="33" max="33" width="18" customWidth="1"/>
+    <col min="34" max="34" width="16" customWidth="1"/>
+    <col min="35" max="35" width="9" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1665,15 +1734,20 @@
       </c>
       <c r="AF1" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">Electrical control</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">PSCAD library</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AH1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">PSCAD definition</t>
         </is>
       </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">PSCAD AC port</t>
         </is>
@@ -1817,15 +1891,20 @@
       </c>
       <c r="AF2" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">PSS/E .dyr -- REEC_A: PV, WT | REEC_C: BESS | REEC_D: PV, BESS, WT4 (blank = REEC_A, BESS REEC_C)</t>
+        </is>
+      </c>
+      <c r="AG2" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">vendor library .pslx (blank = none)</t>
         </is>
       </c>
-      <c r="AG2" s="2" t="inlineStr">
+      <c r="AH2" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">vendor model, library:name (blank = a source: network check)</t>
         </is>
       </c>
-      <c r="AH2" s="2" t="inlineStr">
+      <c r="AI2" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">its AC port (blank = its 3-phase port)</t>
         </is>
@@ -1853,7 +1932,7 @@
         </is>
       </c>
       <c r="E3" s="3">
-        <v>40</v>
+        <v>25</v>
       </c>
       <c r="F3" s="3">
         <v>4.2</v>
@@ -1915,9 +1994,14 @@
       <c r="AC3" s="3"/>
       <c r="AD3" s="3"/>
       <c r="AE3" s="3"/>
-      <c r="AF3" s="3"/>
+      <c r="AF3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REEC_A</t>
+        </is>
+      </c>
       <c r="AG3" s="3"/>
       <c r="AH3" s="3"/>
+      <c r="AI3" s="3"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -1944,19 +2028,19 @@
         <v>25</v>
       </c>
       <c r="F4" s="3">
+        <v>4.4</v>
+      </c>
+      <c r="G4" s="3">
         <v>4.0</v>
       </c>
-      <c r="G4" s="3">
-        <v>3.6</v>
-      </c>
       <c r="H4" s="3">
-        <v>-3.6</v>
+        <v>-4.0</v>
       </c>
       <c r="I4" s="3">
-        <v>1.74</v>
+        <v>1.83</v>
       </c>
       <c r="J4" s="3">
-        <v>-1.74</v>
+        <v>-1.83</v>
       </c>
       <c r="K4" s="3"/>
       <c r="L4" s="3">
@@ -1972,7 +2056,7 @@
       <c r="P4" s="3"/>
       <c r="Q4" s="3"/>
       <c r="R4" s="3">
-        <v>4.0</v>
+        <v>4.4</v>
       </c>
       <c r="S4" s="3">
         <v>34.5</v>
@@ -1994,31 +2078,26 @@
       <c r="X4" s="3"/>
       <c r="Y4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">EQUIVALENT</t>
-        </is>
-      </c>
-      <c r="Z4" s="3">
-        <v>0.004</v>
-      </c>
-      <c r="AA4" s="3">
-        <v>0.003</v>
-      </c>
-      <c r="AB4" s="3">
-        <v>0.015</v>
-      </c>
-      <c r="AC4" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">pu</t>
-        </is>
-      </c>
+          <t xml:space="preserve">FEEDERS</t>
+        </is>
+      </c>
+      <c r="Z4" s="3"/>
+      <c r="AA4" s="3"/>
+      <c r="AB4" s="3"/>
+      <c r="AC4" s="3"/>
       <c r="AD4" s="3"/>
       <c r="AE4" s="3"/>
-      <c r="AF4" s="3"/>
+      <c r="AF4" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REEC_C</t>
+        </is>
+      </c>
       <c r="AG4" s="3"/>
       <c r="AH4" s="3"/>
+      <c r="AI4" s="3"/>
     </row>
   </sheetData>
-  <dataValidations count="4">
+  <dataValidations count="5">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B3:B500">
       <formula1>"PV,BESS,WT4,WT3,SYNC,USER"</formula1>
     </dataValidation>
@@ -2030,6 +2109,9 @@
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="AC3:AC500">
       <formula1>"pu,ohm"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="AF3:AF500">
+      <formula1>"REEC_A,REEC_C,REEC_D"</formula1>
     </dataValidation>
   </dataValidations>
 </worksheet>
@@ -2173,7 +2255,7 @@
         </is>
       </c>
       <c r="C3" s="3">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D3" s="3">
         <v>1</v>
@@ -2185,7 +2267,7 @@
         </is>
       </c>
       <c r="G3" s="3">
-        <v>2.0</v>
+        <v>1.6</v>
       </c>
       <c r="H3" s="3" t="inlineStr">
         <is>
@@ -2210,7 +2292,7 @@
         </is>
       </c>
       <c r="C4" s="3">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D4" s="3">
         <v>2</v>
@@ -2222,7 +2304,7 @@
         </is>
       </c>
       <c r="G4" s="3">
-        <v>0.35</v>
+        <v>0.4</v>
       </c>
       <c r="H4" s="3" t="inlineStr">
         <is>
@@ -2230,7 +2312,7 @@
         </is>
       </c>
       <c r="I4" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J4" s="3"/>
       <c r="K4" s="3"/>
@@ -2247,7 +2329,7 @@
         </is>
       </c>
       <c r="C5" s="3">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D5" s="3">
         <v>3</v>
@@ -2259,7 +2341,7 @@
         </is>
       </c>
       <c r="G5" s="3">
-        <v>0.35</v>
+        <v>0.4</v>
       </c>
       <c r="H5" s="3" t="inlineStr">
         <is>
@@ -2267,7 +2349,7 @@
         </is>
       </c>
       <c r="I5" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J5" s="3"/>
       <c r="K5" s="3"/>
@@ -2284,7 +2366,7 @@
         </is>
       </c>
       <c r="C6" s="3">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D6" s="3">
         <v>4</v>
@@ -2296,7 +2378,7 @@
         </is>
       </c>
       <c r="G6" s="3">
-        <v>0.35</v>
+        <v>0.4</v>
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
@@ -2304,7 +2386,7 @@
         </is>
       </c>
       <c r="I6" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J6" s="3"/>
       <c r="K6" s="3"/>
@@ -2321,7 +2403,7 @@
         </is>
       </c>
       <c r="C7" s="3">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D7" s="3">
         <v>5</v>
@@ -2333,7 +2415,7 @@
         </is>
       </c>
       <c r="G7" s="3">
-        <v>0.35</v>
+        <v>0.4</v>
       </c>
       <c r="H7" s="3" t="inlineStr">
         <is>
@@ -2341,7 +2423,7 @@
         </is>
       </c>
       <c r="I7" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J7" s="3"/>
       <c r="K7" s="3"/>
@@ -2358,7 +2440,7 @@
         </is>
       </c>
       <c r="C8" s="3">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="D8" s="3">
         <v>6</v>
@@ -2370,7 +2452,7 @@
         </is>
       </c>
       <c r="G8" s="3">
-        <v>0.35</v>
+        <v>0.4</v>
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
@@ -2378,10 +2460,232 @@
         </is>
       </c>
       <c r="I8" s="3">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="J8" s="3"/>
       <c r="K8" s="3"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BESS</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">F</t>
+        </is>
+      </c>
+      <c r="C9" s="3">
+        <v>5</v>
+      </c>
+      <c r="D9" s="3">
+        <v>1</v>
+      </c>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1000AL</t>
+        </is>
+      </c>
+      <c r="G9" s="3">
+        <v>0.8</v>
+      </c>
+      <c r="H9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">km</t>
+        </is>
+      </c>
+      <c r="I9" s="3">
+        <v>0</v>
+      </c>
+      <c r="J9" s="3"/>
+      <c r="K9" s="3"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BESS</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">F</t>
+        </is>
+      </c>
+      <c r="C10" s="3">
+        <v>5</v>
+      </c>
+      <c r="D10" s="3">
+        <v>2</v>
+      </c>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">500AL</t>
+        </is>
+      </c>
+      <c r="G10" s="3">
+        <v>0.15</v>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">km</t>
+        </is>
+      </c>
+      <c r="I10" s="3">
+        <v>1</v>
+      </c>
+      <c r="J10" s="3"/>
+      <c r="K10" s="3"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BESS</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">F</t>
+        </is>
+      </c>
+      <c r="C11" s="3">
+        <v>5</v>
+      </c>
+      <c r="D11" s="3">
+        <v>3</v>
+      </c>
+      <c r="E11" s="3"/>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">500AL</t>
+        </is>
+      </c>
+      <c r="G11" s="3">
+        <v>0.15</v>
+      </c>
+      <c r="H11" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">km</t>
+        </is>
+      </c>
+      <c r="I11" s="3">
+        <v>1</v>
+      </c>
+      <c r="J11" s="3"/>
+      <c r="K11" s="3"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BESS</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">F</t>
+        </is>
+      </c>
+      <c r="C12" s="3">
+        <v>5</v>
+      </c>
+      <c r="D12" s="3">
+        <v>4</v>
+      </c>
+      <c r="E12" s="3"/>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4/0AL</t>
+        </is>
+      </c>
+      <c r="G12" s="3">
+        <v>0.15</v>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">km</t>
+        </is>
+      </c>
+      <c r="I12" s="3">
+        <v>1</v>
+      </c>
+      <c r="J12" s="3"/>
+      <c r="K12" s="3"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BESS</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">F</t>
+        </is>
+      </c>
+      <c r="C13" s="3">
+        <v>5</v>
+      </c>
+      <c r="D13" s="3">
+        <v>5</v>
+      </c>
+      <c r="E13" s="3"/>
+      <c r="F13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4/0AL</t>
+        </is>
+      </c>
+      <c r="G13" s="3">
+        <v>0.15</v>
+      </c>
+      <c r="H13" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">km</t>
+        </is>
+      </c>
+      <c r="I13" s="3">
+        <v>1</v>
+      </c>
+      <c r="J13" s="3"/>
+      <c r="K13" s="3"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BESS</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">F</t>
+        </is>
+      </c>
+      <c r="C14" s="3">
+        <v>5</v>
+      </c>
+      <c r="D14" s="3">
+        <v>6</v>
+      </c>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1/0AL</t>
+        </is>
+      </c>
+      <c r="G14" s="3">
+        <v>0.15</v>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">km</t>
+        </is>
+      </c>
+      <c r="I14" s="3">
+        <v>1</v>
+      </c>
+      <c r="J14" s="3"/>
+      <c r="K14" s="3"/>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -2671,10 +2975,10 @@
         </is>
       </c>
       <c r="C3" s="3">
-        <v>0.5</v>
+        <v>1.0</v>
       </c>
       <c r="D3" s="3">
-        <v>0.2</v>
+        <v>0.3</v>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
smib_build: each generator its own collector to the MPT (SMIB); edge-case fixes
- SMIB: PV and BESS each get their own collector equivalent from the MPT
  winding; only one generator's several collector systems are merged
- DETAILED: no crash when a generator spans collectors or a collector starts
  at another's end; terminal / MV names of unit groups skipped in Bus_Numbers
- zero-MVAr shunts, blank / duplicate load names, duplicate cables, blank
  feeder names, section order, feet without unit no longer stop or mislead
- CHECKs: P at POI beyond Pmax / Pmin, units mismatch, 3-winding LV/TV overload
- no half-written output folder on error; outputs titled by model type

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BGsNUhFmVX23f8qnP53zUv
</commit_message>
<xml_diff>
--- a/smib/SMIB_INPUT_TEMPLATE.xlsx
+++ b/smib/SMIB_INPUT_TEMPLATE.xlsx
@@ -224,7 +224,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E (.raw, .dyr) and PSCAD (.pscx) models of a plant from one workbook -- smib_build.py, 2026-10-14</t>
+          <t xml:space="preserve">PSS/E (.raw, .dyr) and PSCAD (.pscx) models of a plant from one workbook -- smib_build.py, 2026-10-15</t>
         </is>
       </c>
       <c r="B2" s="10"/>
@@ -260,7 +260,7 @@
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Plant: Model type -- SMIB: one equivalent feeder per MPT, each generator one machine | DETAILED: every feeder section, the units at each node a machine of their own. PSS/E and PSCAD are built alike.</t>
+          <t xml:space="preserve">Plant: Model type -- SMIB: each generator one machine on its own equivalent feeder | DETAILED: every feeder section, the units at each node a machine of their own. PSS/E and PSCAD are built alike.</t>
         </is>
       </c>
     </row>
@@ -647,7 +647,7 @@
         </is>
       </c>
     </row>
-    <row r="38" ht="69.0" customHeight="1">
+    <row r="38" ht="56.0" customHeight="1">
       <c r="A38" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">MODEL TYPE</t>
@@ -655,7 +655,7 @@
       </c>
       <c r="B38" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Plant: Model type sets PSS/E and PSCAD alike. SMIB (default): the collectors on one MPT winding are one equivalent feeder (WECC, each collector weighed by its MW), each generator one machine behind one GSU at its far end. DETAILED: every feeder section is a branch (identical feeder copies lumped), the units of a generator at each node a machine of their own behind their own GSU; a generator's Dyr_Params, Dyr_Records and PSCAD_Params rows apply to all its machines.</t>
+          <t xml:space="preserve">Plant: Model type sets PSS/E and PSCAD alike. SMIB (default): each generator is one machine behind one GSU on a collector equivalent of its own (WECC, each feeder weighed by its MW) from its MPT winding. DETAILED: every feeder section is a branch (identical feeder copies lumped), the units of a generator at each node a machine of their own behind their own GSU; a generator's Dyr_Params, Dyr_Records and PSCAD_Params rows apply to all its machines.</t>
         </is>
       </c>
     </row>
@@ -1512,7 +1512,7 @@
       </c>
       <c r="G6" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">SMIB: one equivalent feeder (WECC) per MPT, each generator one machine behind one GSU | DETAILED: every feeder section, the units at each node a machine of their own behind their own GSU -- PSS/E and PSCAD alike (blank = SMIB)</t>
+          <t xml:space="preserve">SMIB: each generator one machine behind one GSU on its own equivalent feeder (WECC) from its MPT | DETAILED: every feeder section, the units at each node a machine of their own behind their own GSU -- PSS/E and PSCAD alike (blank = SMIB)</t>
         </is>
       </c>
       <c r="H6" s="13" t="inlineStr">
@@ -6273,7 +6273,7 @@
       <c r="A163" s="8"/>
       <c r="B163" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;MPT&gt;:COLL</t>
+          <t xml:space="preserve">&lt;collector&gt;</t>
         </is>
       </c>
       <c r="C163" s="8"/>
@@ -6282,7 +6282,7 @@
       <c r="F163" s="8"/>
       <c r="G163" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">SMIB: the far end of the MPT's one equivalent feeder</t>
+          <t xml:space="preserve">a shared collector's far end</t>
         </is>
       </c>
       <c r="H163" s="8"/>
@@ -6291,7 +6291,7 @@
       <c r="A164" s="8"/>
       <c r="B164" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;collector&gt;</t>
+          <t xml:space="preserve">&lt;generator&gt;:MV</t>
         </is>
       </c>
       <c r="C164" s="8"/>
@@ -6300,7 +6300,7 @@
       <c r="F164" s="8"/>
       <c r="G164" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">a shared collector's far end (SMIB without merging)</t>
+          <t xml:space="preserve">a generator's GSU HV side</t>
         </is>
       </c>
       <c r="H164" s="8"/>
@@ -6309,7 +6309,7 @@
       <c r="A165" s="8"/>
       <c r="B165" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;generator&gt;:MV</t>
+          <t xml:space="preserve">&lt;generator&gt; or &lt;generator&gt;:LV</t>
         </is>
       </c>
       <c r="C165" s="8"/>
@@ -6318,7 +6318,7 @@
       <c r="F165" s="8"/>
       <c r="G165" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">a generator's GSU HV side</t>
+          <t xml:space="preserve">a generator's terminal</t>
         </is>
       </c>
       <c r="H165" s="8"/>
@@ -6327,7 +6327,7 @@
       <c r="A166" s="8"/>
       <c r="B166" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;generator&gt; or &lt;generator&gt;:LV</t>
+          <t xml:space="preserve">&lt;collector&gt;_&lt;feeder&gt;_S&lt;n&gt;</t>
         </is>
       </c>
       <c r="C166" s="8"/>
@@ -6336,7 +6336,7 @@
       <c r="F166" s="8"/>
       <c r="G166" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">a generator's terminal</t>
+          <t xml:space="preserve">DETAILED: the far end of feeder section n</t>
         </is>
       </c>
       <c r="H166" s="8"/>
@@ -6345,7 +6345,7 @@
       <c r="A167" s="8"/>
       <c r="B167" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;collector&gt;_&lt;feeder&gt;_S&lt;n&gt;</t>
+          <t xml:space="preserve">&lt;generator&gt;_&lt;feeder&gt;_S&lt;n&gt;:LV</t>
         </is>
       </c>
       <c r="C167" s="8"/>
@@ -6354,42 +6354,50 @@
       <c r="F167" s="8"/>
       <c r="G167" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">DETAILED: the far end of feeder section n</t>
+          <t xml:space="preserve">DETAILED: the terminal of the units at that node</t>
         </is>
       </c>
       <c r="H167" s="8"/>
     </row>
-    <row r="168">
-      <c r="A168" s="8"/>
-      <c r="B168" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">&lt;generator&gt;_&lt;feeder&gt;_S&lt;n&gt;:LV</t>
-        </is>
-      </c>
-      <c r="C168" s="8"/>
-      <c r="D168" s="8"/>
-      <c r="E168" s="8"/>
-      <c r="F168" s="8"/>
-      <c r="G168" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DETAILED: the terminal of the units at that node</t>
-        </is>
-      </c>
-      <c r="H168" s="8"/>
-    </row>
-    <row r="169" ht="18" customHeight="1">
-      <c r="A169" s="7" t="inlineStr">
+    <row r="168" ht="18" customHeight="1">
+      <c r="A168" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">PSCAD_Params PLACEHOLDERS -- filled in for each inverter a vendor model stands for</t>
         </is>
       </c>
-      <c r="B169" s="7"/>
-      <c r="C169" s="7"/>
-      <c r="D169" s="7"/>
-      <c r="E169" s="7"/>
-      <c r="F169" s="7"/>
-      <c r="G169" s="7"/>
-      <c r="H169" s="7"/>
+      <c r="B168" s="7"/>
+      <c r="C168" s="7"/>
+      <c r="D168" s="7"/>
+      <c r="E168" s="7"/>
+      <c r="F168" s="7"/>
+      <c r="G168" s="7"/>
+      <c r="H168" s="7"/>
+    </row>
+    <row r="169">
+      <c r="A169" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD_Params</t>
+        </is>
+      </c>
+      <c r="B169" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{UNITS}</t>
+        </is>
+      </c>
+      <c r="C169" s="8"/>
+      <c r="D169" s="8"/>
+      <c r="E169" s="8"/>
+      <c r="F169" s="8"/>
+      <c r="G169" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the units the inverter stands for</t>
+        </is>
+      </c>
+      <c r="H169" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" s="8" t="inlineStr">
@@ -6399,7 +6407,7 @@
       </c>
       <c r="B170" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{UNITS}</t>
+          <t xml:space="preserve">{MVA}</t>
         </is>
       </c>
       <c r="C170" s="8"/>
@@ -6408,7 +6416,7 @@
       <c r="F170" s="8"/>
       <c r="G170" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">the units the inverter stands for</t>
+          <t xml:space="preserve">their MVA</t>
         </is>
       </c>
       <c r="H170" s="13" t="inlineStr">
@@ -6425,7 +6433,7 @@
       </c>
       <c r="B171" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{MVA}</t>
+          <t xml:space="preserve">{P_MW}</t>
         </is>
       </c>
       <c r="C171" s="8"/>
@@ -6434,7 +6442,7 @@
       <c r="F171" s="8"/>
       <c r="G171" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">their MVA</t>
+          <t xml:space="preserve">their P where the inverter connects (MW)</t>
         </is>
       </c>
       <c r="H171" s="13" t="inlineStr">
@@ -6451,7 +6459,7 @@
       </c>
       <c r="B172" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{P_MW}</t>
+          <t xml:space="preserve">{Q_MVAR}</t>
         </is>
       </c>
       <c r="C172" s="8"/>
@@ -6460,7 +6468,7 @@
       <c r="F172" s="8"/>
       <c r="G172" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">their P where the inverter connects (MW)</t>
+          <t xml:space="preserve">their Q there (MVAr)</t>
         </is>
       </c>
       <c r="H172" s="13" t="inlineStr">
@@ -6477,7 +6485,7 @@
       </c>
       <c r="B173" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{Q_MVAR}</t>
+          <t xml:space="preserve">{P_PU}</t>
         </is>
       </c>
       <c r="C173" s="8"/>
@@ -6486,7 +6494,7 @@
       <c r="F173" s="8"/>
       <c r="G173" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">their Q there (MVAr)</t>
+          <t xml:space="preserve">P on {MVA}</t>
         </is>
       </c>
       <c r="H173" s="13" t="inlineStr">
@@ -6503,7 +6511,7 @@
       </c>
       <c r="B174" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{P_PU}</t>
+          <t xml:space="preserve">{Q_PU}</t>
         </is>
       </c>
       <c r="C174" s="8"/>
@@ -6512,7 +6520,7 @@
       <c r="F174" s="8"/>
       <c r="G174" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">P on {MVA}</t>
+          <t xml:space="preserve">Q on {MVA}</t>
         </is>
       </c>
       <c r="H174" s="13" t="inlineStr">
@@ -6529,7 +6537,7 @@
       </c>
       <c r="B175" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{Q_PU}</t>
+          <t xml:space="preserve">{UNIT_MVA}</t>
         </is>
       </c>
       <c r="C175" s="8"/>
@@ -6538,7 +6546,7 @@
       <c r="F175" s="8"/>
       <c r="G175" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q on {MVA}</t>
+          <t xml:space="preserve">one unit's MVA</t>
         </is>
       </c>
       <c r="H175" s="13" t="inlineStr">
@@ -6555,7 +6563,7 @@
       </c>
       <c r="B176" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{UNIT_MVA}</t>
+          <t xml:space="preserve">{UNIT_P_MW}</t>
         </is>
       </c>
       <c r="C176" s="8"/>
@@ -6564,7 +6572,7 @@
       <c r="F176" s="8"/>
       <c r="G176" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">one unit's MVA</t>
+          <t xml:space="preserve">one unit's P (MW)</t>
         </is>
       </c>
       <c r="H176" s="13" t="inlineStr">
@@ -6581,7 +6589,7 @@
       </c>
       <c r="B177" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{UNIT_P_MW}</t>
+          <t xml:space="preserve">{UNIT_Q_MVAR}</t>
         </is>
       </c>
       <c r="C177" s="8"/>
@@ -6590,7 +6598,7 @@
       <c r="F177" s="8"/>
       <c r="G177" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">one unit's P (MW)</t>
+          <t xml:space="preserve">one unit's Q (MVAr)</t>
         </is>
       </c>
       <c r="H177" s="13" t="inlineStr">
@@ -6607,7 +6615,7 @@
       </c>
       <c r="B178" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{UNIT_Q_MVAR}</t>
+          <t xml:space="preserve">{V_PU}</t>
         </is>
       </c>
       <c r="C178" s="8"/>
@@ -6616,7 +6624,7 @@
       <c r="F178" s="8"/>
       <c r="G178" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">one unit's Q (MVAr)</t>
+          <t xml:space="preserve">the voltage where it connects (pu)</t>
         </is>
       </c>
       <c r="H178" s="13" t="inlineStr">
@@ -6633,7 +6641,7 @@
       </c>
       <c r="B179" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{V_PU}</t>
+          <t xml:space="preserve">{V_KV}</t>
         </is>
       </c>
       <c r="C179" s="8"/>
@@ -6642,7 +6650,7 @@
       <c r="F179" s="8"/>
       <c r="G179" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">the voltage where it connects (pu)</t>
+          <t xml:space="preserve">the same in kV</t>
         </is>
       </c>
       <c r="H179" s="13" t="inlineStr">
@@ -6659,7 +6667,7 @@
       </c>
       <c r="B180" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{V_KV}</t>
+          <t xml:space="preserve">{KV}</t>
         </is>
       </c>
       <c r="C180" s="8"/>
@@ -6668,7 +6676,7 @@
       <c r="F180" s="8"/>
       <c r="G180" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">the same in kV</t>
+          <t xml:space="preserve">that bus's base kV</t>
         </is>
       </c>
       <c r="H180" s="13" t="inlineStr">
@@ -6685,7 +6693,7 @@
       </c>
       <c r="B181" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{KV}</t>
+          <t xml:space="preserve">{ANGLE}</t>
         </is>
       </c>
       <c r="C181" s="8"/>
@@ -6694,7 +6702,7 @@
       <c r="F181" s="8"/>
       <c r="G181" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">that bus's base kV</t>
+          <t xml:space="preserve">its PSCAD angle (deg, the transformers' phase shifts included)</t>
         </is>
       </c>
       <c r="H181" s="13" t="inlineStr">
@@ -6711,7 +6719,7 @@
       </c>
       <c r="B182" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{ANGLE}</t>
+          <t xml:space="preserve">{FREQ}</t>
         </is>
       </c>
       <c r="C182" s="8"/>
@@ -6720,7 +6728,7 @@
       <c r="F182" s="8"/>
       <c r="G182" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">its PSCAD angle (deg, the transformers' phase shifts included)</t>
+          <t xml:space="preserve">frequency (Hz)</t>
         </is>
       </c>
       <c r="H182" s="13" t="inlineStr">
@@ -6737,7 +6745,7 @@
       </c>
       <c r="B183" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{FREQ}</t>
+          <t xml:space="preserve">{P_INV_MW}</t>
         </is>
       </c>
       <c r="C183" s="8"/>
@@ -6746,7 +6754,7 @@
       <c r="F183" s="8"/>
       <c r="G183" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">frequency (Hz)</t>
+          <t xml:space="preserve">P at the inverters' own terminals (MW; a UDM on the MV side)</t>
         </is>
       </c>
       <c r="H183" s="13" t="inlineStr">
@@ -6763,7 +6771,7 @@
       </c>
       <c r="B184" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{P_INV_MW}</t>
+          <t xml:space="preserve">{Q_INV_MVAR}</t>
         </is>
       </c>
       <c r="C184" s="8"/>
@@ -6772,7 +6780,7 @@
       <c r="F184" s="8"/>
       <c r="G184" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">P at the inverters' own terminals (MW; a UDM on the MV side)</t>
+          <t xml:space="preserve">Q there (MVAr)</t>
         </is>
       </c>
       <c r="H184" s="13" t="inlineStr">
@@ -6789,7 +6797,7 @@
       </c>
       <c r="B185" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{Q_INV_MVAR}</t>
+          <t xml:space="preserve">{V_INV_PU}</t>
         </is>
       </c>
       <c r="C185" s="8"/>
@@ -6798,36 +6806,10 @@
       <c r="F185" s="8"/>
       <c r="G185" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q there (MVAr)</t>
+          <t xml:space="preserve">the voltage there (pu)</t>
         </is>
       </c>
       <c r="H185" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSCAD</t>
-        </is>
-      </c>
-    </row>
-    <row r="186">
-      <c r="A186" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSCAD_Params</t>
-        </is>
-      </c>
-      <c r="B186" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">{V_INV_PU}</t>
-        </is>
-      </c>
-      <c r="C186" s="8"/>
-      <c r="D186" s="8"/>
-      <c r="E186" s="8"/>
-      <c r="F186" s="8"/>
-      <c r="G186" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">the voltage there (pu)</t>
-        </is>
-      </c>
-      <c r="H186" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">PSCAD</t>
         </is>
@@ -6849,7 +6831,7 @@
     <mergeCell ref="A149:H149"/>
     <mergeCell ref="A152:H152"/>
     <mergeCell ref="A156:H156"/>
-    <mergeCell ref="A169:H169"/>
+    <mergeCell ref="A168:H168"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A4" location="'Plant'!A1" display="Plant"/>
@@ -6863,7 +6845,7 @@
     <hyperlink ref="A144" location="'Dyr_Params'!A1" display="Dyr_Params"/>
     <hyperlink ref="A149" location="'Dyr_Records'!A1" display="Dyr_Records"/>
     <hyperlink ref="A152" location="'PSCAD_Params'!A1" display="PSCAD_Params"/>
-    <hyperlink ref="A169" location="'PSCAD_Params'!A1" display="PSCAD_Params"/>
+    <hyperlink ref="A168" location="'PSCAD_Params'!A1" display="PSCAD_Params"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
@@ -17529,7 +17511,7 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">SMIB: one equivalent feeder (WECC) per MPT, each generator one machine behind one GSU | DETAILED: every feeder section, the units at each node a machine of their own behind their own GSU -- PSS/E and PSCAD alike (blank = SMIB)</t>
+          <t xml:space="preserve">SMIB: each generator one machine behind one GSU on its own equivalent feeder (WECC) from its MPT | DETAILED: every feeder section, the units at each node a machine of their own behind their own GSU -- PSS/E and PSCAD alike (blank = SMIB)</t>
         </is>
       </c>
       <c r="G4" s="13" t="inlineStr">
@@ -22474,7 +22456,7 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">MPT1:COLL</t>
+          <t xml:space="preserve">PV:MV</t>
         </is>
       </c>
       <c r="B7" s="3"/>
@@ -22492,14 +22474,18 @@
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">BESS:LV</t>
+          <t xml:space="preserve">BESS:MV</t>
         </is>
       </c>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
     </row>
     <row r="10">
-      <c r="A10" s="3"/>
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BESS:LV</t>
+        </is>
+      </c>
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
     </row>

</xml_diff>

<commit_message>
smib_build: PSCAD lines as Coupled PI Sections (pu on 100 MVA)
- the gen-tie, each collector and each feeder section: one Coupled PI Section, R, X, B in pu on 100 MVA and
  the line's kV, per metre; its charging inside (no separate capacitors); zero sequence = positive
- the build script finds the PI in the master library and its parameters by their descriptions in its form
- Plant: PSCAD lines as PI (default) or RLC (the R, L and C/2 capacitors as before)
- the wire between two symbols on a row long enough for its node's name

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BGsNUhFmVX23f8qnP53zUv
</commit_message>
<xml_diff>
--- a/smib/SMIB_INPUT_TEMPLATE.xlsx
+++ b/smib/SMIB_INPUT_TEMPLATE.xlsx
@@ -2705,62 +2705,62 @@
       </c>
       <c r="B41" s="12" t="inlineStr">
         <is>
+          <t xml:space="preserve">PSCAD lines as</t>
+        </is>
+      </c>
+      <c r="C41" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pscad_lines</t>
+        </is>
+      </c>
+      <c r="D41" s="8"/>
+      <c r="E41" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PI</t>
+        </is>
+      </c>
+      <c r="F41" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PI | RLC</t>
+        </is>
+      </c>
+      <c r="G41" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PI = the gen-tie, each collector and each feeder section one Coupled PI Section (R, X, B in pu, its charging inside); RLC = an R and an L, the charging a C at each end (blank = PI)</t>
+        </is>
+      </c>
+      <c r="H41" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="30.0" customHeight="1">
+      <c r="A42" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Plant</t>
+        </is>
+      </c>
+      <c r="B42" s="12" t="inlineStr">
+        <is>
           <t xml:space="preserve">PSCAD fault at POI</t>
         </is>
       </c>
-      <c r="C41" s="8" t="inlineStr">
+      <c r="C42" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">pscad_fault</t>
         </is>
       </c>
-      <c r="D41" s="8"/>
-      <c r="E41" s="8"/>
-      <c r="F41" s="8" t="inlineStr">
+      <c r="D42" s="8"/>
+      <c r="E42" s="8"/>
+      <c r="F42" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">YES | NO</t>
         </is>
       </c>
-      <c r="G41" s="8" t="inlineStr">
+      <c r="G42" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">YES = a fault on the grid side of the POI with its timed fault logic, as vendors' test cases have</t>
-        </is>
-      </c>
-      <c r="H41" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSCAD</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="17.0" customHeight="1">
-      <c r="A42" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Plant</t>
-        </is>
-      </c>
-      <c r="B42" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSCAD fault time</t>
-        </is>
-      </c>
-      <c r="C42" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">pscad_fault_s</t>
-        </is>
-      </c>
-      <c r="D42" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">s</t>
-        </is>
-      </c>
-      <c r="E42" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">100: none in the run</t>
-        </is>
-      </c>
-      <c r="F42" s="8"/>
-      <c r="G42" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">when the fault starts (blank = 100: none in the run)</t>
         </is>
       </c>
       <c r="H42" s="13" t="inlineStr">
@@ -2777,12 +2777,12 @@
       </c>
       <c r="B43" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSCAD fault duration</t>
+          <t xml:space="preserve">PSCAD fault time</t>
         </is>
       </c>
       <c r="C43" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">pscad_fault_dur_s</t>
+          <t xml:space="preserve">pscad_fault_s</t>
         </is>
       </c>
       <c r="D43" s="8" t="inlineStr">
@@ -2792,89 +2792,89 @@
       </c>
       <c r="E43" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.15</t>
+          <t xml:space="preserve">100: none in the run</t>
         </is>
       </c>
       <c r="F43" s="8"/>
       <c r="G43" s="8" t="inlineStr">
         <is>
+          <t xml:space="preserve">when the fault starts (blank = 100: none in the run)</t>
+        </is>
+      </c>
+      <c r="H43" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="17.0" customHeight="1">
+      <c r="A44" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Plant</t>
+        </is>
+      </c>
+      <c r="B44" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD fault duration</t>
+        </is>
+      </c>
+      <c r="C44" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pscad_fault_dur_s</t>
+        </is>
+      </c>
+      <c r="D44" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">s</t>
+        </is>
+      </c>
+      <c r="E44" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.15</t>
+        </is>
+      </c>
+      <c r="F44" s="8"/>
+      <c r="G44" s="8" t="inlineStr">
+        <is>
           <t xml:space="preserve">blank = 0.15</t>
         </is>
       </c>
-      <c r="H43" s="13" t="inlineStr">
+      <c r="H44" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">PSCAD</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="43.0" customHeight="1">
-      <c r="A44" s="8" t="inlineStr">
+    <row r="45" ht="43.0" customHeight="1">
+      <c r="A45" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Plant</t>
         </is>
       </c>
-      <c r="B44" s="12" t="inlineStr">
+      <c r="B45" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">PSCAD fault type</t>
         </is>
       </c>
-      <c r="C44" s="8" t="inlineStr">
+      <c r="C45" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">pscad_fault_type</t>
         </is>
       </c>
-      <c r="D44" s="8"/>
-      <c r="E44" s="8" t="inlineStr">
+      <c r="D45" s="8"/>
+      <c r="E45" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">ABCG</t>
         </is>
       </c>
-      <c r="F44" s="8" t="inlineStr">
+      <c r="F45" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">ABCG | ABC | AG | BG | CG | ABG | BCG | ACG | AB | BC | AC</t>
         </is>
       </c>
-      <c r="G44" s="8" t="inlineStr">
+      <c r="G45" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">the phases faulted, G = to ground (blank = ABCG)</t>
-        </is>
-      </c>
-      <c r="H44" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSCAD</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="17.0" customHeight="1">
-      <c r="A45" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Plant</t>
-        </is>
-      </c>
-      <c r="B45" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSCAD fault resistance</t>
-        </is>
-      </c>
-      <c r="C45" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">pscad_fault_ohm</t>
-        </is>
-      </c>
-      <c r="D45" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ohm</t>
-        </is>
-      </c>
-      <c r="E45" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0.01</t>
-        </is>
-      </c>
-      <c r="F45" s="8"/>
-      <c r="G45" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">blank = 0.01</t>
         </is>
       </c>
       <c r="H45" s="13" t="inlineStr">
@@ -2891,71 +2891,79 @@
       </c>
       <c r="B46" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSCAD libraries</t>
+          <t xml:space="preserve">PSCAD fault resistance</t>
         </is>
       </c>
       <c r="C46" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">pscad_libraries</t>
-        </is>
-      </c>
-      <c r="D46" s="8"/>
-      <c r="E46" s="8"/>
+          <t xml:space="preserve">pscad_fault_ohm</t>
+        </is>
+      </c>
+      <c r="D46" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ohm</t>
+        </is>
+      </c>
+      <c r="E46" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.01</t>
+        </is>
+      </c>
       <c r="F46" s="8"/>
       <c r="G46" s="8" t="inlineStr">
         <is>
+          <t xml:space="preserve">blank = 0.01</t>
+        </is>
+      </c>
+      <c r="H46" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="17.0" customHeight="1">
+      <c r="A47" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Plant</t>
+        </is>
+      </c>
+      <c r="B47" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD libraries</t>
+        </is>
+      </c>
+      <c r="C47" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pscad_libraries</t>
+        </is>
+      </c>
+      <c r="D47" s="8"/>
+      <c r="E47" s="8"/>
+      <c r="F47" s="8"/>
+      <c r="G47" s="8" t="inlineStr">
+        <is>
           <t xml:space="preserve">user-model libraries (.pslx) to load, separated by ;</t>
         </is>
       </c>
-      <c r="H46" s="13" t="inlineStr">
+      <c r="H47" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">PSCAD</t>
         </is>
       </c>
     </row>
-    <row r="47" ht="18" customHeight="1">
-      <c r="A47" s="7" t="inlineStr">
+    <row r="48" ht="18" customHeight="1">
+      <c r="A48" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">MPT</t>
         </is>
       </c>
-      <c r="B47" s="7"/>
-      <c r="C47" s="7"/>
-      <c r="D47" s="7"/>
-      <c r="E47" s="7"/>
-      <c r="F47" s="7"/>
-      <c r="G47" s="7"/>
-      <c r="H47" s="7"/>
-    </row>
-    <row r="48" ht="17.0" customHeight="1">
-      <c r="A48" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MPT</t>
-        </is>
-      </c>
-      <c r="B48" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Name</t>
-        </is>
-      </c>
-      <c r="C48" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">name</t>
-        </is>
-      </c>
-      <c r="D48" s="8"/>
-      <c r="E48" s="8"/>
-      <c r="F48" s="8"/>
-      <c r="G48" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MPT name. Its buses: &lt;name&gt; or &lt;name&gt;:LV (LV winding), &lt;name&gt;:TV (tertiary)</t>
-        </is>
-      </c>
-      <c r="H48" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
-        </is>
-      </c>
+      <c r="B48" s="7"/>
+      <c r="C48" s="7"/>
+      <c r="D48" s="7"/>
+      <c r="E48" s="7"/>
+      <c r="F48" s="7"/>
+      <c r="G48" s="7"/>
+      <c r="H48" s="7"/>
     </row>
     <row r="49" ht="17.0" customHeight="1">
       <c r="A49" s="8" t="inlineStr">
@@ -2965,18 +2973,22 @@
       </c>
       <c r="B49" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">HV kV</t>
+          <t xml:space="preserve">Name</t>
         </is>
       </c>
       <c r="C49" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">hv_kv</t>
+          <t xml:space="preserve">name</t>
         </is>
       </c>
       <c r="D49" s="8"/>
       <c r="E49" s="8"/>
       <c r="F49" s="8"/>
-      <c r="G49" s="8"/>
+      <c r="G49" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MPT name. Its buses: &lt;name&gt; or &lt;name&gt;:LV (LV winding), &lt;name&gt;:TV (tertiary)</t>
+        </is>
+      </c>
       <c r="H49" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">PSS/E + PSCAD</t>
@@ -2991,12 +3003,12 @@
       </c>
       <c r="B50" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">LV kV</t>
+          <t xml:space="preserve">HV kV</t>
         </is>
       </c>
       <c r="C50" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">lv_kv</t>
+          <t xml:space="preserve">hv_kv</t>
         </is>
       </c>
       <c r="D50" s="8"/>
@@ -3017,26 +3029,18 @@
       </c>
       <c r="B51" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">TV kV</t>
+          <t xml:space="preserve">LV kV</t>
         </is>
       </c>
       <c r="C51" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">tv_kv</t>
+          <t xml:space="preserve">lv_kv</t>
         </is>
       </c>
       <c r="D51" s="8"/>
-      <c r="E51" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">two windings</t>
-        </is>
-      </c>
+      <c r="E51" s="8"/>
       <c r="F51" s="8"/>
-      <c r="G51" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">tertiary / 2nd LV winding; blank = two windings</t>
-        </is>
-      </c>
+      <c r="G51" s="8"/>
       <c r="H51" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">PSS/E + PSCAD</t>
@@ -3051,20 +3055,24 @@
       </c>
       <c r="B52" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">MVA</t>
+          <t xml:space="preserve">TV kV</t>
         </is>
       </c>
       <c r="C52" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">mva</t>
+          <t xml:space="preserve">tv_kv</t>
         </is>
       </c>
       <c r="D52" s="8"/>
-      <c r="E52" s="8"/>
+      <c r="E52" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">two windings</t>
+        </is>
+      </c>
       <c r="F52" s="8"/>
       <c r="G52" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">the rating (3 windings: HV winding)</t>
+          <t xml:space="preserve">tertiary / 2nd LV winding; blank = two windings</t>
         </is>
       </c>
       <c r="H52" s="13" t="inlineStr">
@@ -3081,12 +3089,12 @@
       </c>
       <c r="B53" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">LV MVA</t>
+          <t xml:space="preserve">MVA</t>
         </is>
       </c>
       <c r="C53" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">lv_mva</t>
+          <t xml:space="preserve">mva</t>
         </is>
       </c>
       <c r="D53" s="8"/>
@@ -3094,7 +3102,7 @@
       <c r="F53" s="8"/>
       <c r="G53" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 windings</t>
+          <t xml:space="preserve">the rating (3 windings: HV winding)</t>
         </is>
       </c>
       <c r="H53" s="13" t="inlineStr">
@@ -3111,12 +3119,12 @@
       </c>
       <c r="B54" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">TV MVA</t>
+          <t xml:space="preserve">LV MVA</t>
         </is>
       </c>
       <c r="C54" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">tv_mva</t>
+          <t xml:space="preserve">lv_mva</t>
         </is>
       </c>
       <c r="D54" s="8"/>
@@ -3141,12 +3149,12 @@
       </c>
       <c r="B55" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Z HV-LV %</t>
+          <t xml:space="preserve">TV MVA</t>
         </is>
       </c>
       <c r="C55" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">z_hl_pct</t>
+          <t xml:space="preserve">tv_mva</t>
         </is>
       </c>
       <c r="D55" s="8"/>
@@ -3154,7 +3162,7 @@
       <c r="F55" s="8"/>
       <c r="G55" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">on its base MVA</t>
+          <t xml:space="preserve">3 windings</t>
         </is>
       </c>
       <c r="H55" s="13" t="inlineStr">
@@ -3171,12 +3179,12 @@
       </c>
       <c r="B56" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Z HV-TV %</t>
+          <t xml:space="preserve">Z HV-LV %</t>
         </is>
       </c>
       <c r="C56" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">z_ht_pct</t>
+          <t xml:space="preserve">z_hl_pct</t>
         </is>
       </c>
       <c r="D56" s="8"/>
@@ -3184,7 +3192,7 @@
       <c r="F56" s="8"/>
       <c r="G56" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 windings</t>
+          <t xml:space="preserve">on its base MVA</t>
         </is>
       </c>
       <c r="H56" s="13" t="inlineStr">
@@ -3201,12 +3209,12 @@
       </c>
       <c r="B57" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Z LV-TV %</t>
+          <t xml:space="preserve">Z HV-TV %</t>
         </is>
       </c>
       <c r="C57" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">z_lt_pct</t>
+          <t xml:space="preserve">z_ht_pct</t>
         </is>
       </c>
       <c r="D57" s="8"/>
@@ -3231,24 +3239,20 @@
       </c>
       <c r="B58" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Z HV-LV base MVA</t>
+          <t xml:space="preserve">Z LV-TV %</t>
         </is>
       </c>
       <c r="C58" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">base_hl_mva</t>
+          <t xml:space="preserve">z_lt_pct</t>
         </is>
       </c>
       <c r="D58" s="8"/>
-      <c r="E58" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MVA</t>
-        </is>
-      </c>
+      <c r="E58" s="8"/>
       <c r="F58" s="8"/>
       <c r="G58" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">blank = MVA</t>
+          <t xml:space="preserve">3 windings</t>
         </is>
       </c>
       <c r="H58" s="13" t="inlineStr">
@@ -3265,12 +3269,12 @@
       </c>
       <c r="B59" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Z HV-TV base MVA</t>
+          <t xml:space="preserve">Z HV-LV base MVA</t>
         </is>
       </c>
       <c r="C59" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">base_ht_mva</t>
+          <t xml:space="preserve">base_hl_mva</t>
         </is>
       </c>
       <c r="D59" s="8"/>
@@ -3299,12 +3303,12 @@
       </c>
       <c r="B60" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Z LV-TV base MVA</t>
+          <t xml:space="preserve">Z HV-TV base MVA</t>
         </is>
       </c>
       <c r="C60" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">base_lt_mva</t>
+          <t xml:space="preserve">base_ht_mva</t>
         </is>
       </c>
       <c r="D60" s="8"/>
@@ -3333,20 +3337,24 @@
       </c>
       <c r="B61" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">X/R</t>
+          <t xml:space="preserve">Z LV-TV base MVA</t>
         </is>
       </c>
       <c r="C61" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">x_r</t>
+          <t xml:space="preserve">base_lt_mva</t>
         </is>
       </c>
       <c r="D61" s="8"/>
-      <c r="E61" s="8"/>
+      <c r="E61" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MVA</t>
+        </is>
+      </c>
       <c r="F61" s="8"/>
       <c r="G61" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">each impedance</t>
+          <t xml:space="preserve">blank = MVA</t>
         </is>
       </c>
       <c r="H61" s="13" t="inlineStr">
@@ -3363,12 +3371,12 @@
       </c>
       <c r="B62" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Load loss kW</t>
+          <t xml:space="preserve">X/R</t>
         </is>
       </c>
       <c r="C62" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">load_loss_kw</t>
+          <t xml:space="preserve">x_r</t>
         </is>
       </c>
       <c r="D62" s="8"/>
@@ -3376,7 +3384,7 @@
       <c r="F62" s="8"/>
       <c r="G62" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">2 windings, at MVA: instead of X/R</t>
+          <t xml:space="preserve">each impedance</t>
         </is>
       </c>
       <c r="H62" s="13" t="inlineStr">
@@ -3393,12 +3401,12 @@
       </c>
       <c r="B63" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Vector group</t>
+          <t xml:space="preserve">Load loss kW</t>
         </is>
       </c>
       <c r="C63" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">vector</t>
+          <t xml:space="preserve">load_loss_kw</t>
         </is>
       </c>
       <c r="D63" s="8"/>
@@ -3406,7 +3414,7 @@
       <c r="F63" s="8"/>
       <c r="G63" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">YNd1, YNd11, Dyn1, YNyn0, YNd1d1 ...</t>
+          <t xml:space="preserve">2 windings, at MVA: instead of X/R</t>
         </is>
       </c>
       <c r="H63" s="13" t="inlineStr">
@@ -3423,24 +3431,20 @@
       </c>
       <c r="B64" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">HV tap</t>
+          <t xml:space="preserve">Vector group</t>
         </is>
       </c>
       <c r="C64" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">tap</t>
+          <t xml:space="preserve">vector</t>
         </is>
       </c>
       <c r="D64" s="8"/>
-      <c r="E64" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
+      <c r="E64" s="8"/>
       <c r="F64" s="8"/>
       <c r="G64" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">HV winding ratio, 1.025 = +2.5 % (blank = 1)</t>
+          <t xml:space="preserve">YNd1, YNd11, Dyn1, YNyn0, YNd1d1 ...</t>
         </is>
       </c>
       <c r="H64" s="13" t="inlineStr">
@@ -3457,12 +3461,12 @@
       </c>
       <c r="B65" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Parallel units</t>
+          <t xml:space="preserve">HV tap</t>
         </is>
       </c>
       <c r="C65" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">count</t>
+          <t xml:space="preserve">tap</t>
         </is>
       </c>
       <c r="D65" s="8"/>
@@ -3474,7 +3478,7 @@
       <c r="F65" s="8"/>
       <c r="G65" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">identical units (blank = 1)</t>
+          <t xml:space="preserve">HV winding ratio, 1.025 = +2.5 % (blank = 1)</t>
         </is>
       </c>
       <c r="H65" s="13" t="inlineStr">
@@ -3491,24 +3495,24 @@
       </c>
       <c r="B66" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">No-load loss %</t>
+          <t xml:space="preserve">Parallel units</t>
         </is>
       </c>
       <c r="C66" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">nll_pct</t>
+          <t xml:space="preserve">count</t>
         </is>
       </c>
       <c r="D66" s="8"/>
       <c r="E66" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">0</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="F66" s="8"/>
       <c r="G66" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">of MVA (blank = 0)</t>
+          <t xml:space="preserve">identical units (blank = 1)</t>
         </is>
       </c>
       <c r="H66" s="13" t="inlineStr">
@@ -3525,12 +3529,12 @@
       </c>
       <c r="B67" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Magnetising current %</t>
+          <t xml:space="preserve">No-load loss %</t>
         </is>
       </c>
       <c r="C67" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">im_pct</t>
+          <t xml:space="preserve">nll_pct</t>
         </is>
       </c>
       <c r="D67" s="8"/>
@@ -3559,24 +3563,24 @@
       </c>
       <c r="B68" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Rating MVA</t>
+          <t xml:space="preserve">Magnetising current %</t>
         </is>
       </c>
       <c r="C68" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">rate_mva</t>
+          <t xml:space="preserve">im_pct</t>
         </is>
       </c>
       <c r="D68" s="8"/>
       <c r="E68" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">MVA</t>
+          <t xml:space="preserve">0</t>
         </is>
       </c>
       <c r="F68" s="8"/>
       <c r="G68" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">blank = MVA</t>
+          <t xml:space="preserve">of MVA (blank = 0)</t>
         </is>
       </c>
       <c r="H68" s="13" t="inlineStr">
@@ -3593,24 +3597,24 @@
       </c>
       <c r="B69" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tie length</t>
+          <t xml:space="preserve">Rating MVA</t>
         </is>
       </c>
       <c r="C69" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">tie_length</t>
+          <t xml:space="preserve">rate_mva</t>
         </is>
       </c>
       <c r="D69" s="8"/>
       <c r="E69" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">none</t>
+          <t xml:space="preserve">MVA</t>
         </is>
       </c>
       <c r="F69" s="8"/>
       <c r="G69" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">a line of its own from HV to this MPT (blank = none)</t>
+          <t xml:space="preserve">blank = MVA</t>
         </is>
       </c>
       <c r="H69" s="13" t="inlineStr">
@@ -3627,22 +3631,26 @@
       </c>
       <c r="B70" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tie length unit</t>
+          <t xml:space="preserve">Tie length</t>
         </is>
       </c>
       <c r="C70" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">tie_unit</t>
+          <t xml:space="preserve">tie_length</t>
         </is>
       </c>
       <c r="D70" s="8"/>
-      <c r="E70" s="8"/>
-      <c r="F70" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">km | mi | kft | m | ft</t>
-        </is>
-      </c>
-      <c r="G70" s="8"/>
+      <c r="E70" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">none</t>
+        </is>
+      </c>
+      <c r="F70" s="8"/>
+      <c r="G70" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a line of its own from HV to this MPT (blank = none)</t>
+        </is>
+      </c>
       <c r="H70" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">PSS/E + PSCAD</t>
@@ -3657,22 +3665,22 @@
       </c>
       <c r="B71" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tie R per length</t>
+          <t xml:space="preserve">Tie length unit</t>
         </is>
       </c>
       <c r="C71" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">tie_r_per</t>
+          <t xml:space="preserve">tie_unit</t>
         </is>
       </c>
       <c r="D71" s="8"/>
       <c r="E71" s="8"/>
-      <c r="F71" s="8"/>
-      <c r="G71" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ohm</t>
-        </is>
-      </c>
+      <c r="F71" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">km | mi | kft | m | ft</t>
+        </is>
+      </c>
+      <c r="G71" s="8"/>
       <c r="H71" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">PSS/E + PSCAD</t>
@@ -3687,12 +3695,12 @@
       </c>
       <c r="B72" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tie X per length</t>
+          <t xml:space="preserve">Tie R per length</t>
         </is>
       </c>
       <c r="C72" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">tie_x_per</t>
+          <t xml:space="preserve">tie_r_per</t>
         </is>
       </c>
       <c r="D72" s="8"/>
@@ -3717,12 +3725,12 @@
       </c>
       <c r="B73" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tie B per length</t>
+          <t xml:space="preserve">Tie X per length</t>
         </is>
       </c>
       <c r="C73" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">tie_b_per</t>
+          <t xml:space="preserve">tie_x_per</t>
         </is>
       </c>
       <c r="D73" s="8"/>
@@ -3730,7 +3738,7 @@
       <c r="F73" s="8"/>
       <c r="G73" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">uS</t>
+          <t xml:space="preserve">ohm</t>
         </is>
       </c>
       <c r="H73" s="13" t="inlineStr">
@@ -3747,128 +3755,124 @@
       </c>
       <c r="B74" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tie rating MVA</t>
+          <t xml:space="preserve">Tie B per length</t>
         </is>
       </c>
       <c r="C74" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">tie_rate_mva</t>
+          <t xml:space="preserve">tie_b_per</t>
         </is>
       </c>
       <c r="D74" s="8"/>
       <c r="E74" s="8"/>
       <c r="F74" s="8"/>
-      <c r="G74" s="8"/>
+      <c r="G74" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">uS</t>
+        </is>
+      </c>
       <c r="H74" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">PSS/E + PSCAD</t>
         </is>
       </c>
     </row>
-    <row r="75" ht="18" customHeight="1">
-      <c r="A75" s="7" t="inlineStr">
+    <row r="75" ht="17.0" customHeight="1">
+      <c r="A75" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MPT</t>
+        </is>
+      </c>
+      <c r="B75" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tie rating MVA</t>
+        </is>
+      </c>
+      <c r="C75" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">tie_rate_mva</t>
+        </is>
+      </c>
+      <c r="D75" s="8"/>
+      <c r="E75" s="8"/>
+      <c r="F75" s="8"/>
+      <c r="G75" s="8"/>
+      <c r="H75" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSS/E + PSCAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="18" customHeight="1">
+      <c r="A76" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Generators</t>
         </is>
       </c>
-      <c r="B75" s="7"/>
-      <c r="C75" s="7"/>
-      <c r="D75" s="7"/>
-      <c r="E75" s="7"/>
-      <c r="F75" s="7"/>
-      <c r="G75" s="7"/>
-      <c r="H75" s="7"/>
-    </row>
-    <row r="76" ht="17.0" customHeight="1">
-      <c r="A76" s="8" t="inlineStr">
+      <c r="B76" s="7"/>
+      <c r="C76" s="7"/>
+      <c r="D76" s="7"/>
+      <c r="E76" s="7"/>
+      <c r="F76" s="7"/>
+      <c r="G76" s="7"/>
+      <c r="H76" s="7"/>
+    </row>
+    <row r="77" ht="17.0" customHeight="1">
+      <c r="A77" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Generators</t>
         </is>
       </c>
-      <c r="B76" s="12" t="inlineStr">
+      <c r="B77" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Name</t>
         </is>
       </c>
-      <c r="C76" s="8" t="inlineStr">
+      <c r="C77" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">name</t>
-        </is>
-      </c>
-      <c r="D76" s="8"/>
-      <c r="E76" s="8"/>
-      <c r="F76" s="8"/>
-      <c r="G76" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">generator name. Its buses: &lt;name&gt;:MV (GSU HV), &lt;name&gt; or &lt;name&gt;:LV (terminal)</t>
-        </is>
-      </c>
-      <c r="H76" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
-        </is>
-      </c>
-    </row>
-    <row r="77" ht="30.0" customHeight="1">
-      <c r="A77" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Generators</t>
-        </is>
-      </c>
-      <c r="B77" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Type</t>
-        </is>
-      </c>
-      <c r="C77" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">type</t>
         </is>
       </c>
       <c r="D77" s="8"/>
       <c r="E77" s="8"/>
-      <c r="F77" s="8" t="inlineStr">
+      <c r="F77" s="8"/>
+      <c r="G77" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">generator name. Its buses: &lt;name&gt;:MV (GSU HV), &lt;name&gt; or &lt;name&gt;:LV (terminal)</t>
+        </is>
+      </c>
+      <c r="H77" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSS/E + PSCAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="30.0" customHeight="1">
+      <c r="A78" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Generators</t>
+        </is>
+      </c>
+      <c r="B78" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Type</t>
+        </is>
+      </c>
+      <c r="C78" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">type</t>
+        </is>
+      </c>
+      <c r="D78" s="8"/>
+      <c r="E78" s="8"/>
+      <c r="F78" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">PV | BESS | WT4 | WT3 | SYNC | USER</t>
         </is>
       </c>
-      <c r="G77" s="8" t="inlineStr">
+      <c r="G78" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">PV BESS WT4 WT3 SYNC USER (USER: Dyr_Records only)</t>
-        </is>
-      </c>
-      <c r="H77" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
-        </is>
-      </c>
-    </row>
-    <row r="78" ht="17.0" customHeight="1">
-      <c r="A78" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Generators</t>
-        </is>
-      </c>
-      <c r="B78" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Machine ID</t>
-        </is>
-      </c>
-      <c r="C78" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">id</t>
-        </is>
-      </c>
-      <c r="D78" s="8"/>
-      <c r="E78" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
-      <c r="F78" s="8"/>
-      <c r="G78" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">blank = 1</t>
         </is>
       </c>
       <c r="H78" s="13" t="inlineStr">
@@ -3885,20 +3889,24 @@
       </c>
       <c r="B79" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Connect to</t>
+          <t xml:space="preserve">Machine ID</t>
         </is>
       </c>
       <c r="C79" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">connect</t>
+          <t xml:space="preserve">id</t>
         </is>
       </c>
       <c r="D79" s="8"/>
-      <c r="E79" s="8"/>
+      <c r="E79" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
       <c r="F79" s="8"/>
       <c r="G79" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">the bus its collector starts from: MPT1 (LV), MPT1:TV, a shared collector, HV, POI</t>
+          <t xml:space="preserve">blank = 1</t>
         </is>
       </c>
       <c r="H79" s="13" t="inlineStr">
@@ -3915,12 +3923,12 @@
       </c>
       <c r="B80" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Units</t>
+          <t xml:space="preserve">Connect to</t>
         </is>
       </c>
       <c r="C80" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">units</t>
+          <t xml:space="preserve">connect</t>
         </is>
       </c>
       <c r="D80" s="8"/>
@@ -3928,7 +3936,7 @@
       <c r="F80" s="8"/>
       <c r="G80" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">number of units</t>
+          <t xml:space="preserve">the bus its collector starts from: MPT1 (LV), MPT1:TV, a shared collector, HV, POI</t>
         </is>
       </c>
       <c r="H80" s="13" t="inlineStr">
@@ -3945,24 +3953,20 @@
       </c>
       <c r="B81" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unit MVA</t>
+          <t xml:space="preserve">Units</t>
         </is>
       </c>
       <c r="C81" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">unit_mva</t>
+          <t xml:space="preserve">units</t>
         </is>
       </c>
       <c r="D81" s="8"/>
-      <c r="E81" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">from P and Q</t>
-        </is>
-      </c>
+      <c r="E81" s="8"/>
       <c r="F81" s="8"/>
       <c r="G81" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">one unit (blank = from P and Q)</t>
+          <t xml:space="preserve">number of units</t>
         </is>
       </c>
       <c r="H81" s="13" t="inlineStr">
@@ -3979,18 +3983,26 @@
       </c>
       <c r="B82" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unit Pmax MW</t>
+          <t xml:space="preserve">Unit MVA</t>
         </is>
       </c>
       <c r="C82" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">unit_pmax_mw</t>
+          <t xml:space="preserve">unit_mva</t>
         </is>
       </c>
       <c r="D82" s="8"/>
-      <c r="E82" s="8"/>
+      <c r="E82" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">from P and Q</t>
+        </is>
+      </c>
       <c r="F82" s="8"/>
-      <c r="G82" s="8"/>
+      <c r="G82" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">one unit (blank = from P and Q)</t>
+        </is>
+      </c>
       <c r="H82" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">PSS/E + PSCAD</t>
@@ -4005,26 +4017,18 @@
       </c>
       <c r="B83" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unit Pmin MW</t>
+          <t xml:space="preserve">Unit Pmax MW</t>
         </is>
       </c>
       <c r="C83" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">unit_pmin_mw</t>
+          <t xml:space="preserve">unit_pmax_mw</t>
         </is>
       </c>
       <c r="D83" s="8"/>
-      <c r="E83" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0</t>
-        </is>
-      </c>
+      <c r="E83" s="8"/>
       <c r="F83" s="8"/>
-      <c r="G83" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">BESS charging: negative (blank = 0)</t>
-        </is>
-      </c>
+      <c r="G83" s="8"/>
       <c r="H83" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">PSS/E + PSCAD</t>
@@ -4039,24 +4043,24 @@
       </c>
       <c r="B84" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unit Qmax MVAr</t>
+          <t xml:space="preserve">Unit Pmin MW</t>
         </is>
       </c>
       <c r="C84" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">unit_qmax_mvar</t>
+          <t xml:space="preserve">unit_pmin_mw</t>
         </is>
       </c>
       <c r="D84" s="8"/>
       <c r="E84" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">from Unit PF</t>
+          <t xml:space="preserve">0</t>
         </is>
       </c>
       <c r="F84" s="8"/>
       <c r="G84" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">blank = from Unit PF</t>
+          <t xml:space="preserve">BESS charging: negative (blank = 0)</t>
         </is>
       </c>
       <c r="H84" s="13" t="inlineStr">
@@ -4073,24 +4077,24 @@
       </c>
       <c r="B85" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unit Qmin MVAr</t>
+          <t xml:space="preserve">Unit Qmax MVAr</t>
         </is>
       </c>
       <c r="C85" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">unit_qmin_mvar</t>
+          <t xml:space="preserve">unit_qmax_mvar</t>
         </is>
       </c>
       <c r="D85" s="8"/>
       <c r="E85" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">-Qmax</t>
+          <t xml:space="preserve">from Unit PF</t>
         </is>
       </c>
       <c r="F85" s="8"/>
       <c r="G85" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">blank = -Qmax</t>
+          <t xml:space="preserve">blank = from Unit PF</t>
         </is>
       </c>
       <c r="H85" s="13" t="inlineStr">
@@ -4107,24 +4111,24 @@
       </c>
       <c r="B86" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Unit PF</t>
+          <t xml:space="preserve">Unit Qmin MVAr</t>
         </is>
       </c>
       <c r="C86" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">unit_pf</t>
+          <t xml:space="preserve">unit_qmin_mvar</t>
         </is>
       </c>
       <c r="D86" s="8"/>
       <c r="E86" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.95</t>
+          <t xml:space="preserve">-Qmax</t>
         </is>
       </c>
       <c r="F86" s="8"/>
       <c r="G86" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q at Pmax when Qmax is blank (blank = 0.95)</t>
+          <t xml:space="preserve">blank = -Qmax</t>
         </is>
       </c>
       <c r="H86" s="13" t="inlineStr">
@@ -4141,24 +4145,24 @@
       </c>
       <c r="B87" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Terminal kV</t>
+          <t xml:space="preserve">Unit PF</t>
         </is>
       </c>
       <c r="C87" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">kv</t>
+          <t xml:space="preserve">unit_pf</t>
         </is>
       </c>
       <c r="D87" s="8"/>
       <c r="E87" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSU LV kV</t>
+          <t xml:space="preserve">0.95</t>
         </is>
       </c>
       <c r="F87" s="8"/>
       <c r="G87" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">blank = GSU LV kV</t>
+          <t xml:space="preserve">Q at Pmax when Qmax is blank (blank = 0.95)</t>
         </is>
       </c>
       <c r="H87" s="13" t="inlineStr">
@@ -4167,7 +4171,7 @@
         </is>
       </c>
     </row>
-    <row r="88" ht="30.0" customHeight="1">
+    <row r="88" ht="17.0" customHeight="1">
       <c r="A88" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Generators</t>
@@ -4175,58 +4179,58 @@
       </c>
       <c r="B88" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dispatch MW</t>
+          <t xml:space="preserve">Terminal kV</t>
         </is>
       </c>
       <c r="C88" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">dispatch_mw</t>
+          <t xml:space="preserve">kv</t>
         </is>
       </c>
       <c r="D88" s="8"/>
       <c r="E88" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pmax (BESS charging: negative</t>
+          <t xml:space="preserve">GSU LV kV</t>
         </is>
       </c>
       <c r="F88" s="8"/>
       <c r="G88" s="8" t="inlineStr">
         <is>
+          <t xml:space="preserve">blank = GSU LV kV</t>
+        </is>
+      </c>
+      <c r="H88" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSS/E + PSCAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="30.0" customHeight="1">
+      <c r="A89" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Generators</t>
+        </is>
+      </c>
+      <c r="B89" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dispatch MW</t>
+        </is>
+      </c>
+      <c r="C89" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">dispatch_mw</t>
+        </is>
+      </c>
+      <c r="D89" s="8"/>
+      <c r="E89" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pmax (BESS charging: negative</t>
+        </is>
+      </c>
+      <c r="F89" s="8"/>
+      <c r="G89" s="8" t="inlineStr">
+        <is>
           <t xml:space="preserve">this generator's total; blank = Pmax (BESS charging: negative)</t>
-        </is>
-      </c>
-      <c r="H88" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
-        </is>
-      </c>
-    </row>
-    <row r="89" ht="17.0" customHeight="1">
-      <c r="A89" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Generators</t>
-        </is>
-      </c>
-      <c r="B89" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Q mode</t>
-        </is>
-      </c>
-      <c r="C89" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">q_mode</t>
-        </is>
-      </c>
-      <c r="D89" s="8"/>
-      <c r="E89" s="8"/>
-      <c r="F89" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">share | fixed</t>
-        </is>
-      </c>
-      <c r="G89" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">share: holds the POI with the other share generators | fixed: its own Q</t>
         </is>
       </c>
       <c r="H89" s="13" t="inlineStr">
@@ -4243,24 +4247,24 @@
       </c>
       <c r="B90" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fixed Q MVAr</t>
+          <t xml:space="preserve">Q mode</t>
         </is>
       </c>
       <c r="C90" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">fixed_q_mvar</t>
+          <t xml:space="preserve">q_mode</t>
         </is>
       </c>
       <c r="D90" s="8"/>
-      <c r="E90" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">0</t>
-        </is>
-      </c>
-      <c r="F90" s="8"/>
+      <c r="E90" s="8"/>
+      <c r="F90" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">share | fixed</t>
+        </is>
+      </c>
       <c r="G90" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q mode fixed (blank = 0)</t>
+          <t xml:space="preserve">share: holds the POI with the other share generators | fixed: its own Q</t>
         </is>
       </c>
       <c r="H90" s="13" t="inlineStr">
@@ -4277,20 +4281,24 @@
       </c>
       <c r="B91" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fixed PF</t>
+          <t xml:space="preserve">Fixed Q MVAr</t>
         </is>
       </c>
       <c r="C91" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">fixed_pf</t>
+          <t xml:space="preserve">fixed_q_mvar</t>
         </is>
       </c>
       <c r="D91" s="8"/>
-      <c r="E91" s="8"/>
+      <c r="E91" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0</t>
+        </is>
+      </c>
       <c r="F91" s="8"/>
       <c r="G91" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q mode fixed, instead of Fixed Q (+ lagging)</t>
+          <t xml:space="preserve">Q mode fixed (blank = 0)</t>
         </is>
       </c>
       <c r="H91" s="13" t="inlineStr">
@@ -4307,24 +4315,20 @@
       </c>
       <c r="B92" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSU count</t>
+          <t xml:space="preserve">Fixed PF</t>
         </is>
       </c>
       <c r="C92" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">gsu_count</t>
+          <t xml:space="preserve">fixed_pf</t>
         </is>
       </c>
       <c r="D92" s="8"/>
-      <c r="E92" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Units</t>
-        </is>
-      </c>
+      <c r="E92" s="8"/>
       <c r="F92" s="8"/>
       <c r="G92" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">blank = Units</t>
+          <t xml:space="preserve">Q mode fixed, instead of Fixed Q (+ lagging)</t>
         </is>
       </c>
       <c r="H92" s="13" t="inlineStr">
@@ -4333,7 +4337,7 @@
         </is>
       </c>
     </row>
-    <row r="93" ht="30.0" customHeight="1">
+    <row r="93" ht="17.0" customHeight="1">
       <c r="A93" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Generators</t>
@@ -4341,52 +4345,60 @@
       </c>
       <c r="B93" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSU MVA</t>
+          <t xml:space="preserve">GSU count</t>
         </is>
       </c>
       <c r="C93" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">gsu_mva</t>
+          <t xml:space="preserve">gsu_count</t>
         </is>
       </c>
       <c r="D93" s="8"/>
       <c r="E93" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">no GSU (units on the MV bus</t>
+          <t xml:space="preserve">Units</t>
         </is>
       </c>
       <c r="F93" s="8"/>
       <c r="G93" s="8" t="inlineStr">
         <is>
+          <t xml:space="preserve">blank = Units</t>
+        </is>
+      </c>
+      <c r="H93" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSS/E + PSCAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="30.0" customHeight="1">
+      <c r="A94" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Generators</t>
+        </is>
+      </c>
+      <c r="B94" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GSU MVA</t>
+        </is>
+      </c>
+      <c r="C94" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">gsu_mva</t>
+        </is>
+      </c>
+      <c r="D94" s="8"/>
+      <c r="E94" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">no GSU (units on the MV bus</t>
+        </is>
+      </c>
+      <c r="F94" s="8"/>
+      <c r="G94" s="8" t="inlineStr">
+        <is>
           <t xml:space="preserve">one GSU; blank = no GSU (units on the MV bus)</t>
         </is>
       </c>
-      <c r="H93" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
-        </is>
-      </c>
-    </row>
-    <row r="94" ht="17.0" customHeight="1">
-      <c r="A94" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Generators</t>
-        </is>
-      </c>
-      <c r="B94" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">GSU HV kV</t>
-        </is>
-      </c>
-      <c r="C94" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">gsu_hv_kv</t>
-        </is>
-      </c>
-      <c r="D94" s="8"/>
-      <c r="E94" s="8"/>
-      <c r="F94" s="8"/>
-      <c r="G94" s="8"/>
       <c r="H94" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">PSS/E + PSCAD</t>
@@ -4401,12 +4413,12 @@
       </c>
       <c r="B95" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSU LV kV</t>
+          <t xml:space="preserve">GSU HV kV</t>
         </is>
       </c>
       <c r="C95" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">gsu_lv_kv</t>
+          <t xml:space="preserve">gsu_hv_kv</t>
         </is>
       </c>
       <c r="D95" s="8"/>
@@ -4427,22 +4439,18 @@
       </c>
       <c r="B96" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSU Z %</t>
+          <t xml:space="preserve">GSU LV kV</t>
         </is>
       </c>
       <c r="C96" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">gsu_z_pct</t>
+          <t xml:space="preserve">gsu_lv_kv</t>
         </is>
       </c>
       <c r="D96" s="8"/>
       <c r="E96" s="8"/>
       <c r="F96" s="8"/>
-      <c r="G96" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">on GSU MVA</t>
-        </is>
-      </c>
+      <c r="G96" s="8"/>
       <c r="H96" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">PSS/E + PSCAD</t>
@@ -4457,18 +4465,22 @@
       </c>
       <c r="B97" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSU X/R</t>
+          <t xml:space="preserve">GSU Z %</t>
         </is>
       </c>
       <c r="C97" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">gsu_x_r</t>
+          <t xml:space="preserve">gsu_z_pct</t>
         </is>
       </c>
       <c r="D97" s="8"/>
       <c r="E97" s="8"/>
       <c r="F97" s="8"/>
-      <c r="G97" s="8"/>
+      <c r="G97" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">on GSU MVA</t>
+        </is>
+      </c>
       <c r="H97" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">PSS/E + PSCAD</t>
@@ -4483,12 +4495,12 @@
       </c>
       <c r="B98" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSU vector group</t>
+          <t xml:space="preserve">GSU X/R</t>
         </is>
       </c>
       <c r="C98" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">gsu_vector</t>
+          <t xml:space="preserve">gsu_x_r</t>
         </is>
       </c>
       <c r="D98" s="8"/>
@@ -4509,26 +4521,18 @@
       </c>
       <c r="B99" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">GSU HV tap</t>
+          <t xml:space="preserve">GSU vector group</t>
         </is>
       </c>
       <c r="C99" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">gsu_tap</t>
+          <t xml:space="preserve">gsu_vector</t>
         </is>
       </c>
       <c r="D99" s="8"/>
-      <c r="E99" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
+      <c r="E99" s="8"/>
       <c r="F99" s="8"/>
-      <c r="G99" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">blank = 1</t>
-        </is>
-      </c>
+      <c r="G99" s="8"/>
       <c r="H99" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">PSS/E + PSCAD</t>
@@ -4543,24 +4547,24 @@
       </c>
       <c r="B100" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Collector</t>
+          <t xml:space="preserve">GSU HV tap</t>
         </is>
       </c>
       <c r="C100" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">collector</t>
+          <t xml:space="preserve">gsu_tap</t>
         </is>
       </c>
       <c r="D100" s="8"/>
-      <c r="E100" s="8"/>
-      <c r="F100" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FEEDERS | EQUIVALENT | NONE</t>
-        </is>
-      </c>
+      <c r="E100" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="F100" s="8"/>
       <c r="G100" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">FEEDERS: WECC equivalent of its Feeders rows | EQUIVALENT: R X B here | NONE</t>
+          <t xml:space="preserve">blank = 1</t>
         </is>
       </c>
       <c r="H100" s="13" t="inlineStr">
@@ -4577,20 +4581,24 @@
       </c>
       <c r="B101" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Collector R</t>
+          <t xml:space="preserve">Collector</t>
         </is>
       </c>
       <c r="C101" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">coll_r</t>
+          <t xml:space="preserve">collector</t>
         </is>
       </c>
       <c r="D101" s="8"/>
       <c r="E101" s="8"/>
-      <c r="F101" s="8"/>
+      <c r="F101" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">FEEDERS | EQUIVALENT | NONE</t>
+        </is>
+      </c>
       <c r="G101" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">EQUIVALENT</t>
+          <t xml:space="preserve">FEEDERS: WECC equivalent of its Feeders rows | EQUIVALENT: R X B here | NONE</t>
         </is>
       </c>
       <c r="H101" s="13" t="inlineStr">
@@ -4607,12 +4615,12 @@
       </c>
       <c r="B102" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Collector X</t>
+          <t xml:space="preserve">Collector R</t>
         </is>
       </c>
       <c r="C102" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">coll_x</t>
+          <t xml:space="preserve">coll_r</t>
         </is>
       </c>
       <c r="D102" s="8"/>
@@ -4637,12 +4645,12 @@
       </c>
       <c r="B103" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Collector B</t>
+          <t xml:space="preserve">Collector X</t>
         </is>
       </c>
       <c r="C103" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">coll_b</t>
+          <t xml:space="preserve">coll_x</t>
         </is>
       </c>
       <c r="D103" s="8"/>
@@ -4650,7 +4658,7 @@
       <c r="F103" s="8"/>
       <c r="G103" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">EQUIVALENT, total charging</t>
+          <t xml:space="preserve">EQUIVALENT</t>
         </is>
       </c>
       <c r="H103" s="13" t="inlineStr">
@@ -4667,24 +4675,20 @@
       </c>
       <c r="B104" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Collector units</t>
+          <t xml:space="preserve">Collector B</t>
         </is>
       </c>
       <c r="C104" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">coll_units</t>
+          <t xml:space="preserve">coll_b</t>
         </is>
       </c>
       <c r="D104" s="8"/>
       <c r="E104" s="8"/>
-      <c r="F104" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">pu | ohm</t>
-        </is>
-      </c>
+      <c r="F104" s="8"/>
       <c r="G104" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">pu: system base at collector kV | ohm: R X in ohm, B in uS</t>
+          <t xml:space="preserve">EQUIVALENT, total charging</t>
         </is>
       </c>
       <c r="H104" s="13" t="inlineStr">
@@ -4701,25 +4705,29 @@
       </c>
       <c r="B105" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">ZSORCE X pu</t>
+          <t xml:space="preserve">Collector units</t>
         </is>
       </c>
       <c r="C105" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">zsorce_x</t>
+          <t xml:space="preserve">coll_units</t>
         </is>
       </c>
       <c r="D105" s="8"/>
       <c r="E105" s="8"/>
-      <c r="F105" s="8"/>
+      <c r="F105" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pu | ohm</t>
+        </is>
+      </c>
       <c r="G105" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">on MBASE (blank: inverters 9999, SYNC X''d)</t>
+          <t xml:space="preserve">pu: system base at collector kV | ohm: R X in ohm, B in uS</t>
         </is>
       </c>
       <c r="H105" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E .dyr</t>
+          <t xml:space="preserve">PSS/E + PSCAD</t>
         </is>
       </c>
     </row>
@@ -4731,12 +4739,12 @@
       </c>
       <c r="B106" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">WMOD</t>
+          <t xml:space="preserve">ZSORCE X pu</t>
         </is>
       </c>
       <c r="C106" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">wmod</t>
+          <t xml:space="preserve">zsorce_x</t>
         </is>
       </c>
       <c r="D106" s="8"/>
@@ -4744,84 +4752,80 @@
       <c r="F106" s="8"/>
       <c r="G106" s="8" t="inlineStr">
         <is>
+          <t xml:space="preserve">on MBASE (blank: inverters 9999, SYNC X''d)</t>
+        </is>
+      </c>
+      <c r="H106" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSS/E .dyr</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="17.0" customHeight="1">
+      <c r="A107" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Generators</t>
+        </is>
+      </c>
+      <c r="B107" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">WMOD</t>
+        </is>
+      </c>
+      <c r="C107" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">wmod</t>
+        </is>
+      </c>
+      <c r="D107" s="8"/>
+      <c r="E107" s="8"/>
+      <c r="F107" s="8"/>
+      <c r="G107" s="8" t="inlineStr">
+        <is>
           <t xml:space="preserve">blank: inverters 1, SYNC 0</t>
         </is>
       </c>
-      <c r="H106" s="13" t="inlineStr">
+      <c r="H107" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">PSS/E .dyr</t>
         </is>
       </c>
     </row>
-    <row r="107" ht="30.0" customHeight="1">
-      <c r="A107" s="8" t="inlineStr">
+    <row r="108" ht="30.0" customHeight="1">
+      <c r="A108" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Generators</t>
         </is>
       </c>
-      <c r="B107" s="12" t="inlineStr">
+      <c r="B108" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Electrical control</t>
         </is>
       </c>
-      <c r="C107" s="8" t="inlineStr">
+      <c r="C108" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">reec</t>
-        </is>
-      </c>
-      <c r="D107" s="8"/>
-      <c r="E107" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">REEC_A, BESS REEC_C</t>
-        </is>
-      </c>
-      <c r="F107" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">REEC_A | REEC_C | REEC_D</t>
-        </is>
-      </c>
-      <c r="G107" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSS/E .dyr -- REEC_A: PV, WT | REEC_C: BESS | REEC_D: PV, BESS, WT4 (blank = REEC_A, BESS REEC_C)</t>
-        </is>
-      </c>
-      <c r="H107" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSS/E .dyr</t>
-        </is>
-      </c>
-    </row>
-    <row r="108" ht="17.0" customHeight="1">
-      <c r="A108" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Generators</t>
-        </is>
-      </c>
-      <c r="B108" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSCAD library</t>
-        </is>
-      </c>
-      <c r="C108" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">pscad_library</t>
         </is>
       </c>
       <c r="D108" s="8"/>
       <c r="E108" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">none</t>
-        </is>
-      </c>
-      <c r="F108" s="8"/>
+          <t xml:space="preserve">REEC_A, BESS REEC_C</t>
+        </is>
+      </c>
+      <c r="F108" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REEC_A | REEC_C | REEC_D</t>
+        </is>
+      </c>
       <c r="G108" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">vendor library .pslx (blank = none)</t>
+          <t xml:space="preserve">PSS/E .dyr -- REEC_A: PV, WT | REEC_C: BESS | REEC_D: PV, BESS, WT4 (blank = REEC_A, BESS REEC_C)</t>
         </is>
       </c>
       <c r="H108" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSCAD</t>
+          <t xml:space="preserve">PSS/E .dyr</t>
         </is>
       </c>
     </row>
@@ -4833,24 +4837,24 @@
       </c>
       <c r="B109" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSCAD definition</t>
+          <t xml:space="preserve">PSCAD library</t>
         </is>
       </c>
       <c r="C109" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">pscad_definition</t>
+          <t xml:space="preserve">pscad_library</t>
         </is>
       </c>
       <c r="D109" s="8"/>
       <c r="E109" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">a source: network check</t>
+          <t xml:space="preserve">none</t>
         </is>
       </c>
       <c r="F109" s="8"/>
       <c r="G109" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">vendor model, library:name (blank = a source: network check)</t>
+          <t xml:space="preserve">vendor library .pslx (blank = none)</t>
         </is>
       </c>
       <c r="H109" s="13" t="inlineStr">
@@ -4867,24 +4871,24 @@
       </c>
       <c r="B110" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSCAD AC port</t>
+          <t xml:space="preserve">PSCAD definition</t>
         </is>
       </c>
       <c r="C110" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">pscad_ac_port</t>
+          <t xml:space="preserve">pscad_definition</t>
         </is>
       </c>
       <c r="D110" s="8"/>
       <c r="E110" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">its 3-phase port</t>
+          <t xml:space="preserve">a source: network check</t>
         </is>
       </c>
       <c r="F110" s="8"/>
       <c r="G110" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">its AC port (blank = its 3-phase port)</t>
+          <t xml:space="preserve">vendor model, library:name (blank = a source: network check)</t>
         </is>
       </c>
       <c r="H110" s="13" t="inlineStr">
@@ -4893,7 +4897,7 @@
         </is>
       </c>
     </row>
-    <row r="111" ht="30.0" customHeight="1">
+    <row r="111" ht="17.0" customHeight="1">
       <c r="A111" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Generators</t>
@@ -4901,79 +4905,83 @@
       </c>
       <c r="B111" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSCAD inverter at</t>
+          <t xml:space="preserve">PSCAD AC port</t>
         </is>
       </c>
       <c r="C111" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">pscad_inv_at</t>
+          <t xml:space="preserve">pscad_ac_port</t>
         </is>
       </c>
       <c r="D111" s="8"/>
       <c r="E111" s="8" t="inlineStr">
         <is>
+          <t xml:space="preserve">its 3-phase port</t>
+        </is>
+      </c>
+      <c r="F111" s="8"/>
+      <c r="G111" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">its AC port (blank = its 3-phase port)</t>
+        </is>
+      </c>
+      <c r="H111" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="112" ht="30.0" customHeight="1">
+      <c r="A112" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Generators</t>
+        </is>
+      </c>
+      <c r="B112" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD inverter at</t>
+        </is>
+      </c>
+      <c r="C112" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pscad_inv_at</t>
+        </is>
+      </c>
+      <c r="D112" s="8"/>
+      <c r="E112" s="8" t="inlineStr">
+        <is>
           <t xml:space="preserve">LV</t>
         </is>
       </c>
-      <c r="F111" s="8" t="inlineStr">
+      <c r="F112" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">LV | MV</t>
         </is>
       </c>
-      <c r="G111" s="8" t="inlineStr">
+      <c r="G112" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">LV: the inverter (your UDM or the stand-in source) on the GSU's LV side, the GSU built | MV: on its HV side, for a UDM with its GSU inside (blank = LV)</t>
         </is>
       </c>
-      <c r="H111" s="13" t="inlineStr">
+      <c r="H112" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">PSCAD</t>
         </is>
       </c>
     </row>
-    <row r="112" ht="18" customHeight="1">
-      <c r="A112" s="7" t="inlineStr">
+    <row r="113" ht="18" customHeight="1">
+      <c r="A113" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Feeders</t>
         </is>
       </c>
-      <c r="B112" s="7"/>
-      <c r="C112" s="7"/>
-      <c r="D112" s="7"/>
-      <c r="E112" s="7"/>
-      <c r="F112" s="7"/>
-      <c r="G112" s="7"/>
-      <c r="H112" s="7"/>
-    </row>
-    <row r="113" ht="17.0" customHeight="1">
-      <c r="A113" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Feeders</t>
-        </is>
-      </c>
-      <c r="B113" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Collector</t>
-        </is>
-      </c>
-      <c r="C113" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">collector</t>
-        </is>
-      </c>
-      <c r="D113" s="8"/>
-      <c r="E113" s="8"/>
-      <c r="F113" s="8"/>
-      <c r="G113" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">the generator (its own collector) or a shared collector</t>
-        </is>
-      </c>
-      <c r="H113" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
-        </is>
-      </c>
+      <c r="B113" s="7"/>
+      <c r="C113" s="7"/>
+      <c r="D113" s="7"/>
+      <c r="E113" s="7"/>
+      <c r="F113" s="7"/>
+      <c r="G113" s="7"/>
+      <c r="H113" s="7"/>
     </row>
     <row r="114" ht="17.0" customHeight="1">
       <c r="A114" s="8" t="inlineStr">
@@ -4983,12 +4991,12 @@
       </c>
       <c r="B114" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Feeder</t>
+          <t xml:space="preserve">Collector</t>
         </is>
       </c>
       <c r="C114" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">feeder</t>
+          <t xml:space="preserve">collector</t>
         </is>
       </c>
       <c r="D114" s="8"/>
@@ -4996,7 +5004,7 @@
       <c r="F114" s="8"/>
       <c r="G114" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">feeder name</t>
+          <t xml:space="preserve">the generator (its own collector) or a shared collector</t>
         </is>
       </c>
       <c r="H114" s="13" t="inlineStr">
@@ -5013,24 +5021,20 @@
       </c>
       <c r="B115" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Copies</t>
+          <t xml:space="preserve">Feeder</t>
         </is>
       </c>
       <c r="C115" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">copies</t>
+          <t xml:space="preserve">feeder</t>
         </is>
       </c>
       <c r="D115" s="8"/>
-      <c r="E115" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
+      <c r="E115" s="8"/>
       <c r="F115" s="8"/>
       <c r="G115" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">identical feeders (blank = 1)</t>
+          <t xml:space="preserve">feeder name</t>
         </is>
       </c>
       <c r="H115" s="13" t="inlineStr">
@@ -5047,20 +5051,24 @@
       </c>
       <c r="B116" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Section</t>
+          <t xml:space="preserve">Copies</t>
         </is>
       </c>
       <c r="C116" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">section</t>
+          <t xml:space="preserve">copies</t>
         </is>
       </c>
       <c r="D116" s="8"/>
-      <c r="E116" s="8"/>
+      <c r="E116" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
       <c r="F116" s="8"/>
       <c r="G116" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">1, 2, 3 ... from the collector bus out</t>
+          <t xml:space="preserve">identical feeders (blank = 1)</t>
         </is>
       </c>
       <c r="H116" s="13" t="inlineStr">
@@ -5069,7 +5077,7 @@
         </is>
       </c>
     </row>
-    <row r="117" ht="30.0" customHeight="1">
+    <row r="117" ht="17.0" customHeight="1">
       <c r="A117" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Feeders</t>
@@ -5077,24 +5085,20 @@
       </c>
       <c r="B117" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">From section</t>
+          <t xml:space="preserve">Section</t>
         </is>
       </c>
       <c r="C117" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">from_section</t>
+          <t xml:space="preserve">section</t>
         </is>
       </c>
       <c r="D117" s="8"/>
-      <c r="E117" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">the one before (daisy chain</t>
-        </is>
-      </c>
+      <c r="E117" s="8"/>
       <c r="F117" s="8"/>
       <c r="G117" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">blank = the one before (daisy chain) | 0 = the collector bus | n = a lateral off the end of section n</t>
+          <t xml:space="preserve">1, 2, 3 ... from the collector bus out</t>
         </is>
       </c>
       <c r="H117" s="13" t="inlineStr">
@@ -5103,7 +5107,7 @@
         </is>
       </c>
     </row>
-    <row r="118" ht="17.0" customHeight="1">
+    <row r="118" ht="30.0" customHeight="1">
       <c r="A118" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Feeders</t>
@@ -5111,20 +5115,24 @@
       </c>
       <c r="B118" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cable</t>
+          <t xml:space="preserve">From section</t>
         </is>
       </c>
       <c r="C118" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">cable</t>
+          <t xml:space="preserve">from_section</t>
         </is>
       </c>
       <c r="D118" s="8"/>
-      <c r="E118" s="8"/>
+      <c r="E118" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the one before (daisy chain</t>
+        </is>
+      </c>
       <c r="F118" s="8"/>
       <c r="G118" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">from Cables</t>
+          <t xml:space="preserve">blank = the one before (daisy chain) | 0 = the collector bus | n = a lateral off the end of section n</t>
         </is>
       </c>
       <c r="H118" s="13" t="inlineStr">
@@ -5141,18 +5149,22 @@
       </c>
       <c r="B119" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Length</t>
+          <t xml:space="preserve">Cable</t>
         </is>
       </c>
       <c r="C119" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">length</t>
+          <t xml:space="preserve">cable</t>
         </is>
       </c>
       <c r="D119" s="8"/>
       <c r="E119" s="8"/>
       <c r="F119" s="8"/>
-      <c r="G119" s="8"/>
+      <c r="G119" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">from Cables</t>
+        </is>
+      </c>
       <c r="H119" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">PSS/E + PSCAD</t>
@@ -5167,30 +5179,18 @@
       </c>
       <c r="B120" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Length unit</t>
+          <t xml:space="preserve">Length</t>
         </is>
       </c>
       <c r="C120" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">unit</t>
+          <t xml:space="preserve">length</t>
         </is>
       </c>
       <c r="D120" s="8"/>
-      <c r="E120" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">km</t>
-        </is>
-      </c>
-      <c r="F120" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">km | mi | kft | m | ft</t>
-        </is>
-      </c>
-      <c r="G120" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">blank = km</t>
-        </is>
-      </c>
+      <c r="E120" s="8"/>
+      <c r="F120" s="8"/>
+      <c r="G120" s="8"/>
       <c r="H120" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">PSS/E + PSCAD</t>
@@ -5205,20 +5205,28 @@
       </c>
       <c r="B121" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Units at end</t>
+          <t xml:space="preserve">Length unit</t>
         </is>
       </c>
       <c r="C121" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">units</t>
+          <t xml:space="preserve">unit</t>
         </is>
       </c>
       <c r="D121" s="8"/>
-      <c r="E121" s="8"/>
-      <c r="F121" s="8"/>
+      <c r="E121" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">km</t>
+        </is>
+      </c>
+      <c r="F121" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">km | mi | kft | m | ft</t>
+        </is>
+      </c>
       <c r="G121" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">units tapped at the far end</t>
+          <t xml:space="preserve">blank = km</t>
         </is>
       </c>
       <c r="H121" s="13" t="inlineStr">
@@ -5235,12 +5243,12 @@
       </c>
       <c r="B122" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Units of</t>
+          <t xml:space="preserve">Units at end</t>
         </is>
       </c>
       <c r="C122" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">units_of</t>
+          <t xml:space="preserve">units</t>
         </is>
       </c>
       <c r="D122" s="8"/>
@@ -5248,7 +5256,7 @@
       <c r="F122" s="8"/>
       <c r="G122" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">shared collectors: whose units (repeat the section for another generator's)</t>
+          <t xml:space="preserve">units tapped at the far end</t>
         </is>
       </c>
       <c r="H122" s="13" t="inlineStr">
@@ -5265,75 +5273,75 @@
       </c>
       <c r="B123" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Parallel cables</t>
+          <t xml:space="preserve">Units of</t>
         </is>
       </c>
       <c r="C123" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">parallel</t>
+          <t xml:space="preserve">units_of</t>
         </is>
       </c>
       <c r="D123" s="8"/>
-      <c r="E123" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
+      <c r="E123" s="8"/>
       <c r="F123" s="8"/>
       <c r="G123" s="8" t="inlineStr">
         <is>
+          <t xml:space="preserve">shared collectors: whose units (repeat the section for another generator's)</t>
+        </is>
+      </c>
+      <c r="H123" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSS/E + PSCAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="124" ht="17.0" customHeight="1">
+      <c r="A124" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Feeders</t>
+        </is>
+      </c>
+      <c r="B124" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Parallel cables</t>
+        </is>
+      </c>
+      <c r="C124" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">parallel</t>
+        </is>
+      </c>
+      <c r="D124" s="8"/>
+      <c r="E124" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
+      <c r="F124" s="8"/>
+      <c r="G124" s="8" t="inlineStr">
+        <is>
           <t xml:space="preserve">blank = 1</t>
         </is>
       </c>
-      <c r="H123" s="13" t="inlineStr">
+      <c r="H124" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">PSS/E + PSCAD</t>
         </is>
       </c>
     </row>
-    <row r="124" ht="18" customHeight="1">
-      <c r="A124" s="7" t="inlineStr">
+    <row r="125" ht="18" customHeight="1">
+      <c r="A125" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Cables</t>
         </is>
       </c>
-      <c r="B124" s="7"/>
-      <c r="C124" s="7"/>
-      <c r="D124" s="7"/>
-      <c r="E124" s="7"/>
-      <c r="F124" s="7"/>
-      <c r="G124" s="7"/>
-      <c r="H124" s="7"/>
-    </row>
-    <row r="125" ht="17.0" customHeight="1">
-      <c r="A125" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Cables</t>
-        </is>
-      </c>
-      <c r="B125" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Cable</t>
-        </is>
-      </c>
-      <c r="C125" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">cable</t>
-        </is>
-      </c>
-      <c r="D125" s="8"/>
-      <c r="E125" s="8"/>
-      <c r="F125" s="8"/>
-      <c r="G125" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">cable type</t>
-        </is>
-      </c>
-      <c r="H125" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
-        </is>
-      </c>
+      <c r="B125" s="7"/>
+      <c r="C125" s="7"/>
+      <c r="D125" s="7"/>
+      <c r="E125" s="7"/>
+      <c r="F125" s="7"/>
+      <c r="G125" s="7"/>
+      <c r="H125" s="7"/>
     </row>
     <row r="126" ht="17.0" customHeight="1">
       <c r="A126" s="8" t="inlineStr">
@@ -5343,24 +5351,20 @@
       </c>
       <c r="B126" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Length unit</t>
+          <t xml:space="preserve">Cable</t>
         </is>
       </c>
       <c r="C126" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">unit</t>
+          <t xml:space="preserve">cable</t>
         </is>
       </c>
       <c r="D126" s="8"/>
       <c r="E126" s="8"/>
-      <c r="F126" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">km | mi | kft | m | ft</t>
-        </is>
-      </c>
+      <c r="F126" s="8"/>
       <c r="G126" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">the values are per</t>
+          <t xml:space="preserve">cable type</t>
         </is>
       </c>
       <c r="H126" s="13" t="inlineStr">
@@ -5377,20 +5381,24 @@
       </c>
       <c r="B127" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">R per length</t>
+          <t xml:space="preserve">Length unit</t>
         </is>
       </c>
       <c r="C127" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">r_per</t>
+          <t xml:space="preserve">unit</t>
         </is>
       </c>
       <c r="D127" s="8"/>
       <c r="E127" s="8"/>
-      <c r="F127" s="8"/>
+      <c r="F127" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">km | mi | kft | m | ft</t>
+        </is>
+      </c>
       <c r="G127" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">ohm, at operating temperature</t>
+          <t xml:space="preserve">the values are per</t>
         </is>
       </c>
       <c r="H127" s="13" t="inlineStr">
@@ -5407,12 +5415,12 @@
       </c>
       <c r="B128" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">X per length</t>
+          <t xml:space="preserve">R per length</t>
         </is>
       </c>
       <c r="C128" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">x_per</t>
+          <t xml:space="preserve">r_per</t>
         </is>
       </c>
       <c r="D128" s="8"/>
@@ -5420,7 +5428,7 @@
       <c r="F128" s="8"/>
       <c r="G128" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">ohm</t>
+          <t xml:space="preserve">ohm, at operating temperature</t>
         </is>
       </c>
       <c r="H128" s="13" t="inlineStr">
@@ -5437,12 +5445,12 @@
       </c>
       <c r="B129" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">C per length</t>
+          <t xml:space="preserve">X per length</t>
         </is>
       </c>
       <c r="C129" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">c_per</t>
+          <t xml:space="preserve">x_per</t>
         </is>
       </c>
       <c r="D129" s="8"/>
@@ -5450,7 +5458,7 @@
       <c r="F129" s="8"/>
       <c r="G129" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">uF</t>
+          <t xml:space="preserve">ohm</t>
         </is>
       </c>
       <c r="H129" s="13" t="inlineStr">
@@ -5467,12 +5475,12 @@
       </c>
       <c r="B130" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">B per length</t>
+          <t xml:space="preserve">C per length</t>
         </is>
       </c>
       <c r="C130" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">b_per</t>
+          <t xml:space="preserve">c_per</t>
         </is>
       </c>
       <c r="D130" s="8"/>
@@ -5480,58 +5488,58 @@
       <c r="F130" s="8"/>
       <c r="G130" s="8" t="inlineStr">
         <is>
+          <t xml:space="preserve">uF</t>
+        </is>
+      </c>
+      <c r="H130" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSS/E + PSCAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="131" ht="17.0" customHeight="1">
+      <c r="A131" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cables</t>
+        </is>
+      </c>
+      <c r="B131" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">B per length</t>
+        </is>
+      </c>
+      <c r="C131" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">b_per</t>
+        </is>
+      </c>
+      <c r="D131" s="8"/>
+      <c r="E131" s="8"/>
+      <c r="F131" s="8"/>
+      <c r="G131" s="8" t="inlineStr">
+        <is>
           <t xml:space="preserve">uS, instead of C</t>
         </is>
       </c>
-      <c r="H130" s="13" t="inlineStr">
+      <c r="H131" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">PSS/E + PSCAD</t>
         </is>
       </c>
     </row>
-    <row r="131" ht="18" customHeight="1">
-      <c r="A131" s="7" t="inlineStr">
+    <row r="132" ht="18" customHeight="1">
+      <c r="A132" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Collectors</t>
         </is>
       </c>
-      <c r="B131" s="7"/>
-      <c r="C131" s="7"/>
-      <c r="D131" s="7"/>
-      <c r="E131" s="7"/>
-      <c r="F131" s="7"/>
-      <c r="G131" s="7"/>
-      <c r="H131" s="7"/>
-    </row>
-    <row r="132" ht="17.0" customHeight="1">
-      <c r="A132" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Collectors</t>
-        </is>
-      </c>
-      <c r="B132" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Name</t>
-        </is>
-      </c>
-      <c r="C132" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">name</t>
-        </is>
-      </c>
-      <c r="D132" s="8"/>
-      <c r="E132" s="8"/>
-      <c r="F132" s="8"/>
-      <c r="G132" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">shared collector: its far-end bus has this name</t>
-        </is>
-      </c>
-      <c r="H132" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
-        </is>
-      </c>
+      <c r="B132" s="7"/>
+      <c r="C132" s="7"/>
+      <c r="D132" s="7"/>
+      <c r="E132" s="7"/>
+      <c r="F132" s="7"/>
+      <c r="G132" s="7"/>
+      <c r="H132" s="7"/>
     </row>
     <row r="133" ht="17.0" customHeight="1">
       <c r="A133" s="8" t="inlineStr">
@@ -5541,12 +5549,12 @@
       </c>
       <c r="B133" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Connect to</t>
+          <t xml:space="preserve">Name</t>
         </is>
       </c>
       <c r="C133" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">connect</t>
+          <t xml:space="preserve">name</t>
         </is>
       </c>
       <c r="D133" s="8"/>
@@ -5554,62 +5562,58 @@
       <c r="F133" s="8"/>
       <c r="G133" s="8" t="inlineStr">
         <is>
+          <t xml:space="preserve">shared collector: its far-end bus has this name</t>
+        </is>
+      </c>
+      <c r="H133" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSS/E + PSCAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="134" ht="17.0" customHeight="1">
+      <c r="A134" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Collectors</t>
+        </is>
+      </c>
+      <c r="B134" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Connect to</t>
+        </is>
+      </c>
+      <c r="C134" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">connect</t>
+        </is>
+      </c>
+      <c r="D134" s="8"/>
+      <c r="E134" s="8"/>
+      <c r="F134" s="8"/>
+      <c r="G134" s="8" t="inlineStr">
+        <is>
           <t xml:space="preserve">the bus it starts from (MPT1, MPT1:TV ...)</t>
         </is>
       </c>
-      <c r="H133" s="13" t="inlineStr">
+      <c r="H134" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">PSS/E + PSCAD</t>
         </is>
       </c>
     </row>
-    <row r="134" ht="18" customHeight="1">
-      <c r="A134" s="7" t="inlineStr">
+    <row r="135" ht="18" customHeight="1">
+      <c r="A135" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Loads_Shunts</t>
         </is>
       </c>
-      <c r="B134" s="7"/>
-      <c r="C134" s="7"/>
-      <c r="D134" s="7"/>
-      <c r="E134" s="7"/>
-      <c r="F134" s="7"/>
-      <c r="G134" s="7"/>
-      <c r="H134" s="7"/>
-    </row>
-    <row r="135" ht="17.0" customHeight="1">
-      <c r="A135" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Loads_Shunts</t>
-        </is>
-      </c>
-      <c r="B135" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Kind</t>
-        </is>
-      </c>
-      <c r="C135" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">kind</t>
-        </is>
-      </c>
-      <c r="D135" s="8"/>
-      <c r="E135" s="8"/>
-      <c r="F135" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LOAD | SHUNT</t>
-        </is>
-      </c>
-      <c r="G135" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LOAD: constant impedance | SHUNT: + capacitor, - reactor</t>
-        </is>
-      </c>
-      <c r="H135" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
-        </is>
-      </c>
+      <c r="B135" s="7"/>
+      <c r="C135" s="7"/>
+      <c r="D135" s="7"/>
+      <c r="E135" s="7"/>
+      <c r="F135" s="7"/>
+      <c r="G135" s="7"/>
+      <c r="H135" s="7"/>
     </row>
     <row r="136" ht="17.0" customHeight="1">
       <c r="A136" s="8" t="inlineStr">
@@ -5619,20 +5623,24 @@
       </c>
       <c r="B136" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">At bus</t>
+          <t xml:space="preserve">Kind</t>
         </is>
       </c>
       <c r="C136" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">at</t>
+          <t xml:space="preserve">kind</t>
         </is>
       </c>
       <c r="D136" s="8"/>
       <c r="E136" s="8"/>
-      <c r="F136" s="8"/>
+      <c r="F136" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LOAD | SHUNT</t>
+        </is>
+      </c>
       <c r="G136" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">POI, HV, MPT1, MPT1:TV, PV:MV, PV ...</t>
+          <t xml:space="preserve">LOAD: constant impedance | SHUNT: + capacitor, - reactor</t>
         </is>
       </c>
       <c r="H136" s="13" t="inlineStr">
@@ -5649,12 +5657,12 @@
       </c>
       <c r="B137" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">MW</t>
+          <t xml:space="preserve">At bus</t>
         </is>
       </c>
       <c r="C137" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">mw</t>
+          <t xml:space="preserve">at</t>
         </is>
       </c>
       <c r="D137" s="8"/>
@@ -5662,7 +5670,7 @@
       <c r="F137" s="8"/>
       <c r="G137" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">LOAD, at 1 pu</t>
+          <t xml:space="preserve">POI, HV, MPT1, MPT1:TV, PV:MV, PV ...</t>
         </is>
       </c>
       <c r="H137" s="13" t="inlineStr">
@@ -5679,12 +5687,12 @@
       </c>
       <c r="B138" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">MVAr</t>
+          <t xml:space="preserve">MW</t>
         </is>
       </c>
       <c r="C138" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">mvar</t>
+          <t xml:space="preserve">mw</t>
         </is>
       </c>
       <c r="D138" s="8"/>
@@ -5692,7 +5700,7 @@
       <c r="F138" s="8"/>
       <c r="G138" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">at 1 pu: LOAD + inductive | SHUNT + capacitive</t>
+          <t xml:space="preserve">LOAD, at 1 pu</t>
         </is>
       </c>
       <c r="H138" s="13" t="inlineStr">
@@ -5709,67 +5717,67 @@
       </c>
       <c r="B139" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Name</t>
+          <t xml:space="preserve">MVAr</t>
         </is>
       </c>
       <c r="C139" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">name</t>
+          <t xml:space="preserve">mvar</t>
         </is>
       </c>
       <c r="D139" s="8"/>
       <c r="E139" s="8"/>
       <c r="F139" s="8"/>
-      <c r="G139" s="8"/>
+      <c r="G139" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">at 1 pu: LOAD + inductive | SHUNT + capacitive</t>
+        </is>
+      </c>
       <c r="H139" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">PSS/E + PSCAD</t>
         </is>
       </c>
     </row>
-    <row r="140" ht="18" customHeight="1">
-      <c r="A140" s="7" t="inlineStr">
+    <row r="140" ht="17.0" customHeight="1">
+      <c r="A140" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Loads_Shunts</t>
+        </is>
+      </c>
+      <c r="B140" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Name</t>
+        </is>
+      </c>
+      <c r="C140" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">name</t>
+        </is>
+      </c>
+      <c r="D140" s="8"/>
+      <c r="E140" s="8"/>
+      <c r="F140" s="8"/>
+      <c r="G140" s="8"/>
+      <c r="H140" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSS/E + PSCAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="141" ht="18" customHeight="1">
+      <c r="A141" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Bus_Numbers</t>
         </is>
       </c>
-      <c r="B140" s="7"/>
-      <c r="C140" s="7"/>
-      <c r="D140" s="7"/>
-      <c r="E140" s="7"/>
-      <c r="F140" s="7"/>
-      <c r="G140" s="7"/>
-      <c r="H140" s="7"/>
-    </row>
-    <row r="141" ht="17.0" customHeight="1">
-      <c r="A141" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bus_Numbers</t>
-        </is>
-      </c>
-      <c r="B141" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bus</t>
-        </is>
-      </c>
-      <c r="C141" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">bus</t>
-        </is>
-      </c>
-      <c r="D141" s="8"/>
-      <c r="E141" s="8"/>
-      <c r="F141" s="8"/>
-      <c r="G141" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">its role: IB, POI, HV, MPT1:LV, PV:MV, PV:LV ...</t>
-        </is>
-      </c>
-      <c r="H141" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
-        </is>
-      </c>
+      <c r="B141" s="7"/>
+      <c r="C141" s="7"/>
+      <c r="D141" s="7"/>
+      <c r="E141" s="7"/>
+      <c r="F141" s="7"/>
+      <c r="G141" s="7"/>
+      <c r="H141" s="7"/>
     </row>
     <row r="142" ht="17.0" customHeight="1">
       <c r="A142" s="8" t="inlineStr">
@@ -5779,24 +5787,20 @@
       </c>
       <c r="B142" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Number</t>
+          <t xml:space="preserve">Bus</t>
         </is>
       </c>
       <c r="C142" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">bus</t>
         </is>
       </c>
       <c r="D142" s="8"/>
-      <c r="E142" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">automatic</t>
-        </is>
-      </c>
+      <c r="E142" s="8"/>
       <c r="F142" s="8"/>
       <c r="G142" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">blank = automatic</t>
+          <t xml:space="preserve">its role: IB, POI, HV, MPT1:LV, PV:MV, PV:LV ...</t>
         </is>
       </c>
       <c r="H142" s="13" t="inlineStr">
@@ -5805,7 +5809,7 @@
         </is>
       </c>
     </row>
-    <row r="143" ht="30.0" customHeight="1">
+    <row r="143" ht="17.0" customHeight="1">
       <c r="A143" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Bus_Numbers</t>
@@ -5813,90 +5817,94 @@
       </c>
       <c r="B143" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Name</t>
+          <t xml:space="preserve">Number</t>
         </is>
       </c>
       <c r="C143" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">name</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D143" s="8"/>
       <c r="E143" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">automatic (12 characters at most</t>
+          <t xml:space="preserve">automatic</t>
         </is>
       </c>
       <c r="F143" s="8"/>
       <c r="G143" s="8" t="inlineStr">
         <is>
+          <t xml:space="preserve">blank = automatic</t>
+        </is>
+      </c>
+      <c r="H143" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSS/E + PSCAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="144" ht="30.0" customHeight="1">
+      <c r="A144" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bus_Numbers</t>
+        </is>
+      </c>
+      <c r="B144" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Name</t>
+        </is>
+      </c>
+      <c r="C144" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">name</t>
+        </is>
+      </c>
+      <c r="D144" s="8"/>
+      <c r="E144" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">automatic (12 characters at most</t>
+        </is>
+      </c>
+      <c r="F144" s="8"/>
+      <c r="G144" s="8" t="inlineStr">
+        <is>
           <t xml:space="preserve">blank = automatic (12 characters at most)</t>
         </is>
       </c>
-      <c r="H143" s="13" t="inlineStr">
+      <c r="H144" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">PSS/E + PSCAD</t>
         </is>
       </c>
     </row>
-    <row r="144" ht="18" customHeight="1">
-      <c r="A144" s="7" t="inlineStr">
+    <row r="145" ht="18" customHeight="1">
+      <c r="A145" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Dyr_Params</t>
         </is>
       </c>
-      <c r="B144" s="7"/>
-      <c r="C144" s="7"/>
-      <c r="D144" s="7"/>
-      <c r="E144" s="7"/>
-      <c r="F144" s="7"/>
-      <c r="G144" s="7"/>
-      <c r="H144" s="7"/>
-    </row>
-    <row r="145" ht="17.0" customHeight="1">
-      <c r="A145" s="8" t="inlineStr">
+      <c r="B145" s="7"/>
+      <c r="C145" s="7"/>
+      <c r="D145" s="7"/>
+      <c r="E145" s="7"/>
+      <c r="F145" s="7"/>
+      <c r="G145" s="7"/>
+      <c r="H145" s="7"/>
+    </row>
+    <row r="146" ht="17.0" customHeight="1">
+      <c r="A146" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Dyr_Params</t>
         </is>
       </c>
-      <c r="B145" s="12" t="inlineStr">
+      <c r="B146" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Generator</t>
         </is>
       </c>
-      <c r="C145" s="8" t="inlineStr">
+      <c r="C146" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">generator</t>
-        </is>
-      </c>
-      <c r="D145" s="8"/>
-      <c r="E145" s="8"/>
-      <c r="F145" s="8"/>
-      <c r="G145" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">IB: the infinite bus | PLANT: the plant controller (REPC_B)</t>
-        </is>
-      </c>
-      <c r="H145" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSS/E .dyr</t>
-        </is>
-      </c>
-    </row>
-    <row r="146" ht="30.0" customHeight="1">
-      <c r="A146" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Dyr_Params</t>
-        </is>
-      </c>
-      <c r="B146" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Model</t>
-        </is>
-      </c>
-      <c r="C146" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">model</t>
         </is>
       </c>
       <c r="D146" s="8"/>
@@ -5904,7 +5912,7 @@
       <c r="F146" s="8"/>
       <c r="G146" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">REGCA1 (REGCAU1) | REECA1 REECCU1 REECDU1 | REPCA1 (REPCAU1) or REAX4BU1 | PLANT: PLNTBU1 | WT3: + WTDTA1 WTARA1 WTPTA1 WTTQA1 | SYNC: GENROU SEXS TGOV1 | IB: GENCLS</t>
+          <t xml:space="preserve">IB: the infinite bus | PLANT: the plant controller (REPC_B)</t>
         </is>
       </c>
       <c r="H146" s="13" t="inlineStr">
@@ -5913,7 +5921,7 @@
         </is>
       </c>
     </row>
-    <row r="147" ht="17.0" customHeight="1">
+    <row r="147" ht="30.0" customHeight="1">
       <c r="A147" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Dyr_Params</t>
@@ -5921,12 +5929,12 @@
       </c>
       <c r="B147" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Parameter</t>
+          <t xml:space="preserve">Model</t>
         </is>
       </c>
       <c r="C147" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">parameter</t>
+          <t xml:space="preserve">model</t>
         </is>
       </c>
       <c r="D147" s="8"/>
@@ -5934,7 +5942,7 @@
       <c r="F147" s="8"/>
       <c r="G147" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E name (the report lists them all) or position: ICON2, CON14</t>
+          <t xml:space="preserve">REGCA1 (REGCAU1) | REECA1 REECCU1 REECDU1 | REPCA1 (REPCAU1) or REAX4BU1 | PLANT: PLNTBU1 | WT3: + WTDTA1 WTARA1 WTPTA1 WTTQA1 | SYNC: GENROU SEXS TGOV1 | IB: GENCLS</t>
         </is>
       </c>
       <c r="H147" s="13" t="inlineStr">
@@ -5951,71 +5959,67 @@
       </c>
       <c r="B148" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Value</t>
+          <t xml:space="preserve">Parameter</t>
         </is>
       </c>
       <c r="C148" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">value</t>
+          <t xml:space="preserve">parameter</t>
         </is>
       </c>
       <c r="D148" s="8"/>
       <c r="E148" s="8"/>
       <c r="F148" s="8"/>
-      <c r="G148" s="8"/>
+      <c r="G148" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSS/E name (the report lists them all) or position: ICON2, CON14</t>
+        </is>
+      </c>
       <c r="H148" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">PSS/E .dyr</t>
         </is>
       </c>
     </row>
-    <row r="149" ht="18" customHeight="1">
-      <c r="A149" s="7" t="inlineStr">
+    <row r="149" ht="17.0" customHeight="1">
+      <c r="A149" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dyr_Params</t>
+        </is>
+      </c>
+      <c r="B149" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Value</t>
+        </is>
+      </c>
+      <c r="C149" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">value</t>
+        </is>
+      </c>
+      <c r="D149" s="8"/>
+      <c r="E149" s="8"/>
+      <c r="F149" s="8"/>
+      <c r="G149" s="8"/>
+      <c r="H149" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSS/E .dyr</t>
+        </is>
+      </c>
+    </row>
+    <row r="150" ht="18" customHeight="1">
+      <c r="A150" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Dyr_Records</t>
         </is>
       </c>
-      <c r="B149" s="7"/>
-      <c r="C149" s="7"/>
-      <c r="D149" s="7"/>
-      <c r="E149" s="7"/>
-      <c r="F149" s="7"/>
-      <c r="G149" s="7"/>
-      <c r="H149" s="7"/>
-    </row>
-    <row r="150" ht="17.0" customHeight="1">
-      <c r="A150" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Dyr_Records</t>
-        </is>
-      </c>
-      <c r="B150" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Generator</t>
-        </is>
-      </c>
-      <c r="C150" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">generator</t>
-        </is>
-      </c>
-      <c r="D150" s="8"/>
-      <c r="E150" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">the plant</t>
-        </is>
-      </c>
-      <c r="F150" s="8"/>
-      <c r="G150" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">blank = the plant</t>
-        </is>
-      </c>
-      <c r="H150" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSS/E .dyr</t>
-        </is>
-      </c>
+      <c r="B150" s="7"/>
+      <c r="C150" s="7"/>
+      <c r="D150" s="7"/>
+      <c r="E150" s="7"/>
+      <c r="F150" s="7"/>
+      <c r="G150" s="7"/>
+      <c r="H150" s="7"/>
     </row>
     <row r="151" ht="17.0" customHeight="1">
       <c r="A151" s="8" t="inlineStr">
@@ -6025,67 +6029,75 @@
       </c>
       <c r="B151" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Record</t>
+          <t xml:space="preserve">Generator</t>
         </is>
       </c>
       <c r="C151" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">record</t>
+          <t xml:space="preserve">generator</t>
         </is>
       </c>
       <c r="D151" s="8"/>
-      <c r="E151" s="8"/>
+      <c r="E151" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the plant</t>
+        </is>
+      </c>
       <c r="F151" s="8"/>
       <c r="G151" s="8" t="inlineStr">
         <is>
+          <t xml:space="preserve">blank = the plant</t>
+        </is>
+      </c>
+      <c r="H151" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSS/E .dyr</t>
+        </is>
+      </c>
+    </row>
+    <row r="152" ht="17.0" customHeight="1">
+      <c r="A152" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dyr_Records</t>
+        </is>
+      </c>
+      <c r="B152" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Record</t>
+        </is>
+      </c>
+      <c r="C152" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">record</t>
+        </is>
+      </c>
+      <c r="D152" s="8"/>
+      <c r="E152" s="8"/>
+      <c r="F152" s="8"/>
+      <c r="G152" s="8" t="inlineStr">
+        <is>
           <t xml:space="preserve">.dyr text ending in / -- {BUS} {ID} {MBASE} {POI} {IB} {HV} {MV} {&lt;bus role&gt;} are filled in</t>
         </is>
       </c>
-      <c r="H151" s="13" t="inlineStr">
+      <c r="H152" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">PSS/E .dyr</t>
         </is>
       </c>
     </row>
-    <row r="152" ht="18" customHeight="1">
-      <c r="A152" s="7" t="inlineStr">
+    <row r="153" ht="18" customHeight="1">
+      <c r="A153" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">PSCAD_Params</t>
         </is>
       </c>
-      <c r="B152" s="7"/>
-      <c r="C152" s="7"/>
-      <c r="D152" s="7"/>
-      <c r="E152" s="7"/>
-      <c r="F152" s="7"/>
-      <c r="G152" s="7"/>
-      <c r="H152" s="7"/>
-    </row>
-    <row r="153" ht="17.0" customHeight="1">
-      <c r="A153" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSCAD_Params</t>
-        </is>
-      </c>
-      <c r="B153" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Generator</t>
-        </is>
-      </c>
-      <c r="C153" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">generator</t>
-        </is>
-      </c>
-      <c r="D153" s="8"/>
-      <c r="E153" s="8"/>
-      <c r="F153" s="8"/>
-      <c r="G153" s="8"/>
-      <c r="H153" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSCAD</t>
-        </is>
-      </c>
+      <c r="B153" s="7"/>
+      <c r="C153" s="7"/>
+      <c r="D153" s="7"/>
+      <c r="E153" s="7"/>
+      <c r="F153" s="7"/>
+      <c r="G153" s="7"/>
+      <c r="H153" s="7"/>
     </row>
     <row r="154" ht="17.0" customHeight="1">
       <c r="A154" s="8" t="inlineStr">
@@ -6095,22 +6107,18 @@
       </c>
       <c r="B154" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Parameter</t>
+          <t xml:space="preserve">Generator</t>
         </is>
       </c>
       <c r="C154" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">parameter</t>
+          <t xml:space="preserve">generator</t>
         </is>
       </c>
       <c r="D154" s="8"/>
       <c r="E154" s="8"/>
       <c r="F154" s="8"/>
-      <c r="G154" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">the vendor model's parameter name</t>
-        </is>
-      </c>
+      <c r="G154" s="8"/>
       <c r="H154" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">PSCAD</t>
@@ -6125,12 +6133,12 @@
       </c>
       <c r="B155" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Value</t>
+          <t xml:space="preserve">Parameter</t>
         </is>
       </c>
       <c r="C155" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">value</t>
+          <t xml:space="preserve">parameter</t>
         </is>
       </c>
       <c r="D155" s="8"/>
@@ -6138,52 +6146,64 @@
       <c r="F155" s="8"/>
       <c r="G155" s="8" t="inlineStr">
         <is>
+          <t xml:space="preserve">the vendor model's parameter name</t>
+        </is>
+      </c>
+      <c r="H155" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="156" ht="17.0" customHeight="1">
+      <c r="A156" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD_Params</t>
+        </is>
+      </c>
+      <c r="B156" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Value</t>
+        </is>
+      </c>
+      <c r="C156" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">value</t>
+        </is>
+      </c>
+      <c r="D156" s="8"/>
+      <c r="E156" s="8"/>
+      <c r="F156" s="8"/>
+      <c r="G156" s="8" t="inlineStr">
+        <is>
           <t xml:space="preserve">as PSCAD takes it (0.63 [kV], 40, {UNITS}, {P_PU} ...)</t>
         </is>
       </c>
-      <c r="H155" s="13" t="inlineStr">
+      <c r="H156" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">PSCAD</t>
         </is>
       </c>
     </row>
-    <row r="156" ht="18" customHeight="1">
-      <c r="A156" s="7" t="inlineStr">
+    <row r="157" ht="18" customHeight="1">
+      <c r="A157" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">BUS NAMES -- Connect to, At, Bus_Numbers and {&lt;bus&gt;} in Dyr_Records take these</t>
         </is>
       </c>
-      <c r="B156" s="7"/>
-      <c r="C156" s="7"/>
-      <c r="D156" s="7"/>
-      <c r="E156" s="7"/>
-      <c r="F156" s="7"/>
-      <c r="G156" s="7"/>
-      <c r="H156" s="7"/>
-    </row>
-    <row r="157">
-      <c r="A157" s="8"/>
-      <c r="B157" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">IB</t>
-        </is>
-      </c>
-      <c r="C157" s="8"/>
-      <c r="D157" s="8"/>
-      <c r="E157" s="8"/>
-      <c r="F157" s="8"/>
-      <c r="G157" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">the infinite bus</t>
-        </is>
-      </c>
-      <c r="H157" s="8"/>
+      <c r="B157" s="7"/>
+      <c r="C157" s="7"/>
+      <c r="D157" s="7"/>
+      <c r="E157" s="7"/>
+      <c r="F157" s="7"/>
+      <c r="G157" s="7"/>
+      <c r="H157" s="7"/>
     </row>
     <row r="158">
       <c r="A158" s="8"/>
       <c r="B158" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">POI</t>
+          <t xml:space="preserve">IB</t>
         </is>
       </c>
       <c r="C158" s="8"/>
@@ -6192,7 +6212,7 @@
       <c r="F158" s="8"/>
       <c r="G158" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">the point of interconnection</t>
+          <t xml:space="preserve">the infinite bus</t>
         </is>
       </c>
       <c r="H158" s="8"/>
@@ -6201,7 +6221,7 @@
       <c r="A159" s="8"/>
       <c r="B159" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">HV</t>
+          <t xml:space="preserve">POI</t>
         </is>
       </c>
       <c r="C159" s="8"/>
@@ -6210,7 +6230,7 @@
       <c r="F159" s="8"/>
       <c r="G159" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">the gen-tie's plant end (the POI when there is no gen-tie)</t>
+          <t xml:space="preserve">the point of interconnection</t>
         </is>
       </c>
       <c r="H159" s="8"/>
@@ -6219,7 +6239,7 @@
       <c r="A160" s="8"/>
       <c r="B160" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;MPT&gt; or &lt;MPT&gt;:LV</t>
+          <t xml:space="preserve">HV</t>
         </is>
       </c>
       <c r="C160" s="8"/>
@@ -6228,7 +6248,7 @@
       <c r="F160" s="8"/>
       <c r="G160" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">an MPT's LV winding</t>
+          <t xml:space="preserve">the gen-tie's plant end (the POI when there is no gen-tie)</t>
         </is>
       </c>
       <c r="H160" s="8"/>
@@ -6237,7 +6257,7 @@
       <c r="A161" s="8"/>
       <c r="B161" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;MPT&gt;:TV</t>
+          <t xml:space="preserve">&lt;MPT&gt; or &lt;MPT&gt;:LV</t>
         </is>
       </c>
       <c r="C161" s="8"/>
@@ -6246,7 +6266,7 @@
       <c r="F161" s="8"/>
       <c r="G161" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">a 3-winding MPT's tertiary</t>
+          <t xml:space="preserve">an MPT's LV winding</t>
         </is>
       </c>
       <c r="H161" s="8"/>
@@ -6255,7 +6275,7 @@
       <c r="A162" s="8"/>
       <c r="B162" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;MPT&gt;:HV</t>
+          <t xml:space="preserve">&lt;MPT&gt;:TV</t>
         </is>
       </c>
       <c r="C162" s="8"/>
@@ -6264,7 +6284,7 @@
       <c r="F162" s="8"/>
       <c r="G162" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">an MPT with a tie line of its own: its HV end</t>
+          <t xml:space="preserve">a 3-winding MPT's tertiary</t>
         </is>
       </c>
       <c r="H162" s="8"/>
@@ -6273,7 +6293,7 @@
       <c r="A163" s="8"/>
       <c r="B163" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;collector&gt;</t>
+          <t xml:space="preserve">&lt;MPT&gt;:HV</t>
         </is>
       </c>
       <c r="C163" s="8"/>
@@ -6282,7 +6302,7 @@
       <c r="F163" s="8"/>
       <c r="G163" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">a shared collector's far end</t>
+          <t xml:space="preserve">an MPT with a tie line of its own: its HV end</t>
         </is>
       </c>
       <c r="H163" s="8"/>
@@ -6291,7 +6311,7 @@
       <c r="A164" s="8"/>
       <c r="B164" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;generator&gt;:MV</t>
+          <t xml:space="preserve">&lt;collector&gt;</t>
         </is>
       </c>
       <c r="C164" s="8"/>
@@ -6300,7 +6320,7 @@
       <c r="F164" s="8"/>
       <c r="G164" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">a generator's GSU HV side</t>
+          <t xml:space="preserve">a shared collector's far end</t>
         </is>
       </c>
       <c r="H164" s="8"/>
@@ -6309,7 +6329,7 @@
       <c r="A165" s="8"/>
       <c r="B165" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;generator&gt; or &lt;generator&gt;:LV</t>
+          <t xml:space="preserve">&lt;generator&gt;:MV</t>
         </is>
       </c>
       <c r="C165" s="8"/>
@@ -6318,7 +6338,7 @@
       <c r="F165" s="8"/>
       <c r="G165" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">a generator's terminal</t>
+          <t xml:space="preserve">a generator's GSU HV side</t>
         </is>
       </c>
       <c r="H165" s="8"/>
@@ -6327,7 +6347,7 @@
       <c r="A166" s="8"/>
       <c r="B166" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;collector&gt;_&lt;feeder&gt;_S&lt;n&gt;</t>
+          <t xml:space="preserve">&lt;generator&gt; or &lt;generator&gt;:LV</t>
         </is>
       </c>
       <c r="C166" s="8"/>
@@ -6336,7 +6356,7 @@
       <c r="F166" s="8"/>
       <c r="G166" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">DETAILED: the far end of feeder section n</t>
+          <t xml:space="preserve">a generator's terminal</t>
         </is>
       </c>
       <c r="H166" s="8"/>
@@ -6345,7 +6365,7 @@
       <c r="A167" s="8"/>
       <c r="B167" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;generator&gt;_&lt;feeder&gt;_S&lt;n&gt;:LV</t>
+          <t xml:space="preserve">&lt;collector&gt;_&lt;feeder&gt;_S&lt;n&gt;</t>
         </is>
       </c>
       <c r="C167" s="8"/>
@@ -6354,50 +6374,42 @@
       <c r="F167" s="8"/>
       <c r="G167" s="8" t="inlineStr">
         <is>
+          <t xml:space="preserve">DETAILED: the far end of feeder section n</t>
+        </is>
+      </c>
+      <c r="H167" s="8"/>
+    </row>
+    <row r="168">
+      <c r="A168" s="8"/>
+      <c r="B168" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;generator&gt;_&lt;feeder&gt;_S&lt;n&gt;:LV</t>
+        </is>
+      </c>
+      <c r="C168" s="8"/>
+      <c r="D168" s="8"/>
+      <c r="E168" s="8"/>
+      <c r="F168" s="8"/>
+      <c r="G168" s="8" t="inlineStr">
+        <is>
           <t xml:space="preserve">DETAILED: the terminal of the units at that node</t>
         </is>
       </c>
-      <c r="H167" s="8"/>
-    </row>
-    <row r="168" ht="18" customHeight="1">
-      <c r="A168" s="7" t="inlineStr">
+      <c r="H168" s="8"/>
+    </row>
+    <row r="169" ht="18" customHeight="1">
+      <c r="A169" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">PSCAD_Params PLACEHOLDERS -- filled in for each inverter a vendor model stands for</t>
         </is>
       </c>
-      <c r="B168" s="7"/>
-      <c r="C168" s="7"/>
-      <c r="D168" s="7"/>
-      <c r="E168" s="7"/>
-      <c r="F168" s="7"/>
-      <c r="G168" s="7"/>
-      <c r="H168" s="7"/>
-    </row>
-    <row r="169">
-      <c r="A169" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSCAD_Params</t>
-        </is>
-      </c>
-      <c r="B169" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">{UNITS}</t>
-        </is>
-      </c>
-      <c r="C169" s="8"/>
-      <c r="D169" s="8"/>
-      <c r="E169" s="8"/>
-      <c r="F169" s="8"/>
-      <c r="G169" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">the units the inverter stands for</t>
-        </is>
-      </c>
-      <c r="H169" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSCAD</t>
-        </is>
-      </c>
+      <c r="B169" s="7"/>
+      <c r="C169" s="7"/>
+      <c r="D169" s="7"/>
+      <c r="E169" s="7"/>
+      <c r="F169" s="7"/>
+      <c r="G169" s="7"/>
+      <c r="H169" s="7"/>
     </row>
     <row r="170">
       <c r="A170" s="8" t="inlineStr">
@@ -6407,7 +6419,7 @@
       </c>
       <c r="B170" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{MVA}</t>
+          <t xml:space="preserve">{UNITS}</t>
         </is>
       </c>
       <c r="C170" s="8"/>
@@ -6416,7 +6428,7 @@
       <c r="F170" s="8"/>
       <c r="G170" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">their MVA</t>
+          <t xml:space="preserve">the units the inverter stands for</t>
         </is>
       </c>
       <c r="H170" s="13" t="inlineStr">
@@ -6433,7 +6445,7 @@
       </c>
       <c r="B171" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{P_MW}</t>
+          <t xml:space="preserve">{MVA}</t>
         </is>
       </c>
       <c r="C171" s="8"/>
@@ -6442,7 +6454,7 @@
       <c r="F171" s="8"/>
       <c r="G171" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">their P where the inverter connects (MW)</t>
+          <t xml:space="preserve">their MVA</t>
         </is>
       </c>
       <c r="H171" s="13" t="inlineStr">
@@ -6459,7 +6471,7 @@
       </c>
       <c r="B172" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{Q_MVAR}</t>
+          <t xml:space="preserve">{P_MW}</t>
         </is>
       </c>
       <c r="C172" s="8"/>
@@ -6468,7 +6480,7 @@
       <c r="F172" s="8"/>
       <c r="G172" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">their Q there (MVAr)</t>
+          <t xml:space="preserve">their P where the inverter connects (MW)</t>
         </is>
       </c>
       <c r="H172" s="13" t="inlineStr">
@@ -6485,7 +6497,7 @@
       </c>
       <c r="B173" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{P_PU}</t>
+          <t xml:space="preserve">{Q_MVAR}</t>
         </is>
       </c>
       <c r="C173" s="8"/>
@@ -6494,7 +6506,7 @@
       <c r="F173" s="8"/>
       <c r="G173" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">P on {MVA}</t>
+          <t xml:space="preserve">their Q there (MVAr)</t>
         </is>
       </c>
       <c r="H173" s="13" t="inlineStr">
@@ -6511,7 +6523,7 @@
       </c>
       <c r="B174" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{Q_PU}</t>
+          <t xml:space="preserve">{P_PU}</t>
         </is>
       </c>
       <c r="C174" s="8"/>
@@ -6520,7 +6532,7 @@
       <c r="F174" s="8"/>
       <c r="G174" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q on {MVA}</t>
+          <t xml:space="preserve">P on {MVA}</t>
         </is>
       </c>
       <c r="H174" s="13" t="inlineStr">
@@ -6537,7 +6549,7 @@
       </c>
       <c r="B175" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{UNIT_MVA}</t>
+          <t xml:space="preserve">{Q_PU}</t>
         </is>
       </c>
       <c r="C175" s="8"/>
@@ -6546,7 +6558,7 @@
       <c r="F175" s="8"/>
       <c r="G175" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">one unit's MVA</t>
+          <t xml:space="preserve">Q on {MVA}</t>
         </is>
       </c>
       <c r="H175" s="13" t="inlineStr">
@@ -6563,7 +6575,7 @@
       </c>
       <c r="B176" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{UNIT_P_MW}</t>
+          <t xml:space="preserve">{UNIT_MVA}</t>
         </is>
       </c>
       <c r="C176" s="8"/>
@@ -6572,7 +6584,7 @@
       <c r="F176" s="8"/>
       <c r="G176" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">one unit's P (MW)</t>
+          <t xml:space="preserve">one unit's MVA</t>
         </is>
       </c>
       <c r="H176" s="13" t="inlineStr">
@@ -6589,7 +6601,7 @@
       </c>
       <c r="B177" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{UNIT_Q_MVAR}</t>
+          <t xml:space="preserve">{UNIT_P_MW}</t>
         </is>
       </c>
       <c r="C177" s="8"/>
@@ -6598,7 +6610,7 @@
       <c r="F177" s="8"/>
       <c r="G177" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">one unit's Q (MVAr)</t>
+          <t xml:space="preserve">one unit's P (MW)</t>
         </is>
       </c>
       <c r="H177" s="13" t="inlineStr">
@@ -6615,7 +6627,7 @@
       </c>
       <c r="B178" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{V_PU}</t>
+          <t xml:space="preserve">{UNIT_Q_MVAR}</t>
         </is>
       </c>
       <c r="C178" s="8"/>
@@ -6624,7 +6636,7 @@
       <c r="F178" s="8"/>
       <c r="G178" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">the voltage where it connects (pu)</t>
+          <t xml:space="preserve">one unit's Q (MVAr)</t>
         </is>
       </c>
       <c r="H178" s="13" t="inlineStr">
@@ -6641,7 +6653,7 @@
       </c>
       <c r="B179" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{V_KV}</t>
+          <t xml:space="preserve">{V_PU}</t>
         </is>
       </c>
       <c r="C179" s="8"/>
@@ -6650,7 +6662,7 @@
       <c r="F179" s="8"/>
       <c r="G179" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">the same in kV</t>
+          <t xml:space="preserve">the voltage where it connects (pu)</t>
         </is>
       </c>
       <c r="H179" s="13" t="inlineStr">
@@ -6667,7 +6679,7 @@
       </c>
       <c r="B180" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{KV}</t>
+          <t xml:space="preserve">{V_KV}</t>
         </is>
       </c>
       <c r="C180" s="8"/>
@@ -6676,7 +6688,7 @@
       <c r="F180" s="8"/>
       <c r="G180" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">that bus's base kV</t>
+          <t xml:space="preserve">the same in kV</t>
         </is>
       </c>
       <c r="H180" s="13" t="inlineStr">
@@ -6693,7 +6705,7 @@
       </c>
       <c r="B181" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{ANGLE}</t>
+          <t xml:space="preserve">{KV}</t>
         </is>
       </c>
       <c r="C181" s="8"/>
@@ -6702,7 +6714,7 @@
       <c r="F181" s="8"/>
       <c r="G181" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">its PSCAD angle (deg, the transformers' phase shifts included)</t>
+          <t xml:space="preserve">that bus's base kV</t>
         </is>
       </c>
       <c r="H181" s="13" t="inlineStr">
@@ -6719,7 +6731,7 @@
       </c>
       <c r="B182" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{FREQ}</t>
+          <t xml:space="preserve">{ANGLE}</t>
         </is>
       </c>
       <c r="C182" s="8"/>
@@ -6728,7 +6740,7 @@
       <c r="F182" s="8"/>
       <c r="G182" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">frequency (Hz)</t>
+          <t xml:space="preserve">its PSCAD angle (deg, the transformers' phase shifts included)</t>
         </is>
       </c>
       <c r="H182" s="13" t="inlineStr">
@@ -6745,7 +6757,7 @@
       </c>
       <c r="B183" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{P_INV_MW}</t>
+          <t xml:space="preserve">{FREQ}</t>
         </is>
       </c>
       <c r="C183" s="8"/>
@@ -6754,7 +6766,7 @@
       <c r="F183" s="8"/>
       <c r="G183" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">P at the inverters' own terminals (MW; a UDM on the MV side)</t>
+          <t xml:space="preserve">frequency (Hz)</t>
         </is>
       </c>
       <c r="H183" s="13" t="inlineStr">
@@ -6771,7 +6783,7 @@
       </c>
       <c r="B184" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{Q_INV_MVAR}</t>
+          <t xml:space="preserve">{P_INV_MW}</t>
         </is>
       </c>
       <c r="C184" s="8"/>
@@ -6780,7 +6792,7 @@
       <c r="F184" s="8"/>
       <c r="G184" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q there (MVAr)</t>
+          <t xml:space="preserve">P at the inverters' own terminals (MW; a UDM on the MV side)</t>
         </is>
       </c>
       <c r="H184" s="13" t="inlineStr">
@@ -6797,7 +6809,7 @@
       </c>
       <c r="B185" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{V_INV_PU}</t>
+          <t xml:space="preserve">{Q_INV_MVAR}</t>
         </is>
       </c>
       <c r="C185" s="8"/>
@@ -6806,10 +6818,36 @@
       <c r="F185" s="8"/>
       <c r="G185" s="8" t="inlineStr">
         <is>
+          <t xml:space="preserve">Q there (MVAr)</t>
+        </is>
+      </c>
+      <c r="H185" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="186">
+      <c r="A186" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD_Params</t>
+        </is>
+      </c>
+      <c r="B186" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{V_INV_PU}</t>
+        </is>
+      </c>
+      <c r="C186" s="8"/>
+      <c r="D186" s="8"/>
+      <c r="E186" s="8"/>
+      <c r="F186" s="8"/>
+      <c r="G186" s="8" t="inlineStr">
+        <is>
           <t xml:space="preserve">the voltage there (pu)</t>
         </is>
       </c>
-      <c r="H185" s="13" t="inlineStr">
+      <c r="H186" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">PSCAD</t>
         </is>
@@ -6820,32 +6858,32 @@
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A4:H4"/>
-    <mergeCell ref="A47:H47"/>
-    <mergeCell ref="A75:H75"/>
-    <mergeCell ref="A112:H112"/>
-    <mergeCell ref="A124:H124"/>
-    <mergeCell ref="A131:H131"/>
-    <mergeCell ref="A134:H134"/>
-    <mergeCell ref="A140:H140"/>
-    <mergeCell ref="A144:H144"/>
-    <mergeCell ref="A149:H149"/>
-    <mergeCell ref="A152:H152"/>
-    <mergeCell ref="A156:H156"/>
-    <mergeCell ref="A168:H168"/>
+    <mergeCell ref="A48:H48"/>
+    <mergeCell ref="A76:H76"/>
+    <mergeCell ref="A113:H113"/>
+    <mergeCell ref="A125:H125"/>
+    <mergeCell ref="A132:H132"/>
+    <mergeCell ref="A135:H135"/>
+    <mergeCell ref="A141:H141"/>
+    <mergeCell ref="A145:H145"/>
+    <mergeCell ref="A150:H150"/>
+    <mergeCell ref="A153:H153"/>
+    <mergeCell ref="A157:H157"/>
+    <mergeCell ref="A169:H169"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A4" location="'Plant'!A1" display="Plant"/>
-    <hyperlink ref="A47" location="'MPT'!A1" display="MPT"/>
-    <hyperlink ref="A75" location="'Generators'!A1" display="Generators"/>
-    <hyperlink ref="A112" location="'Feeders'!A1" display="Feeders"/>
-    <hyperlink ref="A124" location="'Cables'!A1" display="Cables"/>
-    <hyperlink ref="A131" location="'Collectors'!A1" display="Collectors"/>
-    <hyperlink ref="A134" location="'Loads_Shunts'!A1" display="Loads_Shunts"/>
-    <hyperlink ref="A140" location="'Bus_Numbers'!A1" display="Bus_Numbers"/>
-    <hyperlink ref="A144" location="'Dyr_Params'!A1" display="Dyr_Params"/>
-    <hyperlink ref="A149" location="'Dyr_Records'!A1" display="Dyr_Records"/>
-    <hyperlink ref="A152" location="'PSCAD_Params'!A1" display="PSCAD_Params"/>
-    <hyperlink ref="A168" location="'PSCAD_Params'!A1" display="PSCAD_Params"/>
+    <hyperlink ref="A48" location="'MPT'!A1" display="MPT"/>
+    <hyperlink ref="A76" location="'Generators'!A1" display="Generators"/>
+    <hyperlink ref="A113" location="'Feeders'!A1" display="Feeders"/>
+    <hyperlink ref="A125" location="'Cables'!A1" display="Cables"/>
+    <hyperlink ref="A132" location="'Collectors'!A1" display="Collectors"/>
+    <hyperlink ref="A135" location="'Loads_Shunts'!A1" display="Loads_Shunts"/>
+    <hyperlink ref="A141" location="'Bus_Numbers'!A1" display="Bus_Numbers"/>
+    <hyperlink ref="A145" location="'Dyr_Params'!A1" display="Dyr_Params"/>
+    <hyperlink ref="A150" location="'Dyr_Records'!A1" display="Dyr_Records"/>
+    <hyperlink ref="A153" location="'PSCAD_Params'!A1" display="PSCAD_Params"/>
+    <hyperlink ref="A169" location="'PSCAD_Params'!A1" display="PSCAD_Params"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
@@ -18521,69 +18559,73 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="18" customHeight="1">
-      <c r="A44" s="7" t="inlineStr">
+    <row r="44" ht="43.0" customHeight="1">
+      <c r="A44" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD lines as</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PI</t>
+        </is>
+      </c>
+      <c r="C44" s="8"/>
+      <c r="D44" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PI</t>
+        </is>
+      </c>
+      <c r="E44" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PI | RLC</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PI = the gen-tie, each collector and each feeder section one Coupled PI Section (R, X, B in pu, its charging inside); RLC = an R and an L, the charging a C at each end (blank = PI)</t>
+        </is>
+      </c>
+      <c r="G44" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="18" customHeight="1">
+      <c r="A45" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">PSCAD FAULT AT THE POI</t>
         </is>
       </c>
-      <c r="B44" s="7"/>
-      <c r="C44" s="7"/>
-      <c r="D44" s="7"/>
-      <c r="E44" s="7"/>
-      <c r="F44" s="7"/>
-      <c r="G44" s="7"/>
-    </row>
-    <row r="45" ht="30.0" customHeight="1">
-      <c r="A45" s="12" t="inlineStr">
+      <c r="B45" s="7"/>
+      <c r="C45" s="7"/>
+      <c r="D45" s="7"/>
+      <c r="E45" s="7"/>
+      <c r="F45" s="7"/>
+      <c r="G45" s="7"/>
+    </row>
+    <row r="46" ht="30.0" customHeight="1">
+      <c r="A46" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">PSCAD fault at POI</t>
         </is>
       </c>
-      <c r="B45" s="3" t="inlineStr">
+      <c r="B46" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">YES</t>
         </is>
       </c>
-      <c r="C45" s="8"/>
-      <c r="D45" s="8"/>
-      <c r="E45" s="8" t="inlineStr">
+      <c r="C46" s="8"/>
+      <c r="D46" s="8"/>
+      <c r="E46" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">YES | NO</t>
         </is>
       </c>
-      <c r="F45" s="2" t="inlineStr">
+      <c r="F46" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">YES = a fault on the grid side of the POI with its timed fault logic, as vendors' test cases have</t>
-        </is>
-      </c>
-      <c r="G45" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSCAD</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="17.0" customHeight="1">
-      <c r="A46" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSCAD fault time</t>
-        </is>
-      </c>
-      <c r="B46" s="3"/>
-      <c r="C46" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">s</t>
-        </is>
-      </c>
-      <c r="D46" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">100: none in the run</t>
-        </is>
-      </c>
-      <c r="E46" s="8"/>
-      <c r="F46" s="2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">when the fault starts (blank = 100: none in the run)</t>
         </is>
       </c>
       <c r="G46" s="13" t="inlineStr">
@@ -18595,12 +18637,10 @@
     <row r="47" ht="17.0" customHeight="1">
       <c r="A47" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSCAD fault duration</t>
-        </is>
-      </c>
-      <c r="B47" s="3">
-        <v>0.15</v>
-      </c>
+          <t xml:space="preserve">PSCAD fault time</t>
+        </is>
+      </c>
+      <c r="B47" s="3"/>
       <c r="C47" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">s</t>
@@ -18608,114 +18648,145 @@
       </c>
       <c r="D47" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.15</t>
+          <t xml:space="preserve">100: none in the run</t>
         </is>
       </c>
       <c r="E47" s="8"/>
       <c r="F47" s="2" t="inlineStr">
         <is>
+          <t xml:space="preserve">when the fault starts (blank = 100: none in the run)</t>
+        </is>
+      </c>
+      <c r="G47" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="17.0" customHeight="1">
+      <c r="A48" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD fault duration</t>
+        </is>
+      </c>
+      <c r="B48" s="3">
+        <v>0.15</v>
+      </c>
+      <c r="C48" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">s</t>
+        </is>
+      </c>
+      <c r="D48" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">0.15</t>
+        </is>
+      </c>
+      <c r="E48" s="8"/>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
           <t xml:space="preserve">blank = 0.15</t>
         </is>
       </c>
-      <c r="G47" s="13" t="inlineStr">
+      <c r="G48" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">PSCAD</t>
         </is>
       </c>
     </row>
-    <row r="48" ht="43.0" customHeight="1">
-      <c r="A48" s="12" t="inlineStr">
+    <row r="49" ht="43.0" customHeight="1">
+      <c r="A49" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">PSCAD fault type</t>
         </is>
       </c>
-      <c r="B48" s="3" t="inlineStr">
+      <c r="B49" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">ABCG</t>
         </is>
       </c>
-      <c r="C48" s="8"/>
-      <c r="D48" s="8" t="inlineStr">
+      <c r="C49" s="8"/>
+      <c r="D49" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">ABCG</t>
         </is>
       </c>
-      <c r="E48" s="8" t="inlineStr">
+      <c r="E49" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">ABCG | ABC | AG | BG | CG | ABG | BCG | ACG | AB | BC | AC</t>
         </is>
       </c>
-      <c r="F48" s="2" t="inlineStr">
+      <c r="F49" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">the phases faulted, G = to ground (blank = ABCG)</t>
         </is>
       </c>
-      <c r="G48" s="13" t="inlineStr">
+      <c r="G49" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">PSCAD</t>
         </is>
       </c>
     </row>
-    <row r="49" ht="17.0" customHeight="1">
-      <c r="A49" s="12" t="inlineStr">
+    <row r="50" ht="17.0" customHeight="1">
+      <c r="A50" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">PSCAD fault resistance</t>
         </is>
       </c>
-      <c r="B49" s="3">
+      <c r="B50" s="3">
         <v>0.01</v>
       </c>
-      <c r="C49" s="8" t="inlineStr">
+      <c r="C50" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">ohm</t>
         </is>
       </c>
-      <c r="D49" s="8" t="inlineStr">
+      <c r="D50" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">0.01</t>
         </is>
       </c>
-      <c r="E49" s="8"/>
-      <c r="F49" s="2" t="inlineStr">
+      <c r="E50" s="8"/>
+      <c r="F50" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">blank = 0.01</t>
         </is>
       </c>
-      <c r="G49" s="13" t="inlineStr">
+      <c r="G50" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">PSCAD</t>
         </is>
       </c>
     </row>
-    <row r="50" ht="18" customHeight="1">
-      <c r="A50" s="7" t="inlineStr">
+    <row r="51" ht="18" customHeight="1">
+      <c r="A51" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">PSCAD LIBRARIES</t>
         </is>
       </c>
-      <c r="B50" s="7"/>
-      <c r="C50" s="7"/>
-      <c r="D50" s="7"/>
-      <c r="E50" s="7"/>
-      <c r="F50" s="7"/>
-      <c r="G50" s="7"/>
-    </row>
-    <row r="51" ht="17.0" customHeight="1">
-      <c r="A51" s="12" t="inlineStr">
+      <c r="B51" s="7"/>
+      <c r="C51" s="7"/>
+      <c r="D51" s="7"/>
+      <c r="E51" s="7"/>
+      <c r="F51" s="7"/>
+      <c r="G51" s="7"/>
+    </row>
+    <row r="52" ht="17.0" customHeight="1">
+      <c r="A52" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">PSCAD libraries</t>
         </is>
       </c>
-      <c r="B51" s="3"/>
-      <c r="C51" s="8"/>
-      <c r="D51" s="8"/>
-      <c r="E51" s="8"/>
-      <c r="F51" s="2" t="inlineStr">
+      <c r="B52" s="3"/>
+      <c r="C52" s="8"/>
+      <c r="D52" s="8"/>
+      <c r="E52" s="8"/>
+      <c r="F52" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">user-model libraries (.pslx) to load, separated by ;</t>
         </is>
       </c>
-      <c r="G51" s="13" t="inlineStr">
+      <c r="G52" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">PSCAD</t>
         </is>
@@ -18729,10 +18800,10 @@
     <mergeCell ref="A29:G29"/>
     <mergeCell ref="A36:G36"/>
     <mergeCell ref="A39:G39"/>
-    <mergeCell ref="A44:G44"/>
-    <mergeCell ref="A50:G50"/>
+    <mergeCell ref="A45:G45"/>
+    <mergeCell ref="A51:G51"/>
   </mergeCells>
-  <dataValidations count="8">
+  <dataValidations count="9">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B4">
       <formula1>"SMIB,DETAILED"</formula1>
     </dataValidation>
@@ -18751,10 +18822,13 @@
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B43">
       <formula1>"YES,NO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B45">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B44">
+      <formula1>"PI,RLC"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B46">
       <formula1>"YES,NO"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B48">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B49">
       <formula1>"ABCG,ABC,AG,BG,CG,ABG,BCG,ACG,AB,BC,AC"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
smib_build: Machines sheet, Scale up, faster load flow, PSCAD columns
- Machines (DETAILED): a machine's own Pgen, Pmax, Pmin, Qmax, Qmin, fixed Q, MBASE and ID; the GUI lists the
  machines with their values
- Scale up (GUI) / --scale MPTS FEEDERS GSUS INVERTERS: a test plant of copies of the first MPT with its
  generators, feeders per MPT, GSUs per feeder, inverters per GSU; units, GSU count and MVA, dispatch, MPT MVA
  and gen-tie circuits follow
- load flow: sparse elimination (50 feeders: 41 s -> 0.5 s), results unchanged
- PSCAD: a drawing taller than the page goes on in columns, joined by node labels

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BGsNUhFmVX23f8qnP53zUv
</commit_message>
<xml_diff>
--- a/smib/SMIB_INPUT_TEMPLATE.xlsx
+++ b/smib/SMIB_INPUT_TEMPLATE.xlsx
@@ -10,12 +10,13 @@
     <sheet name="Cables" sheetId="6" r:id="rId6"/>
     <sheet name="Collectors" sheetId="7" r:id="rId7"/>
     <sheet name="Loads_Shunts" sheetId="8" r:id="rId8"/>
-    <sheet name="Bus_Numbers" sheetId="9" r:id="rId9"/>
-    <sheet name="Dyr_Params" sheetId="10" r:id="rId10"/>
-    <sheet name="Dyr_Records" sheetId="11" r:id="rId11"/>
-    <sheet name="PSCAD_Params" sheetId="12" r:id="rId12"/>
-    <sheet name="Input_Reference" sheetId="13" r:id="rId13"/>
-    <sheet name="Dynamic_Models" sheetId="14" r:id="rId14"/>
+    <sheet name="Machines" sheetId="9" r:id="rId9"/>
+    <sheet name="Bus_Numbers" sheetId="10" r:id="rId10"/>
+    <sheet name="Dyr_Params" sheetId="11" r:id="rId11"/>
+    <sheet name="Dyr_Records" sheetId="12" r:id="rId12"/>
+    <sheet name="PSCAD_Params" sheetId="13" r:id="rId13"/>
+    <sheet name="Input_Reference" sheetId="14" r:id="rId14"/>
+    <sheet name="Dynamic_Models" sheetId="15" r:id="rId15"/>
   </sheets>
 </workbook>
 </file>
@@ -420,12 +421,12 @@
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bus_Numbers</t>
+          <t xml:space="preserve">Machines</t>
         </is>
       </c>
       <c r="B18" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">bus numbers and names of your own (blank = automatic)</t>
+          <t xml:space="preserve">DETAILED: each machine's own Pgen, P and Q limits, MBASE and ID</t>
         </is>
       </c>
       <c r="C18" s="13" t="inlineStr">
@@ -437,12 +438,12 @@
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dyr_Params</t>
+          <t xml:space="preserve">Bus_Numbers</t>
         </is>
       </c>
       <c r="B19" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">any dynamic model parameter, by generator, model and name</t>
+          <t xml:space="preserve">bus numbers and names of your own (blank = automatic)</t>
         </is>
       </c>
       <c r="C19" s="13" t="inlineStr">
@@ -454,12 +455,12 @@
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dyr_Records</t>
+          <t xml:space="preserve">Dyr_Params</t>
         </is>
       </c>
       <c r="B20" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">.dyr records of your own (vendor models)</t>
+          <t xml:space="preserve">any dynamic model parameter, by generator, model and name</t>
         </is>
       </c>
       <c r="C20" s="13" t="inlineStr">
@@ -471,12 +472,12 @@
     <row r="21">
       <c r="A21" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSCAD_Params</t>
+          <t xml:space="preserve">Dyr_Records</t>
         </is>
       </c>
       <c r="B21" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">the vendor PSCAD model's parameters, by generator</t>
+          <t xml:space="preserve">.dyr records of your own (vendor models)</t>
         </is>
       </c>
       <c r="C21" s="13" t="inlineStr">
@@ -488,320 +489,349 @@
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Input_Reference</t>
+          <t xml:space="preserve">PSCAD_Params</t>
         </is>
       </c>
       <c r="B22" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">every input: what it is, its unit, the default when blank, the choices, which model uses it</t>
+          <t xml:space="preserve">the vendor PSCAD model's parameters, by generator</t>
         </is>
       </c>
       <c r="C22" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">reference</t>
+          <t xml:space="preserve">input</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="9" t="inlineStr">
         <is>
+          <t xml:space="preserve">Input_Reference</t>
+        </is>
+      </c>
+      <c r="B23" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">every input: what it is, its unit, the default when blank, the choices, which model uses it</t>
+        </is>
+      </c>
+      <c r="C23" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">reference</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="9" t="inlineStr">
+        <is>
           <t xml:space="preserve">Dynamic_Models</t>
         </is>
       </c>
-      <c r="B23" s="8" t="inlineStr">
+      <c r="B24" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">every dynamic model's parameters: position, default and meaning</t>
         </is>
       </c>
-      <c r="C23" s="13" t="inlineStr">
+      <c r="C24" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">reference</t>
         </is>
       </c>
     </row>
-    <row r="24"/>
-    <row r="25" ht="20" customHeight="1">
-      <c r="A25" s="7" t="inlineStr">
+    <row r="25"/>
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">COLOURS</t>
         </is>
       </c>
-      <c r="B25" s="7"/>
-      <c r="C25" s="7"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="3"/>
-      <c r="B26" s="8" t="inlineStr">
+      <c r="B26" s="7"/>
+      <c r="C26" s="7"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="3"/>
+      <c r="B27" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">your inputs</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="2" t="inlineStr">
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">note</t>
         </is>
       </c>
-      <c r="B27" s="8" t="inlineStr">
+      <c r="B28" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">what to enter, the default when blank</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="1" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="1" t="inlineStr">
         <is>
           <t xml:space="preserve">Column</t>
         </is>
       </c>
-      <c r="B28" s="8" t="inlineStr">
+      <c r="B29" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">column titles</t>
         </is>
       </c>
     </row>
-    <row r="29">
-      <c r="A29" s="7" t="inlineStr">
+    <row r="30">
+      <c r="A30" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">SECTION</t>
         </is>
       </c>
-      <c r="B29" s="8" t="inlineStr">
+      <c r="B30" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">a group of items</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="13" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">PSS/E + PSCAD</t>
         </is>
       </c>
-      <c r="B30" s="8" t="inlineStr">
+      <c r="B31" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">which model an input goes into</t>
         </is>
       </c>
     </row>
-    <row r="31"/>
-    <row r="32" ht="20" customHeight="1">
-      <c r="A32" s="7" t="inlineStr">
+    <row r="32"/>
+    <row r="33" ht="20" customHeight="1">
+      <c r="A33" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">GUIDE</t>
         </is>
       </c>
-      <c r="B32" s="7"/>
-      <c r="C32" s="7"/>
-    </row>
-    <row r="33" ht="17.0" customHeight="1">
-      <c r="A33" s="12" t="inlineStr">
+      <c r="B33" s="7"/>
+      <c r="C33" s="7"/>
+    </row>
+    <row r="34" ht="17.0" customHeight="1">
+      <c r="A34" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">SMIB INPUT</t>
         </is>
       </c>
-      <c r="B33" s="8" t="inlineStr">
+      <c r="B34" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Fill in the sheets, save, then run:   python smib_build.py &lt;this workbook&gt;.xlsx</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="43.0" customHeight="1">
-      <c r="A34" s="8"/>
-      <c r="B34" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">It writes the PSS/E model (.raw rev 33 and .dyr; with PSS/E found, a solved .sav and a flat-run check) and the PSCAD build script (run it where PSCAD 5 and its Python automation library mhi.pscad are: it builds the .pscx), with a report of every equivalent, the load flow and anything to check.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="30.0" customHeight="1">
+    <row r="35" ht="43.0" customHeight="1">
       <c r="A35" s="8"/>
       <c r="B35" s="8" t="inlineStr">
         <is>
+          <t xml:space="preserve">It writes the PSS/E model (.raw rev 33 and .dyr; with PSS/E found, a solved .sav and a flat-run check) and the PSCAD build script (run it where PSCAD 5 and its Python automation library mhi.pscad are: it builds the .pscx), with a report of every equivalent, the load flow and anything to check.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="30.0" customHeight="1">
+      <c r="A36" s="8"/>
+      <c r="B36" s="8" t="inlineStr">
+        <is>
           <t xml:space="preserve">Blank cells take the default in the column note (row 2 of each sheet). Any row whose first cell starts with # is skipped (row 2 is one).</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="56.0" customHeight="1">
-      <c r="A36" s="12" t="inlineStr">
+    <row r="37" ht="56.0" customHeight="1">
+      <c r="A37" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">BUSES</t>
         </is>
       </c>
-      <c r="B36" s="8" t="inlineStr">
+      <c r="B37" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Name a bus by its role: POI | HV (the gen-tie's end; the POI when there is no gen-tie) | &lt;MPT&gt; or &lt;MPT&gt;:LV | &lt;MPT&gt;:TV (3-winding) | &lt;MPT&gt;:HV (an MPT with a tie of its own) | &lt;shared collector&gt; (its far end) | &lt;generator&gt;:MV (GSU HV side) | &lt;generator&gt; or &lt;generator&gt;:LV (terminal) | IB (infinite bus). Numbers are automatic from First bus number; Bus_Numbers sets any one.</t>
         </is>
       </c>
     </row>
-    <row r="37" ht="30.0" customHeight="1">
-      <c r="A37" s="12" t="inlineStr">
+    <row r="38" ht="30.0" customHeight="1">
+      <c r="A38" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Plant</t>
         </is>
       </c>
-      <c r="B37" s="8" t="inlineStr">
+      <c r="B38" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Bases, the POI, the grid (SCR and X/R, or short-circuit MVA, or R/X), the gen-tie, the operating point, the plant controller and the PSCAD run settings.</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="56.0" customHeight="1">
-      <c r="A38" s="12" t="inlineStr">
+    <row r="39" ht="56.0" customHeight="1">
+      <c r="A39" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">MODEL TYPE</t>
         </is>
       </c>
-      <c r="B38" s="8" t="inlineStr">
+      <c r="B39" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Plant: Model type sets PSS/E and PSCAD alike. SMIB (default): each generator is one machine behind one GSU on a collector equivalent of its own (WECC, each feeder weighed by its MW) from its MPT winding. DETAILED: every feeder section is a branch (identical feeder copies lumped), the units of a generator at each node a machine of their own behind their own GSU; a generator's Dyr_Params, Dyr_Records and PSCAD_Params rows apply to all its machines.</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="43.0" customHeight="1">
-      <c r="A39" s="8"/>
-      <c r="B39" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Control mode Q: the plant holds the POI voltage with Q at POI into the grid; PF: with that power factor; V: the plant holds the POI voltage with the infinite bus at Grid voltage. The infinite-bus voltage (and the generators' Q) come out of the load flow.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="56.0" customHeight="1">
+    <row r="40" ht="43.0" customHeight="1">
       <c r="A40" s="8"/>
       <c r="B40" s="8" t="inlineStr">
         <is>
+          <t xml:space="preserve">Control mode Q: the plant holds the POI voltage with Q at POI into the grid; PF: with that power factor; V: the plant holds the POI voltage with the infinite bus at Grid voltage. The infinite-bus voltage (and the generators' Q) come out of the load flow.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="56.0" customHeight="1">
+      <c r="A41" s="8"/>
+      <c r="B41" s="8" t="inlineStr">
+        <is>
           <t xml:space="preserve">Plant controller (PSS/E .dyr): REPC_A = a REPCA1 on each generator, each holding the POI; REPC_B = one controller for the whole plant (hybrid PV + BESS): PLNTBU1 at the POI, and on each generator a REAX4BU1 that takes its share of the plant's Q (Qmax / sum of Qmax) and P (Pmax / sum of Pmax). REGC_A / REPC_A records: standard = REGCA1 / REPCA1 from the PSS/E library; USRMDL = REGCAU1 / REPCAU1.</t>
         </is>
       </c>
     </row>
-    <row r="41" ht="30.0" customHeight="1">
-      <c r="A41" s="12" t="inlineStr">
+    <row r="42" ht="30.0" customHeight="1">
+      <c r="A42" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">MPT</t>
         </is>
       </c>
-      <c r="B41" s="8" t="inlineStr">
+      <c r="B42" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">One row per main power transformer; HV winding first. Three windings: TV kV, the three impedances and their bases. Parallel units: identical units in parallel. Tie: a line of its own from HV to it.</t>
         </is>
       </c>
     </row>
-    <row r="42" ht="82.0" customHeight="1">
-      <c r="A42" s="12" t="inlineStr">
+    <row r="43" ht="82.0" customHeight="1">
+      <c r="A43" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Generators</t>
         </is>
       </c>
-      <c r="B42" s="8" t="inlineStr">
+      <c r="B43" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">One row per generator (PV, BESS, wind, synchronous ...): the units (count and one unit's data; the model is their aggregate), its GSU (one GSU's data and the count), its collector (FEEDERS: the WECC equivalent of its rows in Feeders; EQUIVALENT: R X B given; NONE), how it shares the POI's Q, its electrical control model in the .dyr (REEC_A: REECA1, PV and wind; REEC_C: REECCU1, BESS; REEC_D: REECDU1, PV, BESS and WT4) and its PSCAD model (vendor library and definition, or blank for a voltage source at the solved terminal voltage: a network check against PSS/E) and where the inverter connects (LV or MV side of the GSU).</t>
         </is>
       </c>
     </row>
-    <row r="43" ht="56.0" customHeight="1">
-      <c r="A43" s="12" t="inlineStr">
+    <row r="44" ht="56.0" customHeight="1">
+      <c r="A44" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Feeders</t>
         </is>
       </c>
-      <c r="B43" s="8" t="inlineStr">
+      <c r="B44" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">The collector feeders section by section from the collector bus out: cable, length and the units tapped at the section's far end. A daisy chain needs no From section; a lateral names the section it leaves from (its far end); 0 = straight from the collector bus. Copies: identical feeders. WECC equivalent: Zeq = sum(Zi Wi^2) / W^2, Beq = sum(Bi), Wi = MW of the units downstream of section i.</t>
         </is>
       </c>
     </row>
-    <row r="44" ht="17.0" customHeight="1">
-      <c r="A44" s="12" t="inlineStr">
+    <row r="45" ht="17.0" customHeight="1">
+      <c r="A45" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Cables</t>
         </is>
       </c>
-      <c r="B44" s="8" t="inlineStr">
+      <c r="B45" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Cable data per length (R, X in ohm; C in uF or B in uS) and the length unit they are per.</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="30.0" customHeight="1">
-      <c r="A45" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Collectors</t>
-        </is>
-      </c>
-      <c r="B45" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Collector systems shared by more than one generator: name and the bus it starts from. Their Feeders rows say whose units each section carries (Units of); the generators on it Connect to its name.</t>
         </is>
       </c>
     </row>
     <row r="46" ht="30.0" customHeight="1">
       <c r="A46" s="12" t="inlineStr">
         <is>
+          <t xml:space="preserve">Collectors</t>
+        </is>
+      </c>
+      <c r="B46" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Collector systems shared by more than one generator: name and the bus it starts from. Their Feeders rows say whose units each section carries (Units of); the generators on it Connect to its name.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="30.0" customHeight="1">
+      <c r="A47" s="12" t="inlineStr">
+        <is>
           <t xml:space="preserve">Loads_Shunts</t>
         </is>
       </c>
-      <c r="B46" s="8" t="inlineStr">
+      <c r="B47" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Auxiliary loads (constant impedance, MW and MVAr at 1 pu) and shunts (MVAr at 1 pu: + capacitor, - reactor) on any bus.</t>
         </is>
       </c>
     </row>
-    <row r="47" ht="17.0" customHeight="1">
-      <c r="A47" s="12" t="inlineStr">
+    <row r="48" ht="56.0" customHeight="1">
+      <c r="A48" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Machines</t>
+        </is>
+      </c>
+      <c r="B48" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DETAILED model only: a machine's own Pgen, Pmax, Pmin, Qmax, Qmin, fixed Q, MBASE and ID in place of its share of its generator's (the GUI's 'List the DETAILED machines' fills in their names and values). Scale up (GUI) or --scale: a test plant -- MPTs (copies of the first, with its generators), feeders per MPT, GSUs per feeder and inverters per GSU.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="17.0" customHeight="1">
+      <c r="A49" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Bus_Numbers</t>
         </is>
       </c>
-      <c r="B47" s="8" t="inlineStr">
+      <c r="B49" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Bus numbers or names of your own, by role (the report lists every role and its number).</t>
         </is>
       </c>
     </row>
-    <row r="48" ht="82.0" customHeight="1">
-      <c r="A48" s="12" t="inlineStr">
+    <row r="50" ht="82.0" customHeight="1">
+      <c r="A50" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Dyr_Params</t>
         </is>
       </c>
-      <c r="B48" s="8" t="inlineStr">
+      <c r="B50" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Any parameter of the WECC-approved generic models, by generator, model and PSS/E name or position (ICON2, CON14) -- IB for the infinite bus, PLANT for the plant controller. Inverters: REGCA1 (REGC_A) + REECA1 / REECCU1 / REECDU1 (REEC_A / C / D) + REPCA1 (REPC_A) or REAX4BU1 (with PLNTBU1, REPC_B); WT3: + WTDTA1 WTARA1 WTPTA1 WTTQA1; SYNC: GENROU SEXS TGOV1. REECCU1, REECDU1, PLNTBU1, REAX4BU1 (and REGCAU1, REPCAU1) are user models: the WECC user-model DLL must be loaded for the PSS/E check (ADDLIB_IDV / DLLS in the script). The report lists every model's parameters with the values used.</t>
         </is>
       </c>
     </row>
-    <row r="49" ht="43.0" customHeight="1">
-      <c r="A49" s="12" t="inlineStr">
+    <row r="51" ht="43.0" customHeight="1">
+      <c r="A51" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Dyr_Records</t>
         </is>
       </c>
-      <c r="B49" s="8" t="inlineStr">
+      <c r="B51" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Records of your own (vendor or user models), one per row, ending in /. {BUS} {ID} {MBASE} {POI} {IB} {HV} {MV} and {&lt;bus role&gt;} are filled in. Type USER generators have only these. Models in user DLLs: list the DLLs in DLLS in the script for the PSS/E check.</t>
         </is>
       </c>
     </row>
-    <row r="50" ht="69.0" customHeight="1">
-      <c r="A50" s="12" t="inlineStr">
+    <row r="52" ht="69.0" customHeight="1">
+      <c r="A52" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">PSCAD_Params</t>
         </is>
       </c>
-      <c r="B50" s="8" t="inlineStr">
+      <c r="B52" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Parameters of each generator's vendor PSCAD model (UDM), as PSCAD takes them. Filled in for each inverter it stands for (DETAILED: each node): {UNITS} units, {MVA} their MVA, {P_MW} {Q_MVAR} their P and Q where it connects, {P_PU} {Q_PU} on {MVA}, {UNIT_MVA} {UNIT_P_MW} {UNIT_Q_MVAR} one unit's, {V_PU} {V_KV} {KV} {ANGLE} the voltage there, its base and PSCAD angle, {P_INV_MW} {Q_INV_MVAR} {V_INV_PU} at the inverters' own terminals (a UDM on the MV side), {FREQ} -- e.g. Ninv = {UNITS}, Vt0 = {V_PU}.</t>
         </is>
       </c>
     </row>
-    <row r="51" ht="108.0" customHeight="1">
-      <c r="A51" s="12" t="inlineStr">
+    <row r="53" ht="108.0" customHeight="1">
+      <c r="A53" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">PSCAD</t>
         </is>
       </c>
-      <c r="B51" s="8" t="inlineStr">
+      <c r="B53" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">The .pscx is built in the same run when PSCAD 5 and its Python library mhi.pscad (pip install mhi.pscad) are on the PC; otherwise run &lt;name&gt;_build_pscad.py where they are. The case holds the grid (source and Thevenin impedance), the gen-tie, the MPTs, each collector (the WECC equivalent as a pi section, or DETAILED: every feeder section, identical feeder copies lumped), the GSUs and, on each GSU's LV side, the inverter: your UDM (PSCAD library, definition and AC port in Generators) or a stand-in source at the solved voltage -- delete it and wire your UDM in its place (the report and the build log list every inverter node). PSCAD inverter at MV: for a UDM with its GSU inside, the inverter on the GSU's HV side and no GSU drawn. It is drawn as a single-line diagram with wires, left to right from the grid; where PSCAD's R, L and C are single-phase, each is drawn three times between breakouts.</t>
         </is>
@@ -813,8 +843,8 @@
     <mergeCell ref="A2:C2"/>
     <mergeCell ref="A4:C4"/>
     <mergeCell ref="A10:C10"/>
-    <mergeCell ref="A25:C25"/>
-    <mergeCell ref="A32:C32"/>
+    <mergeCell ref="A26:C26"/>
+    <mergeCell ref="A33:C33"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A11" location="'Plant'!A1" display="Plant"/>
@@ -824,12 +854,13 @@
     <hyperlink ref="A15" location="'Cables'!A1" display="Cables"/>
     <hyperlink ref="A16" location="'Collectors'!A1" display="Collectors"/>
     <hyperlink ref="A17" location="'Loads_Shunts'!A1" display="Loads_Shunts"/>
-    <hyperlink ref="A18" location="'Bus_Numbers'!A1" display="Bus_Numbers"/>
-    <hyperlink ref="A19" location="'Dyr_Params'!A1" display="Dyr_Params"/>
-    <hyperlink ref="A20" location="'Dyr_Records'!A1" display="Dyr_Records"/>
-    <hyperlink ref="A21" location="'PSCAD_Params'!A1" display="PSCAD_Params"/>
-    <hyperlink ref="A22" location="'Input_Reference'!A1" display="Input_Reference"/>
-    <hyperlink ref="A23" location="'Dynamic_Models'!A1" display="Dynamic_Models"/>
+    <hyperlink ref="A18" location="'Machines'!A1" display="Machines"/>
+    <hyperlink ref="A19" location="'Bus_Numbers'!A1" display="Bus_Numbers"/>
+    <hyperlink ref="A20" location="'Dyr_Params'!A1" display="Dyr_Params"/>
+    <hyperlink ref="A21" location="'Dyr_Records'!A1" display="Dyr_Records"/>
+    <hyperlink ref="A22" location="'PSCAD_Params'!A1" display="PSCAD_Params"/>
+    <hyperlink ref="A23" location="'Input_Reference'!A1" display="Input_Reference"/>
+    <hyperlink ref="A24" location="'Dynamic_Models'!A1" display="Dynamic_Models"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
@@ -837,6 +868,191 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="FF2E75B6"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <sheetFormatPr defaultRowHeight="14"/>
+  <cols>
+    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="2" max="2" width="10" customWidth="1"/>
+    <col min="3" max="3" width="14" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bus</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Number</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Name</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="52.0" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve"># its role: IB, POI, HV, MPT1:LV, PV:MV, PV:LV ...</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">blank = automatic</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">blank = automatic (12 characters at most)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IB</t>
+        </is>
+      </c>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">POI</t>
+        </is>
+      </c>
+      <c r="B4" s="3"/>
+      <c r="C4" s="3"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">HV</t>
+        </is>
+      </c>
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MPT1:LV</t>
+        </is>
+      </c>
+      <c r="B6" s="3"/>
+      <c r="C6" s="3"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PV:MV</t>
+        </is>
+      </c>
+      <c r="B7" s="3"/>
+      <c r="C7" s="3"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PV:LV</t>
+        </is>
+      </c>
+      <c r="B8" s="3"/>
+      <c r="C8" s="3"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BESS:MV</t>
+        </is>
+      </c>
+      <c r="B9" s="3"/>
+      <c r="C9" s="3"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BESS:LV</t>
+        </is>
+      </c>
+      <c r="B10" s="3"/>
+      <c r="C10" s="3"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="3"/>
+      <c r="B11" s="3"/>
+      <c r="C11" s="3"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="3"/>
+      <c r="B12" s="3"/>
+      <c r="C12" s="3"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3"/>
+      <c r="B13" s="3"/>
+      <c r="C13" s="3"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="3"/>
+      <c r="B14" s="3"/>
+      <c r="C14" s="3"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="3"/>
+      <c r="B15" s="3"/>
+      <c r="C15" s="3"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="3"/>
+      <c r="B16" s="3"/>
+      <c r="C16" s="3"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3"/>
+      <c r="B17" s="3"/>
+      <c r="C17" s="3"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="3"/>
+      <c r="B18" s="3"/>
+      <c r="C18" s="3"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="3"/>
+      <c r="B19" s="3"/>
+      <c r="C19" s="3"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="3"/>
+      <c r="B20" s="3"/>
+      <c r="C20" s="3"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="3"/>
+      <c r="B21" s="3"/>
+      <c r="C21" s="3"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="3"/>
+      <c r="B22" s="3"/>
+      <c r="C22" s="3"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
+  <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FF2E75B6"/>
@@ -1044,7 +1260,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FF2E75B6"/>
@@ -1174,7 +1390,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FF2E75B6"/>
@@ -1351,7 +1567,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FF70AD47"/>
@@ -5768,7 +5984,7 @@
     <row r="141" ht="18" customHeight="1">
       <c r="A141" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bus_Numbers</t>
+          <t xml:space="preserve">Machines</t>
         </is>
       </c>
       <c r="B141" s="7"/>
@@ -5779,20 +5995,20 @@
       <c r="G141" s="7"/>
       <c r="H141" s="7"/>
     </row>
-    <row r="142" ht="17.0" customHeight="1">
+    <row r="142" ht="30.0" customHeight="1">
       <c r="A142" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bus_Numbers</t>
+          <t xml:space="preserve">Machines</t>
         </is>
       </c>
       <c r="B142" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bus</t>
+          <t xml:space="preserve">Machine</t>
         </is>
       </c>
       <c r="C142" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">bus</t>
+          <t xml:space="preserve">machine</t>
         </is>
       </c>
       <c r="D142" s="8"/>
@@ -5800,7 +6016,7 @@
       <c r="F142" s="8"/>
       <c r="G142" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">its role: IB, POI, HV, MPT1:LV, PV:MV, PV:LV ...</t>
+          <t xml:space="preserve">DETAILED model: a machine, &lt;generator&gt;_&lt;feeder&gt;_S&lt;section&gt; (the GUI lists them); its values in place of its share of its generator's</t>
         </is>
       </c>
       <c r="H142" s="13" t="inlineStr">
@@ -5812,29 +6028,29 @@
     <row r="143" ht="17.0" customHeight="1">
       <c r="A143" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bus_Numbers</t>
+          <t xml:space="preserve">Machines</t>
         </is>
       </c>
       <c r="B143" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Number</t>
+          <t xml:space="preserve">Machine ID</t>
         </is>
       </c>
       <c r="C143" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">id</t>
         </is>
       </c>
       <c r="D143" s="8"/>
       <c r="E143" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">automatic</t>
+          <t xml:space="preserve">its generator's</t>
         </is>
       </c>
       <c r="F143" s="8"/>
       <c r="G143" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">blank = automatic</t>
+          <t xml:space="preserve">blank = its generator's</t>
         </is>
       </c>
       <c r="H143" s="13" t="inlineStr">
@@ -5846,29 +6062,29 @@
     <row r="144" ht="30.0" customHeight="1">
       <c r="A144" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bus_Numbers</t>
+          <t xml:space="preserve">Machines</t>
         </is>
       </c>
       <c r="B144" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Name</t>
+          <t xml:space="preserve">Pgen MW</t>
         </is>
       </c>
       <c r="C144" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">name</t>
+          <t xml:space="preserve">pgen_mw</t>
         </is>
       </c>
       <c r="D144" s="8"/>
       <c r="E144" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">automatic (12 characters at most</t>
+          <t xml:space="preserve">its share of its generator's Dispatch MW</t>
         </is>
       </c>
       <c r="F144" s="8"/>
       <c r="G144" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">blank = automatic (12 characters at most)</t>
+          <t xml:space="preserve">its dispatch (blank = its share of its generator's Dispatch MW)</t>
         </is>
       </c>
       <c r="H144" s="13" t="inlineStr">
@@ -5877,198 +6093,238 @@
         </is>
       </c>
     </row>
-    <row r="145" ht="18" customHeight="1">
-      <c r="A145" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Dyr_Params</t>
-        </is>
-      </c>
-      <c r="B145" s="7"/>
-      <c r="C145" s="7"/>
-      <c r="D145" s="7"/>
-      <c r="E145" s="7"/>
-      <c r="F145" s="7"/>
-      <c r="G145" s="7"/>
-      <c r="H145" s="7"/>
+    <row r="145" ht="17.0" customHeight="1">
+      <c r="A145" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Machines</t>
+        </is>
+      </c>
+      <c r="B145" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pmax MW</t>
+        </is>
+      </c>
+      <c r="C145" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pmax_mw</t>
+        </is>
+      </c>
+      <c r="D145" s="8"/>
+      <c r="E145" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">its units x Unit Pmax</t>
+        </is>
+      </c>
+      <c r="F145" s="8"/>
+      <c r="G145" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">blank = its units x Unit Pmax</t>
+        </is>
+      </c>
+      <c r="H145" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSS/E + PSCAD</t>
+        </is>
+      </c>
     </row>
     <row r="146" ht="17.0" customHeight="1">
       <c r="A146" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dyr_Params</t>
+          <t xml:space="preserve">Machines</t>
         </is>
       </c>
       <c r="B146" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Generator</t>
+          <t xml:space="preserve">Pmin MW</t>
         </is>
       </c>
       <c r="C146" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">generator</t>
+          <t xml:space="preserve">pmin_mw</t>
         </is>
       </c>
       <c r="D146" s="8"/>
-      <c r="E146" s="8"/>
+      <c r="E146" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">its units x Unit Pmin</t>
+        </is>
+      </c>
       <c r="F146" s="8"/>
       <c r="G146" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">IB: the infinite bus | PLANT: the plant controller (REPC_B)</t>
+          <t xml:space="preserve">blank = its units x Unit Pmin</t>
         </is>
       </c>
       <c r="H146" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E .dyr</t>
-        </is>
-      </c>
-    </row>
-    <row r="147" ht="30.0" customHeight="1">
+          <t xml:space="preserve">PSS/E + PSCAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="147" ht="17.0" customHeight="1">
       <c r="A147" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dyr_Params</t>
+          <t xml:space="preserve">Machines</t>
         </is>
       </c>
       <c r="B147" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Model</t>
+          <t xml:space="preserve">Qmax MVAr</t>
         </is>
       </c>
       <c r="C147" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">model</t>
+          <t xml:space="preserve">qmax_mvar</t>
         </is>
       </c>
       <c r="D147" s="8"/>
-      <c r="E147" s="8"/>
+      <c r="E147" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">its units x Unit Qmax</t>
+        </is>
+      </c>
       <c r="F147" s="8"/>
       <c r="G147" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">REGCA1 (REGCAU1) | REECA1 REECCU1 REECDU1 | REPCA1 (REPCAU1) or REAX4BU1 | PLANT: PLNTBU1 | WT3: + WTDTA1 WTARA1 WTPTA1 WTTQA1 | SYNC: GENROU SEXS TGOV1 | IB: GENCLS</t>
+          <t xml:space="preserve">blank = its units x Unit Qmax</t>
         </is>
       </c>
       <c r="H147" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E .dyr</t>
+          <t xml:space="preserve">PSS/E + PSCAD</t>
         </is>
       </c>
     </row>
     <row r="148" ht="17.0" customHeight="1">
       <c r="A148" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dyr_Params</t>
+          <t xml:space="preserve">Machines</t>
         </is>
       </c>
       <c r="B148" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Parameter</t>
+          <t xml:space="preserve">Qmin MVAr</t>
         </is>
       </c>
       <c r="C148" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">parameter</t>
+          <t xml:space="preserve">qmin_mvar</t>
         </is>
       </c>
       <c r="D148" s="8"/>
-      <c r="E148" s="8"/>
+      <c r="E148" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">its units x Unit Qmin</t>
+        </is>
+      </c>
       <c r="F148" s="8"/>
       <c r="G148" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E name (the report lists them all) or position: ICON2, CON14</t>
+          <t xml:space="preserve">blank = its units x Unit Qmin</t>
         </is>
       </c>
       <c r="H148" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E .dyr</t>
-        </is>
-      </c>
-    </row>
-    <row r="149" ht="17.0" customHeight="1">
+          <t xml:space="preserve">PSS/E + PSCAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="149" ht="30.0" customHeight="1">
       <c r="A149" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dyr_Params</t>
+          <t xml:space="preserve">Machines</t>
         </is>
       </c>
       <c r="B149" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Value</t>
+          <t xml:space="preserve">Fixed Q MVAr</t>
         </is>
       </c>
       <c r="C149" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">value</t>
+          <t xml:space="preserve">q_mvar</t>
         </is>
       </c>
       <c r="D149" s="8"/>
-      <c r="E149" s="8"/>
+      <c r="E149" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">as its generator's Q mode</t>
+        </is>
+      </c>
       <c r="F149" s="8"/>
-      <c r="G149" s="8"/>
+      <c r="G149" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a value: this Q, fixed (blank = as its generator's Q mode)</t>
+        </is>
+      </c>
       <c r="H149" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E .dyr</t>
-        </is>
-      </c>
-    </row>
-    <row r="150" ht="18" customHeight="1">
-      <c r="A150" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Dyr_Records</t>
-        </is>
-      </c>
-      <c r="B150" s="7"/>
-      <c r="C150" s="7"/>
-      <c r="D150" s="7"/>
-      <c r="E150" s="7"/>
-      <c r="F150" s="7"/>
-      <c r="G150" s="7"/>
-      <c r="H150" s="7"/>
-    </row>
-    <row r="151" ht="17.0" customHeight="1">
-      <c r="A151" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Dyr_Records</t>
-        </is>
-      </c>
-      <c r="B151" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Generator</t>
-        </is>
-      </c>
-      <c r="C151" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">generator</t>
-        </is>
-      </c>
-      <c r="D151" s="8"/>
-      <c r="E151" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">the plant</t>
-        </is>
-      </c>
-      <c r="F151" s="8"/>
-      <c r="G151" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">blank = the plant</t>
-        </is>
-      </c>
-      <c r="H151" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSS/E .dyr</t>
-        </is>
-      </c>
+          <t xml:space="preserve">PSS/E + PSCAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="150" ht="17.0" customHeight="1">
+      <c r="A150" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Machines</t>
+        </is>
+      </c>
+      <c r="B150" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MBASE MVA</t>
+        </is>
+      </c>
+      <c r="C150" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mbase_mva</t>
+        </is>
+      </c>
+      <c r="D150" s="8"/>
+      <c r="E150" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">its units x Unit MVA</t>
+        </is>
+      </c>
+      <c r="F150" s="8"/>
+      <c r="G150" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">blank = its units x Unit MVA</t>
+        </is>
+      </c>
+      <c r="H150" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSS/E + PSCAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="151" ht="18" customHeight="1">
+      <c r="A151" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bus_Numbers</t>
+        </is>
+      </c>
+      <c r="B151" s="7"/>
+      <c r="C151" s="7"/>
+      <c r="D151" s="7"/>
+      <c r="E151" s="7"/>
+      <c r="F151" s="7"/>
+      <c r="G151" s="7"/>
+      <c r="H151" s="7"/>
     </row>
     <row r="152" ht="17.0" customHeight="1">
       <c r="A152" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dyr_Records</t>
+          <t xml:space="preserve">Bus_Numbers</t>
         </is>
       </c>
       <c r="B152" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Record</t>
+          <t xml:space="preserve">Bus</t>
         </is>
       </c>
       <c r="C152" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">record</t>
+          <t xml:space="preserve">bus</t>
         </is>
       </c>
       <c r="D152" s="8"/>
@@ -6076,99 +6332,111 @@
       <c r="F152" s="8"/>
       <c r="G152" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">.dyr text ending in / -- {BUS} {ID} {MBASE} {POI} {IB} {HV} {MV} {&lt;bus role&gt;} are filled in</t>
+          <t xml:space="preserve">its role: IB, POI, HV, MPT1:LV, PV:MV, PV:LV ...</t>
         </is>
       </c>
       <c r="H152" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E .dyr</t>
-        </is>
-      </c>
-    </row>
-    <row r="153" ht="18" customHeight="1">
-      <c r="A153" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSCAD_Params</t>
-        </is>
-      </c>
-      <c r="B153" s="7"/>
-      <c r="C153" s="7"/>
-      <c r="D153" s="7"/>
-      <c r="E153" s="7"/>
-      <c r="F153" s="7"/>
-      <c r="G153" s="7"/>
-      <c r="H153" s="7"/>
-    </row>
-    <row r="154" ht="17.0" customHeight="1">
+          <t xml:space="preserve">PSS/E + PSCAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="153" ht="17.0" customHeight="1">
+      <c r="A153" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bus_Numbers</t>
+        </is>
+      </c>
+      <c r="B153" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Number</t>
+        </is>
+      </c>
+      <c r="C153" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">number</t>
+        </is>
+      </c>
+      <c r="D153" s="8"/>
+      <c r="E153" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">automatic</t>
+        </is>
+      </c>
+      <c r="F153" s="8"/>
+      <c r="G153" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">blank = automatic</t>
+        </is>
+      </c>
+      <c r="H153" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSS/E + PSCAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="154" ht="30.0" customHeight="1">
       <c r="A154" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSCAD_Params</t>
+          <t xml:space="preserve">Bus_Numbers</t>
         </is>
       </c>
       <c r="B154" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Generator</t>
+          <t xml:space="preserve">Name</t>
         </is>
       </c>
       <c r="C154" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">generator</t>
+          <t xml:space="preserve">name</t>
         </is>
       </c>
       <c r="D154" s="8"/>
-      <c r="E154" s="8"/>
+      <c r="E154" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">automatic (12 characters at most</t>
+        </is>
+      </c>
       <c r="F154" s="8"/>
-      <c r="G154" s="8"/>
+      <c r="G154" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">blank = automatic (12 characters at most)</t>
+        </is>
+      </c>
       <c r="H154" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSCAD</t>
-        </is>
-      </c>
-    </row>
-    <row r="155" ht="17.0" customHeight="1">
-      <c r="A155" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSCAD_Params</t>
-        </is>
-      </c>
-      <c r="B155" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Parameter</t>
-        </is>
-      </c>
-      <c r="C155" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">parameter</t>
-        </is>
-      </c>
-      <c r="D155" s="8"/>
-      <c r="E155" s="8"/>
-      <c r="F155" s="8"/>
-      <c r="G155" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">the vendor model's parameter name</t>
-        </is>
-      </c>
-      <c r="H155" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSCAD</t>
-        </is>
-      </c>
+          <t xml:space="preserve">PSS/E + PSCAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="155" ht="18" customHeight="1">
+      <c r="A155" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dyr_Params</t>
+        </is>
+      </c>
+      <c r="B155" s="7"/>
+      <c r="C155" s="7"/>
+      <c r="D155" s="7"/>
+      <c r="E155" s="7"/>
+      <c r="F155" s="7"/>
+      <c r="G155" s="7"/>
+      <c r="H155" s="7"/>
     </row>
     <row r="156" ht="17.0" customHeight="1">
       <c r="A156" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSCAD_Params</t>
+          <t xml:space="preserve">Dyr_Params</t>
         </is>
       </c>
       <c r="B156" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Value</t>
+          <t xml:space="preserve">Generator</t>
         </is>
       </c>
       <c r="C156" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">value</t>
+          <t xml:space="preserve">generator</t>
         </is>
       </c>
       <c r="D156" s="8"/>
@@ -6176,214 +6444,298 @@
       <c r="F156" s="8"/>
       <c r="G156" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">as PSCAD takes it (0.63 [kV], 40, {UNITS}, {P_PU} ...)</t>
+          <t xml:space="preserve">IB: the infinite bus | PLANT: the plant controller (REPC_B)</t>
         </is>
       </c>
       <c r="H156" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSCAD</t>
-        </is>
-      </c>
-    </row>
-    <row r="157" ht="18" customHeight="1">
-      <c r="A157" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">BUS NAMES -- Connect to, At, Bus_Numbers and {&lt;bus&gt;} in Dyr_Records take these</t>
-        </is>
-      </c>
-      <c r="B157" s="7"/>
-      <c r="C157" s="7"/>
-      <c r="D157" s="7"/>
-      <c r="E157" s="7"/>
-      <c r="F157" s="7"/>
-      <c r="G157" s="7"/>
-      <c r="H157" s="7"/>
-    </row>
-    <row r="158">
-      <c r="A158" s="8"/>
+          <t xml:space="preserve">PSS/E .dyr</t>
+        </is>
+      </c>
+    </row>
+    <row r="157" ht="30.0" customHeight="1">
+      <c r="A157" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dyr_Params</t>
+        </is>
+      </c>
+      <c r="B157" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Model</t>
+        </is>
+      </c>
+      <c r="C157" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">model</t>
+        </is>
+      </c>
+      <c r="D157" s="8"/>
+      <c r="E157" s="8"/>
+      <c r="F157" s="8"/>
+      <c r="G157" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REGCA1 (REGCAU1) | REECA1 REECCU1 REECDU1 | REPCA1 (REPCAU1) or REAX4BU1 | PLANT: PLNTBU1 | WT3: + WTDTA1 WTARA1 WTPTA1 WTTQA1 | SYNC: GENROU SEXS TGOV1 | IB: GENCLS</t>
+        </is>
+      </c>
+      <c r="H157" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSS/E .dyr</t>
+        </is>
+      </c>
+    </row>
+    <row r="158" ht="17.0" customHeight="1">
+      <c r="A158" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dyr_Params</t>
+        </is>
+      </c>
       <c r="B158" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">IB</t>
-        </is>
-      </c>
-      <c r="C158" s="8"/>
+          <t xml:space="preserve">Parameter</t>
+        </is>
+      </c>
+      <c r="C158" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">parameter</t>
+        </is>
+      </c>
       <c r="D158" s="8"/>
       <c r="E158" s="8"/>
       <c r="F158" s="8"/>
       <c r="G158" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">the infinite bus</t>
-        </is>
-      </c>
-      <c r="H158" s="8"/>
-    </row>
-    <row r="159">
-      <c r="A159" s="8"/>
+          <t xml:space="preserve">PSS/E name (the report lists them all) or position: ICON2, CON14</t>
+        </is>
+      </c>
+      <c r="H158" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSS/E .dyr</t>
+        </is>
+      </c>
+    </row>
+    <row r="159" ht="17.0" customHeight="1">
+      <c r="A159" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dyr_Params</t>
+        </is>
+      </c>
       <c r="B159" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">POI</t>
-        </is>
-      </c>
-      <c r="C159" s="8"/>
+          <t xml:space="preserve">Value</t>
+        </is>
+      </c>
+      <c r="C159" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">value</t>
+        </is>
+      </c>
       <c r="D159" s="8"/>
       <c r="E159" s="8"/>
       <c r="F159" s="8"/>
-      <c r="G159" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">the point of interconnection</t>
-        </is>
-      </c>
-      <c r="H159" s="8"/>
-    </row>
-    <row r="160">
-      <c r="A160" s="8"/>
-      <c r="B160" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HV</t>
-        </is>
-      </c>
-      <c r="C160" s="8"/>
-      <c r="D160" s="8"/>
-      <c r="E160" s="8"/>
-      <c r="F160" s="8"/>
-      <c r="G160" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">the gen-tie's plant end (the POI when there is no gen-tie)</t>
-        </is>
-      </c>
-      <c r="H160" s="8"/>
-    </row>
-    <row r="161">
-      <c r="A161" s="8"/>
+      <c r="G159" s="8"/>
+      <c r="H159" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSS/E .dyr</t>
+        </is>
+      </c>
+    </row>
+    <row r="160" ht="18" customHeight="1">
+      <c r="A160" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dyr_Records</t>
+        </is>
+      </c>
+      <c r="B160" s="7"/>
+      <c r="C160" s="7"/>
+      <c r="D160" s="7"/>
+      <c r="E160" s="7"/>
+      <c r="F160" s="7"/>
+      <c r="G160" s="7"/>
+      <c r="H160" s="7"/>
+    </row>
+    <row r="161" ht="17.0" customHeight="1">
+      <c r="A161" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dyr_Records</t>
+        </is>
+      </c>
       <c r="B161" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;MPT&gt; or &lt;MPT&gt;:LV</t>
-        </is>
-      </c>
-      <c r="C161" s="8"/>
+          <t xml:space="preserve">Generator</t>
+        </is>
+      </c>
+      <c r="C161" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">generator</t>
+        </is>
+      </c>
       <c r="D161" s="8"/>
-      <c r="E161" s="8"/>
+      <c r="E161" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the plant</t>
+        </is>
+      </c>
       <c r="F161" s="8"/>
       <c r="G161" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">an MPT's LV winding</t>
-        </is>
-      </c>
-      <c r="H161" s="8"/>
-    </row>
-    <row r="162">
-      <c r="A162" s="8"/>
+          <t xml:space="preserve">blank = the plant</t>
+        </is>
+      </c>
+      <c r="H161" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSS/E .dyr</t>
+        </is>
+      </c>
+    </row>
+    <row r="162" ht="17.0" customHeight="1">
+      <c r="A162" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dyr_Records</t>
+        </is>
+      </c>
       <c r="B162" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;MPT&gt;:TV</t>
-        </is>
-      </c>
-      <c r="C162" s="8"/>
+          <t xml:space="preserve">Record</t>
+        </is>
+      </c>
+      <c r="C162" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">record</t>
+        </is>
+      </c>
       <c r="D162" s="8"/>
       <c r="E162" s="8"/>
       <c r="F162" s="8"/>
       <c r="G162" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">a 3-winding MPT's tertiary</t>
-        </is>
-      </c>
-      <c r="H162" s="8"/>
-    </row>
-    <row r="163">
-      <c r="A163" s="8"/>
-      <c r="B163" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">&lt;MPT&gt;:HV</t>
-        </is>
-      </c>
-      <c r="C163" s="8"/>
-      <c r="D163" s="8"/>
-      <c r="E163" s="8"/>
-      <c r="F163" s="8"/>
-      <c r="G163" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">an MPT with a tie line of its own: its HV end</t>
-        </is>
-      </c>
-      <c r="H163" s="8"/>
-    </row>
-    <row r="164">
-      <c r="A164" s="8"/>
+          <t xml:space="preserve">.dyr text ending in / -- {BUS} {ID} {MBASE} {POI} {IB} {HV} {MV} {&lt;bus role&gt;} are filled in</t>
+        </is>
+      </c>
+      <c r="H162" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSS/E .dyr</t>
+        </is>
+      </c>
+    </row>
+    <row r="163" ht="18" customHeight="1">
+      <c r="A163" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD_Params</t>
+        </is>
+      </c>
+      <c r="B163" s="7"/>
+      <c r="C163" s="7"/>
+      <c r="D163" s="7"/>
+      <c r="E163" s="7"/>
+      <c r="F163" s="7"/>
+      <c r="G163" s="7"/>
+      <c r="H163" s="7"/>
+    </row>
+    <row r="164" ht="17.0" customHeight="1">
+      <c r="A164" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD_Params</t>
+        </is>
+      </c>
       <c r="B164" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;collector&gt;</t>
-        </is>
-      </c>
-      <c r="C164" s="8"/>
+          <t xml:space="preserve">Generator</t>
+        </is>
+      </c>
+      <c r="C164" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">generator</t>
+        </is>
+      </c>
       <c r="D164" s="8"/>
       <c r="E164" s="8"/>
       <c r="F164" s="8"/>
-      <c r="G164" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">a shared collector's far end</t>
-        </is>
-      </c>
-      <c r="H164" s="8"/>
-    </row>
-    <row r="165">
-      <c r="A165" s="8"/>
+      <c r="G164" s="8"/>
+      <c r="H164" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="165" ht="17.0" customHeight="1">
+      <c r="A165" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD_Params</t>
+        </is>
+      </c>
       <c r="B165" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;generator&gt;:MV</t>
-        </is>
-      </c>
-      <c r="C165" s="8"/>
+          <t xml:space="preserve">Parameter</t>
+        </is>
+      </c>
+      <c r="C165" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">parameter</t>
+        </is>
+      </c>
       <c r="D165" s="8"/>
       <c r="E165" s="8"/>
       <c r="F165" s="8"/>
       <c r="G165" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">a generator's GSU HV side</t>
-        </is>
-      </c>
-      <c r="H165" s="8"/>
-    </row>
-    <row r="166">
-      <c r="A166" s="8"/>
+          <t xml:space="preserve">the vendor model's parameter name</t>
+        </is>
+      </c>
+      <c r="H165" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="166" ht="17.0" customHeight="1">
+      <c r="A166" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD_Params</t>
+        </is>
+      </c>
       <c r="B166" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;generator&gt; or &lt;generator&gt;:LV</t>
-        </is>
-      </c>
-      <c r="C166" s="8"/>
+          <t xml:space="preserve">Value</t>
+        </is>
+      </c>
+      <c r="C166" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">value</t>
+        </is>
+      </c>
       <c r="D166" s="8"/>
       <c r="E166" s="8"/>
       <c r="F166" s="8"/>
       <c r="G166" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">a generator's terminal</t>
-        </is>
-      </c>
-      <c r="H166" s="8"/>
-    </row>
-    <row r="167">
-      <c r="A167" s="8"/>
-      <c r="B167" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">&lt;collector&gt;_&lt;feeder&gt;_S&lt;n&gt;</t>
-        </is>
-      </c>
-      <c r="C167" s="8"/>
-      <c r="D167" s="8"/>
-      <c r="E167" s="8"/>
-      <c r="F167" s="8"/>
-      <c r="G167" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DETAILED: the far end of feeder section n</t>
-        </is>
-      </c>
-      <c r="H167" s="8"/>
+          <t xml:space="preserve">as PSCAD takes it (0.63 [kV], 40, {UNITS}, {P_PU} ...)</t>
+        </is>
+      </c>
+      <c r="H166" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="167" ht="18" customHeight="1">
+      <c r="A167" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BUS NAMES -- Connect to, At, Bus_Numbers and {&lt;bus&gt;} in Dyr_Records take these</t>
+        </is>
+      </c>
+      <c r="B167" s="7"/>
+      <c r="C167" s="7"/>
+      <c r="D167" s="7"/>
+      <c r="E167" s="7"/>
+      <c r="F167" s="7"/>
+      <c r="G167" s="7"/>
+      <c r="H167" s="7"/>
     </row>
     <row r="168">
       <c r="A168" s="8"/>
       <c r="B168" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;generator&gt;_&lt;feeder&gt;_S&lt;n&gt;:LV</t>
+          <t xml:space="preserve">IB</t>
         </is>
       </c>
       <c r="C168" s="8"/>
@@ -6392,34 +6744,34 @@
       <c r="F168" s="8"/>
       <c r="G168" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">DETAILED: the terminal of the units at that node</t>
+          <t xml:space="preserve">the infinite bus</t>
         </is>
       </c>
       <c r="H168" s="8"/>
     </row>
-    <row r="169" ht="18" customHeight="1">
-      <c r="A169" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSCAD_Params PLACEHOLDERS -- filled in for each inverter a vendor model stands for</t>
-        </is>
-      </c>
-      <c r="B169" s="7"/>
-      <c r="C169" s="7"/>
-      <c r="D169" s="7"/>
-      <c r="E169" s="7"/>
-      <c r="F169" s="7"/>
-      <c r="G169" s="7"/>
-      <c r="H169" s="7"/>
+    <row r="169">
+      <c r="A169" s="8"/>
+      <c r="B169" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">POI</t>
+        </is>
+      </c>
+      <c r="C169" s="8"/>
+      <c r="D169" s="8"/>
+      <c r="E169" s="8"/>
+      <c r="F169" s="8"/>
+      <c r="G169" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the point of interconnection</t>
+        </is>
+      </c>
+      <c r="H169" s="8"/>
     </row>
     <row r="170">
-      <c r="A170" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSCAD_Params</t>
-        </is>
-      </c>
+      <c r="A170" s="8"/>
       <c r="B170" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{UNITS}</t>
+          <t xml:space="preserve">HV</t>
         </is>
       </c>
       <c r="C170" s="8"/>
@@ -6428,24 +6780,16 @@
       <c r="F170" s="8"/>
       <c r="G170" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">the units the inverter stands for</t>
-        </is>
-      </c>
-      <c r="H170" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSCAD</t>
-        </is>
-      </c>
+          <t xml:space="preserve">the gen-tie's plant end (the POI when there is no gen-tie)</t>
+        </is>
+      </c>
+      <c r="H170" s="8"/>
     </row>
     <row r="171">
-      <c r="A171" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSCAD_Params</t>
-        </is>
-      </c>
+      <c r="A171" s="8"/>
       <c r="B171" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{MVA}</t>
+          <t xml:space="preserve">&lt;MPT&gt; or &lt;MPT&gt;:LV</t>
         </is>
       </c>
       <c r="C171" s="8"/>
@@ -6454,24 +6798,16 @@
       <c r="F171" s="8"/>
       <c r="G171" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">their MVA</t>
-        </is>
-      </c>
-      <c r="H171" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSCAD</t>
-        </is>
-      </c>
+          <t xml:space="preserve">an MPT's LV winding</t>
+        </is>
+      </c>
+      <c r="H171" s="8"/>
     </row>
     <row r="172">
-      <c r="A172" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSCAD_Params</t>
-        </is>
-      </c>
+      <c r="A172" s="8"/>
       <c r="B172" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{P_MW}</t>
+          <t xml:space="preserve">&lt;MPT&gt;:TV</t>
         </is>
       </c>
       <c r="C172" s="8"/>
@@ -6480,24 +6816,16 @@
       <c r="F172" s="8"/>
       <c r="G172" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">their P where the inverter connects (MW)</t>
-        </is>
-      </c>
-      <c r="H172" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSCAD</t>
-        </is>
-      </c>
+          <t xml:space="preserve">a 3-winding MPT's tertiary</t>
+        </is>
+      </c>
+      <c r="H172" s="8"/>
     </row>
     <row r="173">
-      <c r="A173" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSCAD_Params</t>
-        </is>
-      </c>
+      <c r="A173" s="8"/>
       <c r="B173" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{Q_MVAR}</t>
+          <t xml:space="preserve">&lt;MPT&gt;:HV</t>
         </is>
       </c>
       <c r="C173" s="8"/>
@@ -6506,24 +6834,16 @@
       <c r="F173" s="8"/>
       <c r="G173" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">their Q there (MVAr)</t>
-        </is>
-      </c>
-      <c r="H173" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSCAD</t>
-        </is>
-      </c>
+          <t xml:space="preserve">an MPT with a tie line of its own: its HV end</t>
+        </is>
+      </c>
+      <c r="H173" s="8"/>
     </row>
     <row r="174">
-      <c r="A174" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSCAD_Params</t>
-        </is>
-      </c>
+      <c r="A174" s="8"/>
       <c r="B174" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{P_PU}</t>
+          <t xml:space="preserve">&lt;collector&gt;</t>
         </is>
       </c>
       <c r="C174" s="8"/>
@@ -6532,24 +6852,16 @@
       <c r="F174" s="8"/>
       <c r="G174" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">P on {MVA}</t>
-        </is>
-      </c>
-      <c r="H174" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSCAD</t>
-        </is>
-      </c>
+          <t xml:space="preserve">a shared collector's far end</t>
+        </is>
+      </c>
+      <c r="H174" s="8"/>
     </row>
     <row r="175">
-      <c r="A175" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSCAD_Params</t>
-        </is>
-      </c>
+      <c r="A175" s="8"/>
       <c r="B175" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{Q_PU}</t>
+          <t xml:space="preserve">&lt;generator&gt;:MV</t>
         </is>
       </c>
       <c r="C175" s="8"/>
@@ -6558,24 +6870,16 @@
       <c r="F175" s="8"/>
       <c r="G175" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q on {MVA}</t>
-        </is>
-      </c>
-      <c r="H175" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSCAD</t>
-        </is>
-      </c>
+          <t xml:space="preserve">a generator's GSU HV side</t>
+        </is>
+      </c>
+      <c r="H175" s="8"/>
     </row>
     <row r="176">
-      <c r="A176" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSCAD_Params</t>
-        </is>
-      </c>
+      <c r="A176" s="8"/>
       <c r="B176" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{UNIT_MVA}</t>
+          <t xml:space="preserve">&lt;generator&gt; or &lt;generator&gt;:LV</t>
         </is>
       </c>
       <c r="C176" s="8"/>
@@ -6584,24 +6888,16 @@
       <c r="F176" s="8"/>
       <c r="G176" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">one unit's MVA</t>
-        </is>
-      </c>
-      <c r="H176" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSCAD</t>
-        </is>
-      </c>
+          <t xml:space="preserve">a generator's terminal</t>
+        </is>
+      </c>
+      <c r="H176" s="8"/>
     </row>
     <row r="177">
-      <c r="A177" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSCAD_Params</t>
-        </is>
-      </c>
+      <c r="A177" s="8"/>
       <c r="B177" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{UNIT_P_MW}</t>
+          <t xml:space="preserve">&lt;collector&gt;_&lt;feeder&gt;_S&lt;n&gt;</t>
         </is>
       </c>
       <c r="C177" s="8"/>
@@ -6610,24 +6906,16 @@
       <c r="F177" s="8"/>
       <c r="G177" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">one unit's P (MW)</t>
-        </is>
-      </c>
-      <c r="H177" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSCAD</t>
-        </is>
-      </c>
+          <t xml:space="preserve">DETAILED: the far end of feeder section n</t>
+        </is>
+      </c>
+      <c r="H177" s="8"/>
     </row>
     <row r="178">
-      <c r="A178" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSCAD_Params</t>
-        </is>
-      </c>
+      <c r="A178" s="8"/>
       <c r="B178" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{UNIT_Q_MVAR}</t>
+          <t xml:space="preserve">&lt;generator&gt;_&lt;feeder&gt;_S&lt;n&gt;:LV</t>
         </is>
       </c>
       <c r="C178" s="8"/>
@@ -6636,40 +6924,24 @@
       <c r="F178" s="8"/>
       <c r="G178" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">one unit's Q (MVAr)</t>
-        </is>
-      </c>
-      <c r="H178" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSCAD</t>
-        </is>
-      </c>
-    </row>
-    <row r="179">
-      <c r="A179" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSCAD_Params</t>
-        </is>
-      </c>
-      <c r="B179" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">{V_PU}</t>
-        </is>
-      </c>
-      <c r="C179" s="8"/>
-      <c r="D179" s="8"/>
-      <c r="E179" s="8"/>
-      <c r="F179" s="8"/>
-      <c r="G179" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">the voltage where it connects (pu)</t>
-        </is>
-      </c>
-      <c r="H179" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSCAD</t>
-        </is>
-      </c>
+          <t xml:space="preserve">DETAILED: the terminal of the units at that node</t>
+        </is>
+      </c>
+      <c r="H178" s="8"/>
+    </row>
+    <row r="179" ht="18" customHeight="1">
+      <c r="A179" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD_Params PLACEHOLDERS -- filled in for each inverter a vendor model stands for</t>
+        </is>
+      </c>
+      <c r="B179" s="7"/>
+      <c r="C179" s="7"/>
+      <c r="D179" s="7"/>
+      <c r="E179" s="7"/>
+      <c r="F179" s="7"/>
+      <c r="G179" s="7"/>
+      <c r="H179" s="7"/>
     </row>
     <row r="180">
       <c r="A180" s="8" t="inlineStr">
@@ -6679,7 +6951,7 @@
       </c>
       <c r="B180" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{V_KV}</t>
+          <t xml:space="preserve">{UNITS}</t>
         </is>
       </c>
       <c r="C180" s="8"/>
@@ -6688,7 +6960,7 @@
       <c r="F180" s="8"/>
       <c r="G180" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">the same in kV</t>
+          <t xml:space="preserve">the units the inverter stands for</t>
         </is>
       </c>
       <c r="H180" s="13" t="inlineStr">
@@ -6705,7 +6977,7 @@
       </c>
       <c r="B181" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{KV}</t>
+          <t xml:space="preserve">{MVA}</t>
         </is>
       </c>
       <c r="C181" s="8"/>
@@ -6714,7 +6986,7 @@
       <c r="F181" s="8"/>
       <c r="G181" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">that bus's base kV</t>
+          <t xml:space="preserve">their MVA</t>
         </is>
       </c>
       <c r="H181" s="13" t="inlineStr">
@@ -6731,7 +7003,7 @@
       </c>
       <c r="B182" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{ANGLE}</t>
+          <t xml:space="preserve">{P_MW}</t>
         </is>
       </c>
       <c r="C182" s="8"/>
@@ -6740,7 +7012,7 @@
       <c r="F182" s="8"/>
       <c r="G182" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">its PSCAD angle (deg, the transformers' phase shifts included)</t>
+          <t xml:space="preserve">their P where the inverter connects (MW)</t>
         </is>
       </c>
       <c r="H182" s="13" t="inlineStr">
@@ -6757,7 +7029,7 @@
       </c>
       <c r="B183" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{FREQ}</t>
+          <t xml:space="preserve">{Q_MVAR}</t>
         </is>
       </c>
       <c r="C183" s="8"/>
@@ -6766,7 +7038,7 @@
       <c r="F183" s="8"/>
       <c r="G183" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">frequency (Hz)</t>
+          <t xml:space="preserve">their Q there (MVAr)</t>
         </is>
       </c>
       <c r="H183" s="13" t="inlineStr">
@@ -6783,7 +7055,7 @@
       </c>
       <c r="B184" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{P_INV_MW}</t>
+          <t xml:space="preserve">{P_PU}</t>
         </is>
       </c>
       <c r="C184" s="8"/>
@@ -6792,7 +7064,7 @@
       <c r="F184" s="8"/>
       <c r="G184" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">P at the inverters' own terminals (MW; a UDM on the MV side)</t>
+          <t xml:space="preserve">P on {MVA}</t>
         </is>
       </c>
       <c r="H184" s="13" t="inlineStr">
@@ -6809,7 +7081,7 @@
       </c>
       <c r="B185" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{Q_INV_MVAR}</t>
+          <t xml:space="preserve">{Q_PU}</t>
         </is>
       </c>
       <c r="C185" s="8"/>
@@ -6818,7 +7090,7 @@
       <c r="F185" s="8"/>
       <c r="G185" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q there (MVAr)</t>
+          <t xml:space="preserve">Q on {MVA}</t>
         </is>
       </c>
       <c r="H185" s="13" t="inlineStr">
@@ -6835,7 +7107,7 @@
       </c>
       <c r="B186" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{V_INV_PU}</t>
+          <t xml:space="preserve">{UNIT_MVA}</t>
         </is>
       </c>
       <c r="C186" s="8"/>
@@ -6844,17 +7116,277 @@
       <c r="F186" s="8"/>
       <c r="G186" s="8" t="inlineStr">
         <is>
+          <t xml:space="preserve">one unit's MVA</t>
+        </is>
+      </c>
+      <c r="H186" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="187">
+      <c r="A187" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD_Params</t>
+        </is>
+      </c>
+      <c r="B187" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{UNIT_P_MW}</t>
+        </is>
+      </c>
+      <c r="C187" s="8"/>
+      <c r="D187" s="8"/>
+      <c r="E187" s="8"/>
+      <c r="F187" s="8"/>
+      <c r="G187" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">one unit's P (MW)</t>
+        </is>
+      </c>
+      <c r="H187" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="188">
+      <c r="A188" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD_Params</t>
+        </is>
+      </c>
+      <c r="B188" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{UNIT_Q_MVAR}</t>
+        </is>
+      </c>
+      <c r="C188" s="8"/>
+      <c r="D188" s="8"/>
+      <c r="E188" s="8"/>
+      <c r="F188" s="8"/>
+      <c r="G188" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">one unit's Q (MVAr)</t>
+        </is>
+      </c>
+      <c r="H188" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="189">
+      <c r="A189" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD_Params</t>
+        </is>
+      </c>
+      <c r="B189" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{V_PU}</t>
+        </is>
+      </c>
+      <c r="C189" s="8"/>
+      <c r="D189" s="8"/>
+      <c r="E189" s="8"/>
+      <c r="F189" s="8"/>
+      <c r="G189" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the voltage where it connects (pu)</t>
+        </is>
+      </c>
+      <c r="H189" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="190">
+      <c r="A190" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD_Params</t>
+        </is>
+      </c>
+      <c r="B190" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{V_KV}</t>
+        </is>
+      </c>
+      <c r="C190" s="8"/>
+      <c r="D190" s="8"/>
+      <c r="E190" s="8"/>
+      <c r="F190" s="8"/>
+      <c r="G190" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the same in kV</t>
+        </is>
+      </c>
+      <c r="H190" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD_Params</t>
+        </is>
+      </c>
+      <c r="B191" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{KV}</t>
+        </is>
+      </c>
+      <c r="C191" s="8"/>
+      <c r="D191" s="8"/>
+      <c r="E191" s="8"/>
+      <c r="F191" s="8"/>
+      <c r="G191" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">that bus's base kV</t>
+        </is>
+      </c>
+      <c r="H191" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="192">
+      <c r="A192" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD_Params</t>
+        </is>
+      </c>
+      <c r="B192" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{ANGLE}</t>
+        </is>
+      </c>
+      <c r="C192" s="8"/>
+      <c r="D192" s="8"/>
+      <c r="E192" s="8"/>
+      <c r="F192" s="8"/>
+      <c r="G192" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">its PSCAD angle (deg, the transformers' phase shifts included)</t>
+        </is>
+      </c>
+      <c r="H192" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="193">
+      <c r="A193" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD_Params</t>
+        </is>
+      </c>
+      <c r="B193" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{FREQ}</t>
+        </is>
+      </c>
+      <c r="C193" s="8"/>
+      <c r="D193" s="8"/>
+      <c r="E193" s="8"/>
+      <c r="F193" s="8"/>
+      <c r="G193" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">frequency (Hz)</t>
+        </is>
+      </c>
+      <c r="H193" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="194">
+      <c r="A194" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD_Params</t>
+        </is>
+      </c>
+      <c r="B194" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{P_INV_MW}</t>
+        </is>
+      </c>
+      <c r="C194" s="8"/>
+      <c r="D194" s="8"/>
+      <c r="E194" s="8"/>
+      <c r="F194" s="8"/>
+      <c r="G194" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P at the inverters' own terminals (MW; a UDM on the MV side)</t>
+        </is>
+      </c>
+      <c r="H194" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="195">
+      <c r="A195" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD_Params</t>
+        </is>
+      </c>
+      <c r="B195" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{Q_INV_MVAR}</t>
+        </is>
+      </c>
+      <c r="C195" s="8"/>
+      <c r="D195" s="8"/>
+      <c r="E195" s="8"/>
+      <c r="F195" s="8"/>
+      <c r="G195" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Q there (MVAr)</t>
+        </is>
+      </c>
+      <c r="H195" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="196">
+      <c r="A196" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD_Params</t>
+        </is>
+      </c>
+      <c r="B196" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{V_INV_PU}</t>
+        </is>
+      </c>
+      <c r="C196" s="8"/>
+      <c r="D196" s="8"/>
+      <c r="E196" s="8"/>
+      <c r="F196" s="8"/>
+      <c r="G196" s="8" t="inlineStr">
+        <is>
           <t xml:space="preserve">the voltage there (pu)</t>
         </is>
       </c>
-      <c r="H186" s="13" t="inlineStr">
+      <c r="H196" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">PSCAD</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="15">
+  <mergeCells count="16">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A4:H4"/>
@@ -6865,11 +7397,12 @@
     <mergeCell ref="A132:H132"/>
     <mergeCell ref="A135:H135"/>
     <mergeCell ref="A141:H141"/>
-    <mergeCell ref="A145:H145"/>
-    <mergeCell ref="A150:H150"/>
-    <mergeCell ref="A153:H153"/>
-    <mergeCell ref="A157:H157"/>
-    <mergeCell ref="A169:H169"/>
+    <mergeCell ref="A151:H151"/>
+    <mergeCell ref="A155:H155"/>
+    <mergeCell ref="A160:H160"/>
+    <mergeCell ref="A163:H163"/>
+    <mergeCell ref="A167:H167"/>
+    <mergeCell ref="A179:H179"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A4" location="'Plant'!A1" display="Plant"/>
@@ -6879,18 +7412,19 @@
     <hyperlink ref="A125" location="'Cables'!A1" display="Cables"/>
     <hyperlink ref="A132" location="'Collectors'!A1" display="Collectors"/>
     <hyperlink ref="A135" location="'Loads_Shunts'!A1" display="Loads_Shunts"/>
-    <hyperlink ref="A141" location="'Bus_Numbers'!A1" display="Bus_Numbers"/>
-    <hyperlink ref="A145" location="'Dyr_Params'!A1" display="Dyr_Params"/>
-    <hyperlink ref="A150" location="'Dyr_Records'!A1" display="Dyr_Records"/>
-    <hyperlink ref="A153" location="'PSCAD_Params'!A1" display="PSCAD_Params"/>
-    <hyperlink ref="A169" location="'PSCAD_Params'!A1" display="PSCAD_Params"/>
+    <hyperlink ref="A141" location="'Machines'!A1" display="Machines"/>
+    <hyperlink ref="A151" location="'Bus_Numbers'!A1" display="Bus_Numbers"/>
+    <hyperlink ref="A155" location="'Dyr_Params'!A1" display="Dyr_Params"/>
+    <hyperlink ref="A160" location="'Dyr_Records'!A1" display="Dyr_Records"/>
+    <hyperlink ref="A163" location="'PSCAD_Params'!A1" display="PSCAD_Params"/>
+    <hyperlink ref="A179" location="'PSCAD_Params'!A1" display="PSCAD_Params"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="FF70AD47"/>
@@ -22452,176 +22986,330 @@
   </sheetPr>
   <sheetFormatPr defaultRowHeight="14"/>
   <cols>
-    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="1" max="1" width="16" customWidth="1"/>
     <col min="2" max="2" width="10" customWidth="1"/>
-    <col min="3" max="3" width="14" customWidth="1"/>
+    <col min="3" max="3" width="10" customWidth="1"/>
+    <col min="4" max="4" width="10" customWidth="1"/>
+    <col min="5" max="5" width="10" customWidth="1"/>
+    <col min="6" max="6" width="10" customWidth="1"/>
+    <col min="7" max="7" width="10" customWidth="1"/>
+    <col min="8" max="8" width="10" customWidth="1"/>
+    <col min="9" max="9" width="10" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bus</t>
+          <t xml:space="preserve">Machine</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Number</t>
+          <t xml:space="preserve">Machine ID</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Name</t>
-        </is>
-      </c>
-    </row>
-    <row r="2" ht="52.0" customHeight="1">
+          <t xml:space="preserve">Pgen MW</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pmax MW</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pmin MW</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Qmax MVAr</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Qmin MVAr</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed Q MVAr</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MBASE MVA</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="100.0" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"># its role: IB, POI, HV, MPT1:LV, PV:MV, PV:LV ...</t>
+          <t xml:space="preserve"># DETAILED model: a machine, &lt;generator&gt;_&lt;feeder&gt;_S&lt;section&gt; (the GUI lists them); its values in place of its share of its generator's</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">blank = automatic</t>
+          <t xml:space="preserve">blank = its generator's</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">blank = automatic (12 characters at most)</t>
+          <t xml:space="preserve">its dispatch (blank = its share of its generator's Dispatch MW)</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">blank = its units x Unit Pmax</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">blank = its units x Unit Pmin</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">blank = its units x Unit Qmax</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">blank = its units x Unit Qmin</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a value: this Q, fixed (blank = as its generator's Q mode)</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">blank = its units x Unit MVA</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">IB</t>
-        </is>
-      </c>
+      <c r="A3" s="3"/>
       <c r="B3" s="3"/>
       <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+      <c r="I3" s="3"/>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">POI</t>
-        </is>
-      </c>
+      <c r="A4" s="3"/>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
+      <c r="H4" s="3"/>
+      <c r="I4" s="3"/>
     </row>
     <row r="5">
-      <c r="A5" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HV</t>
-        </is>
-      </c>
+      <c r="A5" s="3"/>
       <c r="B5" s="3"/>
       <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+      <c r="I5" s="3"/>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MPT1:LV</t>
-        </is>
-      </c>
+      <c r="A6" s="3"/>
       <c r="B6" s="3"/>
       <c r="C6" s="3"/>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
+      <c r="H6" s="3"/>
+      <c r="I6" s="3"/>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PV:MV</t>
-        </is>
-      </c>
+      <c r="A7" s="3"/>
       <c r="B7" s="3"/>
       <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="3"/>
+      <c r="I7" s="3"/>
     </row>
     <row r="8">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PV:LV</t>
-        </is>
-      </c>
+      <c r="A8" s="3"/>
       <c r="B8" s="3"/>
       <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
+      <c r="H8" s="3"/>
+      <c r="I8" s="3"/>
     </row>
     <row r="9">
-      <c r="A9" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">BESS:MV</t>
-        </is>
-      </c>
+      <c r="A9" s="3"/>
       <c r="B9" s="3"/>
       <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
+      <c r="H9" s="3"/>
+      <c r="I9" s="3"/>
     </row>
     <row r="10">
-      <c r="A10" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">BESS:LV</t>
-        </is>
-      </c>
+      <c r="A10" s="3"/>
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
+      <c r="H10" s="3"/>
+      <c r="I10" s="3"/>
     </row>
     <row r="11">
       <c r="A11" s="3"/>
       <c r="B11" s="3"/>
       <c r="C11" s="3"/>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
+      <c r="F11" s="3"/>
+      <c r="G11" s="3"/>
+      <c r="H11" s="3"/>
+      <c r="I11" s="3"/>
     </row>
     <row r="12">
       <c r="A12" s="3"/>
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
+      <c r="F12" s="3"/>
+      <c r="G12" s="3"/>
+      <c r="H12" s="3"/>
+      <c r="I12" s="3"/>
     </row>
     <row r="13">
       <c r="A13" s="3"/>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3"/>
+      <c r="F13" s="3"/>
+      <c r="G13" s="3"/>
+      <c r="H13" s="3"/>
+      <c r="I13" s="3"/>
     </row>
     <row r="14">
       <c r="A14" s="3"/>
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="3"/>
+      <c r="H14" s="3"/>
+      <c r="I14" s="3"/>
     </row>
     <row r="15">
       <c r="A15" s="3"/>
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
+      <c r="D15" s="3"/>
+      <c r="E15" s="3"/>
+      <c r="F15" s="3"/>
+      <c r="G15" s="3"/>
+      <c r="H15" s="3"/>
+      <c r="I15" s="3"/>
     </row>
     <row r="16">
       <c r="A16" s="3"/>
       <c r="B16" s="3"/>
       <c r="C16" s="3"/>
+      <c r="D16" s="3"/>
+      <c r="E16" s="3"/>
+      <c r="F16" s="3"/>
+      <c r="G16" s="3"/>
+      <c r="H16" s="3"/>
+      <c r="I16" s="3"/>
     </row>
     <row r="17">
       <c r="A17" s="3"/>
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
+      <c r="D17" s="3"/>
+      <c r="E17" s="3"/>
+      <c r="F17" s="3"/>
+      <c r="G17" s="3"/>
+      <c r="H17" s="3"/>
+      <c r="I17" s="3"/>
     </row>
     <row r="18">
       <c r="A18" s="3"/>
       <c r="B18" s="3"/>
       <c r="C18" s="3"/>
+      <c r="D18" s="3"/>
+      <c r="E18" s="3"/>
+      <c r="F18" s="3"/>
+      <c r="G18" s="3"/>
+      <c r="H18" s="3"/>
+      <c r="I18" s="3"/>
     </row>
     <row r="19">
       <c r="A19" s="3"/>
       <c r="B19" s="3"/>
       <c r="C19" s="3"/>
+      <c r="D19" s="3"/>
+      <c r="E19" s="3"/>
+      <c r="F19" s="3"/>
+      <c r="G19" s="3"/>
+      <c r="H19" s="3"/>
+      <c r="I19" s="3"/>
     </row>
     <row r="20">
       <c r="A20" s="3"/>
       <c r="B20" s="3"/>
       <c r="C20" s="3"/>
+      <c r="D20" s="3"/>
+      <c r="E20" s="3"/>
+      <c r="F20" s="3"/>
+      <c r="G20" s="3"/>
+      <c r="H20" s="3"/>
+      <c r="I20" s="3"/>
     </row>
     <row r="21">
       <c r="A21" s="3"/>
       <c r="B21" s="3"/>
       <c r="C21" s="3"/>
+      <c r="D21" s="3"/>
+      <c r="E21" s="3"/>
+      <c r="F21" s="3"/>
+      <c r="G21" s="3"/>
+      <c r="H21" s="3"/>
+      <c r="I21" s="3"/>
     </row>
     <row r="22">
       <c r="A22" s="3"/>
       <c r="B22" s="3"/>
       <c r="C22" s="3"/>
+      <c r="D22" s="3"/>
+      <c r="E22" s="3"/>
+      <c r="F22" s="3"/>
+      <c r="G22" s="3"/>
+      <c r="H22" s="3"/>
+      <c r="I22" s="3"/>
     </row>
   </sheetData>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
smib_build GUI: every .dyr parameter shown and editable in Dyr_Params
The Dyr_Params tab shows every model's parameters with the values the .dyr gets -- a column per generator
(PV, BESS ..., IB, PLANT), your values marked; double-click one to change it (a Dyr_Params row), clear it to go
back to the default. Your rows stay listed below it.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BGsNUhFmVX23f8qnP53zUv
</commit_message>
<xml_diff>
--- a/smib/SMIB_INPUT_TEMPLATE.xlsx
+++ b/smib/SMIB_INPUT_TEMPLATE.xlsx
@@ -789,7 +789,7 @@
         </is>
       </c>
     </row>
-    <row r="50" ht="82.0" customHeight="1">
+    <row r="50" ht="108.0" customHeight="1">
       <c r="A50" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Dyr_Params</t>
@@ -797,7 +797,7 @@
       </c>
       <c r="B50" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Any parameter of the WECC-approved generic models, by generator, model and PSS/E name or position (ICON2, CON14) -- IB for the infinite bus, PLANT for the plant controller. Inverters: REGCA1 (REGC_A) + REECA1 / REECCU1 / REECDU1 (REEC_A / C / D) + REPCA1 (REPC_A) or REAX4BU1 (with PLNTBU1, REPC_B); WT3: + WTDTA1 WTARA1 WTPTA1 WTTQA1; SYNC: GENROU SEXS TGOV1. REECCU1, REECDU1, PLNTBU1, REAX4BU1 (and REGCAU1, REPCAU1) are user models: the WECC user-model DLL must be loaded for the PSS/E check (ADDLIB_IDV / DLLS in the script). The report lists every model's parameters with the values used.</t>
+          <t xml:space="preserve">Any parameter of the WECC-approved generic models, by generator, model and PSS/E name or position (ICON2, CON14) -- IB for the infinite bus, PLANT for the plant controller. Inverters: REGCA1 (REGC_A) + REECA1 / REECCU1 / REECDU1 (REEC_A / C / D) + REPCA1 (REPC_A) or REAX4BU1 (with PLNTBU1, REPC_B); WT3: + WTDTA1 WTARA1 WTPTA1 WTTQA1; SYNC: GENROU SEXS TGOV1. REECCU1, REECDU1, PLNTBU1, REAX4BU1 (and REGCAU1, REPCAU1) are user models: the WECC user-model DLL must be loaded for the PSS/E check (ADDLIB_IDV / DLLS in the script). The report lists every model's parameters with the values used. In the GUI, the Dyr_Params tab shows every model's parameters with the values the .dyr gets, a column per generator: double-click one to change it (it becomes a row here), clear it to go back to the default.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
smib_build PSCAD: PI Sections wired at their drawn ends; a set-up UDM copied to every GSU
- PI Sections: PSCAD reports their ports away from where it draws them -- the build now centres each PI on its
  place by its drawn extent (bounds) and wires its two drawn ends; the log says what PSCAD reported
- Generators: PSCAD source case + PSCAD component ID -- one UDM set up in a case of its own (a vendor's test
  case) is copied, settings and all, to every GSU of the generator (every DETAILED machine): the first by copy
  and paste with its definition, the rest cloned; the source case's resources (.lib, .obj) added to the case;
  PSCAD_Params ({UNITS}, {P_PU} ...) set on each copy

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BGsNUhFmVX23f8qnP53zUv
</commit_message>
<xml_diff>
--- a/smib/SMIB_INPUT_TEMPLATE.xlsx
+++ b/smib/SMIB_INPUT_TEMPLATE.xlsx
@@ -825,7 +825,7 @@
         </is>
       </c>
     </row>
-    <row r="53" ht="108.0" customHeight="1">
+    <row r="53" ht="160.0" customHeight="1">
       <c r="A53" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">PSCAD</t>
@@ -833,7 +833,7 @@
       </c>
       <c r="B53" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">The .pscx is built in the same run when PSCAD 5 and its Python library mhi.pscad (pip install mhi.pscad) are on the PC; otherwise run &lt;name&gt;_build_pscad.py where they are. The case holds the grid (source and Thevenin impedance), the gen-tie, the MPTs, each collector (the WECC equivalent as a pi section, or DETAILED: every feeder section, identical feeder copies lumped), the GSUs and, on each GSU's LV side, the inverter: your UDM (PSCAD library, definition and AC port in Generators) or a stand-in source at the solved voltage -- delete it and wire your UDM in its place (the report and the build log list every inverter node). PSCAD inverter at MV: for a UDM with its GSU inside, the inverter on the GSU's HV side and no GSU drawn. It is drawn as a single-line diagram with wires, left to right from the grid; where PSCAD's R, L and C are single-phase, each is drawn three times between breakouts.</t>
+          <t xml:space="preserve">The .pscx is built in the same run when PSCAD 5 and its Python library mhi.pscad (pip install mhi.pscad) are on the PC; otherwise run &lt;name&gt;_build_pscad.py where they are. The case holds the grid (source and Thevenin impedance), the gen-tie, the MPTs, each collector (the WECC equivalent as a pi section, or DETAILED: every feeder section, identical feeder copies lumped), the GSUs and, on each GSU's LV side, the inverter: your UDM (PSCAD library, definition and AC port in Generators) or a stand-in source at the solved voltage -- delete it and wire your UDM in its place (the report and the build log list every inverter node). Or set one UDM up in a case of its own (a vendor's test case) and give that case and the UDM's component ID (its Properties) in Generators: PSCAD source case, PSCAD component ID -- it is copied, with its settings, to every GSU of that generator (every machine of the DETAILED model), its definition and the case's resources (.lib, .obj) with it; PSCAD_Params rows ({UNITS}, {P_PU} ...) are set on each copy. PSCAD inverter at MV: for a UDM with its GSU inside, the inverter on the GSU's HV side and no GSU drawn. It is drawn as a single-line diagram with wires, left to right from the grid; where PSCAD's R, L and C are single-phase, each is drawn three times between breakouts.</t>
         </is>
       </c>
     </row>
@@ -5269,109 +5269,109 @@
       </c>
       <c r="B115" s="12" t="inlineStr">
         <is>
+          <t xml:space="preserve">PSCAD source case</t>
+        </is>
+      </c>
+      <c r="C115" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pscad_source</t>
+        </is>
+      </c>
+      <c r="D115" s="8"/>
+      <c r="E115" s="8"/>
+      <c r="F115" s="8"/>
+      <c r="G115" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a .pscx or .pslx (or a project open in PSCAD) with one UDM set up as you want it (with PSCAD component ID)</t>
+        </is>
+      </c>
+      <c r="H115" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="116" ht="17.0" customHeight="1">
+      <c r="A116" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Generators</t>
+        </is>
+      </c>
+      <c r="B116" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD component ID</t>
+        </is>
+      </c>
+      <c r="C116" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">pscad_component_id</t>
+        </is>
+      </c>
+      <c r="D116" s="8"/>
+      <c r="E116" s="8"/>
+      <c r="F116" s="8"/>
+      <c r="G116" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">that UDM's ID in the source case: copied, with its settings, to every GSU of this generator</t>
+        </is>
+      </c>
+      <c r="H116" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="117" ht="30.0" customHeight="1">
+      <c r="A117" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Generators</t>
+        </is>
+      </c>
+      <c r="B117" s="12" t="inlineStr">
+        <is>
           <t xml:space="preserve">PSCAD inverter at</t>
         </is>
       </c>
-      <c r="C115" s="8" t="inlineStr">
+      <c r="C117" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">pscad_inv_at</t>
         </is>
       </c>
-      <c r="D115" s="8"/>
-      <c r="E115" s="8" t="inlineStr">
+      <c r="D117" s="8"/>
+      <c r="E117" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">LV</t>
         </is>
       </c>
-      <c r="F115" s="8" t="inlineStr">
+      <c r="F117" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">LV | MV</t>
         </is>
       </c>
-      <c r="G115" s="8" t="inlineStr">
+      <c r="G117" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">LV: the inverter (your UDM or the stand-in source) on the GSU's LV side, the GSU built | MV: on its HV side, for a UDM with its GSU inside (blank = LV)</t>
         </is>
       </c>
-      <c r="H115" s="13" t="inlineStr">
+      <c r="H117" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">PSCAD</t>
         </is>
       </c>
     </row>
-    <row r="116" ht="18" customHeight="1">
-      <c r="A116" s="7" t="inlineStr">
+    <row r="118" ht="18" customHeight="1">
+      <c r="A118" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Feeders</t>
         </is>
       </c>
-      <c r="B116" s="7"/>
-      <c r="C116" s="7"/>
-      <c r="D116" s="7"/>
-      <c r="E116" s="7"/>
-      <c r="F116" s="7"/>
-      <c r="G116" s="7"/>
-      <c r="H116" s="7"/>
-    </row>
-    <row r="117" ht="17.0" customHeight="1">
-      <c r="A117" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Feeders</t>
-        </is>
-      </c>
-      <c r="B117" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Collector</t>
-        </is>
-      </c>
-      <c r="C117" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">collector</t>
-        </is>
-      </c>
-      <c r="D117" s="8"/>
-      <c r="E117" s="8"/>
-      <c r="F117" s="8"/>
-      <c r="G117" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">the generator (its own collector) or a shared collector</t>
-        </is>
-      </c>
-      <c r="H117" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
-        </is>
-      </c>
-    </row>
-    <row r="118" ht="17.0" customHeight="1">
-      <c r="A118" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Feeders</t>
-        </is>
-      </c>
-      <c r="B118" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Feeder</t>
-        </is>
-      </c>
-      <c r="C118" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">feeder</t>
-        </is>
-      </c>
-      <c r="D118" s="8"/>
-      <c r="E118" s="8"/>
-      <c r="F118" s="8"/>
-      <c r="G118" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">feeder name</t>
-        </is>
-      </c>
-      <c r="H118" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
-        </is>
-      </c>
+      <c r="B118" s="7"/>
+      <c r="C118" s="7"/>
+      <c r="D118" s="7"/>
+      <c r="E118" s="7"/>
+      <c r="F118" s="7"/>
+      <c r="G118" s="7"/>
+      <c r="H118" s="7"/>
     </row>
     <row r="119" ht="17.0" customHeight="1">
       <c r="A119" s="8" t="inlineStr">
@@ -5381,24 +5381,20 @@
       </c>
       <c r="B119" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Copies</t>
+          <t xml:space="preserve">Collector</t>
         </is>
       </c>
       <c r="C119" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">copies</t>
+          <t xml:space="preserve">collector</t>
         </is>
       </c>
       <c r="D119" s="8"/>
-      <c r="E119" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
+      <c r="E119" s="8"/>
       <c r="F119" s="8"/>
       <c r="G119" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">identical feeders (blank = 1)</t>
+          <t xml:space="preserve">the generator (its own collector) or a shared collector</t>
         </is>
       </c>
       <c r="H119" s="13" t="inlineStr">
@@ -5415,12 +5411,12 @@
       </c>
       <c r="B120" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Section</t>
+          <t xml:space="preserve">Feeder</t>
         </is>
       </c>
       <c r="C120" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">section</t>
+          <t xml:space="preserve">feeder</t>
         </is>
       </c>
       <c r="D120" s="8"/>
@@ -5428,7 +5424,7 @@
       <c r="F120" s="8"/>
       <c r="G120" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">1, 2, 3 ... from the collector bus out</t>
+          <t xml:space="preserve">feeder name</t>
         </is>
       </c>
       <c r="H120" s="13" t="inlineStr">
@@ -5437,7 +5433,7 @@
         </is>
       </c>
     </row>
-    <row r="121" ht="30.0" customHeight="1">
+    <row r="121" ht="17.0" customHeight="1">
       <c r="A121" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Feeders</t>
@@ -5445,24 +5441,24 @@
       </c>
       <c r="B121" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">From section</t>
+          <t xml:space="preserve">Copies</t>
         </is>
       </c>
       <c r="C121" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">from_section</t>
+          <t xml:space="preserve">copies</t>
         </is>
       </c>
       <c r="D121" s="8"/>
       <c r="E121" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">the one before (daisy chain</t>
+          <t xml:space="preserve">1</t>
         </is>
       </c>
       <c r="F121" s="8"/>
       <c r="G121" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">blank = the one before (daisy chain) | 0 = the collector bus | n = a lateral off the end of section n</t>
+          <t xml:space="preserve">identical feeders (blank = 1)</t>
         </is>
       </c>
       <c r="H121" s="13" t="inlineStr">
@@ -5479,12 +5475,12 @@
       </c>
       <c r="B122" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cable</t>
+          <t xml:space="preserve">Section</t>
         </is>
       </c>
       <c r="C122" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">cable</t>
+          <t xml:space="preserve">section</t>
         </is>
       </c>
       <c r="D122" s="8"/>
@@ -5492,7 +5488,7 @@
       <c r="F122" s="8"/>
       <c r="G122" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">from Cables</t>
+          <t xml:space="preserve">1, 2, 3 ... from the collector bus out</t>
         </is>
       </c>
       <c r="H122" s="13" t="inlineStr">
@@ -5501,7 +5497,7 @@
         </is>
       </c>
     </row>
-    <row r="123" ht="17.0" customHeight="1">
+    <row r="123" ht="30.0" customHeight="1">
       <c r="A123" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Feeders</t>
@@ -5509,18 +5505,26 @@
       </c>
       <c r="B123" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Length</t>
+          <t xml:space="preserve">From section</t>
         </is>
       </c>
       <c r="C123" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">length</t>
+          <t xml:space="preserve">from_section</t>
         </is>
       </c>
       <c r="D123" s="8"/>
-      <c r="E123" s="8"/>
+      <c r="E123" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the one before (daisy chain</t>
+        </is>
+      </c>
       <c r="F123" s="8"/>
-      <c r="G123" s="8"/>
+      <c r="G123" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">blank = the one before (daisy chain) | 0 = the collector bus | n = a lateral off the end of section n</t>
+        </is>
+      </c>
       <c r="H123" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">PSS/E + PSCAD</t>
@@ -5535,28 +5539,20 @@
       </c>
       <c r="B124" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Length unit</t>
+          <t xml:space="preserve">Cable</t>
         </is>
       </c>
       <c r="C124" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">unit</t>
+          <t xml:space="preserve">cable</t>
         </is>
       </c>
       <c r="D124" s="8"/>
-      <c r="E124" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">km</t>
-        </is>
-      </c>
-      <c r="F124" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">km | mi | kft | m | ft</t>
-        </is>
-      </c>
+      <c r="E124" s="8"/>
+      <c r="F124" s="8"/>
       <c r="G124" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">blank = km</t>
+          <t xml:space="preserve">from Cables</t>
         </is>
       </c>
       <c r="H124" s="13" t="inlineStr">
@@ -5573,22 +5569,18 @@
       </c>
       <c r="B125" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Units at end</t>
+          <t xml:space="preserve">Length</t>
         </is>
       </c>
       <c r="C125" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">units</t>
+          <t xml:space="preserve">length</t>
         </is>
       </c>
       <c r="D125" s="8"/>
       <c r="E125" s="8"/>
       <c r="F125" s="8"/>
-      <c r="G125" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">units tapped at the far end</t>
-        </is>
-      </c>
+      <c r="G125" s="8"/>
       <c r="H125" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">PSS/E + PSCAD</t>
@@ -5603,20 +5595,28 @@
       </c>
       <c r="B126" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Units of</t>
+          <t xml:space="preserve">Length unit</t>
         </is>
       </c>
       <c r="C126" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">units_of</t>
+          <t xml:space="preserve">unit</t>
         </is>
       </c>
       <c r="D126" s="8"/>
-      <c r="E126" s="8"/>
-      <c r="F126" s="8"/>
+      <c r="E126" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">km</t>
+        </is>
+      </c>
+      <c r="F126" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">km | mi | kft | m | ft</t>
+        </is>
+      </c>
       <c r="G126" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">shared collectors: whose units (repeat the section for another generator's)</t>
+          <t xml:space="preserve">blank = km</t>
         </is>
       </c>
       <c r="H126" s="13" t="inlineStr">
@@ -5633,24 +5633,20 @@
       </c>
       <c r="B127" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Parallel cables</t>
+          <t xml:space="preserve">Units at end</t>
         </is>
       </c>
       <c r="C127" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">parallel</t>
+          <t xml:space="preserve">units</t>
         </is>
       </c>
       <c r="D127" s="8"/>
-      <c r="E127" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">1</t>
-        </is>
-      </c>
+      <c r="E127" s="8"/>
       <c r="F127" s="8"/>
       <c r="G127" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">blank = 1</t>
+          <t xml:space="preserve">units tapped at the far end</t>
         </is>
       </c>
       <c r="H127" s="13" t="inlineStr">
@@ -5659,42 +5655,62 @@
         </is>
       </c>
     </row>
-    <row r="128" ht="18" customHeight="1">
-      <c r="A128" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Cables</t>
-        </is>
-      </c>
-      <c r="B128" s="7"/>
-      <c r="C128" s="7"/>
-      <c r="D128" s="7"/>
-      <c r="E128" s="7"/>
-      <c r="F128" s="7"/>
-      <c r="G128" s="7"/>
-      <c r="H128" s="7"/>
+    <row r="128" ht="17.0" customHeight="1">
+      <c r="A128" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Feeders</t>
+        </is>
+      </c>
+      <c r="B128" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Units of</t>
+        </is>
+      </c>
+      <c r="C128" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">units_of</t>
+        </is>
+      </c>
+      <c r="D128" s="8"/>
+      <c r="E128" s="8"/>
+      <c r="F128" s="8"/>
+      <c r="G128" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">shared collectors: whose units (repeat the section for another generator's)</t>
+        </is>
+      </c>
+      <c r="H128" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSS/E + PSCAD</t>
+        </is>
+      </c>
     </row>
     <row r="129" ht="17.0" customHeight="1">
       <c r="A129" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cables</t>
+          <t xml:space="preserve">Feeders</t>
         </is>
       </c>
       <c r="B129" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cable</t>
+          <t xml:space="preserve">Parallel cables</t>
         </is>
       </c>
       <c r="C129" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">cable</t>
+          <t xml:space="preserve">parallel</t>
         </is>
       </c>
       <c r="D129" s="8"/>
-      <c r="E129" s="8"/>
+      <c r="E129" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1</t>
+        </is>
+      </c>
       <c r="F129" s="8"/>
       <c r="G129" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">cable type</t>
+          <t xml:space="preserve">blank = 1</t>
         </is>
       </c>
       <c r="H129" s="13" t="inlineStr">
@@ -5703,39 +5719,19 @@
         </is>
       </c>
     </row>
-    <row r="130" ht="17.0" customHeight="1">
-      <c r="A130" s="8" t="inlineStr">
+    <row r="130" ht="18" customHeight="1">
+      <c r="A130" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Cables</t>
         </is>
       </c>
-      <c r="B130" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Length unit</t>
-        </is>
-      </c>
-      <c r="C130" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">unit</t>
-        </is>
-      </c>
-      <c r="D130" s="8"/>
-      <c r="E130" s="8"/>
-      <c r="F130" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">km | mi | kft | m | ft</t>
-        </is>
-      </c>
-      <c r="G130" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">the values are per</t>
-        </is>
-      </c>
-      <c r="H130" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
-        </is>
-      </c>
+      <c r="B130" s="7"/>
+      <c r="C130" s="7"/>
+      <c r="D130" s="7"/>
+      <c r="E130" s="7"/>
+      <c r="F130" s="7"/>
+      <c r="G130" s="7"/>
+      <c r="H130" s="7"/>
     </row>
     <row r="131" ht="17.0" customHeight="1">
       <c r="A131" s="8" t="inlineStr">
@@ -5745,12 +5741,12 @@
       </c>
       <c r="B131" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">R per length</t>
+          <t xml:space="preserve">Cable</t>
         </is>
       </c>
       <c r="C131" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">r_per</t>
+          <t xml:space="preserve">cable</t>
         </is>
       </c>
       <c r="D131" s="8"/>
@@ -5758,7 +5754,7 @@
       <c r="F131" s="8"/>
       <c r="G131" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">ohm, at operating temperature</t>
+          <t xml:space="preserve">cable type</t>
         </is>
       </c>
       <c r="H131" s="13" t="inlineStr">
@@ -5775,20 +5771,24 @@
       </c>
       <c r="B132" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">X per length</t>
+          <t xml:space="preserve">Length unit</t>
         </is>
       </c>
       <c r="C132" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">x_per</t>
+          <t xml:space="preserve">unit</t>
         </is>
       </c>
       <c r="D132" s="8"/>
       <c r="E132" s="8"/>
-      <c r="F132" s="8"/>
+      <c r="F132" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">km | mi | kft | m | ft</t>
+        </is>
+      </c>
       <c r="G132" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">ohm</t>
+          <t xml:space="preserve">the values are per</t>
         </is>
       </c>
       <c r="H132" s="13" t="inlineStr">
@@ -5805,12 +5805,12 @@
       </c>
       <c r="B133" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">C per length</t>
+          <t xml:space="preserve">R per length</t>
         </is>
       </c>
       <c r="C133" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">c_per</t>
+          <t xml:space="preserve">r_per</t>
         </is>
       </c>
       <c r="D133" s="8"/>
@@ -5818,7 +5818,7 @@
       <c r="F133" s="8"/>
       <c r="G133" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">uF</t>
+          <t xml:space="preserve">ohm, at operating temperature</t>
         </is>
       </c>
       <c r="H133" s="13" t="inlineStr">
@@ -5835,12 +5835,12 @@
       </c>
       <c r="B134" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">B per length</t>
+          <t xml:space="preserve">X per length</t>
         </is>
       </c>
       <c r="C134" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">b_per</t>
+          <t xml:space="preserve">x_per</t>
         </is>
       </c>
       <c r="D134" s="8"/>
@@ -5848,7 +5848,7 @@
       <c r="F134" s="8"/>
       <c r="G134" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">uS, instead of C</t>
+          <t xml:space="preserve">ohm</t>
         </is>
       </c>
       <c r="H134" s="13" t="inlineStr">
@@ -5857,34 +5857,50 @@
         </is>
       </c>
     </row>
-    <row r="135" ht="18" customHeight="1">
-      <c r="A135" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Collectors</t>
-        </is>
-      </c>
-      <c r="B135" s="7"/>
-      <c r="C135" s="7"/>
-      <c r="D135" s="7"/>
-      <c r="E135" s="7"/>
-      <c r="F135" s="7"/>
-      <c r="G135" s="7"/>
-      <c r="H135" s="7"/>
+    <row r="135" ht="17.0" customHeight="1">
+      <c r="A135" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cables</t>
+        </is>
+      </c>
+      <c r="B135" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">C per length</t>
+        </is>
+      </c>
+      <c r="C135" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">c_per</t>
+        </is>
+      </c>
+      <c r="D135" s="8"/>
+      <c r="E135" s="8"/>
+      <c r="F135" s="8"/>
+      <c r="G135" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">uF</t>
+        </is>
+      </c>
+      <c r="H135" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSS/E + PSCAD</t>
+        </is>
+      </c>
     </row>
     <row r="136" ht="17.0" customHeight="1">
       <c r="A136" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Collectors</t>
+          <t xml:space="preserve">Cables</t>
         </is>
       </c>
       <c r="B136" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Name</t>
+          <t xml:space="preserve">B per length</t>
         </is>
       </c>
       <c r="C136" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">name</t>
+          <t xml:space="preserve">b_per</t>
         </is>
       </c>
       <c r="D136" s="8"/>
@@ -5892,85 +5908,81 @@
       <c r="F136" s="8"/>
       <c r="G136" s="8" t="inlineStr">
         <is>
+          <t xml:space="preserve">uS, instead of C</t>
+        </is>
+      </c>
+      <c r="H136" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSS/E + PSCAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="137" ht="18" customHeight="1">
+      <c r="A137" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Collectors</t>
+        </is>
+      </c>
+      <c r="B137" s="7"/>
+      <c r="C137" s="7"/>
+      <c r="D137" s="7"/>
+      <c r="E137" s="7"/>
+      <c r="F137" s="7"/>
+      <c r="G137" s="7"/>
+      <c r="H137" s="7"/>
+    </row>
+    <row r="138" ht="17.0" customHeight="1">
+      <c r="A138" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Collectors</t>
+        </is>
+      </c>
+      <c r="B138" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Name</t>
+        </is>
+      </c>
+      <c r="C138" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">name</t>
+        </is>
+      </c>
+      <c r="D138" s="8"/>
+      <c r="E138" s="8"/>
+      <c r="F138" s="8"/>
+      <c r="G138" s="8" t="inlineStr">
+        <is>
           <t xml:space="preserve">shared collector: its far-end bus has this name</t>
         </is>
       </c>
-      <c r="H136" s="13" t="inlineStr">
+      <c r="H138" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">PSS/E + PSCAD</t>
         </is>
       </c>
-    </row>
-    <row r="137" ht="17.0" customHeight="1">
-      <c r="A137" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Collectors</t>
-        </is>
-      </c>
-      <c r="B137" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Connect to</t>
-        </is>
-      </c>
-      <c r="C137" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">connect</t>
-        </is>
-      </c>
-      <c r="D137" s="8"/>
-      <c r="E137" s="8"/>
-      <c r="F137" s="8"/>
-      <c r="G137" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">the bus it starts from (MPT1, MPT1:TV ...)</t>
-        </is>
-      </c>
-      <c r="H137" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
-        </is>
-      </c>
-    </row>
-    <row r="138" ht="18" customHeight="1">
-      <c r="A138" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Loads_Shunts</t>
-        </is>
-      </c>
-      <c r="B138" s="7"/>
-      <c r="C138" s="7"/>
-      <c r="D138" s="7"/>
-      <c r="E138" s="7"/>
-      <c r="F138" s="7"/>
-      <c r="G138" s="7"/>
-      <c r="H138" s="7"/>
     </row>
     <row r="139" ht="17.0" customHeight="1">
       <c r="A139" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Loads_Shunts</t>
+          <t xml:space="preserve">Collectors</t>
         </is>
       </c>
       <c r="B139" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kind</t>
+          <t xml:space="preserve">Connect to</t>
         </is>
       </c>
       <c r="C139" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">kind</t>
+          <t xml:space="preserve">connect</t>
         </is>
       </c>
       <c r="D139" s="8"/>
       <c r="E139" s="8"/>
-      <c r="F139" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LOAD | SHUNT</t>
-        </is>
-      </c>
+      <c r="F139" s="8"/>
       <c r="G139" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">LOAD: constant impedance | SHUNT: + capacitor, - reactor</t>
+          <t xml:space="preserve">the bus it starts from (MPT1, MPT1:TV ...)</t>
         </is>
       </c>
       <c r="H139" s="13" t="inlineStr">
@@ -5979,35 +5991,19 @@
         </is>
       </c>
     </row>
-    <row r="140" ht="17.0" customHeight="1">
-      <c r="A140" s="8" t="inlineStr">
+    <row r="140" ht="18" customHeight="1">
+      <c r="A140" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Loads_Shunts</t>
         </is>
       </c>
-      <c r="B140" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">At bus</t>
-        </is>
-      </c>
-      <c r="C140" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">at</t>
-        </is>
-      </c>
-      <c r="D140" s="8"/>
-      <c r="E140" s="8"/>
-      <c r="F140" s="8"/>
-      <c r="G140" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">POI, HV, MPT1, MPT1:TV, PV:MV, PV ...</t>
-        </is>
-      </c>
-      <c r="H140" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
-        </is>
-      </c>
+      <c r="B140" s="7"/>
+      <c r="C140" s="7"/>
+      <c r="D140" s="7"/>
+      <c r="E140" s="7"/>
+      <c r="F140" s="7"/>
+      <c r="G140" s="7"/>
+      <c r="H140" s="7"/>
     </row>
     <row r="141" ht="17.0" customHeight="1">
       <c r="A141" s="8" t="inlineStr">
@@ -6017,20 +6013,24 @@
       </c>
       <c r="B141" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">MW</t>
+          <t xml:space="preserve">Kind</t>
         </is>
       </c>
       <c r="C141" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">mw</t>
+          <t xml:space="preserve">kind</t>
         </is>
       </c>
       <c r="D141" s="8"/>
       <c r="E141" s="8"/>
-      <c r="F141" s="8"/>
+      <c r="F141" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LOAD | SHUNT</t>
+        </is>
+      </c>
       <c r="G141" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">LOAD, at 1 pu</t>
+          <t xml:space="preserve">LOAD: constant impedance | SHUNT: + capacitor, - reactor</t>
         </is>
       </c>
       <c r="H141" s="13" t="inlineStr">
@@ -6047,12 +6047,12 @@
       </c>
       <c r="B142" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">MVAr</t>
+          <t xml:space="preserve">At bus</t>
         </is>
       </c>
       <c r="C142" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">mvar</t>
+          <t xml:space="preserve">at</t>
         </is>
       </c>
       <c r="D142" s="8"/>
@@ -6060,7 +6060,7 @@
       <c r="F142" s="8"/>
       <c r="G142" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">at 1 pu: LOAD + inductive | SHUNT + capacitive</t>
+          <t xml:space="preserve">POI, HV, MPT1, MPT1:TV, PV:MV, PV ...</t>
         </is>
       </c>
       <c r="H142" s="13" t="inlineStr">
@@ -6077,101 +6077,97 @@
       </c>
       <c r="B143" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Name</t>
+          <t xml:space="preserve">MW</t>
         </is>
       </c>
       <c r="C143" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">name</t>
+          <t xml:space="preserve">mw</t>
         </is>
       </c>
       <c r="D143" s="8"/>
       <c r="E143" s="8"/>
       <c r="F143" s="8"/>
-      <c r="G143" s="8"/>
+      <c r="G143" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LOAD, at 1 pu</t>
+        </is>
+      </c>
       <c r="H143" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">PSS/E + PSCAD</t>
         </is>
       </c>
     </row>
-    <row r="144" ht="18" customHeight="1">
-      <c r="A144" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Machines</t>
-        </is>
-      </c>
-      <c r="B144" s="7"/>
-      <c r="C144" s="7"/>
-      <c r="D144" s="7"/>
-      <c r="E144" s="7"/>
-      <c r="F144" s="7"/>
-      <c r="G144" s="7"/>
-      <c r="H144" s="7"/>
-    </row>
-    <row r="145" ht="30.0" customHeight="1">
+    <row r="144" ht="17.0" customHeight="1">
+      <c r="A144" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Loads_Shunts</t>
+        </is>
+      </c>
+      <c r="B144" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MVAr</t>
+        </is>
+      </c>
+      <c r="C144" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mvar</t>
+        </is>
+      </c>
+      <c r="D144" s="8"/>
+      <c r="E144" s="8"/>
+      <c r="F144" s="8"/>
+      <c r="G144" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">at 1 pu: LOAD + inductive | SHUNT + capacitive</t>
+        </is>
+      </c>
+      <c r="H144" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSS/E + PSCAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="145" ht="17.0" customHeight="1">
       <c r="A145" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Machines</t>
+          <t xml:space="preserve">Loads_Shunts</t>
         </is>
       </c>
       <c r="B145" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Machine</t>
+          <t xml:space="preserve">Name</t>
         </is>
       </c>
       <c r="C145" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">machine</t>
+          <t xml:space="preserve">name</t>
         </is>
       </c>
       <c r="D145" s="8"/>
       <c r="E145" s="8"/>
       <c r="F145" s="8"/>
-      <c r="G145" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">DETAILED model: a machine, &lt;generator&gt;_&lt;feeder&gt;_S&lt;section&gt; (the GUI lists them); its values in place of its share of its generator's</t>
-        </is>
-      </c>
+      <c r="G145" s="8"/>
       <c r="H145" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">PSS/E + PSCAD</t>
         </is>
       </c>
     </row>
-    <row r="146" ht="17.0" customHeight="1">
-      <c r="A146" s="8" t="inlineStr">
+    <row r="146" ht="18" customHeight="1">
+      <c r="A146" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Machines</t>
         </is>
       </c>
-      <c r="B146" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Machine ID</t>
-        </is>
-      </c>
-      <c r="C146" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">id</t>
-        </is>
-      </c>
-      <c r="D146" s="8"/>
-      <c r="E146" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">its generator's</t>
-        </is>
-      </c>
-      <c r="F146" s="8"/>
-      <c r="G146" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">blank = its generator's</t>
-        </is>
-      </c>
-      <c r="H146" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
-        </is>
-      </c>
+      <c r="B146" s="7"/>
+      <c r="C146" s="7"/>
+      <c r="D146" s="7"/>
+      <c r="E146" s="7"/>
+      <c r="F146" s="7"/>
+      <c r="G146" s="7"/>
+      <c r="H146" s="7"/>
     </row>
     <row r="147" ht="30.0" customHeight="1">
       <c r="A147" s="8" t="inlineStr">
@@ -6181,24 +6177,20 @@
       </c>
       <c r="B147" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pgen MW</t>
+          <t xml:space="preserve">Machine</t>
         </is>
       </c>
       <c r="C147" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">pgen_mw</t>
+          <t xml:space="preserve">machine</t>
         </is>
       </c>
       <c r="D147" s="8"/>
-      <c r="E147" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">its share of its generator's Dispatch MW</t>
-        </is>
-      </c>
+      <c r="E147" s="8"/>
       <c r="F147" s="8"/>
       <c r="G147" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">its dispatch (blank = its share of its generator's Dispatch MW)</t>
+          <t xml:space="preserve">DETAILED model: a machine, &lt;generator&gt;_&lt;feeder&gt;_S&lt;section&gt; (the GUI lists them); its values in place of its share of its generator's</t>
         </is>
       </c>
       <c r="H147" s="13" t="inlineStr">
@@ -6215,24 +6207,24 @@
       </c>
       <c r="B148" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pmax MW</t>
+          <t xml:space="preserve">Machine ID</t>
         </is>
       </c>
       <c r="C148" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">pmax_mw</t>
+          <t xml:space="preserve">id</t>
         </is>
       </c>
       <c r="D148" s="8"/>
       <c r="E148" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">its units x Unit Pmax</t>
+          <t xml:space="preserve">its generator's</t>
         </is>
       </c>
       <c r="F148" s="8"/>
       <c r="G148" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">blank = its units x Unit Pmax</t>
+          <t xml:space="preserve">blank = its generator's</t>
         </is>
       </c>
       <c r="H148" s="13" t="inlineStr">
@@ -6241,7 +6233,7 @@
         </is>
       </c>
     </row>
-    <row r="149" ht="17.0" customHeight="1">
+    <row r="149" ht="30.0" customHeight="1">
       <c r="A149" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Machines</t>
@@ -6249,24 +6241,24 @@
       </c>
       <c r="B149" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pmin MW</t>
+          <t xml:space="preserve">Pgen MW</t>
         </is>
       </c>
       <c r="C149" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">pmin_mw</t>
+          <t xml:space="preserve">pgen_mw</t>
         </is>
       </c>
       <c r="D149" s="8"/>
       <c r="E149" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">its units x Unit Pmin</t>
+          <t xml:space="preserve">its share of its generator's Dispatch MW</t>
         </is>
       </c>
       <c r="F149" s="8"/>
       <c r="G149" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">blank = its units x Unit Pmin</t>
+          <t xml:space="preserve">its dispatch (blank = its share of its generator's Dispatch MW)</t>
         </is>
       </c>
       <c r="H149" s="13" t="inlineStr">
@@ -6283,24 +6275,24 @@
       </c>
       <c r="B150" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Qmax MVAr</t>
+          <t xml:space="preserve">Pmax MW</t>
         </is>
       </c>
       <c r="C150" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">qmax_mvar</t>
+          <t xml:space="preserve">pmax_mw</t>
         </is>
       </c>
       <c r="D150" s="8"/>
       <c r="E150" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">its units x Unit Qmax</t>
+          <t xml:space="preserve">its units x Unit Pmax</t>
         </is>
       </c>
       <c r="F150" s="8"/>
       <c r="G150" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">blank = its units x Unit Qmax</t>
+          <t xml:space="preserve">blank = its units x Unit Pmax</t>
         </is>
       </c>
       <c r="H150" s="13" t="inlineStr">
@@ -6317,24 +6309,24 @@
       </c>
       <c r="B151" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Qmin MVAr</t>
+          <t xml:space="preserve">Pmin MW</t>
         </is>
       </c>
       <c r="C151" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">qmin_mvar</t>
+          <t xml:space="preserve">pmin_mw</t>
         </is>
       </c>
       <c r="D151" s="8"/>
       <c r="E151" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">its units x Unit Qmin</t>
+          <t xml:space="preserve">its units x Unit Pmin</t>
         </is>
       </c>
       <c r="F151" s="8"/>
       <c r="G151" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">blank = its units x Unit Qmin</t>
+          <t xml:space="preserve">blank = its units x Unit Pmin</t>
         </is>
       </c>
       <c r="H151" s="13" t="inlineStr">
@@ -6343,7 +6335,7 @@
         </is>
       </c>
     </row>
-    <row r="152" ht="30.0" customHeight="1">
+    <row r="152" ht="17.0" customHeight="1">
       <c r="A152" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Machines</t>
@@ -6351,24 +6343,24 @@
       </c>
       <c r="B152" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fixed Q MVAr</t>
+          <t xml:space="preserve">Qmax MVAr</t>
         </is>
       </c>
       <c r="C152" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">q_mvar</t>
+          <t xml:space="preserve">qmax_mvar</t>
         </is>
       </c>
       <c r="D152" s="8"/>
       <c r="E152" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">as its generator's Q mode</t>
+          <t xml:space="preserve">its units x Unit Qmax</t>
         </is>
       </c>
       <c r="F152" s="8"/>
       <c r="G152" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">a value: this Q, fixed (blank = as its generator's Q mode)</t>
+          <t xml:space="preserve">blank = its units x Unit Qmax</t>
         </is>
       </c>
       <c r="H152" s="13" t="inlineStr">
@@ -6385,24 +6377,24 @@
       </c>
       <c r="B153" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">MBASE MVA</t>
+          <t xml:space="preserve">Qmin MVAr</t>
         </is>
       </c>
       <c r="C153" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">mbase_mva</t>
+          <t xml:space="preserve">qmin_mvar</t>
         </is>
       </c>
       <c r="D153" s="8"/>
       <c r="E153" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">its units x Unit MVA</t>
+          <t xml:space="preserve">its units x Unit Qmin</t>
         </is>
       </c>
       <c r="F153" s="8"/>
       <c r="G153" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">blank = its units x Unit MVA</t>
+          <t xml:space="preserve">blank = its units x Unit Qmin</t>
         </is>
       </c>
       <c r="H153" s="13" t="inlineStr">
@@ -6411,42 +6403,66 @@
         </is>
       </c>
     </row>
-    <row r="154" ht="18" customHeight="1">
-      <c r="A154" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bus_Numbers</t>
-        </is>
-      </c>
-      <c r="B154" s="7"/>
-      <c r="C154" s="7"/>
-      <c r="D154" s="7"/>
-      <c r="E154" s="7"/>
-      <c r="F154" s="7"/>
-      <c r="G154" s="7"/>
-      <c r="H154" s="7"/>
+    <row r="154" ht="30.0" customHeight="1">
+      <c r="A154" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Machines</t>
+        </is>
+      </c>
+      <c r="B154" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Fixed Q MVAr</t>
+        </is>
+      </c>
+      <c r="C154" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">q_mvar</t>
+        </is>
+      </c>
+      <c r="D154" s="8"/>
+      <c r="E154" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">as its generator's Q mode</t>
+        </is>
+      </c>
+      <c r="F154" s="8"/>
+      <c r="G154" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a value: this Q, fixed (blank = as its generator's Q mode)</t>
+        </is>
+      </c>
+      <c r="H154" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSS/E + PSCAD</t>
+        </is>
+      </c>
     </row>
     <row r="155" ht="17.0" customHeight="1">
       <c r="A155" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bus_Numbers</t>
+          <t xml:space="preserve">Machines</t>
         </is>
       </c>
       <c r="B155" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bus</t>
+          <t xml:space="preserve">MBASE MVA</t>
         </is>
       </c>
       <c r="C155" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">bus</t>
+          <t xml:space="preserve">mbase_mva</t>
         </is>
       </c>
       <c r="D155" s="8"/>
-      <c r="E155" s="8"/>
+      <c r="E155" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">its units x Unit MVA</t>
+        </is>
+      </c>
       <c r="F155" s="8"/>
       <c r="G155" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">its role: IB, POI, HV, MPT1:LV, PV:MV, PV:LV ...</t>
+          <t xml:space="preserve">blank = its units x Unit MVA</t>
         </is>
       </c>
       <c r="H155" s="13" t="inlineStr">
@@ -6455,41 +6471,21 @@
         </is>
       </c>
     </row>
-    <row r="156" ht="17.0" customHeight="1">
-      <c r="A156" s="8" t="inlineStr">
+    <row r="156" ht="18" customHeight="1">
+      <c r="A156" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Bus_Numbers</t>
         </is>
       </c>
-      <c r="B156" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Number</t>
-        </is>
-      </c>
-      <c r="C156" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">number</t>
-        </is>
-      </c>
-      <c r="D156" s="8"/>
-      <c r="E156" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">automatic</t>
-        </is>
-      </c>
-      <c r="F156" s="8"/>
-      <c r="G156" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">blank = automatic</t>
-        </is>
-      </c>
-      <c r="H156" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
-        </is>
-      </c>
-    </row>
-    <row r="157" ht="30.0" customHeight="1">
+      <c r="B156" s="7"/>
+      <c r="C156" s="7"/>
+      <c r="D156" s="7"/>
+      <c r="E156" s="7"/>
+      <c r="F156" s="7"/>
+      <c r="G156" s="7"/>
+      <c r="H156" s="7"/>
+    </row>
+    <row r="157" ht="17.0" customHeight="1">
       <c r="A157" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Bus_Numbers</t>
@@ -6497,24 +6493,20 @@
       </c>
       <c r="B157" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Name</t>
+          <t xml:space="preserve">Bus</t>
         </is>
       </c>
       <c r="C157" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">name</t>
+          <t xml:space="preserve">bus</t>
         </is>
       </c>
       <c r="D157" s="8"/>
-      <c r="E157" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">automatic (12 characters at most</t>
-        </is>
-      </c>
+      <c r="E157" s="8"/>
       <c r="F157" s="8"/>
       <c r="G157" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">blank = automatic (12 characters at most)</t>
+          <t xml:space="preserve">its role: IB, POI, HV, MPT1:LV, PV:MV, PV:LV ...</t>
         </is>
       </c>
       <c r="H157" s="13" t="inlineStr">
@@ -6523,79 +6515,87 @@
         </is>
       </c>
     </row>
-    <row r="158" ht="18" customHeight="1">
-      <c r="A158" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Dyr_Params</t>
-        </is>
-      </c>
-      <c r="B158" s="7"/>
-      <c r="C158" s="7"/>
-      <c r="D158" s="7"/>
-      <c r="E158" s="7"/>
-      <c r="F158" s="7"/>
-      <c r="G158" s="7"/>
-      <c r="H158" s="7"/>
-    </row>
-    <row r="159" ht="17.0" customHeight="1">
+    <row r="158" ht="17.0" customHeight="1">
+      <c r="A158" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bus_Numbers</t>
+        </is>
+      </c>
+      <c r="B158" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Number</t>
+        </is>
+      </c>
+      <c r="C158" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">number</t>
+        </is>
+      </c>
+      <c r="D158" s="8"/>
+      <c r="E158" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">automatic</t>
+        </is>
+      </c>
+      <c r="F158" s="8"/>
+      <c r="G158" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">blank = automatic</t>
+        </is>
+      </c>
+      <c r="H158" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSS/E + PSCAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="159" ht="30.0" customHeight="1">
       <c r="A159" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dyr_Params</t>
+          <t xml:space="preserve">Bus_Numbers</t>
         </is>
       </c>
       <c r="B159" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Generator</t>
+          <t xml:space="preserve">Name</t>
         </is>
       </c>
       <c r="C159" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">generator</t>
+          <t xml:space="preserve">name</t>
         </is>
       </c>
       <c r="D159" s="8"/>
-      <c r="E159" s="8"/>
+      <c r="E159" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">automatic (12 characters at most</t>
+        </is>
+      </c>
       <c r="F159" s="8"/>
       <c r="G159" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">IB: the infinite bus | PLANT: the plant controller (REPC_B)</t>
+          <t xml:space="preserve">blank = automatic (12 characters at most)</t>
         </is>
       </c>
       <c r="H159" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E .dyr</t>
-        </is>
-      </c>
-    </row>
-    <row r="160" ht="30.0" customHeight="1">
-      <c r="A160" s="8" t="inlineStr">
+          <t xml:space="preserve">PSS/E + PSCAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="160" ht="18" customHeight="1">
+      <c r="A160" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Dyr_Params</t>
         </is>
       </c>
-      <c r="B160" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Model</t>
-        </is>
-      </c>
-      <c r="C160" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">model</t>
-        </is>
-      </c>
-      <c r="D160" s="8"/>
-      <c r="E160" s="8"/>
-      <c r="F160" s="8"/>
-      <c r="G160" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">REGCA1 (REGCAU1) | REECA1 REECCU1 REECDU1 | REPCA1 (REPCAU1) or REAX4BU1 | PLANT: PLNTBU1 | WT3: + WTDTA1 WTARA1 WTPTA1 WTTQA1 | SYNC: GENROU SEXS TGOV1 | IB: GENCLS</t>
-        </is>
-      </c>
-      <c r="H160" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSS/E .dyr</t>
-        </is>
-      </c>
+      <c r="B160" s="7"/>
+      <c r="C160" s="7"/>
+      <c r="D160" s="7"/>
+      <c r="E160" s="7"/>
+      <c r="F160" s="7"/>
+      <c r="G160" s="7"/>
+      <c r="H160" s="7"/>
     </row>
     <row r="161" ht="17.0" customHeight="1">
       <c r="A161" s="8" t="inlineStr">
@@ -6605,12 +6605,12 @@
       </c>
       <c r="B161" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Parameter</t>
+          <t xml:space="preserve">Generator</t>
         </is>
       </c>
       <c r="C161" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">parameter</t>
+          <t xml:space="preserve">generator</t>
         </is>
       </c>
       <c r="D161" s="8"/>
@@ -6618,7 +6618,7 @@
       <c r="F161" s="8"/>
       <c r="G161" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E name (the report lists them all) or position: ICON2, CON14</t>
+          <t xml:space="preserve">IB: the infinite bus | PLANT: the plant controller (REPC_B)</t>
         </is>
       </c>
       <c r="H161" s="13" t="inlineStr">
@@ -6627,7 +6627,7 @@
         </is>
       </c>
     </row>
-    <row r="162" ht="17.0" customHeight="1">
+    <row r="162" ht="30.0" customHeight="1">
       <c r="A162" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Dyr_Params</t>
@@ -6635,171 +6635,175 @@
       </c>
       <c r="B162" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Value</t>
+          <t xml:space="preserve">Model</t>
         </is>
       </c>
       <c r="C162" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">value</t>
+          <t xml:space="preserve">model</t>
         </is>
       </c>
       <c r="D162" s="8"/>
       <c r="E162" s="8"/>
       <c r="F162" s="8"/>
-      <c r="G162" s="8"/>
+      <c r="G162" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REGCA1 (REGCAU1) | REECA1 REECCU1 REECDU1 | REPCA1 (REPCAU1) or REAX4BU1 | PLANT: PLNTBU1 | WT3: + WTDTA1 WTARA1 WTPTA1 WTTQA1 | SYNC: GENROU SEXS TGOV1 | IB: GENCLS</t>
+        </is>
+      </c>
       <c r="H162" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">PSS/E .dyr</t>
         </is>
       </c>
     </row>
-    <row r="163" ht="18" customHeight="1">
-      <c r="A163" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Dyr_Records</t>
-        </is>
-      </c>
-      <c r="B163" s="7"/>
-      <c r="C163" s="7"/>
-      <c r="D163" s="7"/>
-      <c r="E163" s="7"/>
-      <c r="F163" s="7"/>
-      <c r="G163" s="7"/>
-      <c r="H163" s="7"/>
+    <row r="163" ht="17.0" customHeight="1">
+      <c r="A163" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dyr_Params</t>
+        </is>
+      </c>
+      <c r="B163" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Parameter</t>
+        </is>
+      </c>
+      <c r="C163" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">parameter</t>
+        </is>
+      </c>
+      <c r="D163" s="8"/>
+      <c r="E163" s="8"/>
+      <c r="F163" s="8"/>
+      <c r="G163" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSS/E name (the report lists them all) or position: ICON2, CON14</t>
+        </is>
+      </c>
+      <c r="H163" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSS/E .dyr</t>
+        </is>
+      </c>
     </row>
     <row r="164" ht="17.0" customHeight="1">
       <c r="A164" s="8" t="inlineStr">
         <is>
+          <t xml:space="preserve">Dyr_Params</t>
+        </is>
+      </c>
+      <c r="B164" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Value</t>
+        </is>
+      </c>
+      <c r="C164" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">value</t>
+        </is>
+      </c>
+      <c r="D164" s="8"/>
+      <c r="E164" s="8"/>
+      <c r="F164" s="8"/>
+      <c r="G164" s="8"/>
+      <c r="H164" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSS/E .dyr</t>
+        </is>
+      </c>
+    </row>
+    <row r="165" ht="18" customHeight="1">
+      <c r="A165" s="7" t="inlineStr">
+        <is>
           <t xml:space="preserve">Dyr_Records</t>
         </is>
       </c>
-      <c r="B164" s="12" t="inlineStr">
+      <c r="B165" s="7"/>
+      <c r="C165" s="7"/>
+      <c r="D165" s="7"/>
+      <c r="E165" s="7"/>
+      <c r="F165" s="7"/>
+      <c r="G165" s="7"/>
+      <c r="H165" s="7"/>
+    </row>
+    <row r="166" ht="17.0" customHeight="1">
+      <c r="A166" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dyr_Records</t>
+        </is>
+      </c>
+      <c r="B166" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Generator</t>
         </is>
       </c>
-      <c r="C164" s="8" t="inlineStr">
+      <c r="C166" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">generator</t>
         </is>
       </c>
-      <c r="D164" s="8"/>
-      <c r="E164" s="8" t="inlineStr">
+      <c r="D166" s="8"/>
+      <c r="E166" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">the plant</t>
         </is>
       </c>
-      <c r="F164" s="8"/>
-      <c r="G164" s="8" t="inlineStr">
+      <c r="F166" s="8"/>
+      <c r="G166" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">blank = the plant</t>
         </is>
       </c>
-      <c r="H164" s="13" t="inlineStr">
+      <c r="H166" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">PSS/E .dyr</t>
         </is>
       </c>
-    </row>
-    <row r="165" ht="17.0" customHeight="1">
-      <c r="A165" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Dyr_Records</t>
-        </is>
-      </c>
-      <c r="B165" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Record</t>
-        </is>
-      </c>
-      <c r="C165" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">record</t>
-        </is>
-      </c>
-      <c r="D165" s="8"/>
-      <c r="E165" s="8"/>
-      <c r="F165" s="8"/>
-      <c r="G165" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">.dyr text ending in / -- {BUS} {ID} {MBASE} {POI} {IB} {HV} {MV} {&lt;bus role&gt;} are filled in</t>
-        </is>
-      </c>
-      <c r="H165" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSS/E .dyr</t>
-        </is>
-      </c>
-    </row>
-    <row r="166" ht="18" customHeight="1">
-      <c r="A166" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSCAD_Params</t>
-        </is>
-      </c>
-      <c r="B166" s="7"/>
-      <c r="C166" s="7"/>
-      <c r="D166" s="7"/>
-      <c r="E166" s="7"/>
-      <c r="F166" s="7"/>
-      <c r="G166" s="7"/>
-      <c r="H166" s="7"/>
     </row>
     <row r="167" ht="17.0" customHeight="1">
       <c r="A167" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSCAD_Params</t>
+          <t xml:space="preserve">Dyr_Records</t>
         </is>
       </c>
       <c r="B167" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Generator</t>
+          <t xml:space="preserve">Record</t>
         </is>
       </c>
       <c r="C167" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">generator</t>
+          <t xml:space="preserve">record</t>
         </is>
       </c>
       <c r="D167" s="8"/>
       <c r="E167" s="8"/>
       <c r="F167" s="8"/>
-      <c r="G167" s="8"/>
+      <c r="G167" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">.dyr text ending in / -- {BUS} {ID} {MBASE} {POI} {IB} {HV} {MV} {&lt;bus role&gt;} are filled in</t>
+        </is>
+      </c>
       <c r="H167" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSCAD</t>
-        </is>
-      </c>
-    </row>
-    <row r="168" ht="17.0" customHeight="1">
-      <c r="A168" s="8" t="inlineStr">
+          <t xml:space="preserve">PSS/E .dyr</t>
+        </is>
+      </c>
+    </row>
+    <row r="168" ht="18" customHeight="1">
+      <c r="A168" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">PSCAD_Params</t>
         </is>
       </c>
-      <c r="B168" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Parameter</t>
-        </is>
-      </c>
-      <c r="C168" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">parameter</t>
-        </is>
-      </c>
-      <c r="D168" s="8"/>
-      <c r="E168" s="8"/>
-      <c r="F168" s="8"/>
-      <c r="G168" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">the vendor model's parameter name</t>
-        </is>
-      </c>
-      <c r="H168" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSCAD</t>
-        </is>
-      </c>
+      <c r="B168" s="7"/>
+      <c r="C168" s="7"/>
+      <c r="D168" s="7"/>
+      <c r="E168" s="7"/>
+      <c r="F168" s="7"/>
+      <c r="G168" s="7"/>
+      <c r="H168" s="7"/>
     </row>
     <row r="169" ht="17.0" customHeight="1">
       <c r="A169" s="8" t="inlineStr">
@@ -6809,83 +6813,103 @@
       </c>
       <c r="B169" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Value</t>
+          <t xml:space="preserve">Generator</t>
         </is>
       </c>
       <c r="C169" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">value</t>
+          <t xml:space="preserve">generator</t>
         </is>
       </c>
       <c r="D169" s="8"/>
       <c r="E169" s="8"/>
       <c r="F169" s="8"/>
-      <c r="G169" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">as PSCAD takes it (0.63 [kV], 40, {UNITS}, {P_PU} ...)</t>
-        </is>
-      </c>
+      <c r="G169" s="8"/>
       <c r="H169" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">PSCAD</t>
         </is>
       </c>
     </row>
-    <row r="170" ht="18" customHeight="1">
-      <c r="A170" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">BUS NAMES -- Connect to, At, Bus_Numbers and {&lt;bus&gt;} in Dyr_Records take these</t>
-        </is>
-      </c>
-      <c r="B170" s="7"/>
-      <c r="C170" s="7"/>
-      <c r="D170" s="7"/>
-      <c r="E170" s="7"/>
-      <c r="F170" s="7"/>
-      <c r="G170" s="7"/>
-      <c r="H170" s="7"/>
-    </row>
-    <row r="171">
-      <c r="A171" s="8"/>
+    <row r="170" ht="17.0" customHeight="1">
+      <c r="A170" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD_Params</t>
+        </is>
+      </c>
+      <c r="B170" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Parameter</t>
+        </is>
+      </c>
+      <c r="C170" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">parameter</t>
+        </is>
+      </c>
+      <c r="D170" s="8"/>
+      <c r="E170" s="8"/>
+      <c r="F170" s="8"/>
+      <c r="G170" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the vendor model's parameter name</t>
+        </is>
+      </c>
+      <c r="H170" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="171" ht="17.0" customHeight="1">
+      <c r="A171" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD_Params</t>
+        </is>
+      </c>
       <c r="B171" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">IB</t>
-        </is>
-      </c>
-      <c r="C171" s="8"/>
+          <t xml:space="preserve">Value</t>
+        </is>
+      </c>
+      <c r="C171" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">value</t>
+        </is>
+      </c>
       <c r="D171" s="8"/>
       <c r="E171" s="8"/>
       <c r="F171" s="8"/>
       <c r="G171" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">the infinite bus</t>
-        </is>
-      </c>
-      <c r="H171" s="8"/>
-    </row>
-    <row r="172">
-      <c r="A172" s="8"/>
-      <c r="B172" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">POI</t>
-        </is>
-      </c>
-      <c r="C172" s="8"/>
-      <c r="D172" s="8"/>
-      <c r="E172" s="8"/>
-      <c r="F172" s="8"/>
-      <c r="G172" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">the point of interconnection</t>
-        </is>
-      </c>
-      <c r="H172" s="8"/>
+          <t xml:space="preserve">as PSCAD takes it (0.63 [kV], 40, {UNITS}, {P_PU} ...)</t>
+        </is>
+      </c>
+      <c r="H171" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="172" ht="18" customHeight="1">
+      <c r="A172" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BUS NAMES -- Connect to, At, Bus_Numbers and {&lt;bus&gt;} in Dyr_Records take these</t>
+        </is>
+      </c>
+      <c r="B172" s="7"/>
+      <c r="C172" s="7"/>
+      <c r="D172" s="7"/>
+      <c r="E172" s="7"/>
+      <c r="F172" s="7"/>
+      <c r="G172" s="7"/>
+      <c r="H172" s="7"/>
     </row>
     <row r="173">
       <c r="A173" s="8"/>
       <c r="B173" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">HV</t>
+          <t xml:space="preserve">IB</t>
         </is>
       </c>
       <c r="C173" s="8"/>
@@ -6894,7 +6918,7 @@
       <c r="F173" s="8"/>
       <c r="G173" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">the gen-tie's plant end (the POI when there is no gen-tie)</t>
+          <t xml:space="preserve">the infinite bus</t>
         </is>
       </c>
       <c r="H173" s="8"/>
@@ -6903,7 +6927,7 @@
       <c r="A174" s="8"/>
       <c r="B174" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;MPT&gt; or &lt;MPT&gt;:LV</t>
+          <t xml:space="preserve">POI</t>
         </is>
       </c>
       <c r="C174" s="8"/>
@@ -6912,7 +6936,7 @@
       <c r="F174" s="8"/>
       <c r="G174" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">an MPT's LV winding</t>
+          <t xml:space="preserve">the point of interconnection</t>
         </is>
       </c>
       <c r="H174" s="8"/>
@@ -6921,7 +6945,7 @@
       <c r="A175" s="8"/>
       <c r="B175" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;MPT&gt;:TV</t>
+          <t xml:space="preserve">HV</t>
         </is>
       </c>
       <c r="C175" s="8"/>
@@ -6930,7 +6954,7 @@
       <c r="F175" s="8"/>
       <c r="G175" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">a 3-winding MPT's tertiary</t>
+          <t xml:space="preserve">the gen-tie's plant end (the POI when there is no gen-tie)</t>
         </is>
       </c>
       <c r="H175" s="8"/>
@@ -6939,7 +6963,7 @@
       <c r="A176" s="8"/>
       <c r="B176" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;MPT&gt;:HV</t>
+          <t xml:space="preserve">&lt;MPT&gt; or &lt;MPT&gt;:LV</t>
         </is>
       </c>
       <c r="C176" s="8"/>
@@ -6948,7 +6972,7 @@
       <c r="F176" s="8"/>
       <c r="G176" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">an MPT with a tie line of its own: its HV end</t>
+          <t xml:space="preserve">an MPT's LV winding</t>
         </is>
       </c>
       <c r="H176" s="8"/>
@@ -6957,7 +6981,7 @@
       <c r="A177" s="8"/>
       <c r="B177" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;collector&gt;</t>
+          <t xml:space="preserve">&lt;MPT&gt;:TV</t>
         </is>
       </c>
       <c r="C177" s="8"/>
@@ -6966,7 +6990,7 @@
       <c r="F177" s="8"/>
       <c r="G177" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">a shared collector's far end</t>
+          <t xml:space="preserve">a 3-winding MPT's tertiary</t>
         </is>
       </c>
       <c r="H177" s="8"/>
@@ -6975,7 +6999,7 @@
       <c r="A178" s="8"/>
       <c r="B178" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;generator&gt;:MV</t>
+          <t xml:space="preserve">&lt;MPT&gt;:HV</t>
         </is>
       </c>
       <c r="C178" s="8"/>
@@ -6984,7 +7008,7 @@
       <c r="F178" s="8"/>
       <c r="G178" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">a generator's GSU HV side</t>
+          <t xml:space="preserve">an MPT with a tie line of its own: its HV end</t>
         </is>
       </c>
       <c r="H178" s="8"/>
@@ -6993,7 +7017,7 @@
       <c r="A179" s="8"/>
       <c r="B179" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;generator&gt; or &lt;generator&gt;:LV</t>
+          <t xml:space="preserve">&lt;collector&gt;</t>
         </is>
       </c>
       <c r="C179" s="8"/>
@@ -7002,7 +7026,7 @@
       <c r="F179" s="8"/>
       <c r="G179" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">a generator's terminal</t>
+          <t xml:space="preserve">a shared collector's far end</t>
         </is>
       </c>
       <c r="H179" s="8"/>
@@ -7011,7 +7035,7 @@
       <c r="A180" s="8"/>
       <c r="B180" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;collector&gt;_&lt;feeder&gt;_S&lt;n&gt;</t>
+          <t xml:space="preserve">&lt;generator&gt;:MV</t>
         </is>
       </c>
       <c r="C180" s="8"/>
@@ -7020,7 +7044,7 @@
       <c r="F180" s="8"/>
       <c r="G180" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">DETAILED: the far end of feeder section n</t>
+          <t xml:space="preserve">a generator's GSU HV side</t>
         </is>
       </c>
       <c r="H180" s="8"/>
@@ -7029,7 +7053,7 @@
       <c r="A181" s="8"/>
       <c r="B181" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;generator&gt;_&lt;feeder&gt;_S&lt;n&gt;:LV</t>
+          <t xml:space="preserve">&lt;generator&gt; or &lt;generator&gt;:LV</t>
         </is>
       </c>
       <c r="C181" s="8"/>
@@ -7038,34 +7062,34 @@
       <c r="F181" s="8"/>
       <c r="G181" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">DETAILED: the terminal of the units at that node</t>
+          <t xml:space="preserve">a generator's terminal</t>
         </is>
       </c>
       <c r="H181" s="8"/>
     </row>
-    <row r="182" ht="18" customHeight="1">
-      <c r="A182" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSCAD_Params PLACEHOLDERS -- filled in for each inverter a vendor model stands for</t>
-        </is>
-      </c>
-      <c r="B182" s="7"/>
-      <c r="C182" s="7"/>
-      <c r="D182" s="7"/>
-      <c r="E182" s="7"/>
-      <c r="F182" s="7"/>
-      <c r="G182" s="7"/>
-      <c r="H182" s="7"/>
+    <row r="182">
+      <c r="A182" s="8"/>
+      <c r="B182" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;collector&gt;_&lt;feeder&gt;_S&lt;n&gt;</t>
+        </is>
+      </c>
+      <c r="C182" s="8"/>
+      <c r="D182" s="8"/>
+      <c r="E182" s="8"/>
+      <c r="F182" s="8"/>
+      <c r="G182" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">DETAILED: the far end of feeder section n</t>
+        </is>
+      </c>
+      <c r="H182" s="8"/>
     </row>
     <row r="183">
-      <c r="A183" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSCAD_Params</t>
-        </is>
-      </c>
+      <c r="A183" s="8"/>
       <c r="B183" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{UNITS}</t>
+          <t xml:space="preserve">&lt;generator&gt;_&lt;feeder&gt;_S&lt;n&gt;:LV</t>
         </is>
       </c>
       <c r="C183" s="8"/>
@@ -7074,40 +7098,24 @@
       <c r="F183" s="8"/>
       <c r="G183" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">the units the inverter stands for</t>
-        </is>
-      </c>
-      <c r="H183" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSCAD</t>
-        </is>
-      </c>
-    </row>
-    <row r="184">
-      <c r="A184" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSCAD_Params</t>
-        </is>
-      </c>
-      <c r="B184" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">{MVA}</t>
-        </is>
-      </c>
-      <c r="C184" s="8"/>
-      <c r="D184" s="8"/>
-      <c r="E184" s="8"/>
-      <c r="F184" s="8"/>
-      <c r="G184" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">their MVA</t>
-        </is>
-      </c>
-      <c r="H184" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSCAD</t>
-        </is>
-      </c>
+          <t xml:space="preserve">DETAILED: the terminal of the units at that node</t>
+        </is>
+      </c>
+      <c r="H183" s="8"/>
+    </row>
+    <row r="184" ht="18" customHeight="1">
+      <c r="A184" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD_Params PLACEHOLDERS -- filled in for each inverter a vendor model stands for</t>
+        </is>
+      </c>
+      <c r="B184" s="7"/>
+      <c r="C184" s="7"/>
+      <c r="D184" s="7"/>
+      <c r="E184" s="7"/>
+      <c r="F184" s="7"/>
+      <c r="G184" s="7"/>
+      <c r="H184" s="7"/>
     </row>
     <row r="185">
       <c r="A185" s="8" t="inlineStr">
@@ -7117,7 +7125,7 @@
       </c>
       <c r="B185" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{P_MW}</t>
+          <t xml:space="preserve">{UNITS}</t>
         </is>
       </c>
       <c r="C185" s="8"/>
@@ -7126,7 +7134,7 @@
       <c r="F185" s="8"/>
       <c r="G185" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">their P where the inverter connects (MW)</t>
+          <t xml:space="preserve">the units the inverter stands for</t>
         </is>
       </c>
       <c r="H185" s="13" t="inlineStr">
@@ -7143,7 +7151,7 @@
       </c>
       <c r="B186" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{Q_MVAR}</t>
+          <t xml:space="preserve">{MVA}</t>
         </is>
       </c>
       <c r="C186" s="8"/>
@@ -7152,7 +7160,7 @@
       <c r="F186" s="8"/>
       <c r="G186" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">their Q there (MVAr)</t>
+          <t xml:space="preserve">their MVA</t>
         </is>
       </c>
       <c r="H186" s="13" t="inlineStr">
@@ -7169,7 +7177,7 @@
       </c>
       <c r="B187" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{P_PU}</t>
+          <t xml:space="preserve">{P_MW}</t>
         </is>
       </c>
       <c r="C187" s="8"/>
@@ -7178,7 +7186,7 @@
       <c r="F187" s="8"/>
       <c r="G187" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">P on {MVA}</t>
+          <t xml:space="preserve">their P where the inverter connects (MW)</t>
         </is>
       </c>
       <c r="H187" s="13" t="inlineStr">
@@ -7195,7 +7203,7 @@
       </c>
       <c r="B188" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{Q_PU}</t>
+          <t xml:space="preserve">{Q_MVAR}</t>
         </is>
       </c>
       <c r="C188" s="8"/>
@@ -7204,7 +7212,7 @@
       <c r="F188" s="8"/>
       <c r="G188" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q on {MVA}</t>
+          <t xml:space="preserve">their Q there (MVAr)</t>
         </is>
       </c>
       <c r="H188" s="13" t="inlineStr">
@@ -7221,7 +7229,7 @@
       </c>
       <c r="B189" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{UNIT_MVA}</t>
+          <t xml:space="preserve">{P_PU}</t>
         </is>
       </c>
       <c r="C189" s="8"/>
@@ -7230,7 +7238,7 @@
       <c r="F189" s="8"/>
       <c r="G189" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">one unit's MVA</t>
+          <t xml:space="preserve">P on {MVA}</t>
         </is>
       </c>
       <c r="H189" s="13" t="inlineStr">
@@ -7247,7 +7255,7 @@
       </c>
       <c r="B190" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{UNIT_P_MW}</t>
+          <t xml:space="preserve">{Q_PU}</t>
         </is>
       </c>
       <c r="C190" s="8"/>
@@ -7256,7 +7264,7 @@
       <c r="F190" s="8"/>
       <c r="G190" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">one unit's P (MW)</t>
+          <t xml:space="preserve">Q on {MVA}</t>
         </is>
       </c>
       <c r="H190" s="13" t="inlineStr">
@@ -7273,7 +7281,7 @@
       </c>
       <c r="B191" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{UNIT_Q_MVAR}</t>
+          <t xml:space="preserve">{UNIT_MVA}</t>
         </is>
       </c>
       <c r="C191" s="8"/>
@@ -7282,7 +7290,7 @@
       <c r="F191" s="8"/>
       <c r="G191" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">one unit's Q (MVAr)</t>
+          <t xml:space="preserve">one unit's MVA</t>
         </is>
       </c>
       <c r="H191" s="13" t="inlineStr">
@@ -7299,7 +7307,7 @@
       </c>
       <c r="B192" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{V_PU}</t>
+          <t xml:space="preserve">{UNIT_P_MW}</t>
         </is>
       </c>
       <c r="C192" s="8"/>
@@ -7308,7 +7316,7 @@
       <c r="F192" s="8"/>
       <c r="G192" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">the voltage where it connects (pu)</t>
+          <t xml:space="preserve">one unit's P (MW)</t>
         </is>
       </c>
       <c r="H192" s="13" t="inlineStr">
@@ -7325,7 +7333,7 @@
       </c>
       <c r="B193" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{V_KV}</t>
+          <t xml:space="preserve">{UNIT_Q_MVAR}</t>
         </is>
       </c>
       <c r="C193" s="8"/>
@@ -7334,7 +7342,7 @@
       <c r="F193" s="8"/>
       <c r="G193" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">the same in kV</t>
+          <t xml:space="preserve">one unit's Q (MVAr)</t>
         </is>
       </c>
       <c r="H193" s="13" t="inlineStr">
@@ -7351,7 +7359,7 @@
       </c>
       <c r="B194" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{KV}</t>
+          <t xml:space="preserve">{V_PU}</t>
         </is>
       </c>
       <c r="C194" s="8"/>
@@ -7360,7 +7368,7 @@
       <c r="F194" s="8"/>
       <c r="G194" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">that bus's base kV</t>
+          <t xml:space="preserve">the voltage where it connects (pu)</t>
         </is>
       </c>
       <c r="H194" s="13" t="inlineStr">
@@ -7377,7 +7385,7 @@
       </c>
       <c r="B195" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{ANGLE}</t>
+          <t xml:space="preserve">{V_KV}</t>
         </is>
       </c>
       <c r="C195" s="8"/>
@@ -7386,7 +7394,7 @@
       <c r="F195" s="8"/>
       <c r="G195" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">its PSCAD angle (deg, the transformers' phase shifts included)</t>
+          <t xml:space="preserve">the same in kV</t>
         </is>
       </c>
       <c r="H195" s="13" t="inlineStr">
@@ -7403,7 +7411,7 @@
       </c>
       <c r="B196" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{FREQ}</t>
+          <t xml:space="preserve">{KV}</t>
         </is>
       </c>
       <c r="C196" s="8"/>
@@ -7412,7 +7420,7 @@
       <c r="F196" s="8"/>
       <c r="G196" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">frequency (Hz)</t>
+          <t xml:space="preserve">that bus's base kV</t>
         </is>
       </c>
       <c r="H196" s="13" t="inlineStr">
@@ -7429,7 +7437,7 @@
       </c>
       <c r="B197" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{P_INV_MW}</t>
+          <t xml:space="preserve">{ANGLE}</t>
         </is>
       </c>
       <c r="C197" s="8"/>
@@ -7438,7 +7446,7 @@
       <c r="F197" s="8"/>
       <c r="G197" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">P at the inverters' own terminals (MW; a UDM on the MV side)</t>
+          <t xml:space="preserve">its PSCAD angle (deg, the transformers' phase shifts included)</t>
         </is>
       </c>
       <c r="H197" s="13" t="inlineStr">
@@ -7455,7 +7463,7 @@
       </c>
       <c r="B198" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{Q_INV_MVAR}</t>
+          <t xml:space="preserve">{FREQ}</t>
         </is>
       </c>
       <c r="C198" s="8"/>
@@ -7464,7 +7472,7 @@
       <c r="F198" s="8"/>
       <c r="G198" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q there (MVAr)</t>
+          <t xml:space="preserve">frequency (Hz)</t>
         </is>
       </c>
       <c r="H198" s="13" t="inlineStr">
@@ -7481,7 +7489,7 @@
       </c>
       <c r="B199" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{V_INV_PU}</t>
+          <t xml:space="preserve">{P_INV_MW}</t>
         </is>
       </c>
       <c r="C199" s="8"/>
@@ -7490,10 +7498,62 @@
       <c r="F199" s="8"/>
       <c r="G199" s="8" t="inlineStr">
         <is>
+          <t xml:space="preserve">P at the inverters' own terminals (MW; a UDM on the MV side)</t>
+        </is>
+      </c>
+      <c r="H199" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD_Params</t>
+        </is>
+      </c>
+      <c r="B200" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{Q_INV_MVAR}</t>
+        </is>
+      </c>
+      <c r="C200" s="8"/>
+      <c r="D200" s="8"/>
+      <c r="E200" s="8"/>
+      <c r="F200" s="8"/>
+      <c r="G200" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Q there (MVAr)</t>
+        </is>
+      </c>
+      <c r="H200" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="201">
+      <c r="A201" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD_Params</t>
+        </is>
+      </c>
+      <c r="B201" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{V_INV_PU}</t>
+        </is>
+      </c>
+      <c r="C201" s="8"/>
+      <c r="D201" s="8"/>
+      <c r="E201" s="8"/>
+      <c r="F201" s="8"/>
+      <c r="G201" s="8" t="inlineStr">
+        <is>
           <t xml:space="preserve">the voltage there (pu)</t>
         </is>
       </c>
-      <c r="H199" s="13" t="inlineStr">
+      <c r="H201" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">PSCAD</t>
         </is>
@@ -7506,32 +7566,32 @@
     <mergeCell ref="A4:H4"/>
     <mergeCell ref="A51:H51"/>
     <mergeCell ref="A79:H79"/>
-    <mergeCell ref="A116:H116"/>
-    <mergeCell ref="A128:H128"/>
-    <mergeCell ref="A135:H135"/>
-    <mergeCell ref="A138:H138"/>
-    <mergeCell ref="A144:H144"/>
-    <mergeCell ref="A154:H154"/>
-    <mergeCell ref="A158:H158"/>
-    <mergeCell ref="A163:H163"/>
-    <mergeCell ref="A166:H166"/>
-    <mergeCell ref="A170:H170"/>
-    <mergeCell ref="A182:H182"/>
+    <mergeCell ref="A118:H118"/>
+    <mergeCell ref="A130:H130"/>
+    <mergeCell ref="A137:H137"/>
+    <mergeCell ref="A140:H140"/>
+    <mergeCell ref="A146:H146"/>
+    <mergeCell ref="A156:H156"/>
+    <mergeCell ref="A160:H160"/>
+    <mergeCell ref="A165:H165"/>
+    <mergeCell ref="A168:H168"/>
+    <mergeCell ref="A172:H172"/>
+    <mergeCell ref="A184:H184"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A4" location="'Plant'!A1" display="Plant"/>
     <hyperlink ref="A51" location="'MPT'!A1" display="MPT"/>
     <hyperlink ref="A79" location="'Generators'!A1" display="Generators"/>
-    <hyperlink ref="A116" location="'Feeders'!A1" display="Feeders"/>
-    <hyperlink ref="A128" location="'Cables'!A1" display="Cables"/>
-    <hyperlink ref="A135" location="'Collectors'!A1" display="Collectors"/>
-    <hyperlink ref="A138" location="'Loads_Shunts'!A1" display="Loads_Shunts"/>
-    <hyperlink ref="A144" location="'Machines'!A1" display="Machines"/>
-    <hyperlink ref="A154" location="'Bus_Numbers'!A1" display="Bus_Numbers"/>
-    <hyperlink ref="A158" location="'Dyr_Params'!A1" display="Dyr_Params"/>
-    <hyperlink ref="A163" location="'Dyr_Records'!A1" display="Dyr_Records"/>
-    <hyperlink ref="A166" location="'PSCAD_Params'!A1" display="PSCAD_Params"/>
-    <hyperlink ref="A182" location="'PSCAD_Params'!A1" display="PSCAD_Params"/>
+    <hyperlink ref="A118" location="'Feeders'!A1" display="Feeders"/>
+    <hyperlink ref="A130" location="'Cables'!A1" display="Cables"/>
+    <hyperlink ref="A137" location="'Collectors'!A1" display="Collectors"/>
+    <hyperlink ref="A140" location="'Loads_Shunts'!A1" display="Loads_Shunts"/>
+    <hyperlink ref="A146" location="'Machines'!A1" display="Machines"/>
+    <hyperlink ref="A156" location="'Bus_Numbers'!A1" display="Bus_Numbers"/>
+    <hyperlink ref="A160" location="'Dyr_Params'!A1" display="Dyr_Params"/>
+    <hyperlink ref="A165" location="'Dyr_Records'!A1" display="Dyr_Records"/>
+    <hyperlink ref="A168" location="'PSCAD_Params'!A1" display="PSCAD_Params"/>
+    <hyperlink ref="A184" location="'PSCAD_Params'!A1" display="PSCAD_Params"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
@@ -20544,7 +20604,9 @@
     <col min="33" max="33" width="18" customWidth="1"/>
     <col min="34" max="34" width="16" customWidth="1"/>
     <col min="35" max="35" width="10" customWidth="1"/>
-    <col min="36" max="36" width="10" customWidth="1"/>
+    <col min="36" max="36" width="18" customWidth="1"/>
+    <col min="37" max="37" width="10" customWidth="1"/>
+    <col min="38" max="38" width="10" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -20725,6 +20787,16 @@
       </c>
       <c r="AJ1" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">PSCAD source case</t>
+        </is>
+      </c>
+      <c r="AK1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD component ID</t>
+        </is>
+      </c>
+      <c r="AL1" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">PSCAD inverter at</t>
         </is>
       </c>
@@ -20886,6 +20958,16 @@
         </is>
       </c>
       <c r="AJ2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a .pscx or .pslx (or a project open in PSCAD) with one UDM set up as you want it (with PSCAD component ID)</t>
+        </is>
+      </c>
+      <c r="AK2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">that UDM's ID in the source case: copied, with its settings, to every GSU of this generator</t>
+        </is>
+      </c>
+      <c r="AL2" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">LV: the inverter (your UDM or the stand-in source) on the GSU's LV side, the GSU built | MV: on its HV side, for a UDM with its GSU inside (blank = LV)</t>
         </is>
@@ -20983,7 +21065,9 @@
       <c r="AG3" s="3"/>
       <c r="AH3" s="3"/>
       <c r="AI3" s="3"/>
-      <c r="AJ3" s="3" t="inlineStr">
+      <c r="AJ3" s="3"/>
+      <c r="AK3" s="3"/>
+      <c r="AL3" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">LV</t>
         </is>
@@ -21081,7 +21165,9 @@
       <c r="AG4" s="3"/>
       <c r="AH4" s="3"/>
       <c r="AI4" s="3"/>
-      <c r="AJ4" s="3" t="inlineStr">
+      <c r="AJ4" s="3"/>
+      <c r="AK4" s="3"/>
+      <c r="AL4" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">LV</t>
         </is>
@@ -21124,6 +21210,8 @@
       <c r="AH5" s="3"/>
       <c r="AI5" s="3"/>
       <c r="AJ5" s="3"/>
+      <c r="AK5" s="3"/>
+      <c r="AL5" s="3"/>
     </row>
     <row r="6">
       <c r="A6" s="3"/>
@@ -21162,6 +21250,8 @@
       <c r="AH6" s="3"/>
       <c r="AI6" s="3"/>
       <c r="AJ6" s="3"/>
+      <c r="AK6" s="3"/>
+      <c r="AL6" s="3"/>
     </row>
     <row r="7">
       <c r="A7" s="3"/>
@@ -21200,6 +21290,8 @@
       <c r="AH7" s="3"/>
       <c r="AI7" s="3"/>
       <c r="AJ7" s="3"/>
+      <c r="AK7" s="3"/>
+      <c r="AL7" s="3"/>
     </row>
     <row r="8">
       <c r="A8" s="3"/>
@@ -21238,6 +21330,8 @@
       <c r="AH8" s="3"/>
       <c r="AI8" s="3"/>
       <c r="AJ8" s="3"/>
+      <c r="AK8" s="3"/>
+      <c r="AL8" s="3"/>
     </row>
     <row r="9">
       <c r="A9" s="3"/>
@@ -21276,6 +21370,8 @@
       <c r="AH9" s="3"/>
       <c r="AI9" s="3"/>
       <c r="AJ9" s="3"/>
+      <c r="AK9" s="3"/>
+      <c r="AL9" s="3"/>
     </row>
     <row r="10">
       <c r="A10" s="3"/>
@@ -21314,6 +21410,8 @@
       <c r="AH10" s="3"/>
       <c r="AI10" s="3"/>
       <c r="AJ10" s="3"/>
+      <c r="AK10" s="3"/>
+      <c r="AL10" s="3"/>
     </row>
     <row r="11">
       <c r="A11" s="3"/>
@@ -21352,6 +21450,8 @@
       <c r="AH11" s="3"/>
       <c r="AI11" s="3"/>
       <c r="AJ11" s="3"/>
+      <c r="AK11" s="3"/>
+      <c r="AL11" s="3"/>
     </row>
     <row r="12">
       <c r="A12" s="3"/>
@@ -21390,6 +21490,8 @@
       <c r="AH12" s="3"/>
       <c r="AI12" s="3"/>
       <c r="AJ12" s="3"/>
+      <c r="AK12" s="3"/>
+      <c r="AL12" s="3"/>
     </row>
     <row r="13">
       <c r="A13" s="3"/>
@@ -21428,6 +21530,8 @@
       <c r="AH13" s="3"/>
       <c r="AI13" s="3"/>
       <c r="AJ13" s="3"/>
+      <c r="AK13" s="3"/>
+      <c r="AL13" s="3"/>
     </row>
     <row r="14">
       <c r="A14" s="3"/>
@@ -21466,6 +21570,8 @@
       <c r="AH14" s="3"/>
       <c r="AI14" s="3"/>
       <c r="AJ14" s="3"/>
+      <c r="AK14" s="3"/>
+      <c r="AL14" s="3"/>
     </row>
     <row r="15">
       <c r="A15" s="3"/>
@@ -21504,6 +21610,8 @@
       <c r="AH15" s="3"/>
       <c r="AI15" s="3"/>
       <c r="AJ15" s="3"/>
+      <c r="AK15" s="3"/>
+      <c r="AL15" s="3"/>
     </row>
     <row r="16">
       <c r="A16" s="3"/>
@@ -21542,6 +21650,8 @@
       <c r="AH16" s="3"/>
       <c r="AI16" s="3"/>
       <c r="AJ16" s="3"/>
+      <c r="AK16" s="3"/>
+      <c r="AL16" s="3"/>
     </row>
     <row r="17">
       <c r="A17" s="3"/>
@@ -21580,6 +21690,8 @@
       <c r="AH17" s="3"/>
       <c r="AI17" s="3"/>
       <c r="AJ17" s="3"/>
+      <c r="AK17" s="3"/>
+      <c r="AL17" s="3"/>
     </row>
     <row r="18">
       <c r="A18" s="3"/>
@@ -21618,6 +21730,8 @@
       <c r="AH18" s="3"/>
       <c r="AI18" s="3"/>
       <c r="AJ18" s="3"/>
+      <c r="AK18" s="3"/>
+      <c r="AL18" s="3"/>
     </row>
     <row r="19">
       <c r="A19" s="3"/>
@@ -21656,6 +21770,8 @@
       <c r="AH19" s="3"/>
       <c r="AI19" s="3"/>
       <c r="AJ19" s="3"/>
+      <c r="AK19" s="3"/>
+      <c r="AL19" s="3"/>
     </row>
     <row r="20">
       <c r="A20" s="3"/>
@@ -21694,6 +21810,8 @@
       <c r="AH20" s="3"/>
       <c r="AI20" s="3"/>
       <c r="AJ20" s="3"/>
+      <c r="AK20" s="3"/>
+      <c r="AL20" s="3"/>
     </row>
     <row r="21">
       <c r="A21" s="3"/>
@@ -21732,6 +21850,8 @@
       <c r="AH21" s="3"/>
       <c r="AI21" s="3"/>
       <c r="AJ21" s="3"/>
+      <c r="AK21" s="3"/>
+      <c r="AL21" s="3"/>
     </row>
     <row r="22">
       <c r="A22" s="3"/>
@@ -21770,6 +21890,8 @@
       <c r="AH22" s="3"/>
       <c r="AI22" s="3"/>
       <c r="AJ22" s="3"/>
+      <c r="AK22" s="3"/>
+      <c r="AL22" s="3"/>
     </row>
   </sheetData>
   <dataValidations count="6">
@@ -21788,7 +21910,7 @@
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="AF3:AF500">
       <formula1>"REEC_A,REEC_C,REEC_D"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="AJ3:AJ500">
+    <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="AL3:AL500">
       <formula1>"LV,MV"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
smib_build: feeder sections' own R, X, B; the UDM picked from the OEM's PSCAD model
- Feeders: R ohm / X ohm / B uS per section in place of Cable x Length (blank = as before); GUI: Fill R, X, B
  from cables shows the values to change, Clear R, X, B goes back; a section by R and X needs no cable; the
  report marks a section with its own values (*)
- Generators, Pick UDM from OEM model (GUI): the OEM's .pscx / .pslx read as XML -- its definitions listed with
  their ports, parameters and placed component IDs; the one picked (and the definitions it uses) is added to
  the case's definitions from that file, with the model's resources, and put at every GSU; a component ID
  copies the placed one instead, its settings kept

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BGsNUhFmVX23f8qnP53zUv
</commit_message>
<xml_diff>
--- a/smib/SMIB_INPUT_TEMPLATE.xlsx
+++ b/smib/SMIB_INPUT_TEMPLATE.xlsx
@@ -717,7 +717,7 @@
         </is>
       </c>
     </row>
-    <row r="44" ht="56.0" customHeight="1">
+    <row r="44" ht="82.0" customHeight="1">
       <c r="A44" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Feeders</t>
@@ -725,7 +725,7 @@
       </c>
       <c r="B44" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">The collector feeders section by section from the collector bus out: cable, length and the units tapped at the section's far end. A daisy chain needs no From section; a lateral names the section it leaves from (its far end); 0 = straight from the collector bus. Copies: identical feeders. WECC equivalent: Zeq = sum(Zi Wi^2) / W^2, Beq = sum(Bi), Wi = MW of the units downstream of section i.</t>
+          <t xml:space="preserve">The collector feeders section by section from the collector bus out: cable, length and the units tapped at the section's far end. A daisy chain needs no From section; a lateral names the section it leaves from (its far end); 0 = straight from the collector bus. Copies: identical feeders. WECC equivalent: Zeq = sum(Zi Wi^2) / W^2, Beq = sum(Bi), Wi = MW of the units downstream of section i. R ohm, X ohm, B uS: a section's own values (its parallel cables together) in place of Cable x Length -- the GUI's Fill R, X, B from cables shows them to change; Clear R, X, B goes back. A section with R and X needs no cable.</t>
         </is>
       </c>
     </row>
@@ -833,7 +833,7 @@
       </c>
       <c r="B53" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">The .pscx is built in the same run when PSCAD 5 and its Python library mhi.pscad (pip install mhi.pscad) are on the PC; otherwise run &lt;name&gt;_build_pscad.py where they are. The case holds the grid (source and Thevenin impedance), the gen-tie, the MPTs, each collector (the WECC equivalent as a pi section, or DETAILED: every feeder section, identical feeder copies lumped), the GSUs and, on each GSU's LV side, the inverter: your UDM (PSCAD library, definition and AC port in Generators) or a stand-in source at the solved voltage -- delete it and wire your UDM in its place (the report and the build log list every inverter node). Or set one UDM up in a case of its own (a vendor's test case) and give that case and the UDM's component ID (its Properties) in Generators: PSCAD source case, PSCAD component ID -- it is copied, with its settings, to every GSU of that generator (every machine of the DETAILED model), its definition and the case's resources (.lib, .obj) with it; PSCAD_Params rows ({UNITS}, {P_PU} ...) are set on each copy. PSCAD inverter at MV: for a UDM with its GSU inside, the inverter on the GSU's HV side and no GSU drawn. It is drawn as a single-line diagram with wires, left to right from the grid; where PSCAD's R, L and C are single-phase, each is drawn three times between breakouts.</t>
+          <t xml:space="preserve">The .pscx is built in the same run when PSCAD 5 and its Python library mhi.pscad (pip install mhi.pscad) are on the PC; otherwise run &lt;name&gt;_build_pscad.py where they are. The case holds the grid (source and Thevenin impedance), the gen-tie, the MPTs, each collector (the WECC equivalent as a pi section, or DETAILED: every feeder section, identical feeder copies lumped), the GSUs and, on each GSU's LV side, the inverter: your UDM (PSCAD library, definition and AC port in Generators) or a stand-in source at the solved voltage -- delete it and wire your UDM in its place (the report and the build log list every inverter node). Or take the UDM from the OEM's PSCAD model: Generators, Pick UDM from OEM model -- the model's definitions are listed (their ports, parameters and the IDs of the ones placed in it); the one picked is added to the case's definitions (with the ones it uses and the model's resources, .lib / .obj) and put at every GSU of that generator (every machine of the DETAILED model), PSCAD_Params rows ({UNITS}, {P_PU} ...) set on each; or, with a component ID, that placed one is copied instead, its settings and all. PSCAD inverter at MV: for a UDM with its GSU inside, the inverter on the GSU's HV side and no GSU drawn. It is drawn as a single-line diagram with wires, left to right from the grid; where PSCAD's R, L and C are single-phase, each is drawn three times between breakouts.</t>
         </is>
       </c>
     </row>
@@ -5282,7 +5282,7 @@
       <c r="F115" s="8"/>
       <c r="G115" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">a .pscx or .pslx (or a project open in PSCAD) with one UDM set up as you want it (with PSCAD component ID)</t>
+          <t xml:space="preserve">the OEM's PSCAD model (.pscx / .pslx) the UDM comes from: its PSCAD definition added to the case (GUI: Pick UDM from OEM model)</t>
         </is>
       </c>
       <c r="H115" s="13" t="inlineStr">
@@ -5291,7 +5291,7 @@
         </is>
       </c>
     </row>
-    <row r="116" ht="17.0" customHeight="1">
+    <row r="116" ht="30.0" customHeight="1">
       <c r="A116" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Generators</t>
@@ -5308,11 +5308,15 @@
         </is>
       </c>
       <c r="D116" s="8"/>
-      <c r="E116" s="8"/>
+      <c r="E116" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the definition, its values from PSCAD_Params</t>
+        </is>
+      </c>
       <c r="F116" s="8"/>
       <c r="G116" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">that UDM's ID in the source case: copied, with its settings, to every GSU of this generator</t>
+          <t xml:space="preserve">a UDM placed in the source case: copied with its settings instead (blank = the definition, its values from PSCAD_Params)</t>
         </is>
       </c>
       <c r="H116" s="13" t="inlineStr">
@@ -5719,42 +5723,66 @@
         </is>
       </c>
     </row>
-    <row r="130" ht="18" customHeight="1">
-      <c r="A130" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Cables</t>
-        </is>
-      </c>
-      <c r="B130" s="7"/>
-      <c r="C130" s="7"/>
-      <c r="D130" s="7"/>
-      <c r="E130" s="7"/>
-      <c r="F130" s="7"/>
-      <c r="G130" s="7"/>
-      <c r="H130" s="7"/>
+    <row r="130" ht="17.0" customHeight="1">
+      <c r="A130" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Feeders</t>
+        </is>
+      </c>
+      <c r="B130" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R ohm</t>
+        </is>
+      </c>
+      <c r="C130" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">r_ohm</t>
+        </is>
+      </c>
+      <c r="D130" s="8"/>
+      <c r="E130" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cable x Length</t>
+        </is>
+      </c>
+      <c r="F130" s="8"/>
+      <c r="G130" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the section's R, its parallel cables together (blank = Cable x Length)</t>
+        </is>
+      </c>
+      <c r="H130" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSS/E + PSCAD</t>
+        </is>
+      </c>
     </row>
     <row r="131" ht="17.0" customHeight="1">
       <c r="A131" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cables</t>
+          <t xml:space="preserve">Feeders</t>
         </is>
       </c>
       <c r="B131" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cable</t>
+          <t xml:space="preserve">X ohm</t>
         </is>
       </c>
       <c r="C131" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">cable</t>
+          <t xml:space="preserve">x_ohm</t>
         </is>
       </c>
       <c r="D131" s="8"/>
-      <c r="E131" s="8"/>
+      <c r="E131" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cable x Length</t>
+        </is>
+      </c>
       <c r="F131" s="8"/>
       <c r="G131" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">cable type</t>
+          <t xml:space="preserve">the section's X (blank = Cable x Length)</t>
         </is>
       </c>
       <c r="H131" s="13" t="inlineStr">
@@ -5766,66 +5794,50 @@
     <row r="132" ht="17.0" customHeight="1">
       <c r="A132" s="8" t="inlineStr">
         <is>
+          <t xml:space="preserve">Feeders</t>
+        </is>
+      </c>
+      <c r="B132" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">B uS</t>
+        </is>
+      </c>
+      <c r="C132" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">b_us</t>
+        </is>
+      </c>
+      <c r="D132" s="8"/>
+      <c r="E132" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cable x Length</t>
+        </is>
+      </c>
+      <c r="F132" s="8"/>
+      <c r="G132" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the section's charging B, total (blank = Cable x Length)</t>
+        </is>
+      </c>
+      <c r="H132" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSS/E + PSCAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="133" ht="18" customHeight="1">
+      <c r="A133" s="7" t="inlineStr">
+        <is>
           <t xml:space="preserve">Cables</t>
         </is>
       </c>
-      <c r="B132" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Length unit</t>
-        </is>
-      </c>
-      <c r="C132" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">unit</t>
-        </is>
-      </c>
-      <c r="D132" s="8"/>
-      <c r="E132" s="8"/>
-      <c r="F132" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">km | mi | kft | m | ft</t>
-        </is>
-      </c>
-      <c r="G132" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">the values are per</t>
-        </is>
-      </c>
-      <c r="H132" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
-        </is>
-      </c>
-    </row>
-    <row r="133" ht="17.0" customHeight="1">
-      <c r="A133" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Cables</t>
-        </is>
-      </c>
-      <c r="B133" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">R per length</t>
-        </is>
-      </c>
-      <c r="C133" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">r_per</t>
-        </is>
-      </c>
-      <c r="D133" s="8"/>
-      <c r="E133" s="8"/>
-      <c r="F133" s="8"/>
-      <c r="G133" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ohm, at operating temperature</t>
-        </is>
-      </c>
-      <c r="H133" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
-        </is>
-      </c>
+      <c r="B133" s="7"/>
+      <c r="C133" s="7"/>
+      <c r="D133" s="7"/>
+      <c r="E133" s="7"/>
+      <c r="F133" s="7"/>
+      <c r="G133" s="7"/>
+      <c r="H133" s="7"/>
     </row>
     <row r="134" ht="17.0" customHeight="1">
       <c r="A134" s="8" t="inlineStr">
@@ -5835,12 +5847,12 @@
       </c>
       <c r="B134" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">X per length</t>
+          <t xml:space="preserve">Cable</t>
         </is>
       </c>
       <c r="C134" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">x_per</t>
+          <t xml:space="preserve">cable</t>
         </is>
       </c>
       <c r="D134" s="8"/>
@@ -5848,7 +5860,7 @@
       <c r="F134" s="8"/>
       <c r="G134" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">ohm</t>
+          <t xml:space="preserve">cable type</t>
         </is>
       </c>
       <c r="H134" s="13" t="inlineStr">
@@ -5865,20 +5877,24 @@
       </c>
       <c r="B135" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">C per length</t>
+          <t xml:space="preserve">Length unit</t>
         </is>
       </c>
       <c r="C135" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">c_per</t>
+          <t xml:space="preserve">unit</t>
         </is>
       </c>
       <c r="D135" s="8"/>
       <c r="E135" s="8"/>
-      <c r="F135" s="8"/>
+      <c r="F135" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">km | mi | kft | m | ft</t>
+        </is>
+      </c>
       <c r="G135" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">uF</t>
+          <t xml:space="preserve">the values are per</t>
         </is>
       </c>
       <c r="H135" s="13" t="inlineStr">
@@ -5895,12 +5911,12 @@
       </c>
       <c r="B136" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">B per length</t>
+          <t xml:space="preserve">R per length</t>
         </is>
       </c>
       <c r="C136" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">b_per</t>
+          <t xml:space="preserve">r_per</t>
         </is>
       </c>
       <c r="D136" s="8"/>
@@ -5908,7 +5924,7 @@
       <c r="F136" s="8"/>
       <c r="G136" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">uS, instead of C</t>
+          <t xml:space="preserve">ohm, at operating temperature</t>
         </is>
       </c>
       <c r="H136" s="13" t="inlineStr">
@@ -5917,34 +5933,50 @@
         </is>
       </c>
     </row>
-    <row r="137" ht="18" customHeight="1">
-      <c r="A137" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Collectors</t>
-        </is>
-      </c>
-      <c r="B137" s="7"/>
-      <c r="C137" s="7"/>
-      <c r="D137" s="7"/>
-      <c r="E137" s="7"/>
-      <c r="F137" s="7"/>
-      <c r="G137" s="7"/>
-      <c r="H137" s="7"/>
+    <row r="137" ht="17.0" customHeight="1">
+      <c r="A137" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Cables</t>
+        </is>
+      </c>
+      <c r="B137" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">X per length</t>
+        </is>
+      </c>
+      <c r="C137" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">x_per</t>
+        </is>
+      </c>
+      <c r="D137" s="8"/>
+      <c r="E137" s="8"/>
+      <c r="F137" s="8"/>
+      <c r="G137" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ohm</t>
+        </is>
+      </c>
+      <c r="H137" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSS/E + PSCAD</t>
+        </is>
+      </c>
     </row>
     <row r="138" ht="17.0" customHeight="1">
       <c r="A138" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Collectors</t>
+          <t xml:space="preserve">Cables</t>
         </is>
       </c>
       <c r="B138" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Name</t>
+          <t xml:space="preserve">C per length</t>
         </is>
       </c>
       <c r="C138" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">name</t>
+          <t xml:space="preserve">c_per</t>
         </is>
       </c>
       <c r="D138" s="8"/>
@@ -5952,7 +5984,7 @@
       <c r="F138" s="8"/>
       <c r="G138" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">shared collector: its far-end bus has this name</t>
+          <t xml:space="preserve">uF</t>
         </is>
       </c>
       <c r="H138" s="13" t="inlineStr">
@@ -5964,17 +5996,17 @@
     <row r="139" ht="17.0" customHeight="1">
       <c r="A139" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Collectors</t>
+          <t xml:space="preserve">Cables</t>
         </is>
       </c>
       <c r="B139" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Connect to</t>
+          <t xml:space="preserve">B per length</t>
         </is>
       </c>
       <c r="C139" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">connect</t>
+          <t xml:space="preserve">b_per</t>
         </is>
       </c>
       <c r="D139" s="8"/>
@@ -5982,7 +6014,7 @@
       <c r="F139" s="8"/>
       <c r="G139" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">the bus it starts from (MPT1, MPT1:TV ...)</t>
+          <t xml:space="preserve">uS, instead of C</t>
         </is>
       </c>
       <c r="H139" s="13" t="inlineStr">
@@ -5994,7 +6026,7 @@
     <row r="140" ht="18" customHeight="1">
       <c r="A140" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">Loads_Shunts</t>
+          <t xml:space="preserve">Collectors</t>
         </is>
       </c>
       <c r="B140" s="7"/>
@@ -6008,29 +6040,25 @@
     <row r="141" ht="17.0" customHeight="1">
       <c r="A141" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Loads_Shunts</t>
+          <t xml:space="preserve">Collectors</t>
         </is>
       </c>
       <c r="B141" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Kind</t>
+          <t xml:space="preserve">Name</t>
         </is>
       </c>
       <c r="C141" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">kind</t>
+          <t xml:space="preserve">name</t>
         </is>
       </c>
       <c r="D141" s="8"/>
       <c r="E141" s="8"/>
-      <c r="F141" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LOAD | SHUNT</t>
-        </is>
-      </c>
+      <c r="F141" s="8"/>
       <c r="G141" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">LOAD: constant impedance | SHUNT: + capacitor, - reactor</t>
+          <t xml:space="preserve">shared collector: its far-end bus has this name</t>
         </is>
       </c>
       <c r="H141" s="13" t="inlineStr">
@@ -6042,17 +6070,17 @@
     <row r="142" ht="17.0" customHeight="1">
       <c r="A142" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Loads_Shunts</t>
+          <t xml:space="preserve">Collectors</t>
         </is>
       </c>
       <c r="B142" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">At bus</t>
+          <t xml:space="preserve">Connect to</t>
         </is>
       </c>
       <c r="C142" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">at</t>
+          <t xml:space="preserve">connect</t>
         </is>
       </c>
       <c r="D142" s="8"/>
@@ -6060,7 +6088,7 @@
       <c r="F142" s="8"/>
       <c r="G142" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">POI, HV, MPT1, MPT1:TV, PV:MV, PV ...</t>
+          <t xml:space="preserve">the bus it starts from (MPT1, MPT1:TV ...)</t>
         </is>
       </c>
       <c r="H142" s="13" t="inlineStr">
@@ -6069,35 +6097,19 @@
         </is>
       </c>
     </row>
-    <row r="143" ht="17.0" customHeight="1">
-      <c r="A143" s="8" t="inlineStr">
+    <row r="143" ht="18" customHeight="1">
+      <c r="A143" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Loads_Shunts</t>
         </is>
       </c>
-      <c r="B143" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">MW</t>
-        </is>
-      </c>
-      <c r="C143" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">mw</t>
-        </is>
-      </c>
-      <c r="D143" s="8"/>
-      <c r="E143" s="8"/>
-      <c r="F143" s="8"/>
-      <c r="G143" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">LOAD, at 1 pu</t>
-        </is>
-      </c>
-      <c r="H143" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
-        </is>
-      </c>
+      <c r="B143" s="7"/>
+      <c r="C143" s="7"/>
+      <c r="D143" s="7"/>
+      <c r="E143" s="7"/>
+      <c r="F143" s="7"/>
+      <c r="G143" s="7"/>
+      <c r="H143" s="7"/>
     </row>
     <row r="144" ht="17.0" customHeight="1">
       <c r="A144" s="8" t="inlineStr">
@@ -6107,20 +6119,24 @@
       </c>
       <c r="B144" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">MVAr</t>
+          <t xml:space="preserve">Kind</t>
         </is>
       </c>
       <c r="C144" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">mvar</t>
+          <t xml:space="preserve">kind</t>
         </is>
       </c>
       <c r="D144" s="8"/>
       <c r="E144" s="8"/>
-      <c r="F144" s="8"/>
+      <c r="F144" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LOAD | SHUNT</t>
+        </is>
+      </c>
       <c r="G144" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">at 1 pu: LOAD + inductive | SHUNT + capacitive</t>
+          <t xml:space="preserve">LOAD: constant impedance | SHUNT: + capacitor, - reactor</t>
         </is>
       </c>
       <c r="H144" s="13" t="inlineStr">
@@ -6137,52 +6153,72 @@
       </c>
       <c r="B145" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Name</t>
+          <t xml:space="preserve">At bus</t>
         </is>
       </c>
       <c r="C145" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">name</t>
+          <t xml:space="preserve">at</t>
         </is>
       </c>
       <c r="D145" s="8"/>
       <c r="E145" s="8"/>
       <c r="F145" s="8"/>
-      <c r="G145" s="8"/>
+      <c r="G145" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">POI, HV, MPT1, MPT1:TV, PV:MV, PV ...</t>
+        </is>
+      </c>
       <c r="H145" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">PSS/E + PSCAD</t>
         </is>
       </c>
     </row>
-    <row r="146" ht="18" customHeight="1">
-      <c r="A146" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Machines</t>
-        </is>
-      </c>
-      <c r="B146" s="7"/>
-      <c r="C146" s="7"/>
-      <c r="D146" s="7"/>
-      <c r="E146" s="7"/>
-      <c r="F146" s="7"/>
-      <c r="G146" s="7"/>
-      <c r="H146" s="7"/>
-    </row>
-    <row r="147" ht="30.0" customHeight="1">
+    <row r="146" ht="17.0" customHeight="1">
+      <c r="A146" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Loads_Shunts</t>
+        </is>
+      </c>
+      <c r="B146" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MW</t>
+        </is>
+      </c>
+      <c r="C146" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">mw</t>
+        </is>
+      </c>
+      <c r="D146" s="8"/>
+      <c r="E146" s="8"/>
+      <c r="F146" s="8"/>
+      <c r="G146" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LOAD, at 1 pu</t>
+        </is>
+      </c>
+      <c r="H146" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSS/E + PSCAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="147" ht="17.0" customHeight="1">
       <c r="A147" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Machines</t>
+          <t xml:space="preserve">Loads_Shunts</t>
         </is>
       </c>
       <c r="B147" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Machine</t>
+          <t xml:space="preserve">MVAr</t>
         </is>
       </c>
       <c r="C147" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">machine</t>
+          <t xml:space="preserve">mvar</t>
         </is>
       </c>
       <c r="D147" s="8"/>
@@ -6190,7 +6226,7 @@
       <c r="F147" s="8"/>
       <c r="G147" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">DETAILED model: a machine, &lt;generator&gt;_&lt;feeder&gt;_S&lt;section&gt; (the GUI lists them); its values in place of its share of its generator's</t>
+          <t xml:space="preserve">at 1 pu: LOAD + inductive | SHUNT + capacitive</t>
         </is>
       </c>
       <c r="H147" s="13" t="inlineStr">
@@ -6202,97 +6238,65 @@
     <row r="148" ht="17.0" customHeight="1">
       <c r="A148" s="8" t="inlineStr">
         <is>
+          <t xml:space="preserve">Loads_Shunts</t>
+        </is>
+      </c>
+      <c r="B148" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Name</t>
+        </is>
+      </c>
+      <c r="C148" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">name</t>
+        </is>
+      </c>
+      <c r="D148" s="8"/>
+      <c r="E148" s="8"/>
+      <c r="F148" s="8"/>
+      <c r="G148" s="8"/>
+      <c r="H148" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSS/E + PSCAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="149" ht="18" customHeight="1">
+      <c r="A149" s="7" t="inlineStr">
+        <is>
           <t xml:space="preserve">Machines</t>
         </is>
       </c>
-      <c r="B148" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Machine ID</t>
-        </is>
-      </c>
-      <c r="C148" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">id</t>
-        </is>
-      </c>
-      <c r="D148" s="8"/>
-      <c r="E148" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">its generator's</t>
-        </is>
-      </c>
-      <c r="F148" s="8"/>
-      <c r="G148" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">blank = its generator's</t>
-        </is>
-      </c>
-      <c r="H148" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
-        </is>
-      </c>
-    </row>
-    <row r="149" ht="30.0" customHeight="1">
-      <c r="A149" s="8" t="inlineStr">
+      <c r="B149" s="7"/>
+      <c r="C149" s="7"/>
+      <c r="D149" s="7"/>
+      <c r="E149" s="7"/>
+      <c r="F149" s="7"/>
+      <c r="G149" s="7"/>
+      <c r="H149" s="7"/>
+    </row>
+    <row r="150" ht="30.0" customHeight="1">
+      <c r="A150" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Machines</t>
         </is>
       </c>
-      <c r="B149" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Pgen MW</t>
-        </is>
-      </c>
-      <c r="C149" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">pgen_mw</t>
-        </is>
-      </c>
-      <c r="D149" s="8"/>
-      <c r="E149" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">its share of its generator's Dispatch MW</t>
-        </is>
-      </c>
-      <c r="F149" s="8"/>
-      <c r="G149" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">its dispatch (blank = its share of its generator's Dispatch MW)</t>
-        </is>
-      </c>
-      <c r="H149" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
-        </is>
-      </c>
-    </row>
-    <row r="150" ht="17.0" customHeight="1">
-      <c r="A150" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Machines</t>
-        </is>
-      </c>
       <c r="B150" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pmax MW</t>
+          <t xml:space="preserve">Machine</t>
         </is>
       </c>
       <c r="C150" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">pmax_mw</t>
+          <t xml:space="preserve">machine</t>
         </is>
       </c>
       <c r="D150" s="8"/>
-      <c r="E150" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">its units x Unit Pmax</t>
-        </is>
-      </c>
+      <c r="E150" s="8"/>
       <c r="F150" s="8"/>
       <c r="G150" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">blank = its units x Unit Pmax</t>
+          <t xml:space="preserve">DETAILED model: a machine, &lt;generator&gt;_&lt;feeder&gt;_S&lt;section&gt; (the GUI lists them); its values in place of its share of its generator's</t>
         </is>
       </c>
       <c r="H150" s="13" t="inlineStr">
@@ -6309,24 +6313,24 @@
       </c>
       <c r="B151" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pmin MW</t>
+          <t xml:space="preserve">Machine ID</t>
         </is>
       </c>
       <c r="C151" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">pmin_mw</t>
+          <t xml:space="preserve">id</t>
         </is>
       </c>
       <c r="D151" s="8"/>
       <c r="E151" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">its units x Unit Pmin</t>
+          <t xml:space="preserve">its generator's</t>
         </is>
       </c>
       <c r="F151" s="8"/>
       <c r="G151" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">blank = its units x Unit Pmin</t>
+          <t xml:space="preserve">blank = its generator's</t>
         </is>
       </c>
       <c r="H151" s="13" t="inlineStr">
@@ -6335,7 +6339,7 @@
         </is>
       </c>
     </row>
-    <row r="152" ht="17.0" customHeight="1">
+    <row r="152" ht="30.0" customHeight="1">
       <c r="A152" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Machines</t>
@@ -6343,24 +6347,24 @@
       </c>
       <c r="B152" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Qmax MVAr</t>
+          <t xml:space="preserve">Pgen MW</t>
         </is>
       </c>
       <c r="C152" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">qmax_mvar</t>
+          <t xml:space="preserve">pgen_mw</t>
         </is>
       </c>
       <c r="D152" s="8"/>
       <c r="E152" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">its units x Unit Qmax</t>
+          <t xml:space="preserve">its share of its generator's Dispatch MW</t>
         </is>
       </c>
       <c r="F152" s="8"/>
       <c r="G152" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">blank = its units x Unit Qmax</t>
+          <t xml:space="preserve">its dispatch (blank = its share of its generator's Dispatch MW)</t>
         </is>
       </c>
       <c r="H152" s="13" t="inlineStr">
@@ -6377,24 +6381,24 @@
       </c>
       <c r="B153" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Qmin MVAr</t>
+          <t xml:space="preserve">Pmax MW</t>
         </is>
       </c>
       <c r="C153" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">qmin_mvar</t>
+          <t xml:space="preserve">pmax_mw</t>
         </is>
       </c>
       <c r="D153" s="8"/>
       <c r="E153" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">its units x Unit Qmin</t>
+          <t xml:space="preserve">its units x Unit Pmax</t>
         </is>
       </c>
       <c r="F153" s="8"/>
       <c r="G153" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">blank = its units x Unit Qmin</t>
+          <t xml:space="preserve">blank = its units x Unit Pmax</t>
         </is>
       </c>
       <c r="H153" s="13" t="inlineStr">
@@ -6403,7 +6407,7 @@
         </is>
       </c>
     </row>
-    <row r="154" ht="30.0" customHeight="1">
+    <row r="154" ht="17.0" customHeight="1">
       <c r="A154" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Machines</t>
@@ -6411,24 +6415,24 @@
       </c>
       <c r="B154" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fixed Q MVAr</t>
+          <t xml:space="preserve">Pmin MW</t>
         </is>
       </c>
       <c r="C154" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">q_mvar</t>
+          <t xml:space="preserve">pmin_mw</t>
         </is>
       </c>
       <c r="D154" s="8"/>
       <c r="E154" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">as its generator's Q mode</t>
+          <t xml:space="preserve">its units x Unit Pmin</t>
         </is>
       </c>
       <c r="F154" s="8"/>
       <c r="G154" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">a value: this Q, fixed (blank = as its generator's Q mode)</t>
+          <t xml:space="preserve">blank = its units x Unit Pmin</t>
         </is>
       </c>
       <c r="H154" s="13" t="inlineStr">
@@ -6445,24 +6449,24 @@
       </c>
       <c r="B155" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">MBASE MVA</t>
+          <t xml:space="preserve">Qmax MVAr</t>
         </is>
       </c>
       <c r="C155" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">mbase_mva</t>
+          <t xml:space="preserve">qmax_mvar</t>
         </is>
       </c>
       <c r="D155" s="8"/>
       <c r="E155" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">its units x Unit MVA</t>
+          <t xml:space="preserve">its units x Unit Qmax</t>
         </is>
       </c>
       <c r="F155" s="8"/>
       <c r="G155" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">blank = its units x Unit MVA</t>
+          <t xml:space="preserve">blank = its units x Unit Qmax</t>
         </is>
       </c>
       <c r="H155" s="13" t="inlineStr">
@@ -6471,42 +6475,66 @@
         </is>
       </c>
     </row>
-    <row r="156" ht="18" customHeight="1">
-      <c r="A156" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Bus_Numbers</t>
-        </is>
-      </c>
-      <c r="B156" s="7"/>
-      <c r="C156" s="7"/>
-      <c r="D156" s="7"/>
-      <c r="E156" s="7"/>
-      <c r="F156" s="7"/>
-      <c r="G156" s="7"/>
-      <c r="H156" s="7"/>
-    </row>
-    <row r="157" ht="17.0" customHeight="1">
+    <row r="156" ht="17.0" customHeight="1">
+      <c r="A156" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Machines</t>
+        </is>
+      </c>
+      <c r="B156" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Qmin MVAr</t>
+        </is>
+      </c>
+      <c r="C156" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">qmin_mvar</t>
+        </is>
+      </c>
+      <c r="D156" s="8"/>
+      <c r="E156" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">its units x Unit Qmin</t>
+        </is>
+      </c>
+      <c r="F156" s="8"/>
+      <c r="G156" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">blank = its units x Unit Qmin</t>
+        </is>
+      </c>
+      <c r="H156" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSS/E + PSCAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="157" ht="30.0" customHeight="1">
       <c r="A157" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bus_Numbers</t>
+          <t xml:space="preserve">Machines</t>
         </is>
       </c>
       <c r="B157" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bus</t>
+          <t xml:space="preserve">Fixed Q MVAr</t>
         </is>
       </c>
       <c r="C157" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">bus</t>
+          <t xml:space="preserve">q_mvar</t>
         </is>
       </c>
       <c r="D157" s="8"/>
-      <c r="E157" s="8"/>
+      <c r="E157" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">as its generator's Q mode</t>
+        </is>
+      </c>
       <c r="F157" s="8"/>
       <c r="G157" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">its role: IB, POI, HV, MPT1:LV, PV:MV, PV:LV ...</t>
+          <t xml:space="preserve">a value: this Q, fixed (blank = as its generator's Q mode)</t>
         </is>
       </c>
       <c r="H157" s="13" t="inlineStr">
@@ -6518,29 +6546,29 @@
     <row r="158" ht="17.0" customHeight="1">
       <c r="A158" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bus_Numbers</t>
+          <t xml:space="preserve">Machines</t>
         </is>
       </c>
       <c r="B158" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Number</t>
+          <t xml:space="preserve">MBASE MVA</t>
         </is>
       </c>
       <c r="C158" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">number</t>
+          <t xml:space="preserve">mbase_mva</t>
         </is>
       </c>
       <c r="D158" s="8"/>
       <c r="E158" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">automatic</t>
+          <t xml:space="preserve">its units x Unit MVA</t>
         </is>
       </c>
       <c r="F158" s="8"/>
       <c r="G158" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">blank = automatic</t>
+          <t xml:space="preserve">blank = its units x Unit MVA</t>
         </is>
       </c>
       <c r="H158" s="13" t="inlineStr">
@@ -6549,143 +6577,131 @@
         </is>
       </c>
     </row>
-    <row r="159" ht="30.0" customHeight="1">
-      <c r="A159" s="8" t="inlineStr">
+    <row r="159" ht="18" customHeight="1">
+      <c r="A159" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Bus_Numbers</t>
         </is>
       </c>
-      <c r="B159" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Name</t>
-        </is>
-      </c>
-      <c r="C159" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">name</t>
-        </is>
-      </c>
-      <c r="D159" s="8"/>
-      <c r="E159" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">automatic (12 characters at most</t>
-        </is>
-      </c>
-      <c r="F159" s="8"/>
-      <c r="G159" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">blank = automatic (12 characters at most)</t>
-        </is>
-      </c>
-      <c r="H159" s="13" t="inlineStr">
+      <c r="B159" s="7"/>
+      <c r="C159" s="7"/>
+      <c r="D159" s="7"/>
+      <c r="E159" s="7"/>
+      <c r="F159" s="7"/>
+      <c r="G159" s="7"/>
+      <c r="H159" s="7"/>
+    </row>
+    <row r="160" ht="17.0" customHeight="1">
+      <c r="A160" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bus_Numbers</t>
+        </is>
+      </c>
+      <c r="B160" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bus</t>
+        </is>
+      </c>
+      <c r="C160" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">bus</t>
+        </is>
+      </c>
+      <c r="D160" s="8"/>
+      <c r="E160" s="8"/>
+      <c r="F160" s="8"/>
+      <c r="G160" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">its role: IB, POI, HV, MPT1:LV, PV:MV, PV:LV ...</t>
+        </is>
+      </c>
+      <c r="H160" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">PSS/E + PSCAD</t>
         </is>
       </c>
-    </row>
-    <row r="160" ht="18" customHeight="1">
-      <c r="A160" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Dyr_Params</t>
-        </is>
-      </c>
-      <c r="B160" s="7"/>
-      <c r="C160" s="7"/>
-      <c r="D160" s="7"/>
-      <c r="E160" s="7"/>
-      <c r="F160" s="7"/>
-      <c r="G160" s="7"/>
-      <c r="H160" s="7"/>
     </row>
     <row r="161" ht="17.0" customHeight="1">
       <c r="A161" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dyr_Params</t>
+          <t xml:space="preserve">Bus_Numbers</t>
         </is>
       </c>
       <c r="B161" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Generator</t>
+          <t xml:space="preserve">Number</t>
         </is>
       </c>
       <c r="C161" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">generator</t>
+          <t xml:space="preserve">number</t>
         </is>
       </c>
       <c r="D161" s="8"/>
-      <c r="E161" s="8"/>
+      <c r="E161" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">automatic</t>
+        </is>
+      </c>
       <c r="F161" s="8"/>
       <c r="G161" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">IB: the infinite bus | PLANT: the plant controller (REPC_B)</t>
+          <t xml:space="preserve">blank = automatic</t>
         </is>
       </c>
       <c r="H161" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E .dyr</t>
+          <t xml:space="preserve">PSS/E + PSCAD</t>
         </is>
       </c>
     </row>
     <row r="162" ht="30.0" customHeight="1">
       <c r="A162" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dyr_Params</t>
+          <t xml:space="preserve">Bus_Numbers</t>
         </is>
       </c>
       <c r="B162" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Model</t>
+          <t xml:space="preserve">Name</t>
         </is>
       </c>
       <c r="C162" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">model</t>
+          <t xml:space="preserve">name</t>
         </is>
       </c>
       <c r="D162" s="8"/>
-      <c r="E162" s="8"/>
+      <c r="E162" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">automatic (12 characters at most</t>
+        </is>
+      </c>
       <c r="F162" s="8"/>
       <c r="G162" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">REGCA1 (REGCAU1) | REECA1 REECCU1 REECDU1 | REPCA1 (REPCAU1) or REAX4BU1 | PLANT: PLNTBU1 | WT3: + WTDTA1 WTARA1 WTPTA1 WTTQA1 | SYNC: GENROU SEXS TGOV1 | IB: GENCLS</t>
+          <t xml:space="preserve">blank = automatic (12 characters at most)</t>
         </is>
       </c>
       <c r="H162" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E .dyr</t>
-        </is>
-      </c>
-    </row>
-    <row r="163" ht="17.0" customHeight="1">
-      <c r="A163" s="8" t="inlineStr">
+          <t xml:space="preserve">PSS/E + PSCAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="163" ht="18" customHeight="1">
+      <c r="A163" s="7" t="inlineStr">
         <is>
           <t xml:space="preserve">Dyr_Params</t>
         </is>
       </c>
-      <c r="B163" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Parameter</t>
-        </is>
-      </c>
-      <c r="C163" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">parameter</t>
-        </is>
-      </c>
-      <c r="D163" s="8"/>
-      <c r="E163" s="8"/>
-      <c r="F163" s="8"/>
-      <c r="G163" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSS/E name (the report lists them all) or position: ICON2, CON14</t>
-        </is>
-      </c>
-      <c r="H163" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSS/E .dyr</t>
-        </is>
-      </c>
+      <c r="B163" s="7"/>
+      <c r="C163" s="7"/>
+      <c r="D163" s="7"/>
+      <c r="E163" s="7"/>
+      <c r="F163" s="7"/>
+      <c r="G163" s="7"/>
+      <c r="H163" s="7"/>
     </row>
     <row r="164" ht="17.0" customHeight="1">
       <c r="A164" s="8" t="inlineStr">
@@ -6695,64 +6711,80 @@
       </c>
       <c r="B164" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Value</t>
+          <t xml:space="preserve">Generator</t>
         </is>
       </c>
       <c r="C164" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">value</t>
+          <t xml:space="preserve">generator</t>
         </is>
       </c>
       <c r="D164" s="8"/>
       <c r="E164" s="8"/>
       <c r="F164" s="8"/>
-      <c r="G164" s="8"/>
+      <c r="G164" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">IB: the infinite bus | PLANT: the plant controller (REPC_B)</t>
+        </is>
+      </c>
       <c r="H164" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">PSS/E .dyr</t>
         </is>
       </c>
     </row>
-    <row r="165" ht="18" customHeight="1">
-      <c r="A165" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Dyr_Records</t>
-        </is>
-      </c>
-      <c r="B165" s="7"/>
-      <c r="C165" s="7"/>
-      <c r="D165" s="7"/>
-      <c r="E165" s="7"/>
-      <c r="F165" s="7"/>
-      <c r="G165" s="7"/>
-      <c r="H165" s="7"/>
+    <row r="165" ht="30.0" customHeight="1">
+      <c r="A165" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Dyr_Params</t>
+        </is>
+      </c>
+      <c r="B165" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Model</t>
+        </is>
+      </c>
+      <c r="C165" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">model</t>
+        </is>
+      </c>
+      <c r="D165" s="8"/>
+      <c r="E165" s="8"/>
+      <c r="F165" s="8"/>
+      <c r="G165" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">REGCA1 (REGCAU1) | REECA1 REECCU1 REECDU1 | REPCA1 (REPCAU1) or REAX4BU1 | PLANT: PLNTBU1 | WT3: + WTDTA1 WTARA1 WTPTA1 WTTQA1 | SYNC: GENROU SEXS TGOV1 | IB: GENCLS</t>
+        </is>
+      </c>
+      <c r="H165" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSS/E .dyr</t>
+        </is>
+      </c>
     </row>
     <row r="166" ht="17.0" customHeight="1">
       <c r="A166" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dyr_Records</t>
+          <t xml:space="preserve">Dyr_Params</t>
         </is>
       </c>
       <c r="B166" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Generator</t>
+          <t xml:space="preserve">Parameter</t>
         </is>
       </c>
       <c r="C166" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">generator</t>
+          <t xml:space="preserve">parameter</t>
         </is>
       </c>
       <c r="D166" s="8"/>
-      <c r="E166" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">the plant</t>
-        </is>
-      </c>
+      <c r="E166" s="8"/>
       <c r="F166" s="8"/>
       <c r="G166" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">blank = the plant</t>
+          <t xml:space="preserve">PSS/E name (the report lists them all) or position: ICON2, CON14</t>
         </is>
       </c>
       <c r="H166" s="13" t="inlineStr">
@@ -6764,27 +6796,23 @@
     <row r="167" ht="17.0" customHeight="1">
       <c r="A167" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Dyr_Records</t>
+          <t xml:space="preserve">Dyr_Params</t>
         </is>
       </c>
       <c r="B167" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Record</t>
+          <t xml:space="preserve">Value</t>
         </is>
       </c>
       <c r="C167" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">record</t>
+          <t xml:space="preserve">value</t>
         </is>
       </c>
       <c r="D167" s="8"/>
       <c r="E167" s="8"/>
       <c r="F167" s="8"/>
-      <c r="G167" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">.dyr text ending in / -- {BUS} {ID} {MBASE} {POI} {IB} {HV} {MV} {&lt;bus role&gt;} are filled in</t>
-        </is>
-      </c>
+      <c r="G167" s="8"/>
       <c r="H167" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">PSS/E .dyr</t>
@@ -6794,7 +6822,7 @@
     <row r="168" ht="18" customHeight="1">
       <c r="A168" s="7" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSCAD_Params</t>
+          <t xml:space="preserve">Dyr_Records</t>
         </is>
       </c>
       <c r="B168" s="7"/>
@@ -6808,7 +6836,7 @@
     <row r="169" ht="17.0" customHeight="1">
       <c r="A169" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSCAD_Params</t>
+          <t xml:space="preserve">Dyr_Records</t>
         </is>
       </c>
       <c r="B169" s="12" t="inlineStr">
@@ -6822,29 +6850,37 @@
         </is>
       </c>
       <c r="D169" s="8"/>
-      <c r="E169" s="8"/>
+      <c r="E169" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the plant</t>
+        </is>
+      </c>
       <c r="F169" s="8"/>
-      <c r="G169" s="8"/>
+      <c r="G169" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">blank = the plant</t>
+        </is>
+      </c>
       <c r="H169" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSCAD</t>
+          <t xml:space="preserve">PSS/E .dyr</t>
         </is>
       </c>
     </row>
     <row r="170" ht="17.0" customHeight="1">
       <c r="A170" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSCAD_Params</t>
+          <t xml:space="preserve">Dyr_Records</t>
         </is>
       </c>
       <c r="B170" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Parameter</t>
+          <t xml:space="preserve">Record</t>
         </is>
       </c>
       <c r="C170" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">parameter</t>
+          <t xml:space="preserve">record</t>
         </is>
       </c>
       <c r="D170" s="8"/>
@@ -6852,118 +6888,134 @@
       <c r="F170" s="8"/>
       <c r="G170" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">the vendor model's parameter name</t>
+          <t xml:space="preserve">.dyr text ending in / -- {BUS} {ID} {MBASE} {POI} {IB} {HV} {MV} {&lt;bus role&gt;} are filled in</t>
         </is>
       </c>
       <c r="H170" s="13" t="inlineStr">
         <is>
+          <t xml:space="preserve">PSS/E .dyr</t>
+        </is>
+      </c>
+    </row>
+    <row r="171" ht="18" customHeight="1">
+      <c r="A171" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD_Params</t>
+        </is>
+      </c>
+      <c r="B171" s="7"/>
+      <c r="C171" s="7"/>
+      <c r="D171" s="7"/>
+      <c r="E171" s="7"/>
+      <c r="F171" s="7"/>
+      <c r="G171" s="7"/>
+      <c r="H171" s="7"/>
+    </row>
+    <row r="172" ht="17.0" customHeight="1">
+      <c r="A172" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD_Params</t>
+        </is>
+      </c>
+      <c r="B172" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Generator</t>
+        </is>
+      </c>
+      <c r="C172" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">generator</t>
+        </is>
+      </c>
+      <c r="D172" s="8"/>
+      <c r="E172" s="8"/>
+      <c r="F172" s="8"/>
+      <c r="G172" s="8"/>
+      <c r="H172" s="13" t="inlineStr">
+        <is>
           <t xml:space="preserve">PSCAD</t>
         </is>
       </c>
     </row>
-    <row r="171" ht="17.0" customHeight="1">
-      <c r="A171" s="8" t="inlineStr">
+    <row r="173" ht="17.0" customHeight="1">
+      <c r="A173" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">PSCAD_Params</t>
         </is>
       </c>
-      <c r="B171" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Value</t>
-        </is>
-      </c>
-      <c r="C171" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">value</t>
-        </is>
-      </c>
-      <c r="D171" s="8"/>
-      <c r="E171" s="8"/>
-      <c r="F171" s="8"/>
-      <c r="G171" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">as PSCAD takes it (0.63 [kV], 40, {UNITS}, {P_PU} ...)</t>
-        </is>
-      </c>
-      <c r="H171" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSCAD</t>
-        </is>
-      </c>
-    </row>
-    <row r="172" ht="18" customHeight="1">
-      <c r="A172" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">BUS NAMES -- Connect to, At, Bus_Numbers and {&lt;bus&gt;} in Dyr_Records take these</t>
-        </is>
-      </c>
-      <c r="B172" s="7"/>
-      <c r="C172" s="7"/>
-      <c r="D172" s="7"/>
-      <c r="E172" s="7"/>
-      <c r="F172" s="7"/>
-      <c r="G172" s="7"/>
-      <c r="H172" s="7"/>
-    </row>
-    <row r="173">
-      <c r="A173" s="8"/>
       <c r="B173" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">IB</t>
-        </is>
-      </c>
-      <c r="C173" s="8"/>
+          <t xml:space="preserve">Parameter</t>
+        </is>
+      </c>
+      <c r="C173" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">parameter</t>
+        </is>
+      </c>
       <c r="D173" s="8"/>
       <c r="E173" s="8"/>
       <c r="F173" s="8"/>
       <c r="G173" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">the infinite bus</t>
-        </is>
-      </c>
-      <c r="H173" s="8"/>
-    </row>
-    <row r="174">
-      <c r="A174" s="8"/>
+          <t xml:space="preserve">the vendor model's parameter name</t>
+        </is>
+      </c>
+      <c r="H173" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="174" ht="17.0" customHeight="1">
+      <c r="A174" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD_Params</t>
+        </is>
+      </c>
       <c r="B174" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">POI</t>
-        </is>
-      </c>
-      <c r="C174" s="8"/>
+          <t xml:space="preserve">Value</t>
+        </is>
+      </c>
+      <c r="C174" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">value</t>
+        </is>
+      </c>
       <c r="D174" s="8"/>
       <c r="E174" s="8"/>
       <c r="F174" s="8"/>
       <c r="G174" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">the point of interconnection</t>
-        </is>
-      </c>
-      <c r="H174" s="8"/>
-    </row>
-    <row r="175">
-      <c r="A175" s="8"/>
-      <c r="B175" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">HV</t>
-        </is>
-      </c>
-      <c r="C175" s="8"/>
-      <c r="D175" s="8"/>
-      <c r="E175" s="8"/>
-      <c r="F175" s="8"/>
-      <c r="G175" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">the gen-tie's plant end (the POI when there is no gen-tie)</t>
-        </is>
-      </c>
-      <c r="H175" s="8"/>
+          <t xml:space="preserve">as PSCAD takes it (0.63 [kV], 40, {UNITS}, {P_PU} ...)</t>
+        </is>
+      </c>
+      <c r="H174" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="175" ht="18" customHeight="1">
+      <c r="A175" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BUS NAMES -- Connect to, At, Bus_Numbers and {&lt;bus&gt;} in Dyr_Records take these</t>
+        </is>
+      </c>
+      <c r="B175" s="7"/>
+      <c r="C175" s="7"/>
+      <c r="D175" s="7"/>
+      <c r="E175" s="7"/>
+      <c r="F175" s="7"/>
+      <c r="G175" s="7"/>
+      <c r="H175" s="7"/>
     </row>
     <row r="176">
       <c r="A176" s="8"/>
       <c r="B176" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;MPT&gt; or &lt;MPT&gt;:LV</t>
+          <t xml:space="preserve">IB</t>
         </is>
       </c>
       <c r="C176" s="8"/>
@@ -6972,7 +7024,7 @@
       <c r="F176" s="8"/>
       <c r="G176" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">an MPT's LV winding</t>
+          <t xml:space="preserve">the infinite bus</t>
         </is>
       </c>
       <c r="H176" s="8"/>
@@ -6981,7 +7033,7 @@
       <c r="A177" s="8"/>
       <c r="B177" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;MPT&gt;:TV</t>
+          <t xml:space="preserve">POI</t>
         </is>
       </c>
       <c r="C177" s="8"/>
@@ -6990,7 +7042,7 @@
       <c r="F177" s="8"/>
       <c r="G177" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">a 3-winding MPT's tertiary</t>
+          <t xml:space="preserve">the point of interconnection</t>
         </is>
       </c>
       <c r="H177" s="8"/>
@@ -6999,7 +7051,7 @@
       <c r="A178" s="8"/>
       <c r="B178" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;MPT&gt;:HV</t>
+          <t xml:space="preserve">HV</t>
         </is>
       </c>
       <c r="C178" s="8"/>
@@ -7008,7 +7060,7 @@
       <c r="F178" s="8"/>
       <c r="G178" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">an MPT with a tie line of its own: its HV end</t>
+          <t xml:space="preserve">the gen-tie's plant end (the POI when there is no gen-tie)</t>
         </is>
       </c>
       <c r="H178" s="8"/>
@@ -7017,7 +7069,7 @@
       <c r="A179" s="8"/>
       <c r="B179" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;collector&gt;</t>
+          <t xml:space="preserve">&lt;MPT&gt; or &lt;MPT&gt;:LV</t>
         </is>
       </c>
       <c r="C179" s="8"/>
@@ -7026,7 +7078,7 @@
       <c r="F179" s="8"/>
       <c r="G179" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">a shared collector's far end</t>
+          <t xml:space="preserve">an MPT's LV winding</t>
         </is>
       </c>
       <c r="H179" s="8"/>
@@ -7035,7 +7087,7 @@
       <c r="A180" s="8"/>
       <c r="B180" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;generator&gt;:MV</t>
+          <t xml:space="preserve">&lt;MPT&gt;:TV</t>
         </is>
       </c>
       <c r="C180" s="8"/>
@@ -7044,7 +7096,7 @@
       <c r="F180" s="8"/>
       <c r="G180" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">a generator's GSU HV side</t>
+          <t xml:space="preserve">a 3-winding MPT's tertiary</t>
         </is>
       </c>
       <c r="H180" s="8"/>
@@ -7053,7 +7105,7 @@
       <c r="A181" s="8"/>
       <c r="B181" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;generator&gt; or &lt;generator&gt;:LV</t>
+          <t xml:space="preserve">&lt;MPT&gt;:HV</t>
         </is>
       </c>
       <c r="C181" s="8"/>
@@ -7062,7 +7114,7 @@
       <c r="F181" s="8"/>
       <c r="G181" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">a generator's terminal</t>
+          <t xml:space="preserve">an MPT with a tie line of its own: its HV end</t>
         </is>
       </c>
       <c r="H181" s="8"/>
@@ -7071,7 +7123,7 @@
       <c r="A182" s="8"/>
       <c r="B182" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;collector&gt;_&lt;feeder&gt;_S&lt;n&gt;</t>
+          <t xml:space="preserve">&lt;collector&gt;</t>
         </is>
       </c>
       <c r="C182" s="8"/>
@@ -7080,7 +7132,7 @@
       <c r="F182" s="8"/>
       <c r="G182" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">DETAILED: the far end of feeder section n</t>
+          <t xml:space="preserve">a shared collector's far end</t>
         </is>
       </c>
       <c r="H182" s="8"/>
@@ -7089,7 +7141,7 @@
       <c r="A183" s="8"/>
       <c r="B183" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">&lt;generator&gt;_&lt;feeder&gt;_S&lt;n&gt;:LV</t>
+          <t xml:space="preserve">&lt;generator&gt;:MV</t>
         </is>
       </c>
       <c r="C183" s="8"/>
@@ -7098,34 +7150,34 @@
       <c r="F183" s="8"/>
       <c r="G183" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">DETAILED: the terminal of the units at that node</t>
+          <t xml:space="preserve">a generator's GSU HV side</t>
         </is>
       </c>
       <c r="H183" s="8"/>
     </row>
-    <row r="184" ht="18" customHeight="1">
-      <c r="A184" s="7" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSCAD_Params PLACEHOLDERS -- filled in for each inverter a vendor model stands for</t>
-        </is>
-      </c>
-      <c r="B184" s="7"/>
-      <c r="C184" s="7"/>
-      <c r="D184" s="7"/>
-      <c r="E184" s="7"/>
-      <c r="F184" s="7"/>
-      <c r="G184" s="7"/>
-      <c r="H184" s="7"/>
+    <row r="184">
+      <c r="A184" s="8"/>
+      <c r="B184" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">&lt;generator&gt; or &lt;generator&gt;:LV</t>
+        </is>
+      </c>
+      <c r="C184" s="8"/>
+      <c r="D184" s="8"/>
+      <c r="E184" s="8"/>
+      <c r="F184" s="8"/>
+      <c r="G184" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">a generator's terminal</t>
+        </is>
+      </c>
+      <c r="H184" s="8"/>
     </row>
     <row r="185">
-      <c r="A185" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSCAD_Params</t>
-        </is>
-      </c>
+      <c r="A185" s="8"/>
       <c r="B185" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{UNITS}</t>
+          <t xml:space="preserve">&lt;collector&gt;_&lt;feeder&gt;_S&lt;n&gt;</t>
         </is>
       </c>
       <c r="C185" s="8"/>
@@ -7134,24 +7186,16 @@
       <c r="F185" s="8"/>
       <c r="G185" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">the units the inverter stands for</t>
-        </is>
-      </c>
-      <c r="H185" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSCAD</t>
-        </is>
-      </c>
+          <t xml:space="preserve">DETAILED: the far end of feeder section n</t>
+        </is>
+      </c>
+      <c r="H185" s="8"/>
     </row>
     <row r="186">
-      <c r="A186" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSCAD_Params</t>
-        </is>
-      </c>
+      <c r="A186" s="8"/>
       <c r="B186" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{MVA}</t>
+          <t xml:space="preserve">&lt;generator&gt;_&lt;feeder&gt;_S&lt;n&gt;:LV</t>
         </is>
       </c>
       <c r="C186" s="8"/>
@@ -7160,40 +7204,24 @@
       <c r="F186" s="8"/>
       <c r="G186" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">their MVA</t>
-        </is>
-      </c>
-      <c r="H186" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSCAD</t>
-        </is>
-      </c>
-    </row>
-    <row r="187">
-      <c r="A187" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSCAD_Params</t>
-        </is>
-      </c>
-      <c r="B187" s="12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">{P_MW}</t>
-        </is>
-      </c>
-      <c r="C187" s="8"/>
-      <c r="D187" s="8"/>
-      <c r="E187" s="8"/>
-      <c r="F187" s="8"/>
-      <c r="G187" s="8" t="inlineStr">
-        <is>
-          <t xml:space="preserve">their P where the inverter connects (MW)</t>
-        </is>
-      </c>
-      <c r="H187" s="13" t="inlineStr">
-        <is>
-          <t xml:space="preserve">PSCAD</t>
-        </is>
-      </c>
+          <t xml:space="preserve">DETAILED: the terminal of the units at that node</t>
+        </is>
+      </c>
+      <c r="H186" s="8"/>
+    </row>
+    <row r="187" ht="18" customHeight="1">
+      <c r="A187" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD_Params PLACEHOLDERS -- filled in for each inverter a vendor model stands for</t>
+        </is>
+      </c>
+      <c r="B187" s="7"/>
+      <c r="C187" s="7"/>
+      <c r="D187" s="7"/>
+      <c r="E187" s="7"/>
+      <c r="F187" s="7"/>
+      <c r="G187" s="7"/>
+      <c r="H187" s="7"/>
     </row>
     <row r="188">
       <c r="A188" s="8" t="inlineStr">
@@ -7203,7 +7231,7 @@
       </c>
       <c r="B188" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{Q_MVAR}</t>
+          <t xml:space="preserve">{UNITS}</t>
         </is>
       </c>
       <c r="C188" s="8"/>
@@ -7212,7 +7240,7 @@
       <c r="F188" s="8"/>
       <c r="G188" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">their Q there (MVAr)</t>
+          <t xml:space="preserve">the units the inverter stands for</t>
         </is>
       </c>
       <c r="H188" s="13" t="inlineStr">
@@ -7229,7 +7257,7 @@
       </c>
       <c r="B189" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{P_PU}</t>
+          <t xml:space="preserve">{MVA}</t>
         </is>
       </c>
       <c r="C189" s="8"/>
@@ -7238,7 +7266,7 @@
       <c r="F189" s="8"/>
       <c r="G189" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">P on {MVA}</t>
+          <t xml:space="preserve">their MVA</t>
         </is>
       </c>
       <c r="H189" s="13" t="inlineStr">
@@ -7255,7 +7283,7 @@
       </c>
       <c r="B190" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{Q_PU}</t>
+          <t xml:space="preserve">{P_MW}</t>
         </is>
       </c>
       <c r="C190" s="8"/>
@@ -7264,7 +7292,7 @@
       <c r="F190" s="8"/>
       <c r="G190" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q on {MVA}</t>
+          <t xml:space="preserve">their P where the inverter connects (MW)</t>
         </is>
       </c>
       <c r="H190" s="13" t="inlineStr">
@@ -7281,7 +7309,7 @@
       </c>
       <c r="B191" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{UNIT_MVA}</t>
+          <t xml:space="preserve">{Q_MVAR}</t>
         </is>
       </c>
       <c r="C191" s="8"/>
@@ -7290,7 +7318,7 @@
       <c r="F191" s="8"/>
       <c r="G191" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">one unit's MVA</t>
+          <t xml:space="preserve">their Q there (MVAr)</t>
         </is>
       </c>
       <c r="H191" s="13" t="inlineStr">
@@ -7307,7 +7335,7 @@
       </c>
       <c r="B192" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{UNIT_P_MW}</t>
+          <t xml:space="preserve">{P_PU}</t>
         </is>
       </c>
       <c r="C192" s="8"/>
@@ -7316,7 +7344,7 @@
       <c r="F192" s="8"/>
       <c r="G192" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">one unit's P (MW)</t>
+          <t xml:space="preserve">P on {MVA}</t>
         </is>
       </c>
       <c r="H192" s="13" t="inlineStr">
@@ -7333,7 +7361,7 @@
       </c>
       <c r="B193" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{UNIT_Q_MVAR}</t>
+          <t xml:space="preserve">{Q_PU}</t>
         </is>
       </c>
       <c r="C193" s="8"/>
@@ -7342,7 +7370,7 @@
       <c r="F193" s="8"/>
       <c r="G193" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">one unit's Q (MVAr)</t>
+          <t xml:space="preserve">Q on {MVA}</t>
         </is>
       </c>
       <c r="H193" s="13" t="inlineStr">
@@ -7359,7 +7387,7 @@
       </c>
       <c r="B194" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{V_PU}</t>
+          <t xml:space="preserve">{UNIT_MVA}</t>
         </is>
       </c>
       <c r="C194" s="8"/>
@@ -7368,7 +7396,7 @@
       <c r="F194" s="8"/>
       <c r="G194" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">the voltage where it connects (pu)</t>
+          <t xml:space="preserve">one unit's MVA</t>
         </is>
       </c>
       <c r="H194" s="13" t="inlineStr">
@@ -7385,7 +7413,7 @@
       </c>
       <c r="B195" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{V_KV}</t>
+          <t xml:space="preserve">{UNIT_P_MW}</t>
         </is>
       </c>
       <c r="C195" s="8"/>
@@ -7394,7 +7422,7 @@
       <c r="F195" s="8"/>
       <c r="G195" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">the same in kV</t>
+          <t xml:space="preserve">one unit's P (MW)</t>
         </is>
       </c>
       <c r="H195" s="13" t="inlineStr">
@@ -7411,7 +7439,7 @@
       </c>
       <c r="B196" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{KV}</t>
+          <t xml:space="preserve">{UNIT_Q_MVAR}</t>
         </is>
       </c>
       <c r="C196" s="8"/>
@@ -7420,7 +7448,7 @@
       <c r="F196" s="8"/>
       <c r="G196" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">that bus's base kV</t>
+          <t xml:space="preserve">one unit's Q (MVAr)</t>
         </is>
       </c>
       <c r="H196" s="13" t="inlineStr">
@@ -7437,7 +7465,7 @@
       </c>
       <c r="B197" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{ANGLE}</t>
+          <t xml:space="preserve">{V_PU}</t>
         </is>
       </c>
       <c r="C197" s="8"/>
@@ -7446,7 +7474,7 @@
       <c r="F197" s="8"/>
       <c r="G197" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">its PSCAD angle (deg, the transformers' phase shifts included)</t>
+          <t xml:space="preserve">the voltage where it connects (pu)</t>
         </is>
       </c>
       <c r="H197" s="13" t="inlineStr">
@@ -7463,7 +7491,7 @@
       </c>
       <c r="B198" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{FREQ}</t>
+          <t xml:space="preserve">{V_KV}</t>
         </is>
       </c>
       <c r="C198" s="8"/>
@@ -7472,7 +7500,7 @@
       <c r="F198" s="8"/>
       <c r="G198" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">frequency (Hz)</t>
+          <t xml:space="preserve">the same in kV</t>
         </is>
       </c>
       <c r="H198" s="13" t="inlineStr">
@@ -7489,7 +7517,7 @@
       </c>
       <c r="B199" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{P_INV_MW}</t>
+          <t xml:space="preserve">{KV}</t>
         </is>
       </c>
       <c r="C199" s="8"/>
@@ -7498,7 +7526,7 @@
       <c r="F199" s="8"/>
       <c r="G199" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">P at the inverters' own terminals (MW; a UDM on the MV side)</t>
+          <t xml:space="preserve">that bus's base kV</t>
         </is>
       </c>
       <c r="H199" s="13" t="inlineStr">
@@ -7515,7 +7543,7 @@
       </c>
       <c r="B200" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{Q_INV_MVAR}</t>
+          <t xml:space="preserve">{ANGLE}</t>
         </is>
       </c>
       <c r="C200" s="8"/>
@@ -7524,7 +7552,7 @@
       <c r="F200" s="8"/>
       <c r="G200" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q there (MVAr)</t>
+          <t xml:space="preserve">its PSCAD angle (deg, the transformers' phase shifts included)</t>
         </is>
       </c>
       <c r="H200" s="13" t="inlineStr">
@@ -7541,7 +7569,7 @@
       </c>
       <c r="B201" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">{V_INV_PU}</t>
+          <t xml:space="preserve">{FREQ}</t>
         </is>
       </c>
       <c r="C201" s="8"/>
@@ -7550,10 +7578,88 @@
       <c r="F201" s="8"/>
       <c r="G201" s="8" t="inlineStr">
         <is>
+          <t xml:space="preserve">frequency (Hz)</t>
+        </is>
+      </c>
+      <c r="H201" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="202">
+      <c r="A202" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD_Params</t>
+        </is>
+      </c>
+      <c r="B202" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{P_INV_MW}</t>
+        </is>
+      </c>
+      <c r="C202" s="8"/>
+      <c r="D202" s="8"/>
+      <c r="E202" s="8"/>
+      <c r="F202" s="8"/>
+      <c r="G202" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">P at the inverters' own terminals (MW; a UDM on the MV side)</t>
+        </is>
+      </c>
+      <c r="H202" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="203">
+      <c r="A203" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD_Params</t>
+        </is>
+      </c>
+      <c r="B203" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{Q_INV_MVAR}</t>
+        </is>
+      </c>
+      <c r="C203" s="8"/>
+      <c r="D203" s="8"/>
+      <c r="E203" s="8"/>
+      <c r="F203" s="8"/>
+      <c r="G203" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Q there (MVAr)</t>
+        </is>
+      </c>
+      <c r="H203" s="13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD</t>
+        </is>
+      </c>
+    </row>
+    <row r="204">
+      <c r="A204" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PSCAD_Params</t>
+        </is>
+      </c>
+      <c r="B204" s="12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">{V_INV_PU}</t>
+        </is>
+      </c>
+      <c r="C204" s="8"/>
+      <c r="D204" s="8"/>
+      <c r="E204" s="8"/>
+      <c r="F204" s="8"/>
+      <c r="G204" s="8" t="inlineStr">
+        <is>
           <t xml:space="preserve">the voltage there (pu)</t>
         </is>
       </c>
-      <c r="H201" s="13" t="inlineStr">
+      <c r="H204" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">PSCAD</t>
         </is>
@@ -7567,31 +7673,31 @@
     <mergeCell ref="A51:H51"/>
     <mergeCell ref="A79:H79"/>
     <mergeCell ref="A118:H118"/>
-    <mergeCell ref="A130:H130"/>
-    <mergeCell ref="A137:H137"/>
+    <mergeCell ref="A133:H133"/>
     <mergeCell ref="A140:H140"/>
-    <mergeCell ref="A146:H146"/>
-    <mergeCell ref="A156:H156"/>
-    <mergeCell ref="A160:H160"/>
-    <mergeCell ref="A165:H165"/>
+    <mergeCell ref="A143:H143"/>
+    <mergeCell ref="A149:H149"/>
+    <mergeCell ref="A159:H159"/>
+    <mergeCell ref="A163:H163"/>
     <mergeCell ref="A168:H168"/>
-    <mergeCell ref="A172:H172"/>
-    <mergeCell ref="A184:H184"/>
+    <mergeCell ref="A171:H171"/>
+    <mergeCell ref="A175:H175"/>
+    <mergeCell ref="A187:H187"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="A4" location="'Plant'!A1" display="Plant"/>
     <hyperlink ref="A51" location="'MPT'!A1" display="MPT"/>
     <hyperlink ref="A79" location="'Generators'!A1" display="Generators"/>
     <hyperlink ref="A118" location="'Feeders'!A1" display="Feeders"/>
-    <hyperlink ref="A130" location="'Cables'!A1" display="Cables"/>
-    <hyperlink ref="A137" location="'Collectors'!A1" display="Collectors"/>
-    <hyperlink ref="A140" location="'Loads_Shunts'!A1" display="Loads_Shunts"/>
-    <hyperlink ref="A146" location="'Machines'!A1" display="Machines"/>
-    <hyperlink ref="A156" location="'Bus_Numbers'!A1" display="Bus_Numbers"/>
-    <hyperlink ref="A160" location="'Dyr_Params'!A1" display="Dyr_Params"/>
-    <hyperlink ref="A165" location="'Dyr_Records'!A1" display="Dyr_Records"/>
-    <hyperlink ref="A168" location="'PSCAD_Params'!A1" display="PSCAD_Params"/>
-    <hyperlink ref="A184" location="'PSCAD_Params'!A1" display="PSCAD_Params"/>
+    <hyperlink ref="A133" location="'Cables'!A1" display="Cables"/>
+    <hyperlink ref="A140" location="'Collectors'!A1" display="Collectors"/>
+    <hyperlink ref="A143" location="'Loads_Shunts'!A1" display="Loads_Shunts"/>
+    <hyperlink ref="A149" location="'Machines'!A1" display="Machines"/>
+    <hyperlink ref="A159" location="'Bus_Numbers'!A1" display="Bus_Numbers"/>
+    <hyperlink ref="A163" location="'Dyr_Params'!A1" display="Dyr_Params"/>
+    <hyperlink ref="A168" location="'Dyr_Records'!A1" display="Dyr_Records"/>
+    <hyperlink ref="A171" location="'PSCAD_Params'!A1" display="PSCAD_Params"/>
+    <hyperlink ref="A187" location="'PSCAD_Params'!A1" display="PSCAD_Params"/>
   </hyperlinks>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
   <pageSetup orientation="landscape" fitToWidth="1" fitToHeight="0"/>
@@ -20959,12 +21065,12 @@
       </c>
       <c r="AJ2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">a .pscx or .pslx (or a project open in PSCAD) with one UDM set up as you want it (with PSCAD component ID)</t>
+          <t xml:space="preserve">the OEM's PSCAD model (.pscx / .pslx) the UDM comes from: its PSCAD definition added to the case (GUI: Pick UDM from OEM model)</t>
         </is>
       </c>
       <c r="AK2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">that UDM's ID in the source case: copied, with its settings, to every GSU of this generator</t>
+          <t xml:space="preserve">a UDM placed in the source case: copied with its settings instead (blank = the definition, its values from PSCAD_Params)</t>
         </is>
       </c>
       <c r="AL2" s="2" t="inlineStr">
@@ -21938,6 +22044,9 @@
     <col min="9" max="9" width="10" customWidth="1"/>
     <col min="10" max="10" width="10" customWidth="1"/>
     <col min="11" max="11" width="10" customWidth="1"/>
+    <col min="12" max="12" width="10" customWidth="1"/>
+    <col min="13" max="13" width="10" customWidth="1"/>
+    <col min="14" max="14" width="10" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -21996,6 +22105,21 @@
           <t xml:space="preserve">Parallel cables</t>
         </is>
       </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">R ohm</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">X ohm</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">B uS</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="124.0" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -22049,6 +22173,21 @@
           <t xml:space="preserve">blank = 1</t>
         </is>
       </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the section's R, its parallel cables together (blank = Cable x Length)</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the section's X (blank = Cable x Length)</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">the section's charging B, total (blank = Cable x Length)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -22086,6 +22225,9 @@
       </c>
       <c r="J3" s="3"/>
       <c r="K3" s="3"/>
+      <c r="L3" s="3"/>
+      <c r="M3" s="3"/>
+      <c r="N3" s="3"/>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
@@ -22123,6 +22265,9 @@
       </c>
       <c r="J4" s="3"/>
       <c r="K4" s="3"/>
+      <c r="L4" s="3"/>
+      <c r="M4" s="3"/>
+      <c r="N4" s="3"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -22160,6 +22305,9 @@
       </c>
       <c r="J5" s="3"/>
       <c r="K5" s="3"/>
+      <c r="L5" s="3"/>
+      <c r="M5" s="3"/>
+      <c r="N5" s="3"/>
     </row>
     <row r="6">
       <c r="A6" s="3" t="inlineStr">
@@ -22197,6 +22345,9 @@
       </c>
       <c r="J6" s="3"/>
       <c r="K6" s="3"/>
+      <c r="L6" s="3"/>
+      <c r="M6" s="3"/>
+      <c r="N6" s="3"/>
     </row>
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
@@ -22234,6 +22385,9 @@
       </c>
       <c r="J7" s="3"/>
       <c r="K7" s="3"/>
+      <c r="L7" s="3"/>
+      <c r="M7" s="3"/>
+      <c r="N7" s="3"/>
     </row>
     <row r="8">
       <c r="A8" s="3" t="inlineStr">
@@ -22271,6 +22425,9 @@
       </c>
       <c r="J8" s="3"/>
       <c r="K8" s="3"/>
+      <c r="L8" s="3"/>
+      <c r="M8" s="3"/>
+      <c r="N8" s="3"/>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
@@ -22308,6 +22465,9 @@
       </c>
       <c r="J9" s="3"/>
       <c r="K9" s="3"/>
+      <c r="L9" s="3"/>
+      <c r="M9" s="3"/>
+      <c r="N9" s="3"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -22345,6 +22505,9 @@
       </c>
       <c r="J10" s="3"/>
       <c r="K10" s="3"/>
+      <c r="L10" s="3"/>
+      <c r="M10" s="3"/>
+      <c r="N10" s="3"/>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -22382,6 +22545,9 @@
       </c>
       <c r="J11" s="3"/>
       <c r="K11" s="3"/>
+      <c r="L11" s="3"/>
+      <c r="M11" s="3"/>
+      <c r="N11" s="3"/>
     </row>
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
@@ -22419,6 +22585,9 @@
       </c>
       <c r="J12" s="3"/>
       <c r="K12" s="3"/>
+      <c r="L12" s="3"/>
+      <c r="M12" s="3"/>
+      <c r="N12" s="3"/>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
@@ -22456,6 +22625,9 @@
       </c>
       <c r="J13" s="3"/>
       <c r="K13" s="3"/>
+      <c r="L13" s="3"/>
+      <c r="M13" s="3"/>
+      <c r="N13" s="3"/>
     </row>
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
@@ -22493,6 +22665,9 @@
       </c>
       <c r="J14" s="3"/>
       <c r="K14" s="3"/>
+      <c r="L14" s="3"/>
+      <c r="M14" s="3"/>
+      <c r="N14" s="3"/>
     </row>
     <row r="15">
       <c r="A15" s="3"/>
@@ -22506,6 +22681,9 @@
       <c r="I15" s="3"/>
       <c r="J15" s="3"/>
       <c r="K15" s="3"/>
+      <c r="L15" s="3"/>
+      <c r="M15" s="3"/>
+      <c r="N15" s="3"/>
     </row>
     <row r="16">
       <c r="A16" s="3"/>
@@ -22519,6 +22697,9 @@
       <c r="I16" s="3"/>
       <c r="J16" s="3"/>
       <c r="K16" s="3"/>
+      <c r="L16" s="3"/>
+      <c r="M16" s="3"/>
+      <c r="N16" s="3"/>
     </row>
     <row r="17">
       <c r="A17" s="3"/>
@@ -22532,6 +22713,9 @@
       <c r="I17" s="3"/>
       <c r="J17" s="3"/>
       <c r="K17" s="3"/>
+      <c r="L17" s="3"/>
+      <c r="M17" s="3"/>
+      <c r="N17" s="3"/>
     </row>
     <row r="18">
       <c r="A18" s="3"/>
@@ -22545,6 +22729,9 @@
       <c r="I18" s="3"/>
       <c r="J18" s="3"/>
       <c r="K18" s="3"/>
+      <c r="L18" s="3"/>
+      <c r="M18" s="3"/>
+      <c r="N18" s="3"/>
     </row>
     <row r="19">
       <c r="A19" s="3"/>
@@ -22558,6 +22745,9 @@
       <c r="I19" s="3"/>
       <c r="J19" s="3"/>
       <c r="K19" s="3"/>
+      <c r="L19" s="3"/>
+      <c r="M19" s="3"/>
+      <c r="N19" s="3"/>
     </row>
     <row r="20">
       <c r="A20" s="3"/>
@@ -22571,6 +22761,9 @@
       <c r="I20" s="3"/>
       <c r="J20" s="3"/>
       <c r="K20" s="3"/>
+      <c r="L20" s="3"/>
+      <c r="M20" s="3"/>
+      <c r="N20" s="3"/>
     </row>
     <row r="21">
       <c r="A21" s="3"/>
@@ -22584,6 +22777,9 @@
       <c r="I21" s="3"/>
       <c r="J21" s="3"/>
       <c r="K21" s="3"/>
+      <c r="L21" s="3"/>
+      <c r="M21" s="3"/>
+      <c r="N21" s="3"/>
     </row>
     <row r="22">
       <c r="A22" s="3"/>
@@ -22597,6 +22793,9 @@
       <c r="I22" s="3"/>
       <c r="J22" s="3"/>
       <c r="K22" s="3"/>
+      <c r="L22" s="3"/>
+      <c r="M22" s="3"/>
+      <c r="N22" s="3"/>
     </row>
     <row r="23">
       <c r="A23" s="3"/>
@@ -22610,6 +22809,9 @@
       <c r="I23" s="3"/>
       <c r="J23" s="3"/>
       <c r="K23" s="3"/>
+      <c r="L23" s="3"/>
+      <c r="M23" s="3"/>
+      <c r="N23" s="3"/>
     </row>
     <row r="24">
       <c r="A24" s="3"/>
@@ -22623,6 +22825,9 @@
       <c r="I24" s="3"/>
       <c r="J24" s="3"/>
       <c r="K24" s="3"/>
+      <c r="L24" s="3"/>
+      <c r="M24" s="3"/>
+      <c r="N24" s="3"/>
     </row>
     <row r="25">
       <c r="A25" s="3"/>
@@ -22636,6 +22841,9 @@
       <c r="I25" s="3"/>
       <c r="J25" s="3"/>
       <c r="K25" s="3"/>
+      <c r="L25" s="3"/>
+      <c r="M25" s="3"/>
+      <c r="N25" s="3"/>
     </row>
     <row r="26">
       <c r="A26" s="3"/>
@@ -22649,6 +22857,9 @@
       <c r="I26" s="3"/>
       <c r="J26" s="3"/>
       <c r="K26" s="3"/>
+      <c r="L26" s="3"/>
+      <c r="M26" s="3"/>
+      <c r="N26" s="3"/>
     </row>
   </sheetData>
   <dataValidations count="1">

</xml_diff>

<commit_message>
smib_build: gen-tie in feet; a few feet of line solves; its R, X, B shown as typed
- 'values per' blank: per km or per mile, whichever brings the R, X, B nearer
  a typical line of the POI kV (a NOTE says which) -- no longer the length's
  own unit, so a length in ft with per-km values works. Values per ft that
  are far off say to set 'values per'.
- The load flow takes a series impedance of at least 1e-4 pu, PSS/E's and
  PSLF's jumper threshold: a gen-tie of a few feet (1e-8 pu) made it fail.
- GUI Plant: the gen-tie's R, X (ohm, pu) and B as the build will take them,
  beside its totals, updated as its fields change.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BGsNUhFmVX23f8qnP53zUv
</commit_message>
<xml_diff>
--- a/smib/SMIB_INPUT_TEMPLATE.xlsx
+++ b/smib/SMIB_INPUT_TEMPLATE.xlsx
@@ -2365,7 +2365,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="17.0" customHeight="1">
+    <row r="25" ht="43.0" customHeight="1">
       <c r="A25" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Plant</t>
@@ -2384,7 +2384,7 @@
       <c r="D25" s="8"/>
       <c r="E25" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">the Gen-tie length unit</t>
+          <t xml:space="preserve">km or mi, whichever matches a line of the POI kV</t>
         </is>
       </c>
       <c r="F25" s="8" t="inlineStr">
@@ -2394,7 +2394,7 @@
       </c>
       <c r="G25" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">the length R, X, B, C below are per: km, mi, kft, m, ft (blank = the Gen-tie length unit)</t>
+          <t xml:space="preserve">the length R, X, B, C below are per: km, mi, kft, m, ft (blank = km or mi, whichever matches a line of the POI kV)</t>
         </is>
       </c>
       <c r="H25" s="13" t="inlineStr">
@@ -4185,7 +4185,7 @@
         </is>
       </c>
     </row>
-    <row r="79" ht="17.0" customHeight="1">
+    <row r="79" ht="30.0" customHeight="1">
       <c r="A79" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">MPT</t>
@@ -4204,7 +4204,7 @@
       <c r="D79" s="8"/>
       <c r="E79" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tie length unit</t>
+          <t xml:space="preserve">km or mi, whichever matches a line of its kV</t>
         </is>
       </c>
       <c r="F79" s="8" t="inlineStr">
@@ -4214,7 +4214,7 @@
       </c>
       <c r="G79" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">the length R, X, B are per (blank = Tie length unit)</t>
+          <t xml:space="preserve">the length R, X, B are per (blank = km or mi, whichever matches a line of its kV)</t>
         </is>
       </c>
       <c r="H79" s="13" t="inlineStr">
@@ -20407,7 +20407,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="30.0" customHeight="1">
+    <row r="25" ht="43.0" customHeight="1">
       <c r="A25" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Gen-tie values per</t>
@@ -20421,7 +20421,7 @@
       <c r="C25" s="8"/>
       <c r="D25" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">the Gen-tie length unit</t>
+          <t xml:space="preserve">km or mi, whichever matches a line of the POI kV</t>
         </is>
       </c>
       <c r="E25" s="8" t="inlineStr">
@@ -20431,7 +20431,7 @@
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">the length R, X, B, C below are per: km, mi, kft, m, ft (blank = the Gen-tie length unit)</t>
+          <t xml:space="preserve">the length R, X, B, C below are per: km, mi, kft, m, ft (blank = km or mi, whichever matches a line of the POI kV)</t>
         </is>
       </c>
       <c r="G25" s="13" t="inlineStr">
@@ -21565,7 +21565,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="88.0" customHeight="1">
+    <row r="2" ht="100.0" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve"># MPT name. Its buses: &lt;name&gt; or &lt;name&gt;:LV (LV winding), &lt;name&gt;:TV (tertiary)</t>
@@ -21676,7 +21676,7 @@
       <c r="X2" s="2"/>
       <c r="Y2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">the length R, X, B are per (blank = Tie length unit)</t>
+          <t xml:space="preserve">the length R, X, B are per (blank = km or mi, whichever matches a line of its kV)</t>
         </is>
       </c>
       <c r="Z2" s="2" t="inlineStr">

</xml_diff>

<commit_message>
smib_build GUI: converter model and electrical control drop-downs per generator type
Generators: Converter model and Electrical control open with one click and
list only what the generator's Type takes (REGC_A / REGC_B; PV REEC_A /
REEC_D, BESS REEC_C / REEC_D ...), each with what it is for; the code is
what is kept. A blank cell shows the model the build takes, in brackets; a
Type that does not take the model chosen drops it. Each input says which
programs it goes into (PSS/E, PSLF, PSCAD).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BGsNUhFmVX23f8qnP53zUv
</commit_message>
<xml_diff>
--- a/smib/SMIB_INPUT_TEMPLATE.xlsx
+++ b/smib/SMIB_INPUT_TEMPLATE.xlsx
@@ -594,7 +594,7 @@
     <row r="31">
       <c r="A31" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
       <c r="B31" s="8" t="inlineStr">
@@ -1695,7 +1695,7 @@
       </c>
       <c r="H5" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -1733,7 +1733,7 @@
       </c>
       <c r="H6" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -1771,7 +1771,7 @@
       </c>
       <c r="H7" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -1809,7 +1809,7 @@
       </c>
       <c r="H8" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -1847,7 +1847,7 @@
       </c>
       <c r="H9" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -1885,7 +1885,7 @@
       </c>
       <c r="H10" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -1923,7 +1923,7 @@
       </c>
       <c r="H11" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSLF</t>
         </is>
       </c>
     </row>
@@ -1961,7 +1961,7 @@
       </c>
       <c r="H12" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSLF</t>
         </is>
       </c>
     </row>
@@ -1999,7 +1999,7 @@
       </c>
       <c r="H13" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -2029,7 +2029,7 @@
       </c>
       <c r="H14" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -2063,7 +2063,7 @@
       <c r="G15" s="8"/>
       <c r="H15" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -2093,7 +2093,7 @@
       </c>
       <c r="H16" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -2123,7 +2123,7 @@
       </c>
       <c r="H17" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -2149,7 +2149,7 @@
       <c r="G18" s="8"/>
       <c r="H18" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -2187,7 +2187,7 @@
       </c>
       <c r="H19" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -2221,7 +2221,7 @@
       </c>
       <c r="H20" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -2255,7 +2255,7 @@
       </c>
       <c r="H21" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -2289,7 +2289,7 @@
       </c>
       <c r="H22" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -2323,7 +2323,7 @@
       </c>
       <c r="H23" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -2361,7 +2361,7 @@
       </c>
       <c r="H24" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -2399,7 +2399,7 @@
       </c>
       <c r="H25" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -2437,7 +2437,7 @@
       </c>
       <c r="H26" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -2475,7 +2475,7 @@
       </c>
       <c r="H27" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -2513,7 +2513,7 @@
       </c>
       <c r="H28" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -2547,7 +2547,7 @@
       </c>
       <c r="H29" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -2581,7 +2581,7 @@
       </c>
       <c r="H30" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -2611,7 +2611,7 @@
       <c r="G31" s="8"/>
       <c r="H31" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -2641,7 +2641,7 @@
       <c r="G32" s="8"/>
       <c r="H32" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -2675,7 +2675,7 @@
       </c>
       <c r="H33" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -2713,7 +2713,7 @@
       </c>
       <c r="H34" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -2747,7 +2747,7 @@
       </c>
       <c r="H35" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -2785,7 +2785,7 @@
       </c>
       <c r="H36" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -2823,7 +2823,7 @@
       </c>
       <c r="H37" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -2853,7 +2853,7 @@
       </c>
       <c r="H38" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -2891,7 +2891,7 @@
       </c>
       <c r="H39" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -2929,7 +2929,7 @@
       </c>
       <c r="H40" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -2967,7 +2967,7 @@
       </c>
       <c r="H41" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E .dyr</t>
+          <t xml:space="preserve">PSS/E + PSLF</t>
         </is>
       </c>
     </row>
@@ -3005,7 +3005,7 @@
       </c>
       <c r="H42" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E .dyr</t>
+          <t xml:space="preserve">PSS/E</t>
         </is>
       </c>
     </row>
@@ -3451,7 +3451,7 @@
       </c>
       <c r="H55" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -3489,7 +3489,7 @@
       </c>
       <c r="H56" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -3515,7 +3515,7 @@
       <c r="G57" s="8"/>
       <c r="H57" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -3541,7 +3541,7 @@
       <c r="G58" s="8"/>
       <c r="H58" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -3575,7 +3575,7 @@
       </c>
       <c r="H59" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -3605,7 +3605,7 @@
       </c>
       <c r="H60" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -3635,7 +3635,7 @@
       </c>
       <c r="H61" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -3665,7 +3665,7 @@
       </c>
       <c r="H62" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -3695,7 +3695,7 @@
       </c>
       <c r="H63" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -3725,7 +3725,7 @@
       </c>
       <c r="H64" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -3755,7 +3755,7 @@
       </c>
       <c r="H65" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -3789,7 +3789,7 @@
       </c>
       <c r="H66" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -3823,7 +3823,7 @@
       </c>
       <c r="H67" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -3857,7 +3857,7 @@
       </c>
       <c r="H68" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -3887,7 +3887,7 @@
       </c>
       <c r="H69" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -3917,7 +3917,7 @@
       </c>
       <c r="H70" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -3947,7 +3947,7 @@
       </c>
       <c r="H71" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -3981,7 +3981,7 @@
       </c>
       <c r="H72" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -4015,7 +4015,7 @@
       </c>
       <c r="H73" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -4049,7 +4049,7 @@
       </c>
       <c r="H74" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -4083,7 +4083,7 @@
       </c>
       <c r="H75" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -4117,7 +4117,7 @@
       </c>
       <c r="H76" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -4151,7 +4151,7 @@
       </c>
       <c r="H77" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -4181,7 +4181,7 @@
       <c r="G78" s="8"/>
       <c r="H78" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -4219,7 +4219,7 @@
       </c>
       <c r="H79" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -4253,7 +4253,7 @@
       </c>
       <c r="H80" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -4287,7 +4287,7 @@
       </c>
       <c r="H81" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -4321,7 +4321,7 @@
       </c>
       <c r="H82" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -4355,7 +4355,7 @@
       </c>
       <c r="H83" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -4399,7 +4399,7 @@
       </c>
       <c r="H85" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -4433,7 +4433,7 @@
       </c>
       <c r="H86" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -4467,7 +4467,7 @@
       </c>
       <c r="H87" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -4497,7 +4497,7 @@
       </c>
       <c r="H88" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -4527,7 +4527,7 @@
       </c>
       <c r="H89" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -4561,7 +4561,7 @@
       </c>
       <c r="H90" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -4587,7 +4587,7 @@
       <c r="G91" s="8"/>
       <c r="H91" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -4621,7 +4621,7 @@
       </c>
       <c r="H92" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -4655,7 +4655,7 @@
       </c>
       <c r="H93" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -4689,7 +4689,7 @@
       </c>
       <c r="H94" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -4723,7 +4723,7 @@
       </c>
       <c r="H95" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -4757,7 +4757,7 @@
       </c>
       <c r="H96" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -4791,7 +4791,7 @@
       </c>
       <c r="H97" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -4825,7 +4825,7 @@
       </c>
       <c r="H98" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -4859,7 +4859,7 @@
       </c>
       <c r="H99" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -4889,7 +4889,7 @@
       </c>
       <c r="H100" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -4923,7 +4923,7 @@
       </c>
       <c r="H101" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -4957,7 +4957,7 @@
       </c>
       <c r="H102" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -4983,7 +4983,7 @@
       <c r="G103" s="8"/>
       <c r="H103" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -5009,7 +5009,7 @@
       <c r="G104" s="8"/>
       <c r="H104" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -5039,7 +5039,7 @@
       </c>
       <c r="H105" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -5065,7 +5065,7 @@
       <c r="G106" s="8"/>
       <c r="H106" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -5091,7 +5091,7 @@
       <c r="G107" s="8"/>
       <c r="H107" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -5125,7 +5125,7 @@
       </c>
       <c r="H108" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -5159,7 +5159,7 @@
       </c>
       <c r="H109" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -5189,7 +5189,7 @@
       </c>
       <c r="H110" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -5219,7 +5219,7 @@
       </c>
       <c r="H111" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -5249,7 +5249,7 @@
       </c>
       <c r="H112" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -5283,7 +5283,7 @@
       </c>
       <c r="H113" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -5313,7 +5313,7 @@
       </c>
       <c r="H114" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E .dyr</t>
+          <t xml:space="preserve">PSS/E + PSLF</t>
         </is>
       </c>
     </row>
@@ -5343,11 +5343,11 @@
       </c>
       <c r="H115" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E .dyr</t>
-        </is>
-      </c>
-    </row>
-    <row r="116" ht="30.0" customHeight="1">
+          <t xml:space="preserve">PSS/E</t>
+        </is>
+      </c>
+    </row>
+    <row r="116" ht="43.0" customHeight="1">
       <c r="A116" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Generators</t>
@@ -5376,12 +5376,12 @@
       </c>
       <c r="G116" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E .dyr -- REGC_A: a current source (REGCA1) | REGC_B: a voltage source behind ZSORCE R + jX, for weak grids (REGCBU1; ZSORCE X its Xe) -- PV, BESS, WT4 (blank = REGC_A)</t>
+          <t xml:space="preserve">REGC_A: a current source, the standard | REGC_B: a voltage source behind ZSORCE R + jX, for weak grids (ZSORCE X its Xe) -- PV, BESS, WT4; .dyr REGCA1 / REGCBU1, .dyd regc_a / regc_b (blank = REGC_A)</t>
         </is>
       </c>
       <c r="H116" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E .dyr</t>
+          <t xml:space="preserve">PSS/E + PSLF</t>
         </is>
       </c>
     </row>
@@ -5414,12 +5414,12 @@
       </c>
       <c r="G117" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E .dyr -- REEC_A: PV, WT | REEC_C: BESS | REEC_D: PV, BESS, WT4 (blank = REEC_A, BESS REEC_C)</t>
+          <t xml:space="preserve">REEC_A: PV, WT | REEC_C: BESS (state of charge) | REEC_D: PV, BESS, WT4, the newest (voltage-dependent limits, momentary cessation) -- .dyr and .dyd alike (blank = REEC_A, BESS REEC_C)</t>
         </is>
       </c>
       <c r="H117" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E .dyr</t>
+          <t xml:space="preserve">PSS/E + PSLF</t>
         </is>
       </c>
     </row>
@@ -5667,7 +5667,7 @@
       </c>
       <c r="H125" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -5697,7 +5697,7 @@
       </c>
       <c r="H126" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -5731,7 +5731,7 @@
       </c>
       <c r="H127" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -5761,7 +5761,7 @@
       </c>
       <c r="H128" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -5795,7 +5795,7 @@
       </c>
       <c r="H129" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -5825,7 +5825,7 @@
       </c>
       <c r="H130" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -5851,7 +5851,7 @@
       <c r="G131" s="8"/>
       <c r="H131" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -5889,7 +5889,7 @@
       </c>
       <c r="H132" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -5919,7 +5919,7 @@
       </c>
       <c r="H133" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -5949,7 +5949,7 @@
       </c>
       <c r="H134" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -5983,7 +5983,7 @@
       </c>
       <c r="H135" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -6017,7 +6017,7 @@
       </c>
       <c r="H136" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -6051,7 +6051,7 @@
       </c>
       <c r="H137" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -6085,7 +6085,7 @@
       </c>
       <c r="H138" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -6129,7 +6129,7 @@
       </c>
       <c r="H140" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -6163,7 +6163,7 @@
       </c>
       <c r="H141" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -6193,7 +6193,7 @@
       </c>
       <c r="H142" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -6223,7 +6223,7 @@
       </c>
       <c r="H143" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -6253,7 +6253,7 @@
       </c>
       <c r="H144" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -6283,7 +6283,7 @@
       </c>
       <c r="H145" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -6327,7 +6327,7 @@
       </c>
       <c r="H147" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -6357,7 +6357,7 @@
       </c>
       <c r="H148" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -6405,7 +6405,7 @@
       </c>
       <c r="H150" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -6435,7 +6435,7 @@
       </c>
       <c r="H151" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -6465,7 +6465,7 @@
       </c>
       <c r="H152" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -6495,7 +6495,7 @@
       </c>
       <c r="H153" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -6521,7 +6521,7 @@
       <c r="G154" s="8"/>
       <c r="H154" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -6565,7 +6565,7 @@
       </c>
       <c r="H156" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -6599,7 +6599,7 @@
       </c>
       <c r="H157" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -6633,7 +6633,7 @@
       </c>
       <c r="H158" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -6667,7 +6667,7 @@
       </c>
       <c r="H159" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -6701,7 +6701,7 @@
       </c>
       <c r="H160" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -6735,7 +6735,7 @@
       </c>
       <c r="H161" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -6769,7 +6769,7 @@
       </c>
       <c r="H162" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -6803,7 +6803,7 @@
       </c>
       <c r="H163" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -6837,7 +6837,7 @@
       </c>
       <c r="H164" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -6881,7 +6881,7 @@
       </c>
       <c r="H166" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -6915,7 +6915,7 @@
       </c>
       <c r="H167" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -6949,7 +6949,7 @@
       </c>
       <c r="H168" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -6993,7 +6993,7 @@
       </c>
       <c r="H170" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E .dyr</t>
+          <t xml:space="preserve">PSS/E + PSLF</t>
         </is>
       </c>
     </row>
@@ -7023,7 +7023,7 @@
       </c>
       <c r="H171" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E .dyr</t>
+          <t xml:space="preserve">PSS/E + PSLF</t>
         </is>
       </c>
     </row>
@@ -7053,7 +7053,7 @@
       </c>
       <c r="H172" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E .dyr</t>
+          <t xml:space="preserve">PSS/E + PSLF</t>
         </is>
       </c>
     </row>
@@ -7079,7 +7079,7 @@
       <c r="G173" s="8"/>
       <c r="H173" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E .dyr</t>
+          <t xml:space="preserve">PSS/E + PSLF</t>
         </is>
       </c>
     </row>
@@ -7127,7 +7127,7 @@
       </c>
       <c r="H175" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E .dyr</t>
+          <t xml:space="preserve">PSS/E</t>
         </is>
       </c>
     </row>
@@ -7157,7 +7157,7 @@
       </c>
       <c r="H176" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E .dyr</t>
+          <t xml:space="preserve">PSS/E</t>
         </is>
       </c>
     </row>
@@ -19832,7 +19832,7 @@
       </c>
       <c r="G3" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -19865,7 +19865,7 @@
       </c>
       <c r="G4" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -19896,7 +19896,7 @@
       </c>
       <c r="G5" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -19929,7 +19929,7 @@
       </c>
       <c r="G6" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -19962,7 +19962,7 @@
       </c>
       <c r="G7" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -19995,7 +19995,7 @@
       </c>
       <c r="G8" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -20028,7 +20028,7 @@
       </c>
       <c r="G9" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSLF</t>
         </is>
       </c>
     </row>
@@ -20061,7 +20061,7 @@
       </c>
       <c r="G10" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSLF</t>
         </is>
       </c>
     </row>
@@ -20092,7 +20092,7 @@
       </c>
       <c r="G11" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -20115,7 +20115,7 @@
       </c>
       <c r="G12" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -20155,7 +20155,7 @@
       <c r="F14" s="2"/>
       <c r="G14" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -20180,7 +20180,7 @@
       </c>
       <c r="G15" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -20207,7 +20207,7 @@
       </c>
       <c r="G16" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -20226,7 +20226,7 @@
       <c r="F17" s="2"/>
       <c r="G17" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -20255,7 +20255,7 @@
       </c>
       <c r="G18" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -20280,7 +20280,7 @@
       </c>
       <c r="G19" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -20305,7 +20305,7 @@
       </c>
       <c r="G20" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -20330,7 +20330,7 @@
       </c>
       <c r="G21" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -20370,7 +20370,7 @@
       </c>
       <c r="G23" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -20403,7 +20403,7 @@
       </c>
       <c r="G24" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -20436,7 +20436,7 @@
       </c>
       <c r="G25" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -20467,7 +20467,7 @@
       </c>
       <c r="G26" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -20498,7 +20498,7 @@
       </c>
       <c r="G27" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -20529,7 +20529,7 @@
       </c>
       <c r="G28" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -20554,7 +20554,7 @@
       </c>
       <c r="G29" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -20579,7 +20579,7 @@
       </c>
       <c r="G30" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -20600,7 +20600,7 @@
       <c r="F31" s="2"/>
       <c r="G31" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -20621,7 +20621,7 @@
       <c r="F32" s="2"/>
       <c r="G32" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -20648,7 +20648,7 @@
       </c>
       <c r="G33" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -20679,7 +20679,7 @@
       </c>
       <c r="G34" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -20721,7 +20721,7 @@
       </c>
       <c r="G36" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -20752,7 +20752,7 @@
       </c>
       <c r="G37" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -20783,7 +20783,7 @@
       </c>
       <c r="G38" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -20806,7 +20806,7 @@
       </c>
       <c r="G39" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -20837,7 +20837,7 @@
       </c>
       <c r="G40" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -20866,7 +20866,7 @@
       </c>
       <c r="G41" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E + PSCAD</t>
+          <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
         </is>
       </c>
     </row>
@@ -20912,7 +20912,7 @@
       </c>
       <c r="G43" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E .dyr</t>
+          <t xml:space="preserve">PSS/E + PSLF</t>
         </is>
       </c>
     </row>
@@ -20945,7 +20945,7 @@
       </c>
       <c r="G44" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E .dyr</t>
+          <t xml:space="preserve">PSS/E</t>
         </is>
       </c>
     </row>
@@ -22748,12 +22748,12 @@
       </c>
       <c r="AF2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E .dyr -- REGC_A: a current source (REGCA1) | REGC_B: a voltage source behind ZSORCE R + jX, for weak grids (REGCBU1; ZSORCE X its Xe) -- PV, BESS, WT4 (blank = REGC_A)</t>
+          <t xml:space="preserve">REGC_A: a current source, the standard | REGC_B: a voltage source behind ZSORCE R + jX, for weak grids (ZSORCE X its Xe) -- PV, BESS, WT4; .dyr REGCA1 / REGCBU1, .dyd regc_a / regc_b (blank = REGC_A)</t>
         </is>
       </c>
       <c r="AG2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E .dyr -- REEC_A: PV, WT | REEC_C: BESS | REEC_D: PV, BESS, WT4 (blank = REEC_A, BESS REEC_C)</t>
+          <t xml:space="preserve">REEC_A: PV, WT | REEC_C: BESS (state of charge) | REEC_D: PV, BESS, WT4, the newest (voltage-dependent limits, momentary cessation) -- .dyr and .dyd alike (blank = REEC_A, BESS REEC_C)</t>
         </is>
       </c>
       <c r="AH2" s="2" t="inlineStr">

</xml_diff>

<commit_message>
smib_build GUI: edit each UDM's PSCAD parameters, read from its definition
The PSCAD_Params tab lists every parameter of each generator's vendor
model, read from its definition in the OEM's file -- name, meaning, type,
unit, range, choices, default (a copied component: its own values) -- a
column per generator. Double-click to change one: a choice from its list,
a number checked against its range, a {KEY} placeholder; clear it to go
back to the model's own. Changes are PSCAD_Params rows, set on the UDM
when the PSCAD case is built.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BGsNUhFmVX23f8qnP53zUv
</commit_message>
<xml_diff>
--- a/smib/SMIB_INPUT_TEMPLATE.xlsx
+++ b/smib/SMIB_INPUT_TEMPLATE.xlsx
@@ -225,7 +225,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="10" t="inlineStr">
         <is>
-          <t xml:space="preserve">PSS/E (.raw, .dyr) and PSCAD (.pscx) models of a plant from one workbook -- smib_build.py, 2026-10-15</t>
+          <t xml:space="preserve">PSS/E (.raw, .dyr) and PSCAD (.pscx) models of a plant from one workbook -- smib_build.py, 2026-10-16</t>
         </is>
       </c>
       <c r="B2" s="10"/>
@@ -813,7 +813,7 @@
         </is>
       </c>
     </row>
-    <row r="52" ht="69.0" customHeight="1">
+    <row r="52" ht="95.0" customHeight="1">
       <c r="A52" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">PSCAD_Params</t>
@@ -821,7 +821,7 @@
       </c>
       <c r="B52" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Parameters of each generator's vendor PSCAD model (UDM), as PSCAD takes them. Filled in for each inverter it stands for (DETAILED: each node): {UNITS} units, {MVA} their MVA, {P_MW} {Q_MVAR} their P and Q where it connects, {P_PU} {Q_PU} on {MVA}, {UNIT_MVA} {UNIT_P_MW} {UNIT_Q_MVAR} one unit's, {V_PU} {V_KV} {KV} {ANGLE} the voltage there, its base and PSCAD angle, {P_INV_MW} {Q_INV_MVAR} {V_INV_PU} at the inverters' own terminals (a UDM on the MV side), {FREQ} -- e.g. Ninv = {UNITS}, Vt0 = {V_PU}.</t>
+          <t xml:space="preserve">Parameters of each generator's vendor PSCAD model (UDM), as PSCAD takes them. Filled in for each inverter it stands for (DETAILED: each node): {UNITS} units, {MVA} their MVA, {P_MW} {Q_MVAR} their P and Q where it connects, {P_PU} {Q_PU} on {MVA}, {UNIT_MVA} {UNIT_P_MW} {UNIT_Q_MVAR} one unit's, {V_PU} {V_KV} {KV} {ANGLE} the voltage there, its base and PSCAD angle, {P_INV_MW} {Q_INV_MVAR} {V_INV_PU} at the inverters' own terminals (a UDM on the MV side), {FREQ} -- e.g. Ninv = {UNITS}, Vt0 = {V_PU}. In the GUI, the PSCAD_Params tab shows each vendor model's parameters, read from its definition in its file, a column per generator: double-click one to change it (a choice from its list), clear it to go back to the model's own.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
smib_build GUI: change settings inside a UDM -- its controller, its signals
PSCAD_Params tab, Definition drop-down: the UDM itself, each part inside
its definition made from the OEM file's own definitions (Controller4 ...,
at any depth, its settings as that part has them), the signals set inside
it by a constant, slider or switch wired to their data label (FreqDroop,
RampRate ...), and on request the library's parts too. A change is a
PSCAD_Params row Part/Setting (Controller4/UFLevel1) or Source/Value
(var_switch#5/Value): the build script writes it into a copy of the
definition of the generator's own (<definition>_<generator>), added to the
case in its place; a UDM to be copied by component ID is then made from
its definition, its own values set on it.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BGsNUhFmVX23f8qnP53zUv
</commit_message>
<xml_diff>
--- a/smib/SMIB_INPUT_TEMPLATE.xlsx
+++ b/smib/SMIB_INPUT_TEMPLATE.xlsx
@@ -813,7 +813,7 @@
         </is>
       </c>
     </row>
-    <row r="52" ht="95.0" customHeight="1">
+    <row r="52" ht="134.0" customHeight="1">
       <c r="A52" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">PSCAD_Params</t>
@@ -821,7 +821,7 @@
       </c>
       <c r="B52" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Parameters of each generator's vendor PSCAD model (UDM), as PSCAD takes them. Filled in for each inverter it stands for (DETAILED: each node): {UNITS} units, {MVA} their MVA, {P_MW} {Q_MVAR} their P and Q where it connects, {P_PU} {Q_PU} on {MVA}, {UNIT_MVA} {UNIT_P_MW} {UNIT_Q_MVAR} one unit's, {V_PU} {V_KV} {KV} {ANGLE} the voltage there, its base and PSCAD angle, {P_INV_MW} {Q_INV_MVAR} {V_INV_PU} at the inverters' own terminals (a UDM on the MV side), {FREQ} -- e.g. Ninv = {UNITS}, Vt0 = {V_PU}. In the GUI, the PSCAD_Params tab shows each vendor model's parameters, read from its definition in its file, a column per generator: double-click one to change it (a choice from its list), clear it to go back to the model's own.</t>
+          <t xml:space="preserve">Parameters of each generator's vendor PSCAD model (UDM), as PSCAD takes them. Filled in for each inverter it stands for (DETAILED: each node): {UNITS} units, {MVA} their MVA, {P_MW} {Q_MVAR} their P and Q where it connects, {P_PU} {Q_PU} on {MVA}, {UNIT_MVA} {UNIT_P_MW} {UNIT_Q_MVAR} one unit's, {V_PU} {V_KV} {KV} {ANGLE} the voltage there, its base and PSCAD angle, {P_INV_MW} {Q_INV_MVAR} {V_INV_PU} at the inverters' own terminals (a UDM on the MV side), {FREQ} -- e.g. Ninv = {UNITS}, Vt0 = {V_PU}. In the GUI, the PSCAD_Params tab shows each vendor model's parameters, read from its definition in its file, a column per generator -- and, picked under Definition, those of the parts inside it (its controller ...) and its signals set by a constant, slider or switch (FreqDroop ...): double-click one to change it (a choice from its list), clear it to go back to the model's own. A part's setting is Part/Setting (Controller4/UFLevel1), a signal's its source's Value (var_switch#5/Value); they change a copy of the definition of the generator's own.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Plant Model Builder: gen-tie and MPT ties in feet; Q from MVA and P
- The gen-tie's and an MPT's own tie length: blank unit ft (drop-down ft,
  kft, m, km, mi); the example's gen-tie 16400 ft.
- Unit Qmax blank: the MVA left at full P, sqrt(Unit MVA^2 - P^2), when
  Unit MVA is given (Unit PF given: from it, as before); no Q left at full
  P is CHECKed. In the GUI, a Unit Qmax (and Qmin) on that circle follows a
  change of Unit MVA or P.
- What blanks meant when a file was saved is kept: projects carry a format
  mark, workbooks are read by their notes; older ones get km and Unit PF
  0.95 written in, said.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BGsNUhFmVX23f8qnP53zUv
</commit_message>
<xml_diff>
--- a/smib/SMIB_INPUT_TEMPLATE.xlsx
+++ b/smib/SMIB_INPUT_TEMPLATE.xlsx
@@ -2350,17 +2350,17 @@
       <c r="D24" s="8"/>
       <c r="E24" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">km</t>
+          <t xml:space="preserve">ft</t>
         </is>
       </c>
       <c r="F24" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">km | mi | kft | m | ft</t>
+          <t xml:space="preserve">ft | kft | m | km | mi</t>
         </is>
       </c>
       <c r="G24" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">km, mi, kft, m, ft (blank = km)</t>
+          <t xml:space="preserve">ft, kft, m, km, mi (blank = ft)</t>
         </is>
       </c>
       <c r="H24" s="13" t="inlineStr">
@@ -4298,13 +4298,21 @@
         </is>
       </c>
       <c r="D81" s="8"/>
-      <c r="E81" s="8"/>
+      <c r="E81" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ft</t>
+        </is>
+      </c>
       <c r="F81" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">km | mi | kft | m | ft</t>
-        </is>
-      </c>
-      <c r="G81" s="8"/>
+          <t xml:space="preserve">ft | kft | m | km | mi</t>
+        </is>
+      </c>
+      <c r="G81" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">blank = ft</t>
+        </is>
+      </c>
       <c r="H81" s="13" t="inlineStr">
         <is>
           <t xml:space="preserve">PSS/E + PSLF + PSCAD</t>
@@ -4751,7 +4759,7 @@
         </is>
       </c>
     </row>
-    <row r="96" ht="17.0" customHeight="1">
+    <row r="96" ht="43.0" customHeight="1">
       <c r="A96" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Generators</t>
@@ -4770,13 +4778,13 @@
       <c r="D96" s="8"/>
       <c r="E96" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">from Unit PF</t>
+          <t xml:space="preserve">the MVA left at full P: sqrt(Unit MVA^2 - Pmax^2</t>
         </is>
       </c>
       <c r="F96" s="8"/>
       <c r="G96" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">blank = from Unit PF</t>
+          <t xml:space="preserve">blank = the MVA left at full P: sqrt(Unit MVA^2 - Pmax^2), or from Unit PF</t>
         </is>
       </c>
       <c r="H96" s="13" t="inlineStr">
@@ -4819,7 +4827,7 @@
         </is>
       </c>
     </row>
-    <row r="98" ht="17.0" customHeight="1">
+    <row r="98" ht="30.0" customHeight="1">
       <c r="A98" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">Generators</t>
@@ -4838,13 +4846,13 @@
       <c r="D98" s="8"/>
       <c r="E98" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">0.95</t>
+          <t xml:space="preserve">0.95 where Unit MVA is blank too</t>
         </is>
       </c>
       <c r="F98" s="8"/>
       <c r="G98" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q at Pmax when Qmax is blank (blank = 0.95)</t>
+          <t xml:space="preserve">Q at Pmax when Qmax is blank, instead of from Unit MVA (blank = 0.95 where Unit MVA is blank too)</t>
         </is>
       </c>
       <c r="H98" s="13" t="inlineStr">
@@ -20742,7 +20750,7 @@
         </is>
       </c>
       <c r="B23" s="3">
-        <v>5.0</v>
+        <v>16400</v>
       </c>
       <c r="C23" s="8"/>
       <c r="D23" s="8" t="inlineStr">
@@ -20770,23 +20778,23 @@
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">km</t>
+          <t xml:space="preserve">ft</t>
         </is>
       </c>
       <c r="C24" s="8"/>
       <c r="D24" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">km</t>
+          <t xml:space="preserve">ft</t>
         </is>
       </c>
       <c r="E24" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">km | mi | kft | m | ft</t>
+          <t xml:space="preserve">ft | kft | m | km | mi</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">km, mi, kft, m, ft (blank = km)</t>
+          <t xml:space="preserve">ft, kft, m, km, mi (blank = ft)</t>
         </is>
       </c>
       <c r="G24" s="13" t="inlineStr">
@@ -21777,7 +21785,7 @@
       <formula1>"YES,NO"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B24">
-      <formula1>"km,mi,kft,m,ft"</formula1>
+      <formula1>"ft,kft,m,km,mi"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B25">
       <formula1>"km,mi,kft,m,ft"</formula1>
@@ -22127,7 +22135,11 @@
           <t xml:space="preserve">a line of its own from HV to this MPT (blank = none)</t>
         </is>
       </c>
-      <c r="Z2" s="2"/>
+      <c r="Z2" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">blank = ft</t>
+        </is>
+      </c>
       <c r="AA2" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">the length R, X, B are per (blank = km or mi, whichever matches a line of its kV)</t>
@@ -22848,7 +22860,7 @@
       <formula1>"2,3"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="Z3:Z500">
-      <formula1>"km,mi,kft,m,ft"</formula1>
+      <formula1>"ft,kft,m,km,mi"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="AA3:AA500">
       <formula1>"km,mi,kft,m,ft"</formula1>
@@ -23167,7 +23179,7 @@
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">blank = from Unit PF</t>
+          <t xml:space="preserve">blank = the MVA left at full P: sqrt(Unit MVA^2 - Pmax^2), or from Unit PF</t>
         </is>
       </c>
       <c r="J2" s="2" t="inlineStr">
@@ -23177,7 +23189,7 @@
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Q at Pmax when Qmax is blank (blank = 0.95)</t>
+          <t xml:space="preserve">Q at Pmax when Qmax is blank, instead of from Unit MVA (blank = 0.95 where Unit MVA is blank too)</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Plant Model Builder: defaults for a three-winding MPT
LV and TV MVA blank: the MVA shared out by the units on each winding (none
on the TV: MVA/2 on a split LV winding, MVA/3 a tertiary); Z HV-TV blank =
Z HV-LV, Z LV-TV blank = 1.8 x Z HV-LV (a split LV winding's), each on its
own base. The GUI's MPT page shows a blank cell's value in brackets (TV kV,
LV / TV MVA, Z HV-TV, Z LV-TV, MVA, Rate A / B / C, Windings). Files saved
before (format 3) keep their meaning: LV / TV MVA written in as the MPT's MVA.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BGsNUhFmVX23f8qnP53zUv
</commit_message>
<xml_diff>
--- a/smib/SMIB_INPUT_TEMPLATE.xlsx
+++ b/smib/SMIB_INPUT_TEMPLATE.xlsx
@@ -693,7 +693,7 @@
         </is>
       </c>
     </row>
-    <row r="42" ht="56.0" customHeight="1">
+    <row r="42" ht="82.0" customHeight="1">
       <c r="A42" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">MPT</t>
@@ -701,7 +701,7 @@
       </c>
       <c r="B42" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">One row per main power transformer; HV winding first. Three windings: TV kV, the three impedances and their bases. Parallel units: identical units in parallel. Tie: a line of its own from HV to it. MVA blank: the MVA of the units on it (Unit MVA x Units), following them -- the GUI's Size MPTs from the generators suggests a rating. Rate A, B, C: its normal and emergency ratings (PSS/E RATEA, RATEB, RATEC; PSLF rate1, rate2, rate3).</t>
+          <t xml:space="preserve">One row per main power transformer; HV winding first. Three windings: TV kV (blank: the LV's, a split LV winding), the LV and TV MVA (blank: the MVA shared out by the units on each), the three impedances (Z HV-TV blank: Z HV-LV; Z LV-TV blank: 1.8 x Z HV-LV, a split LV winding's) and their bases. Parallel units: identical units in parallel. Tie: a line of its own from HV to it. MVA blank: the MVA of the units on it (Unit MVA x Units), following them -- the GUI's Size MPTs from the generators suggests a rating. Rate A, B, C: its normal and emergency ratings (PSS/E RATEA, RATEB, RATEC; PSLF rate1, rate2, rate3).</t>
         </is>
       </c>
     </row>
@@ -3671,7 +3671,7 @@
         </is>
       </c>
     </row>
-    <row r="62" ht="17.0" customHeight="1">
+    <row r="62" ht="56.0" customHeight="1">
       <c r="A62" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">MPT</t>
@@ -3688,11 +3688,15 @@
         </is>
       </c>
       <c r="D62" s="8"/>
-      <c r="E62" s="8"/>
+      <c r="E62" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MVA x the LV units' share of the units on LV and TV -- none on TV: MVA</t>
+        </is>
+      </c>
       <c r="F62" s="8"/>
       <c r="G62" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 windings</t>
+          <t xml:space="preserve">3 windings (blank = MVA x the LV units' share of the units on LV and TV -- none on TV: MVA)</t>
         </is>
       </c>
       <c r="H62" s="13" t="inlineStr">
@@ -3701,7 +3705,7 @@
         </is>
       </c>
     </row>
-    <row r="63" ht="17.0" customHeight="1">
+    <row r="63" ht="56.0" customHeight="1">
       <c r="A63" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">MPT</t>
@@ -3718,11 +3722,15 @@
         </is>
       </c>
       <c r="D63" s="8"/>
-      <c r="E63" s="8"/>
+      <c r="E63" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">MVA x the TV units' share -- none on it: MVA/2 on a split LV winding (TV kV the LV's</t>
+        </is>
+      </c>
       <c r="F63" s="8"/>
       <c r="G63" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 windings</t>
+          <t xml:space="preserve">3 windings (blank = MVA x the TV units' share -- none on it: MVA/2 on a split LV winding (TV kV the LV's), MVA/3 a tertiary)</t>
         </is>
       </c>
       <c r="H63" s="13" t="inlineStr">
@@ -3880,11 +3888,15 @@
         </is>
       </c>
       <c r="D68" s="8"/>
-      <c r="E68" s="8"/>
+      <c r="E68" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Z HV-LV</t>
+        </is>
+      </c>
       <c r="F68" s="8"/>
       <c r="G68" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 windings</t>
+          <t xml:space="preserve">3 windings, on its base MVA (blank = Z HV-LV)</t>
         </is>
       </c>
       <c r="H68" s="13" t="inlineStr">
@@ -3893,7 +3905,7 @@
         </is>
       </c>
     </row>
-    <row r="69" ht="17.0" customHeight="1">
+    <row r="69" ht="30.0" customHeight="1">
       <c r="A69" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">MPT</t>
@@ -3910,11 +3922,15 @@
         </is>
       </c>
       <c r="D69" s="8"/>
-      <c r="E69" s="8"/>
+      <c r="E69" s="8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1.8 x Z HV-LV, a split LV winding's</t>
+        </is>
+      </c>
       <c r="F69" s="8"/>
       <c r="G69" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 windings</t>
+          <t xml:space="preserve">3 windings, on its base MVA (blank = 1.8 x Z HV-LV, a split LV winding's)</t>
         </is>
       </c>
       <c r="H69" s="13" t="inlineStr">
@@ -24893,12 +24909,12 @@
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 windings</t>
+          <t xml:space="preserve">3 windings (blank = MVA x the LV units' share of the units on LV and TV -- none on TV: MVA)</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 windings</t>
+          <t xml:space="preserve">3 windings (blank = MVA x the TV units' share -- none on it: MVA/2 on a split LV winding (TV kV the LV's), MVA/3 a tertiary)</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -24923,12 +24939,12 @@
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 windings</t>
+          <t xml:space="preserve">3 windings, on its base MVA (blank = Z HV-LV)</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">3 windings</t>
+          <t xml:space="preserve">3 windings, on its base MVA (blank = 1.8 x Z HV-LV, a split LV winding's)</t>
         </is>
       </c>
       <c r="O2" s="2" t="inlineStr">

</xml_diff>

<commit_message>
Plant Model Builder: cables in B per length
B per length (uS) comes before C on the Cables sheet, and the example cables
are given in B; C stays as the alternative (B = 2 pi f C). The GUI's Cables
page: a cable given by C shows its B in brackets, C to B turns every C into
B at the Plant's frequency, and the simple view hides C where no cable has
it. The models are unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BGsNUhFmVX23f8qnP53zUv
</commit_message>
<xml_diff>
--- a/smib/SMIB_INPUT_TEMPLATE.xlsx
+++ b/smib/SMIB_INPUT_TEMPLATE.xlsx
@@ -737,7 +737,7 @@
       </c>
       <c r="B45" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">Cable data per length (R, X in ohm; C in uF or B in uS) and the length unit they are per; Rate A, B, C one cable's ratings in MVA at its collector's kV (sqrt(3) x kV x amps / 1000): a section's x its parallel cables, a collector equivalent's its sections from the collector bus together.</t>
+          <t xml:space="preserve">Cable data per length (R, X in ohm; B in uS, or C in uF instead -- the GUI's C to B turns C into B) and the length unit they are per; Rate A, B, C one cable's ratings in MVA at its collector's kV (sqrt(3) x kV x amps / 1000): a section's x its parallel cables, a collector equivalent's its sections from the collector bus together.</t>
         </is>
       </c>
     </row>
@@ -6655,12 +6655,12 @@
       </c>
       <c r="B154" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">C per length</t>
+          <t xml:space="preserve">B per length</t>
         </is>
       </c>
       <c r="C154" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">c_per</t>
+          <t xml:space="preserve">b_per</t>
         </is>
       </c>
       <c r="D154" s="8"/>
@@ -6668,7 +6668,7 @@
       <c r="F154" s="8"/>
       <c r="G154" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">uF</t>
+          <t xml:space="preserve">uS, the charging susceptance (GUI: Cables page, C to B)</t>
         </is>
       </c>
       <c r="H154" s="13" t="inlineStr">
@@ -6685,12 +6685,12 @@
       </c>
       <c r="B155" s="12" t="inlineStr">
         <is>
-          <t xml:space="preserve">B per length</t>
+          <t xml:space="preserve">C per length</t>
         </is>
       </c>
       <c r="C155" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">b_per</t>
+          <t xml:space="preserve">c_per</t>
         </is>
       </c>
       <c r="D155" s="8"/>
@@ -6698,7 +6698,7 @@
       <c r="F155" s="8"/>
       <c r="G155" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">uS, instead of C</t>
+          <t xml:space="preserve">uF, instead of B (B = 2 pi f C)</t>
         </is>
       </c>
       <c r="H155" s="13" t="inlineStr">
@@ -28244,12 +28244,12 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
+          <t xml:space="preserve">B per length</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
           <t xml:space="preserve">C per length</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">B per length</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -28291,12 +28291,12 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">uF</t>
+          <t xml:space="preserve">uS, the charging susceptance (GUI: Cables page, C to B)</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">uS, instead of C</t>
+          <t xml:space="preserve">uF, instead of B (B = 2 pi f C)</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
@@ -28333,7 +28333,7 @@
         <v>0.105</v>
       </c>
       <c r="E3" s="3">
-        <v>0.39</v>
+        <v>147.027</v>
       </c>
       <c r="F3" s="3"/>
       <c r="G3" s="3"/>
@@ -28358,7 +28358,7 @@
         <v>0.118</v>
       </c>
       <c r="E4" s="3">
-        <v>0.3</v>
+        <v>113.097</v>
       </c>
       <c r="F4" s="3"/>
       <c r="G4" s="3"/>
@@ -28383,7 +28383,7 @@
         <v>0.133</v>
       </c>
       <c r="E5" s="3">
-        <v>0.22</v>
+        <v>82.938</v>
       </c>
       <c r="F5" s="3"/>
       <c r="G5" s="3"/>
@@ -28408,7 +28408,7 @@
         <v>0.148</v>
       </c>
       <c r="E6" s="3">
-        <v>0.17</v>
+        <v>64.0885</v>
       </c>
       <c r="F6" s="3"/>
       <c r="G6" s="3"/>

</xml_diff>

<commit_message>
Plant Model Builder: every length and value per length in ft; the plant's name shown in its box
A cable's values per length are per ft when its Length unit is blank (files
saved before: km, written in and said); a gen-tie's or MPT tie's blank
'values per' is ft, kft, km or mi, whichever matches a line of its kV (ft
first). The example's cables and gen-tie are per ft, the report gives
lengths in ft, and a cable whose X is no cable's in its unit is named with
the unit its values look per. The GUI's Plant page: All lengths in ft turns
the gen-tie, the MPT ties, the cables and the feeders into ft, the same
lines; a blank Name shows the name from the generators in its box, in
grey, and the window title follows it. The models are unchanged.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BGsNUhFmVX23f8qnP53zUv
</commit_message>
<xml_diff>
--- a/smib/SMIB_INPUT_TEMPLATE.xlsx
+++ b/smib/SMIB_INPUT_TEMPLATE.xlsx
@@ -2392,17 +2392,17 @@
       <c r="D25" s="8"/>
       <c r="E25" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">km or mi, whichever matches a line of the POI kV</t>
+          <t xml:space="preserve">ft, kft, km or mi, whichever matches a line of the POI kV</t>
         </is>
       </c>
       <c r="F25" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">km | mi | kft | m | ft</t>
+          <t xml:space="preserve">ft | kft | m | km | mi</t>
         </is>
       </c>
       <c r="G25" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">the length R, X, B, C below are per: km, mi, kft, m, ft (blank = km or mi, whichever matches a line of the POI kV)</t>
+          <t xml:space="preserve">the length R, X, B, C below are per: ft, kft, m, km, mi (blank = ft, kft, km or mi, whichever matches a line of the POI kV)</t>
         </is>
       </c>
       <c r="H25" s="13" t="inlineStr">
@@ -4339,7 +4339,7 @@
         </is>
       </c>
     </row>
-    <row r="82" ht="30.0" customHeight="1">
+    <row r="82" ht="43.0" customHeight="1">
       <c r="A82" s="8" t="inlineStr">
         <is>
           <t xml:space="preserve">MPT</t>
@@ -4358,17 +4358,17 @@
       <c r="D82" s="8"/>
       <c r="E82" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">km or mi, whichever matches a line of its kV</t>
+          <t xml:space="preserve">ft, kft, km or mi, whichever matches a line of its kV</t>
         </is>
       </c>
       <c r="F82" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">km | mi | kft | m | ft</t>
+          <t xml:space="preserve">ft | kft | m | km | mi</t>
         </is>
       </c>
       <c r="G82" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">the length R, X, B are per (blank = km or mi, whichever matches a line of its kV)</t>
+          <t xml:space="preserve">the length R, X, B are per (blank = ft, kft, km or mi, whichever matches a line of its kV)</t>
         </is>
       </c>
       <c r="H82" s="13" t="inlineStr">
@@ -6568,17 +6568,17 @@
       <c r="D151" s="8"/>
       <c r="E151" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">km</t>
+          <t xml:space="preserve">ft</t>
         </is>
       </c>
       <c r="F151" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">km | mi | kft | m | ft</t>
+          <t xml:space="preserve">ft | kft | m | km | mi</t>
         </is>
       </c>
       <c r="G151" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">the values are per (blank = km)</t>
+          <t xml:space="preserve">the values are per (blank = ft)</t>
         </is>
       </c>
       <c r="H151" s="13" t="inlineStr">
@@ -23678,23 +23678,23 @@
       </c>
       <c r="B25" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">km</t>
+          <t xml:space="preserve">ft</t>
         </is>
       </c>
       <c r="C25" s="8"/>
       <c r="D25" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">km or mi, whichever matches a line of the POI kV</t>
+          <t xml:space="preserve">ft, kft, km or mi, whichever matches a line of the POI kV</t>
         </is>
       </c>
       <c r="E25" s="8" t="inlineStr">
         <is>
-          <t xml:space="preserve">km | mi | kft | m | ft</t>
+          <t xml:space="preserve">ft | kft | m | km | mi</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">the length R, X, B, C below are per: km, mi, kft, m, ft (blank = km or mi, whichever matches a line of the POI kV)</t>
+          <t xml:space="preserve">the length R, X, B, C below are per: ft, kft, m, km, mi (blank = ft, kft, km or mi, whichever matches a line of the POI kV)</t>
         </is>
       </c>
       <c r="G25" s="13" t="inlineStr">
@@ -23710,7 +23710,7 @@
         </is>
       </c>
       <c r="B26" s="3">
-        <v>0.072</v>
+        <v>2.19456e-05</v>
       </c>
       <c r="C26" s="8" t="inlineStr">
         <is>
@@ -23741,7 +23741,7 @@
         </is>
       </c>
       <c r="B27" s="3">
-        <v>0.495</v>
+        <v>0.000150876</v>
       </c>
       <c r="C27" s="8" t="inlineStr">
         <is>
@@ -23772,7 +23772,7 @@
         </is>
       </c>
       <c r="B28" s="3">
-        <v>3.35</v>
+        <v>0.00102108</v>
       </c>
       <c r="C28" s="8" t="inlineStr">
         <is>
@@ -24655,7 +24655,7 @@
       <formula1>"ft,kft,m,km,mi"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B25">
-      <formula1>"km,mi,kft,m,ft"</formula1>
+      <formula1>"ft,kft,m,km,mi"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B36">
       <formula1>"Q,PF,V"</formula1>
@@ -25009,7 +25009,7 @@
       </c>
       <c r="AA2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">the length R, X, B are per (blank = km or mi, whichever matches a line of its kV)</t>
+          <t xml:space="preserve">the length R, X, B are per (blank = ft, kft, km or mi, whichever matches a line of its kV)</t>
         </is>
       </c>
       <c r="AB2" s="2" t="inlineStr">
@@ -25730,7 +25730,7 @@
       <formula1>"ft,kft,m,km,mi"</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="AA3:AA500">
-      <formula1>"km,mi,kft,m,ft"</formula1>
+      <formula1>"ft,kft,m,km,mi"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>
@@ -28276,7 +28276,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">the values are per (blank = km)</t>
+          <t xml:space="preserve">the values are per (blank = ft)</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
@@ -28323,17 +28323,17 @@
       </c>
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">km</t>
+          <t xml:space="preserve">ft</t>
         </is>
       </c>
       <c r="C3" s="3">
-        <v>0.046</v>
+        <v>1.40208e-05</v>
       </c>
       <c r="D3" s="3">
-        <v>0.105</v>
+        <v>3.2004e-05</v>
       </c>
       <c r="E3" s="3">
-        <v>147.027</v>
+        <v>0.0448138296</v>
       </c>
       <c r="F3" s="3"/>
       <c r="G3" s="3"/>
@@ -28348,17 +28348,17 @@
       </c>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">km</t>
+          <t xml:space="preserve">ft</t>
         </is>
       </c>
       <c r="C4" s="3">
-        <v>0.09</v>
+        <v>2.7432e-05</v>
       </c>
       <c r="D4" s="3">
-        <v>0.118</v>
+        <v>3.59664e-05</v>
       </c>
       <c r="E4" s="3">
-        <v>113.097</v>
+        <v>0.0344719656</v>
       </c>
       <c r="F4" s="3"/>
       <c r="G4" s="3"/>
@@ -28373,17 +28373,17 @@
       </c>
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">km</t>
+          <t xml:space="preserve">ft</t>
         </is>
       </c>
       <c r="C5" s="3">
-        <v>0.201</v>
+        <v>6.12648e-05</v>
       </c>
       <c r="D5" s="3">
-        <v>0.133</v>
+        <v>4.05384e-05</v>
       </c>
       <c r="E5" s="3">
-        <v>82.938</v>
+        <v>0.0252795024</v>
       </c>
       <c r="F5" s="3"/>
       <c r="G5" s="3"/>
@@ -28398,17 +28398,17 @@
       </c>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">km</t>
+          <t xml:space="preserve">ft</t>
         </is>
       </c>
       <c r="C6" s="3">
-        <v>0.404</v>
+        <v>0.0001231392</v>
       </c>
       <c r="D6" s="3">
-        <v>0.148</v>
+        <v>4.51104e-05</v>
       </c>
       <c r="E6" s="3">
-        <v>64.0885</v>
+        <v>0.0195341748</v>
       </c>
       <c r="F6" s="3"/>
       <c r="G6" s="3"/>
@@ -28594,7 +28594,7 @@
   </sheetData>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B3:B500">
-      <formula1>"km,mi,kft,m,ft"</formula1>
+      <formula1>"ft,kft,m,km,mi"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.4" right="0.4" top="0.5" bottom="0.5" header="0.3" footer="0.3"/>

</xml_diff>